<commit_message>
Definicion de funciones en R
</commit_message>
<xml_diff>
--- a/Inputs.xlsx
+++ b/Inputs.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30110"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ausenco.sharepoint.com/sites/tg-santiago-waterresources/Shared Documents/General/Hidrología - Hidráulica/Biblioteca/Repositorio/Planillas/Tiempo concentracion/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Codigos\HU_SCS\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="11" documentId="13_ncr:1_{32D9CF2F-367B-4BF6-899F-E31136CAE2F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5F11900D-AF93-4AF4-8EC8-327C24A2954B}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-24630" yWindow="2760" windowWidth="21600" windowHeight="11235" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Info Cuencas" sheetId="1" r:id="rId1"/>
@@ -96,7 +96,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -516,15 +516,15 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:R20"/>
-  <sheetFormatPr defaultRowHeight="14.45"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="14.7109375" customWidth="1"/>
-    <col min="2" max="11" width="12.7109375" customWidth="1"/>
-    <col min="13" max="17" width="12.7109375" customWidth="1"/>
-    <col min="18" max="18" width="14.28515625" customWidth="1"/>
+    <col min="1" max="1" width="14.6640625" customWidth="1"/>
+    <col min="2" max="11" width="12.6640625" customWidth="1"/>
+    <col min="13" max="17" width="12.6640625" customWidth="1"/>
+    <col min="18" max="18" width="14.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" ht="55.15" customHeight="1">
+    <row r="1" spans="1:18" ht="55.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="7" t="s">
         <v>0</v>
       </c>
@@ -578,7 +578,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="2" spans="1:18">
+    <row r="2" spans="1:18" x14ac:dyDescent="0.3">
       <c r="B2" s="4"/>
       <c r="D2" s="5"/>
       <c r="E2" s="5"/>
@@ -609,7 +609,7 @@
         <v/>
       </c>
     </row>
-    <row r="3" spans="1:18">
+    <row r="3" spans="1:18" x14ac:dyDescent="0.3">
       <c r="B3" s="4"/>
       <c r="D3" s="5"/>
       <c r="E3" s="5"/>
@@ -640,7 +640,7 @@
         <v/>
       </c>
     </row>
-    <row r="4" spans="1:18">
+    <row r="4" spans="1:18" x14ac:dyDescent="0.3">
       <c r="B4" s="4"/>
       <c r="D4" s="5"/>
       <c r="E4" s="5"/>
@@ -669,7 +669,7 @@
         <v/>
       </c>
     </row>
-    <row r="5" spans="1:18">
+    <row r="5" spans="1:18" x14ac:dyDescent="0.3">
       <c r="B5" s="4"/>
       <c r="D5" s="5"/>
       <c r="E5" s="5"/>
@@ -698,7 +698,7 @@
         <v/>
       </c>
     </row>
-    <row r="6" spans="1:18">
+    <row r="6" spans="1:18" x14ac:dyDescent="0.3">
       <c r="B6" s="4"/>
       <c r="D6" s="5"/>
       <c r="E6" s="5"/>
@@ -727,7 +727,7 @@
         <v/>
       </c>
     </row>
-    <row r="7" spans="1:18">
+    <row r="7" spans="1:18" x14ac:dyDescent="0.3">
       <c r="B7" s="4"/>
       <c r="D7" s="5"/>
       <c r="E7" s="5"/>
@@ -756,7 +756,7 @@
         <v/>
       </c>
     </row>
-    <row r="8" spans="1:18">
+    <row r="8" spans="1:18" x14ac:dyDescent="0.3">
       <c r="B8" s="4"/>
       <c r="D8" s="5"/>
       <c r="E8" s="5"/>
@@ -785,7 +785,7 @@
         <v/>
       </c>
     </row>
-    <row r="9" spans="1:18">
+    <row r="9" spans="1:18" x14ac:dyDescent="0.3">
       <c r="B9" s="4"/>
       <c r="D9" s="5"/>
       <c r="E9" s="5"/>
@@ -814,7 +814,7 @@
         <v/>
       </c>
     </row>
-    <row r="10" spans="1:18">
+    <row r="10" spans="1:18" x14ac:dyDescent="0.3">
       <c r="B10" s="4"/>
       <c r="D10" s="5"/>
       <c r="E10" s="5"/>
@@ -843,7 +843,7 @@
         <v/>
       </c>
     </row>
-    <row r="11" spans="1:18">
+    <row r="11" spans="1:18" x14ac:dyDescent="0.3">
       <c r="B11" s="4"/>
       <c r="D11" s="5"/>
       <c r="E11" s="5"/>
@@ -872,7 +872,7 @@
         <v/>
       </c>
     </row>
-    <row r="12" spans="1:18">
+    <row r="12" spans="1:18" x14ac:dyDescent="0.3">
       <c r="B12" s="4"/>
       <c r="D12" s="5"/>
       <c r="E12" s="5"/>
@@ -901,7 +901,7 @@
         <v/>
       </c>
     </row>
-    <row r="13" spans="1:18">
+    <row r="13" spans="1:18" x14ac:dyDescent="0.3">
       <c r="B13" s="4"/>
       <c r="D13" s="5"/>
       <c r="E13" s="5"/>
@@ -930,7 +930,7 @@
         <v/>
       </c>
     </row>
-    <row r="14" spans="1:18">
+    <row r="14" spans="1:18" x14ac:dyDescent="0.3">
       <c r="B14" s="4"/>
       <c r="D14" s="5"/>
       <c r="E14" s="5"/>
@@ -959,10 +959,10 @@
         <v/>
       </c>
     </row>
-    <row r="19" spans="8:8">
+    <row r="19" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H19" s="3"/>
     </row>
-    <row r="20" spans="8:8">
+    <row r="20" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H20" s="3"/>
     </row>
   </sheetData>
@@ -1227,15 +1227,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <TaxCatchAll xmlns="40414187-dd76-4ef8-b04f-ccddae734140" xsi:nil="true"/>
@@ -1246,14 +1237,49 @@
 </p:properties>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{124384BF-B442-43EF-BEBD-26F0C03197F3}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{124384BF-B442-43EF-BEBD-26F0C03197F3}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="63768118-86e2-4829-8a12-b72c47658d02"/>
+    <ds:schemaRef ds:uri="40414187-dd76-4ef8-b04f-ccddae734140"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{26BC43C4-0DE4-4398-8C07-F13A3433226F}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2A4DA3E6-B8B6-48A6-81EC-CAAD4DEE707B}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="40414187-dd76-4ef8-b04f-ccddae734140"/>
+    <ds:schemaRef ds:uri="63768118-86e2-4829-8a12-b72c47658d02"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2A4DA3E6-B8B6-48A6-81EC-CAAD4DEE707B}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{26BC43C4-0DE4-4398-8C07-F13A3433226F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Se dterminan Pp de diseño
</commit_message>
<xml_diff>
--- a/Inputs.xlsx
+++ b/Inputs.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Codigos\HU_SCS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{34CF6988-A617-4447-8A92-CAB330465311}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72404BA4-EBF0-4ED1-9610-FA9E114747AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Info Cuencas" sheetId="1" r:id="rId1"/>
@@ -62,7 +62,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="31">
   <si>
     <t>Cuenca</t>
   </si>
@@ -152,6 +152,9 @@
   </si>
   <si>
     <t>T</t>
+  </si>
+  <si>
+    <t>% Tiempo</t>
   </si>
 </sst>
 </file>
@@ -16955,15 +16958,15 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CC7FBFDF-ABB4-4287-9F76-768D0CF54D44}">
-  <dimension ref="A1:E242"/>
+  <dimension ref="A1:F242"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="9.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" s="9" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="B1" s="9" t="s">
         <v>28</v>
@@ -16978,8 +16981,8 @@
         <v>25</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A2" s="9">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A2" s="4">
         <v>0</v>
       </c>
       <c r="B2" s="4">
@@ -16994,10 +16997,11 @@
       <c r="E2" s="4">
         <v>0</v>
       </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F2" s="4"/>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" s="4">
-        <v>0.1</v>
+        <v>0.41666666666666669</v>
       </c>
       <c r="B3" s="4">
         <v>0.17399999999999999</v>
@@ -17011,10 +17015,11 @@
       <c r="E3" s="4">
         <v>0.1</v>
       </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F3" s="4"/>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" s="4">
-        <v>0.2</v>
+        <v>0.83333333333333337</v>
       </c>
       <c r="B4" s="4">
         <v>0.34799999999999998</v>
@@ -17028,10 +17033,11 @@
       <c r="E4" s="4">
         <v>0.2</v>
       </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F4" s="4"/>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" s="4">
-        <v>0.30000000000000004</v>
+        <v>1.25</v>
       </c>
       <c r="B5" s="4">
         <v>0.52200000000000002</v>
@@ -17045,10 +17051,11 @@
       <c r="E5" s="4">
         <v>0.3</v>
       </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F5" s="4"/>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" s="4">
-        <v>0.4</v>
+        <v>1.6666666666666667</v>
       </c>
       <c r="B6" s="4">
         <v>0.69699999999999995</v>
@@ -17062,10 +17069,11 @@
       <c r="E6" s="4">
         <v>0.4</v>
       </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F6" s="4"/>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" s="4">
-        <v>0.5</v>
+        <v>2.083333333333333</v>
       </c>
       <c r="B7" s="4">
         <v>0.87100000000000011</v>
@@ -17079,10 +17087,11 @@
       <c r="E7" s="4">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F7" s="4"/>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" s="4">
-        <v>0.6</v>
+        <v>2.5</v>
       </c>
       <c r="B8" s="4">
         <v>1.046</v>
@@ -17096,10 +17105,11 @@
       <c r="E8" s="4">
         <v>0.6</v>
       </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F8" s="4"/>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9" s="4">
-        <v>0.7</v>
+        <v>2.9166666666666665</v>
       </c>
       <c r="B9" s="4">
         <v>1.22</v>
@@ -17113,10 +17123,11 @@
       <c r="E9" s="4">
         <v>0.70000000000000007</v>
       </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F9" s="4"/>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10" s="4">
-        <v>0.79999999999999993</v>
+        <v>3.3333333333333335</v>
       </c>
       <c r="B10" s="4">
         <v>1.395</v>
@@ -17130,10 +17141,11 @@
       <c r="E10" s="4">
         <v>0.8</v>
       </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F10" s="4"/>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11" s="4">
-        <v>0.89999999999999991</v>
+        <v>3.75</v>
       </c>
       <c r="B11" s="4">
         <v>1.5699999999999998</v>
@@ -17147,10 +17159,11 @@
       <c r="E11" s="4">
         <v>0.89999999999999991</v>
       </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F11" s="4"/>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12" s="4">
-        <v>0.99999999999999989</v>
+        <v>4.1666666666666661</v>
       </c>
       <c r="B12" s="4">
         <v>1.7450000000000001</v>
@@ -17164,10 +17177,11 @@
       <c r="E12" s="4">
         <v>1</v>
       </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F12" s="4"/>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A13" s="4">
-        <v>1.0999999999999999</v>
+        <v>4.5833333333333339</v>
       </c>
       <c r="B13" s="4">
         <v>1.92</v>
@@ -17181,10 +17195,11 @@
       <c r="E13" s="4">
         <v>1.0999999999999999</v>
       </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F13" s="4"/>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A14" s="4">
-        <v>1.2</v>
+        <v>5</v>
       </c>
       <c r="B14" s="4">
         <v>2.0950000000000002</v>
@@ -17198,10 +17213,11 @@
       <c r="E14" s="4">
         <v>1.2</v>
       </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F14" s="4"/>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A15" s="4">
-        <v>1.3</v>
+        <v>5.416666666666667</v>
       </c>
       <c r="B15" s="4">
         <v>2.27</v>
@@ -17215,10 +17231,11 @@
       <c r="E15" s="4">
         <v>1.3</v>
       </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F15" s="4"/>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A16" s="4">
-        <v>1.4000000000000001</v>
+        <v>5.833333333333333</v>
       </c>
       <c r="B16" s="4">
         <v>2.4459999999999997</v>
@@ -17232,10 +17249,11 @@
       <c r="E16" s="4">
         <v>1.4000000000000001</v>
       </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F16" s="4"/>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A17" s="4">
-        <v>1.5000000000000002</v>
+        <v>6.25</v>
       </c>
       <c r="B17" s="4">
         <v>2.621</v>
@@ -17249,10 +17267,11 @@
       <c r="E17" s="4">
         <v>1.5</v>
       </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F17" s="4"/>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A18" s="4">
-        <v>1.6000000000000003</v>
+        <v>6.666666666666667</v>
       </c>
       <c r="B18" s="4">
         <v>2.7969999999999997</v>
@@ -17266,10 +17285,11 @@
       <c r="E18" s="4">
         <v>1.6</v>
       </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F18" s="4"/>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A19" s="4">
-        <v>1.7000000000000004</v>
+        <v>7.083333333333333</v>
       </c>
       <c r="B19" s="4">
         <v>2.972</v>
@@ -17283,10 +17303,11 @@
       <c r="E19" s="4">
         <v>1.7000000000000002</v>
       </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F19" s="4"/>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A20" s="4">
-        <v>1.8000000000000005</v>
+        <v>7.5</v>
       </c>
       <c r="B20" s="4">
         <v>3.1480000000000001</v>
@@ -17300,10 +17321,11 @@
       <c r="E20" s="4">
         <v>1.7999999999999998</v>
       </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F20" s="4"/>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A21" s="4">
-        <v>1.9000000000000006</v>
+        <v>7.9166666666666661</v>
       </c>
       <c r="B21" s="4">
         <v>3.3239999999999998</v>
@@ -17317,10 +17339,11 @@
       <c r="E21" s="4">
         <v>1.9</v>
       </c>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F21" s="4"/>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A22" s="4">
-        <v>2.0000000000000004</v>
+        <v>8.3333333333333321</v>
       </c>
       <c r="B22" s="4">
         <v>3.5000000000000004</v>
@@ -17334,10 +17357,11 @@
       <c r="E22" s="4">
         <v>2</v>
       </c>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F22" s="4"/>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A23" s="4">
-        <v>2.1000000000000005</v>
+        <v>8.75</v>
       </c>
       <c r="B23" s="4">
         <v>3.6769999999999996</v>
@@ -17351,10 +17375,11 @@
       <c r="E23" s="4">
         <v>2.101</v>
       </c>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F23" s="4"/>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A24" s="4">
-        <v>2.2000000000000006</v>
+        <v>9.1666666666666679</v>
       </c>
       <c r="B24" s="4">
         <v>3.8580000000000005</v>
@@ -17368,10 +17393,11 @@
       <c r="E24" s="4">
         <v>2.2030000000000003</v>
       </c>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F24" s="4"/>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A25" s="4">
-        <v>2.3000000000000007</v>
+        <v>9.5833333333333321</v>
       </c>
       <c r="B25" s="4">
         <v>4.0410000000000004</v>
@@ -17385,10 +17411,11 @@
       <c r="E25" s="4">
         <v>2.3069999999999999</v>
       </c>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F25" s="4"/>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A26" s="4">
-        <v>2.4000000000000008</v>
+        <v>10</v>
       </c>
       <c r="B26" s="4">
         <v>4.2270000000000003</v>
@@ -17402,10 +17429,11 @@
       <c r="E26" s="4">
         <v>2.4119999999999999</v>
       </c>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F26" s="4"/>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A27" s="4">
-        <v>2.5000000000000009</v>
+        <v>10.416666666666668</v>
       </c>
       <c r="B27" s="4">
         <v>4.4159999999999995</v>
@@ -17419,10 +17447,11 @@
       <c r="E27" s="4">
         <v>2.5190000000000001</v>
       </c>
-    </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F27" s="4"/>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A28" s="4">
-        <v>2.600000000000001</v>
+        <v>10.833333333333334</v>
       </c>
       <c r="B28" s="4">
         <v>4.6080000000000005</v>
@@ -17436,10 +17465,11 @@
       <c r="E28" s="4">
         <v>2.6270000000000002</v>
       </c>
-    </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F28" s="4"/>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A29" s="4">
-        <v>2.7000000000000011</v>
+        <v>11.25</v>
       </c>
       <c r="B29" s="4">
         <v>4.8029999999999999</v>
@@ -17453,10 +17483,11 @@
       <c r="E29" s="4">
         <v>2.7369999999999997</v>
       </c>
-    </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F29" s="4"/>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A30" s="4">
-        <v>2.8000000000000012</v>
+        <v>11.666666666666666</v>
       </c>
       <c r="B30" s="4">
         <v>5.0009999999999994</v>
@@ -17470,10 +17501,11 @@
       <c r="E30" s="4">
         <v>2.8479999999999999</v>
       </c>
-    </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F30" s="4"/>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A31" s="4">
-        <v>2.9000000000000012</v>
+        <v>12.083333333333334</v>
       </c>
       <c r="B31" s="4">
         <v>5.2010000000000005</v>
@@ -17487,10 +17519,11 @@
       <c r="E31" s="4">
         <v>2.9610000000000003</v>
       </c>
-    </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F31" s="4"/>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A32" s="4">
-        <v>3.0000000000000013</v>
+        <v>12.5</v>
       </c>
       <c r="B32" s="4">
         <v>5.4050000000000002</v>
@@ -17504,10 +17537,11 @@
       <c r="E32" s="4">
         <v>3.0750000000000002</v>
       </c>
-    </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F32" s="4"/>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A33" s="4">
-        <v>3.1000000000000014</v>
+        <v>12.916666666666668</v>
       </c>
       <c r="B33" s="4">
         <v>5.6109999999999998</v>
@@ -17521,10 +17555,11 @@
       <c r="E33" s="4">
         <v>3.1910000000000003</v>
       </c>
-    </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F33" s="4"/>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A34" s="4">
-        <v>3.2000000000000015</v>
+        <v>13.333333333333334</v>
       </c>
       <c r="B34" s="4">
         <v>5.8209999999999997</v>
@@ -17538,10 +17573,11 @@
       <c r="E34" s="4">
         <v>3.3079999999999998</v>
       </c>
-    </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F34" s="4"/>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A35" s="4">
-        <v>3.3000000000000016</v>
+        <v>13.749999999999998</v>
       </c>
       <c r="B35" s="4">
         <v>6.0330000000000004</v>
@@ -17555,10 +17591,11 @@
       <c r="E35" s="4">
         <v>3.427</v>
       </c>
-    </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F35" s="4"/>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A36" s="4">
-        <v>3.4000000000000017</v>
+        <v>14.166666666666666</v>
       </c>
       <c r="B36" s="4">
         <v>6.2480000000000002</v>
@@ -17572,10 +17609,11 @@
       <c r="E36" s="4">
         <v>3.5470000000000002</v>
       </c>
-    </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F36" s="4"/>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A37" s="4">
-        <v>3.5000000000000018</v>
+        <v>14.583333333333334</v>
       </c>
       <c r="B37" s="4">
         <v>6.4659999999999993</v>
@@ -17589,10 +17627,11 @@
       <c r="E37" s="4">
         <v>3.669</v>
       </c>
-    </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F37" s="4"/>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A38" s="4">
-        <v>3.6000000000000019</v>
+        <v>15</v>
       </c>
       <c r="B38" s="4">
         <v>6.6870000000000003</v>
@@ -17606,10 +17645,11 @@
       <c r="E38" s="4">
         <v>3.7920000000000003</v>
       </c>
-    </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F38" s="4"/>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A39" s="4">
-        <v>3.700000000000002</v>
+        <v>15.416666666666668</v>
       </c>
       <c r="B39" s="4">
         <v>6.9110000000000005</v>
@@ -17623,10 +17663,11 @@
       <c r="E39" s="4">
         <v>3.9170000000000003</v>
       </c>
-    </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F39" s="4"/>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A40" s="4">
-        <v>3.800000000000002</v>
+        <v>15.833333333333332</v>
       </c>
       <c r="B40" s="4">
         <v>7.1379999999999999</v>
@@ -17640,10 +17681,11 @@
       <c r="E40" s="4">
         <v>4.0430000000000001</v>
       </c>
-    </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F40" s="4"/>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A41" s="4">
-        <v>3.9000000000000021</v>
+        <v>16.25</v>
       </c>
       <c r="B41" s="4">
         <v>7.367</v>
@@ -17657,10 +17699,11 @@
       <c r="E41" s="4">
         <v>4.1709999999999994</v>
       </c>
-    </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F41" s="4"/>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A42" s="4">
-        <v>4.0000000000000018</v>
+        <v>16.666666666666664</v>
       </c>
       <c r="B42" s="4">
         <v>7.6</v>
@@ -17674,10 +17717,11 @@
       <c r="E42" s="4">
         <v>4.3</v>
       </c>
-    </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F42" s="4"/>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A43" s="4">
-        <v>4.1000000000000014</v>
+        <v>17.083333333333332</v>
       </c>
       <c r="B43" s="4">
         <v>7.835</v>
@@ -17691,10 +17735,11 @@
       <c r="E43" s="4">
         <v>4.431</v>
       </c>
-    </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F43" s="4"/>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A44" s="4">
-        <v>4.2000000000000011</v>
+        <v>17.5</v>
       </c>
       <c r="B44" s="4">
         <v>8.07</v>
@@ -17708,10 +17753,11 @@
       <c r="E44" s="4">
         <v>4.5629999999999997</v>
       </c>
-    </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F44" s="4"/>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A45" s="4">
-        <v>4.3000000000000007</v>
+        <v>17.916666666666668</v>
       </c>
       <c r="B45" s="4">
         <v>8.3070000000000004</v>
@@ -17725,10 +17771,11 @@
       <c r="E45" s="4">
         <v>4.6970000000000001</v>
       </c>
-    </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F45" s="4"/>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A46" s="4">
-        <v>4.4000000000000004</v>
+        <v>18.333333333333336</v>
       </c>
       <c r="B46" s="4">
         <v>8.5449999999999999</v>
@@ -17742,10 +17789,11 @@
       <c r="E46" s="4">
         <v>4.8319999999999999</v>
       </c>
-    </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F46" s="4"/>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A47" s="4">
-        <v>4.5</v>
+        <v>18.75</v>
       </c>
       <c r="B47" s="4">
         <v>8.7840000000000007</v>
@@ -17759,10 +17807,11 @@
       <c r="E47" s="4">
         <v>4.9689999999999994</v>
       </c>
-    </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F47" s="4"/>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A48" s="4">
-        <v>4.5999999999999996</v>
+        <v>19.166666666666664</v>
       </c>
       <c r="B48" s="4">
         <v>9.0240000000000009</v>
@@ -17776,10 +17825,11 @@
       <c r="E48" s="4">
         <v>5.1069999999999993</v>
       </c>
-    </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F48" s="4"/>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A49" s="4">
-        <v>4.6999999999999993</v>
+        <v>19.583333333333332</v>
       </c>
       <c r="B49" s="4">
         <v>9.2649999999999988</v>
@@ -17793,10 +17843,11 @@
       <c r="E49" s="4">
         <v>5.2469999999999999</v>
       </c>
-    </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F49" s="4"/>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A50" s="4">
-        <v>4.7999999999999989</v>
+        <v>20</v>
       </c>
       <c r="B50" s="4">
         <v>9.5069999999999997</v>
@@ -17810,10 +17861,11 @@
       <c r="E50" s="4">
         <v>5.3879999999999999</v>
       </c>
-    </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F50" s="4"/>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A51" s="4">
-        <v>4.8999999999999986</v>
+        <v>20.416666666666668</v>
       </c>
       <c r="B51" s="4">
         <v>9.7509999999999994</v>
@@ -17827,10 +17879,11 @@
       <c r="E51" s="4">
         <v>5.5309999999999997</v>
       </c>
-    </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F51" s="4"/>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A52" s="4">
-        <v>4.9999999999999982</v>
+        <v>20.833333333333336</v>
       </c>
       <c r="B52" s="4">
         <v>9.9949999999999992</v>
@@ -17844,10 +17897,11 @@
       <c r="E52" s="4">
         <v>5.6749999999999998</v>
       </c>
-    </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F52" s="4"/>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A53" s="4">
-        <v>5.0999999999999979</v>
+        <v>21.25</v>
       </c>
       <c r="B53" s="4">
         <v>10.241</v>
@@ -17861,10 +17915,11 @@
       <c r="E53" s="4">
         <v>5.8209999999999997</v>
       </c>
-    </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F53" s="4"/>
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A54" s="4">
-        <v>5.1999999999999975</v>
+        <v>21.666666666666668</v>
       </c>
       <c r="B54" s="4">
         <v>10.487</v>
@@ -17878,10 +17933,11 @@
       <c r="E54" s="4">
         <v>5.968</v>
       </c>
-    </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F54" s="4"/>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A55" s="4">
-        <v>5.2999999999999972</v>
+        <v>22.083333333333332</v>
       </c>
       <c r="B55" s="4">
         <v>10.734999999999999</v>
@@ -17895,10 +17951,11 @@
       <c r="E55" s="4">
         <v>6.117</v>
       </c>
-    </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F55" s="4"/>
+    </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A56" s="4">
-        <v>5.3999999999999968</v>
+        <v>22.5</v>
       </c>
       <c r="B56" s="4">
         <v>10.984</v>
@@ -17912,10 +17969,11 @@
       <c r="E56" s="4">
         <v>6.2670000000000003</v>
       </c>
-    </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F56" s="4"/>
+    </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A57" s="4">
-        <v>5.4999999999999964</v>
+        <v>22.916666666666664</v>
       </c>
       <c r="B57" s="4">
         <v>11.234</v>
@@ -17929,10 +17987,11 @@
       <c r="E57" s="4">
         <v>6.4189999999999996</v>
       </c>
-    </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F57" s="4"/>
+    </row>
+    <row r="58" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A58" s="4">
-        <v>5.5999999999999961</v>
+        <v>23.333333333333332</v>
       </c>
       <c r="B58" s="4">
         <v>11.484999999999999</v>
@@ -17946,10 +18005,11 @@
       <c r="E58" s="4">
         <v>6.5720000000000001</v>
       </c>
-    </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F58" s="4"/>
+    </row>
+    <row r="59" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A59" s="4">
-        <v>5.6999999999999957</v>
+        <v>23.75</v>
       </c>
       <c r="B59" s="4">
         <v>11.737</v>
@@ -17963,10 +18023,11 @@
       <c r="E59" s="4">
         <v>6.7269999999999994</v>
       </c>
-    </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F59" s="4"/>
+    </row>
+    <row r="60" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A60" s="4">
-        <v>5.7999999999999954</v>
+        <v>24.166666666666668</v>
       </c>
       <c r="B60" s="4">
         <v>11.99</v>
@@ -17980,10 +18041,11 @@
       <c r="E60" s="4">
         <v>6.883</v>
       </c>
-    </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F60" s="4"/>
+    </row>
+    <row r="61" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A61" s="4">
-        <v>5.899999999999995</v>
+        <v>24.583333333333336</v>
       </c>
       <c r="B61" s="4">
         <v>12.245000000000001</v>
@@ -17997,10 +18059,11 @@
       <c r="E61" s="4">
         <v>7.0410000000000004</v>
       </c>
-    </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F61" s="4"/>
+    </row>
+    <row r="62" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A62" s="4">
-        <v>5.9999999999999947</v>
+        <v>25</v>
       </c>
       <c r="B62" s="4">
         <v>12.5</v>
@@ -18014,10 +18077,11 @@
       <c r="E62" s="4">
         <v>7.1999999999999993</v>
       </c>
-    </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F62" s="4"/>
+    </row>
+    <row r="63" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A63" s="4">
-        <v>6.0999999999999943</v>
+        <v>25.416666666666664</v>
       </c>
       <c r="B63" s="4">
         <v>12.760999999999999</v>
@@ -18031,10 +18095,11 @@
       <c r="E63" s="4">
         <v>7.3630000000000004</v>
       </c>
-    </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F63" s="4"/>
+    </row>
+    <row r="64" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A64" s="4">
-        <v>6.199999999999994</v>
+        <v>25.833333333333336</v>
       </c>
       <c r="B64" s="4">
         <v>13.034000000000001</v>
@@ -18048,10 +18113,11 @@
       <c r="E64" s="4">
         <v>7.53</v>
       </c>
-    </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F64" s="4"/>
+    </row>
+    <row r="65" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A65" s="4">
-        <v>6.2999999999999936</v>
+        <v>26.25</v>
       </c>
       <c r="B65" s="4">
         <v>13.317</v>
@@ -18065,10 +18131,11 @@
       <c r="E65" s="4">
         <v>7.7030000000000003</v>
       </c>
-    </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F65" s="4"/>
+    </row>
+    <row r="66" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A66" s="4">
-        <v>6.3999999999999932</v>
+        <v>26.666666666666668</v>
       </c>
       <c r="B66" s="4">
         <v>13.61</v>
@@ -18082,10 +18149,11 @@
       <c r="E66" s="4">
         <v>7.88</v>
       </c>
-    </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F66" s="4"/>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A67" s="4">
-        <v>6.4999999999999929</v>
+        <v>27.083333333333332</v>
       </c>
       <c r="B67" s="4">
         <v>13.914999999999999</v>
@@ -18099,10 +18167,11 @@
       <c r="E67" s="4">
         <v>8.0629999999999988</v>
       </c>
-    </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F67" s="4"/>
+    </row>
+    <row r="68" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A68" s="4">
-        <v>6.5999999999999925</v>
+        <v>27.499999999999996</v>
       </c>
       <c r="B68" s="4">
         <v>14.23</v>
@@ -18116,10 +18185,11 @@
       <c r="E68" s="4">
         <v>8.25</v>
       </c>
-    </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F68" s="4"/>
+    </row>
+    <row r="69" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A69" s="4">
-        <v>6.6999999999999922</v>
+        <v>27.916666666666668</v>
       </c>
       <c r="B69" s="4">
         <v>14.557</v>
@@ -18133,10 +18203,11 @@
       <c r="E69" s="4">
         <v>8.4430000000000014</v>
       </c>
-    </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F69" s="4"/>
+    </row>
+    <row r="70" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A70" s="4">
-        <v>6.7999999999999918</v>
+        <v>28.333333333333332</v>
       </c>
       <c r="B70" s="4">
         <v>14.893999999999998</v>
@@ -18150,10 +18221,11 @@
       <c r="E70" s="4">
         <v>8.64</v>
       </c>
-    </row>
-    <row r="71" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F70" s="4"/>
+    </row>
+    <row r="71" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A71" s="4">
-        <v>6.8999999999999915</v>
+        <v>28.750000000000004</v>
       </c>
       <c r="B71" s="4">
         <v>15.241</v>
@@ -18167,10 +18239,11 @@
       <c r="E71" s="4">
         <v>8.843</v>
       </c>
-    </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F71" s="4"/>
+    </row>
+    <row r="72" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A72" s="4">
-        <v>6.9999999999999911</v>
+        <v>29.166666666666668</v>
       </c>
       <c r="B72" s="4">
         <v>15.6</v>
@@ -18184,10 +18257,11 @@
       <c r="E72" s="4">
         <v>9.0499999999999989</v>
       </c>
-    </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F72" s="4"/>
+    </row>
+    <row r="73" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A73" s="4">
-        <v>7.0999999999999908</v>
+        <v>29.583333333333332</v>
       </c>
       <c r="B73" s="4">
         <v>15.965999999999999</v>
@@ -18201,10 +18275,11 @@
       <c r="E73" s="4">
         <v>9.2629999999999999</v>
       </c>
-    </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F73" s="4"/>
+    </row>
+    <row r="74" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A74" s="4">
-        <v>7.1999999999999904</v>
+        <v>30</v>
       </c>
       <c r="B74" s="4">
         <v>16.334</v>
@@ -18218,10 +18293,11 @@
       <c r="E74" s="4">
         <v>9.48</v>
       </c>
-    </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F74" s="4"/>
+    </row>
+    <row r="75" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A75" s="4">
-        <v>7.2999999999999901</v>
+        <v>30.416666666666664</v>
       </c>
       <c r="B75" s="4">
         <v>16.706</v>
@@ -18235,10 +18311,11 @@
       <c r="E75" s="4">
         <v>9.7030000000000012</v>
       </c>
-    </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F75" s="4"/>
+    </row>
+    <row r="76" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A76" s="4">
-        <v>7.3999999999999897</v>
+        <v>30.833333333333336</v>
       </c>
       <c r="B76" s="4">
         <v>17.082000000000001</v>
@@ -18252,10 +18329,11 @@
       <c r="E76" s="4">
         <v>9.93</v>
       </c>
-    </row>
-    <row r="77" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F76" s="4"/>
+    </row>
+    <row r="77" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A77" s="4">
-        <v>7.4999999999999893</v>
+        <v>31.25</v>
       </c>
       <c r="B77" s="4">
         <v>17.46</v>
@@ -18269,10 +18347,11 @@
       <c r="E77" s="4">
         <v>10.163</v>
       </c>
-    </row>
-    <row r="78" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F77" s="4"/>
+    </row>
+    <row r="78" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A78" s="4">
-        <v>7.599999999999989</v>
+        <v>31.666666666666664</v>
       </c>
       <c r="B78" s="4">
         <v>17.841999999999999</v>
@@ -18286,10 +18365,11 @@
       <c r="E78" s="4">
         <v>10.4</v>
       </c>
-    </row>
-    <row r="79" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F78" s="4"/>
+    </row>
+    <row r="79" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A79" s="4">
-        <v>7.6999999999999886</v>
+        <v>32.083333333333336</v>
       </c>
       <c r="B79" s="4">
         <v>18.225999999999999</v>
@@ -18303,10 +18383,11 @@
       <c r="E79" s="4">
         <v>10.642999999999999</v>
       </c>
-    </row>
-    <row r="80" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F79" s="4"/>
+    </row>
+    <row r="80" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A80" s="4">
-        <v>7.7999999999999883</v>
+        <v>32.5</v>
       </c>
       <c r="B80" s="4">
         <v>18.614000000000001</v>
@@ -18320,10 +18401,11 @@
       <c r="E80" s="4">
         <v>10.89</v>
       </c>
-    </row>
-    <row r="81" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F80" s="4"/>
+    </row>
+    <row r="81" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A81" s="4">
-        <v>7.8999999999999879</v>
+        <v>32.916666666666664</v>
       </c>
       <c r="B81" s="4">
         <v>19.006</v>
@@ -18337,10 +18419,11 @@
       <c r="E81" s="4">
         <v>11.143000000000001</v>
       </c>
-    </row>
-    <row r="82" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F81" s="4"/>
+    </row>
+    <row r="82" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A82" s="4">
-        <v>7.9999999999999876</v>
+        <v>33.333333333333329</v>
       </c>
       <c r="B82" s="4">
         <v>19.400000000000002</v>
@@ -18354,10 +18437,11 @@
       <c r="E82" s="4">
         <v>11.4</v>
       </c>
-    </row>
-    <row r="83" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F82" s="4"/>
+    </row>
+    <row r="83" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A83" s="4">
-        <v>8.0999999999999872</v>
+        <v>33.75</v>
       </c>
       <c r="B83" s="4">
         <v>19.817</v>
@@ -18371,10 +18455,11 @@
       <c r="E83" s="4">
         <v>11.666</v>
       </c>
-    </row>
-    <row r="84" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F83" s="4"/>
+    </row>
+    <row r="84" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A84" s="4">
-        <v>8.1999999999999869</v>
+        <v>34.166666666666664</v>
       </c>
       <c r="B84" s="4">
         <v>20.275000000000002</v>
@@ -18388,10 +18473,11 @@
       <c r="E84" s="4">
         <v>11.943</v>
       </c>
-    </row>
-    <row r="85" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F84" s="4"/>
+    </row>
+    <row r="85" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A85" s="4">
-        <v>8.2999999999999865</v>
+        <v>34.583333333333336</v>
       </c>
       <c r="B85" s="4">
         <v>20.774999999999999</v>
@@ -18405,10 +18491,11 @@
       <c r="E85" s="4">
         <v>12.231999999999999</v>
       </c>
-    </row>
-    <row r="86" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F85" s="4"/>
+    </row>
+    <row r="86" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A86" s="4">
-        <v>8.3999999999999861</v>
+        <v>35</v>
       </c>
       <c r="B86" s="4">
         <v>21.317</v>
@@ -18422,10 +18509,11 @@
       <c r="E86" s="4">
         <v>12.531999999999998</v>
       </c>
-    </row>
-    <row r="87" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F86" s="4"/>
+    </row>
+    <row r="87" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A87" s="4">
-        <v>8.4999999999999858</v>
+        <v>35.416666666666671</v>
       </c>
       <c r="B87" s="4">
         <v>21.9</v>
@@ -18439,10 +18527,11 @@
       <c r="E87" s="4">
         <v>12.843999999999999</v>
       </c>
-    </row>
-    <row r="88" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F87" s="4"/>
+    </row>
+    <row r="88" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A88" s="4">
-        <v>8.5999999999999854</v>
+        <v>35.833333333333336</v>
       </c>
       <c r="B88" s="4">
         <v>22.523</v>
@@ -18456,10 +18545,11 @@
       <c r="E88" s="4">
         <v>13.167000000000002</v>
       </c>
-    </row>
-    <row r="89" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F88" s="4"/>
+    </row>
+    <row r="89" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A89" s="4">
-        <v>8.6999999999999851</v>
+        <v>36.25</v>
       </c>
       <c r="B89" s="4">
         <v>23.184999999999999</v>
@@ -18473,10 +18563,11 @@
       <c r="E89" s="4">
         <v>13.502000000000001</v>
       </c>
-    </row>
-    <row r="90" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F89" s="4"/>
+    </row>
+    <row r="90" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A90" s="4">
-        <v>8.7999999999999847</v>
+        <v>36.666666666666671</v>
       </c>
       <c r="B90" s="4">
         <v>23.885000000000002</v>
@@ -18490,10 +18581,11 @@
       <c r="E90" s="4">
         <v>13.847999999999999</v>
       </c>
-    </row>
-    <row r="91" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F90" s="4"/>
+    </row>
+    <row r="91" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A91" s="4">
-        <v>8.8999999999999844</v>
+        <v>37.083333333333336</v>
       </c>
       <c r="B91" s="4">
         <v>24.623000000000001</v>
@@ -18507,10 +18599,11 @@
       <c r="E91" s="4">
         <v>14.206</v>
       </c>
-    </row>
-    <row r="92" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F91" s="4"/>
+    </row>
+    <row r="92" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A92" s="4">
-        <v>8.999999999999984</v>
+        <v>37.5</v>
       </c>
       <c r="B92" s="4">
         <v>25.4</v>
@@ -18524,10 +18617,11 @@
       <c r="E92" s="4">
         <v>14.574999999999999</v>
       </c>
-    </row>
-    <row r="93" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F92" s="4"/>
+    </row>
+    <row r="93" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A93" s="4">
-        <v>9.0999999999999837</v>
+        <v>37.916666666666664</v>
       </c>
       <c r="B93" s="4">
         <v>26.233000000000001</v>
@@ -18541,10 +18635,11 @@
       <c r="E93" s="4">
         <v>14.956</v>
       </c>
-    </row>
-    <row r="94" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F93" s="4"/>
+    </row>
+    <row r="94" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A94" s="4">
-        <v>9.1999999999999833</v>
+        <v>38.333333333333329</v>
       </c>
       <c r="B94" s="4">
         <v>27.139000000000003</v>
@@ -18558,10 +18653,11 @@
       <c r="E94" s="4">
         <v>15.348000000000001</v>
       </c>
-    </row>
-    <row r="95" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F94" s="4"/>
+    </row>
+    <row r="95" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A95" s="4">
-        <v>9.2999999999999829</v>
+        <v>38.75</v>
       </c>
       <c r="B95" s="4">
         <v>28.119</v>
@@ -18575,10 +18671,11 @@
       <c r="E95" s="4">
         <v>15.751999999999999</v>
       </c>
-    </row>
-    <row r="96" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F95" s="4"/>
+    </row>
+    <row r="96" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A96" s="4">
-        <v>9.3999999999999826</v>
+        <v>39.166666666666664</v>
       </c>
       <c r="B96" s="4">
         <v>29.172999999999998</v>
@@ -18592,10 +18689,11 @@
       <c r="E96" s="4">
         <v>16.167000000000002</v>
       </c>
-    </row>
-    <row r="97" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F96" s="4"/>
+    </row>
+    <row r="97" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A97" s="4">
-        <v>9.4999999999999822</v>
+        <v>39.583333333333329</v>
       </c>
       <c r="B97" s="4">
         <v>30.3</v>
@@ -18609,10 +18707,11 @@
       <c r="E97" s="4">
         <v>16.594000000000001</v>
       </c>
-    </row>
-    <row r="98" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F97" s="4"/>
+    </row>
+    <row r="98" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A98" s="4">
-        <v>9.5999999999999819</v>
+        <v>40</v>
       </c>
       <c r="B98" s="4">
         <v>31.941999999999997</v>
@@ -18626,10 +18725,11 @@
       <c r="E98" s="4">
         <v>17.032</v>
       </c>
-    </row>
-    <row r="99" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F98" s="4"/>
+    </row>
+    <row r="99" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A99" s="4">
-        <v>9.6999999999999815</v>
+        <v>40.416666666666664</v>
       </c>
       <c r="B99" s="4">
         <v>34.542000000000002</v>
@@ -18643,10 +18743,11 @@
       <c r="E99" s="4">
         <v>17.481999999999999</v>
       </c>
-    </row>
-    <row r="100" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F99" s="4"/>
+    </row>
+    <row r="100" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A100" s="4">
-        <v>9.7999999999999812</v>
+        <v>40.833333333333336</v>
       </c>
       <c r="B100" s="4">
         <v>38.783999999999999</v>
@@ -18660,10 +18761,11 @@
       <c r="E100" s="4">
         <v>17.943000000000001</v>
       </c>
-    </row>
-    <row r="101" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F100" s="4"/>
+    </row>
+    <row r="101" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A101" s="4">
-        <v>9.8999999999999808</v>
+        <v>41.25</v>
       </c>
       <c r="B101" s="4">
         <v>46.316000000000003</v>
@@ -18677,10 +18779,11 @@
       <c r="E101" s="4">
         <v>18.416</v>
       </c>
-    </row>
-    <row r="102" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F101" s="4"/>
+    </row>
+    <row r="102" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A102" s="4">
-        <v>9.9999999999999805</v>
+        <v>41.666666666666671</v>
       </c>
       <c r="B102" s="4">
         <v>51.5</v>
@@ -18694,10 +18797,11 @@
       <c r="E102" s="4">
         <v>18.899999999999999</v>
       </c>
-    </row>
-    <row r="103" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F102" s="4"/>
+    </row>
+    <row r="103" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A103" s="4">
-        <v>10.09999999999998</v>
+        <v>42.083333333333336</v>
       </c>
       <c r="B103" s="4">
         <v>53.22</v>
@@ -18711,10 +18815,11 @@
       <c r="E103" s="4">
         <v>19.402000000000001</v>
       </c>
-    </row>
-    <row r="104" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F103" s="4"/>
+    </row>
+    <row r="104" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A104" s="4">
-        <v>10.19999999999998</v>
+        <v>42.5</v>
       </c>
       <c r="B104" s="4">
         <v>54.76</v>
@@ -18728,10 +18833,11 @@
       <c r="E104" s="4">
         <v>19.928000000000001</v>
       </c>
-    </row>
-    <row r="105" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F104" s="4"/>
+    </row>
+    <row r="105" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A105" s="4">
-        <v>10.299999999999979</v>
+        <v>42.916666666666671</v>
       </c>
       <c r="B105" s="4">
         <v>56.120000000000005</v>
@@ -18745,10 +18851,11 @@
       <c r="E105" s="4">
         <v>20.477999999999998</v>
       </c>
-    </row>
-    <row r="106" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F105" s="4"/>
+    </row>
+    <row r="106" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A106" s="4">
-        <v>10.399999999999979</v>
+        <v>43.333333333333336</v>
       </c>
       <c r="B106" s="4">
         <v>57.3</v>
@@ -18762,10 +18869,11 @@
       <c r="E106" s="4">
         <v>21.052</v>
       </c>
-    </row>
-    <row r="107" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F106" s="4"/>
+    </row>
+    <row r="107" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A107" s="4">
-        <v>10.499999999999979</v>
+        <v>43.75</v>
       </c>
       <c r="B107" s="4">
         <v>58.3</v>
@@ -18779,10 +18887,11 @@
       <c r="E107" s="4">
         <v>21.65</v>
       </c>
-    </row>
-    <row r="108" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F107" s="4"/>
+    </row>
+    <row r="108" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A108" s="4">
-        <v>10.599999999999978</v>
+        <v>44.166666666666664</v>
       </c>
       <c r="B108" s="4">
         <v>59.187999999999995</v>
@@ -18796,10 +18905,11 @@
       <c r="E108" s="4">
         <v>22.271999999999998</v>
       </c>
-    </row>
-    <row r="109" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F108" s="4"/>
+    </row>
+    <row r="109" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A109" s="4">
-        <v>10.699999999999978</v>
+        <v>44.583333333333329</v>
       </c>
       <c r="B109" s="4">
         <v>60.031999999999996</v>
@@ -18813,10 +18923,11 @@
       <c r="E109" s="4">
         <v>22.917999999999999</v>
       </c>
-    </row>
-    <row r="110" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F109" s="4"/>
+    </row>
+    <row r="110" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A110" s="4">
-        <v>10.799999999999978</v>
+        <v>45</v>
       </c>
       <c r="B110" s="4">
         <v>60.831999999999994</v>
@@ -18830,10 +18941,11 @@
       <c r="E110" s="4">
         <v>23.588000000000001</v>
       </c>
-    </row>
-    <row r="111" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F110" s="4"/>
+    </row>
+    <row r="111" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A111" s="4">
-        <v>10.899999999999977</v>
+        <v>45.416666666666664</v>
       </c>
       <c r="B111" s="4">
         <v>61.588000000000001</v>
@@ -18847,10 +18959,11 @@
       <c r="E111" s="4">
         <v>24.282</v>
       </c>
-    </row>
-    <row r="112" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F111" s="4"/>
+    </row>
+    <row r="112" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A112" s="4">
-        <v>10.999999999999977</v>
+        <v>45.833333333333329</v>
       </c>
       <c r="B112" s="4">
         <v>62.3</v>
@@ -18864,10 +18977,11 @@
       <c r="E112" s="4">
         <v>25</v>
       </c>
-    </row>
-    <row r="113" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F112" s="4"/>
+    </row>
+    <row r="113" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A113" s="4">
-        <v>11.099999999999977</v>
+        <v>46.25</v>
       </c>
       <c r="B113" s="4">
         <v>62.982000000000006</v>
@@ -18881,10 +18995,11 @@
       <c r="E113" s="4">
         <v>25.776</v>
       </c>
-    </row>
-    <row r="114" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F113" s="4"/>
+    </row>
+    <row r="114" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A114" s="4">
-        <v>11.199999999999976</v>
+        <v>46.666666666666664</v>
       </c>
       <c r="B114" s="4">
         <v>63.648000000000003</v>
@@ -18898,10 +19013,11 @@
       <c r="E114" s="4">
         <v>26.644000000000002</v>
       </c>
-    </row>
-    <row r="115" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F114" s="4"/>
+    </row>
+    <row r="115" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A115" s="4">
-        <v>11.299999999999976</v>
+        <v>47.083333333333336</v>
       </c>
       <c r="B115" s="4">
         <v>64.298000000000002</v>
@@ -18915,10 +19031,11 @@
       <c r="E115" s="4">
         <v>27.603999999999999</v>
       </c>
-    </row>
-    <row r="116" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F115" s="4"/>
+    </row>
+    <row r="116" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A116" s="4">
-        <v>11.399999999999975</v>
+        <v>47.5</v>
       </c>
       <c r="B116" s="4">
         <v>64.932000000000002</v>
@@ -18932,10 +19049,11 @@
       <c r="E116" s="4">
         <v>28.655999999999999</v>
       </c>
-    </row>
-    <row r="117" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F116" s="4"/>
+    </row>
+    <row r="117" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A117" s="4">
-        <v>11.499999999999975</v>
+        <v>47.916666666666671</v>
       </c>
       <c r="B117" s="4">
         <v>65.55</v>
@@ -18949,10 +19067,11 @@
       <c r="E117" s="4">
         <v>29.799999999999997</v>
       </c>
-    </row>
-    <row r="118" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F117" s="4"/>
+    </row>
+    <row r="118" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A118" s="4">
-        <v>11.599999999999975</v>
+        <v>48.333333333333336</v>
       </c>
       <c r="B118" s="4">
         <v>66.152000000000001</v>
@@ -18966,10 +19085,11 @@
       <c r="E118" s="4">
         <v>31.430000000000003</v>
       </c>
-    </row>
-    <row r="119" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F118" s="4"/>
+    </row>
+    <row r="119" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A119" s="4">
-        <v>11.699999999999974</v>
+        <v>48.75</v>
       </c>
       <c r="B119" s="4">
         <v>66.738</v>
@@ -18983,10 +19103,11 @@
       <c r="E119" s="4">
         <v>33.94</v>
       </c>
-    </row>
-    <row r="120" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F119" s="4"/>
+    </row>
+    <row r="120" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A120" s="4">
-        <v>11.799999999999974</v>
+        <v>49.166666666666671</v>
       </c>
       <c r="B120" s="4">
         <v>67.308000000000007</v>
@@ -19000,10 +19121,11 @@
       <c r="E120" s="4">
         <v>37.330000000000005</v>
       </c>
-    </row>
-    <row r="121" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F120" s="4"/>
+    </row>
+    <row r="121" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A121" s="4">
-        <v>11.899999999999974</v>
+        <v>49.583333333333336</v>
       </c>
       <c r="B121" s="4">
         <v>67.861999999999995</v>
@@ -19017,10 +19139,11 @@
       <c r="E121" s="4">
         <v>41.6</v>
       </c>
-    </row>
-    <row r="122" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F121" s="4"/>
+    </row>
+    <row r="122" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A122" s="4">
-        <v>11.999999999999973</v>
+        <v>50</v>
       </c>
       <c r="B122" s="4">
         <v>68.400000000000006</v>
@@ -19034,10 +19157,11 @@
       <c r="E122" s="4">
         <v>50</v>
       </c>
-    </row>
-    <row r="123" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F122" s="4"/>
+    </row>
+    <row r="123" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A123" s="4">
-        <v>12.099999999999973</v>
+        <v>50.416666666666664</v>
       </c>
       <c r="B123" s="4">
         <v>68.924999999999997</v>
@@ -19051,10 +19175,11 @@
       <c r="E123" s="4">
         <v>58.4</v>
       </c>
-    </row>
-    <row r="124" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F123" s="4"/>
+    </row>
+    <row r="124" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A124" s="4">
-        <v>12.199999999999973</v>
+        <v>50.833333333333329</v>
       </c>
       <c r="B124" s="4">
         <v>69.44</v>
@@ -19068,10 +19193,11 @@
       <c r="E124" s="4">
         <v>62.67</v>
       </c>
-    </row>
-    <row r="125" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F124" s="4"/>
+    </row>
+    <row r="125" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A125" s="4">
-        <v>12.299999999999972</v>
+        <v>51.250000000000007</v>
       </c>
       <c r="B125" s="4">
         <v>69.945000000000007</v>
@@ -19085,10 +19211,11 @@
       <c r="E125" s="4">
         <v>66.06</v>
       </c>
-    </row>
-    <row r="126" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F125" s="4"/>
+    </row>
+    <row r="126" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A126" s="4">
-        <v>12.399999999999972</v>
+        <v>51.666666666666671</v>
       </c>
       <c r="B126" s="4">
         <v>70.44</v>
@@ -19102,10 +19229,11 @@
       <c r="E126" s="4">
         <v>68.569999999999993</v>
       </c>
-    </row>
-    <row r="127" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F126" s="4"/>
+    </row>
+    <row r="127" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A127" s="4">
-        <v>12.499999999999972</v>
+        <v>52.083333333333336</v>
       </c>
       <c r="B127" s="4">
         <v>70.925000000000011</v>
@@ -19119,10 +19247,11 @@
       <c r="E127" s="4">
         <v>70.199999999999989</v>
       </c>
-    </row>
-    <row r="128" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F127" s="4"/>
+    </row>
+    <row r="128" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A128" s="4">
-        <v>12.599999999999971</v>
+        <v>52.5</v>
       </c>
       <c r="B128" s="4">
         <v>71.399999999999991</v>
@@ -19136,10 +19265,11 @@
       <c r="E128" s="4">
         <v>71.343999999999994</v>
       </c>
-    </row>
-    <row r="129" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F128" s="4"/>
+    </row>
+    <row r="129" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A129" s="4">
-        <v>12.699999999999971</v>
+        <v>52.916666666666664</v>
       </c>
       <c r="B129" s="4">
         <v>71.864999999999995</v>
@@ -19153,10 +19283,11 @@
       <c r="E129" s="4">
         <v>72.396000000000001</v>
       </c>
-    </row>
-    <row r="130" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F129" s="4"/>
+    </row>
+    <row r="130" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A130" s="4">
-        <v>12.799999999999971</v>
+        <v>53.333333333333336</v>
       </c>
       <c r="B130" s="4">
         <v>72.319999999999993</v>
@@ -19170,10 +19301,11 @@
       <c r="E130" s="4">
         <v>73.355999999999995</v>
       </c>
-    </row>
-    <row r="131" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F130" s="4"/>
+    </row>
+    <row r="131" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A131" s="4">
-        <v>12.89999999999997</v>
+        <v>53.75</v>
       </c>
       <c r="B131" s="4">
         <v>72.765000000000001</v>
@@ -19187,10 +19319,11 @@
       <c r="E131" s="4">
         <v>74.224000000000004</v>
       </c>
-    </row>
-    <row r="132" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F131" s="4"/>
+    </row>
+    <row r="132" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A132" s="4">
-        <v>12.99999999999997</v>
+        <v>54.166666666666664</v>
       </c>
       <c r="B132" s="4">
         <v>73.2</v>
@@ -19204,10 +19337,11 @@
       <c r="E132" s="4">
         <v>75</v>
       </c>
-    </row>
-    <row r="133" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F132" s="4"/>
+    </row>
+    <row r="133" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A133" s="4">
-        <v>13.099999999999969</v>
+        <v>54.583333333333329</v>
       </c>
       <c r="B133" s="4">
         <v>73.625</v>
@@ -19221,10 +19355,11 @@
       <c r="E133" s="4">
         <v>75.717999999999989</v>
       </c>
-    </row>
-    <row r="134" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F133" s="4"/>
+    </row>
+    <row r="134" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A134" s="4">
-        <v>13.199999999999969</v>
+        <v>54.999999999999993</v>
       </c>
       <c r="B134" s="4">
         <v>74.039999999999992</v>
@@ -19238,10 +19373,11 @@
       <c r="E134" s="4">
         <v>76.412000000000006</v>
       </c>
-    </row>
-    <row r="135" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F134" s="4"/>
+    </row>
+    <row r="135" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A135" s="4">
-        <v>13.299999999999969</v>
+        <v>55.416666666666671</v>
       </c>
       <c r="B135" s="4">
         <v>74.444999999999993</v>
@@ -19255,10 +19391,11 @@
       <c r="E135" s="4">
         <v>77.081999999999994</v>
       </c>
-    </row>
-    <row r="136" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F135" s="4"/>
+    </row>
+    <row r="136" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A136" s="4">
-        <v>13.399999999999968</v>
+        <v>55.833333333333336</v>
       </c>
       <c r="B136" s="4">
         <v>74.839999999999989</v>
@@ -19272,10 +19409,11 @@
       <c r="E136" s="4">
         <v>77.727999999999994</v>
       </c>
-    </row>
-    <row r="137" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F136" s="4"/>
+    </row>
+    <row r="137" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A137" s="4">
-        <v>13.499999999999968</v>
+        <v>56.25</v>
       </c>
       <c r="B137" s="4">
         <v>75.224999999999994</v>
@@ -19289,10 +19427,11 @@
       <c r="E137" s="4">
         <v>78.349999999999994</v>
       </c>
-    </row>
-    <row r="138" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F137" s="4"/>
+    </row>
+    <row r="138" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A138" s="4">
-        <v>13.599999999999968</v>
+        <v>56.666666666666664</v>
       </c>
       <c r="B138" s="4">
         <v>75.599999999999994</v>
@@ -19306,10 +19445,11 @@
       <c r="E138" s="4">
         <v>78.947999999999993</v>
       </c>
-    </row>
-    <row r="139" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F138" s="4"/>
+    </row>
+    <row r="139" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A139" s="4">
-        <v>13.699999999999967</v>
+        <v>57.083333333333329</v>
       </c>
       <c r="B139" s="4">
         <v>75.965000000000003</v>
@@ -19323,10 +19463,11 @@
       <c r="E139" s="4">
         <v>79.522000000000006</v>
       </c>
-    </row>
-    <row r="140" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F139" s="4"/>
+    </row>
+    <row r="140" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A140" s="4">
-        <v>13.799999999999967</v>
+        <v>57.500000000000007</v>
       </c>
       <c r="B140" s="4">
         <v>76.319999999999993</v>
@@ -19340,10 +19481,11 @@
       <c r="E140" s="4">
         <v>80.072000000000003</v>
       </c>
-    </row>
-    <row r="141" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F140" s="4"/>
+    </row>
+    <row r="141" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A141" s="4">
-        <v>13.899999999999967</v>
+        <v>57.916666666666671</v>
       </c>
       <c r="B141" s="4">
         <v>76.665000000000006</v>
@@ -19357,10 +19499,11 @@
       <c r="E141" s="4">
         <v>80.597999999999999</v>
       </c>
-    </row>
-    <row r="142" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F141" s="4"/>
+    </row>
+    <row r="142" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A142" s="4">
-        <v>13.999999999999966</v>
+        <v>58.333333333333336</v>
       </c>
       <c r="B142" s="4">
         <v>77</v>
@@ -19374,10 +19517,11 @@
       <c r="E142" s="4">
         <v>81.100000000000009</v>
       </c>
-    </row>
-    <row r="143" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F142" s="4"/>
+    </row>
+    <row r="143" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A143" s="4">
-        <v>14.099999999999966</v>
+        <v>58.75</v>
       </c>
       <c r="B143" s="4">
         <v>77.329000000000008</v>
@@ -19391,10 +19535,11 @@
       <c r="E143" s="4">
         <v>81.584000000000003</v>
       </c>
-    </row>
-    <row r="144" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F143" s="4"/>
+    </row>
+    <row r="144" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A144" s="4">
-        <v>14.199999999999966</v>
+        <v>59.166666666666664</v>
       </c>
       <c r="B144" s="4">
         <v>77.656000000000006</v>
@@ -19408,10 +19553,11 @@
       <c r="E144" s="4">
         <v>82.057000000000002</v>
       </c>
-    </row>
-    <row r="145" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F144" s="4"/>
+    </row>
+    <row r="145" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A145" s="4">
-        <v>14.299999999999965</v>
+        <v>59.583333333333336</v>
       </c>
       <c r="B145" s="4">
         <v>77.980999999999995</v>
@@ -19425,10 +19571,11 @@
       <c r="E145" s="4">
         <v>82.518000000000001</v>
       </c>
-    </row>
-    <row r="146" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F145" s="4"/>
+    </row>
+    <row r="146" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A146" s="4">
-        <v>14.399999999999965</v>
+        <v>60</v>
       </c>
       <c r="B146" s="4">
         <v>78.304000000000002</v>
@@ -19442,10 +19589,11 @@
       <c r="E146" s="4">
         <v>82.968000000000004</v>
       </c>
-    </row>
-    <row r="147" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F146" s="4"/>
+    </row>
+    <row r="147" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A147" s="4">
-        <v>14.499999999999964</v>
+        <v>60.416666666666664</v>
       </c>
       <c r="B147" s="4">
         <v>78.625</v>
@@ -19459,10 +19607,11 @@
       <c r="E147" s="4">
         <v>83.406000000000006</v>
       </c>
-    </row>
-    <row r="148" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F147" s="4"/>
+    </row>
+    <row r="148" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A148" s="4">
-        <v>14.599999999999964</v>
+        <v>60.833333333333329</v>
       </c>
       <c r="B148" s="4">
         <v>78.944000000000003</v>
@@ -19476,10 +19625,11 @@
       <c r="E148" s="4">
         <v>83.832999999999998</v>
       </c>
-    </row>
-    <row r="149" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F148" s="4"/>
+    </row>
+    <row r="149" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A149" s="4">
-        <v>14.699999999999964</v>
+        <v>61.249999999999993</v>
       </c>
       <c r="B149" s="4">
         <v>79.26100000000001</v>
@@ -19493,10 +19643,11 @@
       <c r="E149" s="4">
         <v>84.248000000000005</v>
       </c>
-    </row>
-    <row r="150" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F149" s="4"/>
+    </row>
+    <row r="150" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A150" s="4">
-        <v>14.799999999999963</v>
+        <v>61.666666666666671</v>
       </c>
       <c r="B150" s="4">
         <v>79.576000000000008</v>
@@ -19510,10 +19661,11 @@
       <c r="E150" s="4">
         <v>84.652000000000001</v>
       </c>
-    </row>
-    <row r="151" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F150" s="4"/>
+    </row>
+    <row r="151" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A151" s="4">
-        <v>14.899999999999963</v>
+        <v>62.083333333333336</v>
       </c>
       <c r="B151" s="4">
         <v>79.888999999999996</v>
@@ -19527,10 +19679,11 @@
       <c r="E151" s="4">
         <v>85.043999999999997</v>
       </c>
-    </row>
-    <row r="152" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F151" s="4"/>
+    </row>
+    <row r="152" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A152" s="4">
-        <v>14.999999999999963</v>
+        <v>62.5</v>
       </c>
       <c r="B152" s="4">
         <v>80.2</v>
@@ -19544,10 +19697,11 @@
       <c r="E152" s="4">
         <v>85.424999999999997</v>
       </c>
-    </row>
-    <row r="153" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F152" s="4"/>
+    </row>
+    <row r="153" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A153" s="4">
-        <v>15.099999999999962</v>
+        <v>62.916666666666664</v>
       </c>
       <c r="B153" s="4">
         <v>80.509</v>
@@ -19561,10 +19715,11 @@
       <c r="E153" s="4">
         <v>85.793999999999997</v>
       </c>
-    </row>
-    <row r="154" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F153" s="4"/>
+    </row>
+    <row r="154" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A154" s="4">
-        <v>15.199999999999962</v>
+        <v>63.333333333333329</v>
       </c>
       <c r="B154" s="4">
         <v>80.816000000000003</v>
@@ -19578,10 +19733,11 @@
       <c r="E154" s="4">
         <v>86.152000000000001</v>
       </c>
-    </row>
-    <row r="155" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F154" s="4"/>
+    </row>
+    <row r="155" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A155" s="4">
-        <v>15.299999999999962</v>
+        <v>63.750000000000007</v>
       </c>
       <c r="B155" s="4">
         <v>81.120999999999995</v>
@@ -19595,10 +19751,11 @@
       <c r="E155" s="4">
         <v>86.49799999999999</v>
       </c>
-    </row>
-    <row r="156" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F155" s="4"/>
+    </row>
+    <row r="156" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A156" s="4">
-        <v>15.399999999999961</v>
+        <v>64.166666666666671</v>
       </c>
       <c r="B156" s="4">
         <v>81.423999999999992</v>
@@ -19612,10 +19769,11 @@
       <c r="E156" s="4">
         <v>86.832999999999998</v>
       </c>
-    </row>
-    <row r="157" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F156" s="4"/>
+    </row>
+    <row r="157" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A157" s="4">
-        <v>15.499999999999961</v>
+        <v>64.583333333333343</v>
       </c>
       <c r="B157" s="4">
         <v>81.725000000000009</v>
@@ -19629,10 +19787,11 @@
       <c r="E157" s="4">
         <v>87.156000000000006</v>
       </c>
-    </row>
-    <row r="158" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F157" s="4"/>
+    </row>
+    <row r="158" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A158" s="4">
-        <v>15.599999999999961</v>
+        <v>65</v>
       </c>
       <c r="B158" s="4">
         <v>82.024000000000001</v>
@@ -19646,10 +19805,11 @@
       <c r="E158" s="4">
         <v>87.468000000000004</v>
       </c>
-    </row>
-    <row r="159" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F158" s="4"/>
+    </row>
+    <row r="159" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A159" s="4">
-        <v>15.69999999999996</v>
+        <v>65.416666666666671</v>
       </c>
       <c r="B159" s="4">
         <v>82.320999999999998</v>
@@ -19663,10 +19823,11 @@
       <c r="E159" s="4">
         <v>87.768000000000001</v>
       </c>
-    </row>
-    <row r="160" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F159" s="4"/>
+    </row>
+    <row r="160" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A160" s="4">
-        <v>15.79999999999996</v>
+        <v>65.833333333333329</v>
       </c>
       <c r="B160" s="4">
         <v>82.616</v>
@@ -19680,10 +19841,11 @@
       <c r="E160" s="4">
         <v>88.057000000000002</v>
       </c>
-    </row>
-    <row r="161" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F160" s="4"/>
+    </row>
+    <row r="161" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A161" s="4">
-        <v>15.899999999999959</v>
+        <v>66.25</v>
       </c>
       <c r="B161" s="4">
         <v>82.909000000000006</v>
@@ -19697,10 +19859,11 @@
       <c r="E161" s="4">
         <v>88.334000000000003</v>
       </c>
-    </row>
-    <row r="162" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F161" s="4"/>
+    </row>
+    <row r="162" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A162" s="4">
-        <v>15.999999999999959</v>
+        <v>66.666666666666657</v>
       </c>
       <c r="B162" s="4">
         <v>83.2</v>
@@ -19714,10 +19877,11 @@
       <c r="E162" s="4">
         <v>88.6</v>
       </c>
-    </row>
-    <row r="163" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F162" s="4"/>
+    </row>
+    <row r="163" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A163" s="4">
-        <v>16.099999999999959</v>
+        <v>67.083333333333343</v>
       </c>
       <c r="B163" s="4">
         <v>83.489000000000004</v>
@@ -19731,10 +19895,11 @@
       <c r="E163" s="4">
         <v>88.858000000000004</v>
       </c>
-    </row>
-    <row r="164" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F163" s="4"/>
+    </row>
+    <row r="164" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A164" s="4">
-        <v>16.19999999999996</v>
+        <v>67.5</v>
       </c>
       <c r="B164" s="4">
         <v>83.775999999999996</v>
@@ -19748,10 +19913,11 @@
       <c r="E164" s="4">
         <v>89.11</v>
       </c>
-    </row>
-    <row r="165" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F164" s="4"/>
+    </row>
+    <row r="165" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A165" s="4">
-        <v>16.299999999999962</v>
+        <v>67.916666666666671</v>
       </c>
       <c r="B165" s="4">
         <v>84.060999999999993</v>
@@ -19765,10 +19931,11 @@
       <c r="E165" s="4">
         <v>89.358000000000004</v>
       </c>
-    </row>
-    <row r="166" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F165" s="4"/>
+    </row>
+    <row r="166" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A166" s="4">
-        <v>16.399999999999963</v>
+        <v>68.333333333333329</v>
       </c>
       <c r="B166" s="4">
         <v>84.343999999999994</v>
@@ -19782,10 +19949,11 @@
       <c r="E166" s="4">
         <v>89.600000000000009</v>
       </c>
-    </row>
-    <row r="167" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F166" s="4"/>
+    </row>
+    <row r="167" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A167" s="4">
-        <v>16.499999999999964</v>
+        <v>68.75</v>
       </c>
       <c r="B167" s="4">
         <v>84.625</v>
@@ -19799,10 +19967,11 @@
       <c r="E167" s="4">
         <v>89.837999999999994</v>
       </c>
-    </row>
-    <row r="168" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F167" s="4"/>
+    </row>
+    <row r="168" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A168" s="4">
-        <v>16.599999999999966</v>
+        <v>69.166666666666671</v>
       </c>
       <c r="B168" s="4">
         <v>84.903999999999996</v>
@@ -19816,10 +19985,11 @@
       <c r="E168" s="4">
         <v>90.07</v>
       </c>
-    </row>
-    <row r="169" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F168" s="4"/>
+    </row>
+    <row r="169" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A169" s="4">
-        <v>16.699999999999967</v>
+        <v>69.583333333333329</v>
       </c>
       <c r="B169" s="4">
         <v>85.180999999999997</v>
@@ -19833,10 +20003,11 @@
       <c r="E169" s="4">
         <v>90.298000000000002</v>
       </c>
-    </row>
-    <row r="170" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F169" s="4"/>
+    </row>
+    <row r="170" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A170" s="4">
-        <v>16.799999999999969</v>
+        <v>70</v>
       </c>
       <c r="B170" s="4">
         <v>85.456000000000003</v>
@@ -19850,10 +20021,11 @@
       <c r="E170" s="4">
         <v>90.52</v>
       </c>
-    </row>
-    <row r="171" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F170" s="4"/>
+    </row>
+    <row r="171" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A171" s="4">
-        <v>16.89999999999997</v>
+        <v>70.416666666666657</v>
       </c>
       <c r="B171" s="4">
         <v>85.728999999999999</v>
@@ -19867,10 +20039,11 @@
       <c r="E171" s="4">
         <v>90.738</v>
       </c>
-    </row>
-    <row r="172" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F171" s="4"/>
+    </row>
+    <row r="172" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A172" s="4">
-        <v>16.999999999999972</v>
+        <v>70.833333333333343</v>
       </c>
       <c r="B172" s="4">
         <v>86</v>
@@ -19884,10 +20057,11 @@
       <c r="E172" s="4">
         <v>90.95</v>
       </c>
-    </row>
-    <row r="173" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F172" s="4"/>
+    </row>
+    <row r="173" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A173" s="4">
-        <v>17.099999999999973</v>
+        <v>71.25</v>
       </c>
       <c r="B173" s="4">
         <v>86.268999999999991</v>
@@ -19901,10 +20075,11 @@
       <c r="E173" s="4">
         <v>91.158000000000001</v>
       </c>
-    </row>
-    <row r="174" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F173" s="4"/>
+    </row>
+    <row r="174" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A174" s="4">
-        <v>17.199999999999974</v>
+        <v>71.666666666666671</v>
       </c>
       <c r="B174" s="4">
         <v>86.536000000000001</v>
@@ -19918,10 +20093,11 @@
       <c r="E174" s="4">
         <v>91.36</v>
       </c>
-    </row>
-    <row r="175" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F174" s="4"/>
+    </row>
+    <row r="175" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A175" s="4">
-        <v>17.299999999999976</v>
+        <v>72.083333333333329</v>
       </c>
       <c r="B175" s="4">
         <v>86.800999999999988</v>
@@ -19935,10 +20111,11 @@
       <c r="E175" s="4">
         <v>91.557999999999993</v>
       </c>
-    </row>
-    <row r="176" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F175" s="4"/>
+    </row>
+    <row r="176" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A176" s="4">
-        <v>17.399999999999977</v>
+        <v>72.5</v>
       </c>
       <c r="B176" s="4">
         <v>87.063999999999993</v>
@@ -19952,10 +20129,11 @@
       <c r="E176" s="4">
         <v>91.75</v>
       </c>
-    </row>
-    <row r="177" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F176" s="4"/>
+    </row>
+    <row r="177" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A177" s="4">
-        <v>17.499999999999979</v>
+        <v>72.916666666666657</v>
       </c>
       <c r="B177" s="4">
         <v>87.325000000000003</v>
@@ -19969,10 +20147,11 @@
       <c r="E177" s="4">
         <v>91.938000000000002</v>
       </c>
-    </row>
-    <row r="178" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F177" s="4"/>
+    </row>
+    <row r="178" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A178" s="4">
-        <v>17.59999999999998</v>
+        <v>73.333333333333343</v>
       </c>
       <c r="B178" s="4">
         <v>87.583999999999989</v>
@@ -19986,10 +20165,11 @@
       <c r="E178" s="4">
         <v>92.12</v>
       </c>
-    </row>
-    <row r="179" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F178" s="4"/>
+    </row>
+    <row r="179" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A179" s="4">
-        <v>17.699999999999982</v>
+        <v>73.75</v>
       </c>
       <c r="B179" s="4">
         <v>87.841000000000008</v>
@@ -20003,10 +20183,11 @@
       <c r="E179" s="4">
         <v>92.298000000000002</v>
       </c>
-    </row>
-    <row r="180" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F179" s="4"/>
+    </row>
+    <row r="180" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A180" s="4">
-        <v>17.799999999999983</v>
+        <v>74.166666666666671</v>
       </c>
       <c r="B180" s="4">
         <v>88.096000000000004</v>
@@ -20020,10 +20201,11 @@
       <c r="E180" s="4">
         <v>92.47</v>
       </c>
-    </row>
-    <row r="181" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F180" s="4"/>
+    </row>
+    <row r="181" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A181" s="4">
-        <v>17.899999999999984</v>
+        <v>74.583333333333329</v>
       </c>
       <c r="B181" s="4">
         <v>88.349000000000004</v>
@@ -20037,10 +20219,11 @@
       <c r="E181" s="4">
         <v>92.638000000000005</v>
       </c>
-    </row>
-    <row r="182" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F181" s="4"/>
+    </row>
+    <row r="182" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A182" s="4">
-        <v>17.999999999999986</v>
+        <v>75</v>
       </c>
       <c r="B182" s="4">
         <v>88.6</v>
@@ -20054,10 +20237,11 @@
       <c r="E182" s="4">
         <v>92.800000000000011</v>
       </c>
-    </row>
-    <row r="183" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F182" s="4"/>
+    </row>
+    <row r="183" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A183" s="4">
-        <v>18.099999999999987</v>
+        <v>75.416666666666671</v>
       </c>
       <c r="B183" s="4">
         <v>88.849000000000004</v>
@@ -20071,10 +20255,11 @@
       <c r="E183" s="4">
         <v>92.959000000000003</v>
       </c>
-    </row>
-    <row r="184" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F183" s="4"/>
+    </row>
+    <row r="184" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A184" s="4">
-        <v>18.199999999999989</v>
+        <v>75.833333333333329</v>
       </c>
       <c r="B184" s="4">
         <v>89.096000000000004</v>
@@ -20088,10 +20273,11 @@
       <c r="E184" s="4">
         <v>93.117000000000004</v>
       </c>
-    </row>
-    <row r="185" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F184" s="4"/>
+    </row>
+    <row r="185" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A185" s="4">
-        <v>18.29999999999999</v>
+        <v>76.25</v>
       </c>
       <c r="B185" s="4">
         <v>89.341000000000008</v>
@@ -20105,10 +20291,11 @@
       <c r="E185" s="4">
         <v>93.272999999999996</v>
       </c>
-    </row>
-    <row r="186" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F185" s="4"/>
+    </row>
+    <row r="186" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A186" s="4">
-        <v>18.399999999999991</v>
+        <v>76.666666666666657</v>
       </c>
       <c r="B186" s="4">
         <v>89.584000000000003</v>
@@ -20122,10 +20309,11 @@
       <c r="E186" s="4">
         <v>93.427999999999997</v>
       </c>
-    </row>
-    <row r="187" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F186" s="4"/>
+    </row>
+    <row r="187" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A187" s="4">
-        <v>18.499999999999993</v>
+        <v>77.083333333333343</v>
       </c>
       <c r="B187" s="4">
         <v>89.825000000000003</v>
@@ -20139,10 +20327,11 @@
       <c r="E187" s="4">
         <v>93.581000000000003</v>
       </c>
-    </row>
-    <row r="188" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F187" s="4"/>
+    </row>
+    <row r="188" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A188" s="4">
-        <v>18.599999999999994</v>
+        <v>77.5</v>
       </c>
       <c r="B188" s="4">
         <v>90.063999999999993</v>
@@ -20156,10 +20345,11 @@
       <c r="E188" s="4">
         <v>93.733000000000004</v>
       </c>
-    </row>
-    <row r="189" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F188" s="4"/>
+    </row>
+    <row r="189" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A189" s="4">
-        <v>18.699999999999996</v>
+        <v>77.916666666666671</v>
       </c>
       <c r="B189" s="4">
         <v>90.301000000000002</v>
@@ -20173,10 +20363,11 @@
       <c r="E189" s="4">
         <v>93.88300000000001</v>
       </c>
-    </row>
-    <row r="190" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F189" s="4"/>
+    </row>
+    <row r="190" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A190" s="4">
-        <v>18.799999999999997</v>
+        <v>78.333333333333329</v>
       </c>
       <c r="B190" s="4">
         <v>90.536000000000001</v>
@@ -20190,10 +20381,11 @@
       <c r="E190" s="4">
         <v>94.032000000000011</v>
       </c>
-    </row>
-    <row r="191" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F190" s="4"/>
+    </row>
+    <row r="191" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A191" s="4">
-        <v>18.899999999999999</v>
+        <v>78.75</v>
       </c>
       <c r="B191" s="4">
         <v>90.769000000000005</v>
@@ -20207,10 +20399,11 @@
       <c r="E191" s="4">
         <v>94.179000000000002</v>
       </c>
-    </row>
-    <row r="192" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F191" s="4"/>
+    </row>
+    <row r="192" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A192" s="4">
-        <v>19</v>
+        <v>79.166666666666657</v>
       </c>
       <c r="B192" s="4">
         <v>91</v>
@@ -20224,10 +20417,11 @@
       <c r="E192" s="4">
         <v>94.325000000000003</v>
       </c>
-    </row>
-    <row r="193" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F192" s="4"/>
+    </row>
+    <row r="193" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A193" s="4">
-        <v>19.100000000000001</v>
+        <v>79.583333333333343</v>
       </c>
       <c r="B193" s="4">
         <v>91.228999999999999</v>
@@ -20241,10 +20435,11 @@
       <c r="E193" s="4">
         <v>94.469000000000008</v>
       </c>
-    </row>
-    <row r="194" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F193" s="4"/>
+    </row>
+    <row r="194" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A194" s="4">
-        <v>19.200000000000003</v>
+        <v>80</v>
       </c>
       <c r="B194" s="4">
         <v>91.456000000000003</v>
@@ -20258,10 +20453,11 @@
       <c r="E194" s="4">
         <v>94.611999999999995</v>
       </c>
-    </row>
-    <row r="195" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F194" s="4"/>
+    </row>
+    <row r="195" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A195" s="4">
-        <v>19.300000000000004</v>
+        <v>80.416666666666671</v>
       </c>
       <c r="B195" s="4">
         <v>91.680999999999997</v>
@@ -20275,10 +20471,11 @@
       <c r="E195" s="4">
         <v>94.753</v>
       </c>
-    </row>
-    <row r="196" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F195" s="4"/>
+    </row>
+    <row r="196" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A196" s="4">
-        <v>19.400000000000006</v>
+        <v>80.833333333333329</v>
       </c>
       <c r="B196" s="4">
         <v>91.903999999999996</v>
@@ -20292,10 +20489,11 @@
       <c r="E196" s="4">
         <v>94.893000000000001</v>
       </c>
-    </row>
-    <row r="197" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F196" s="4"/>
+    </row>
+    <row r="197" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A197" s="4">
-        <v>19.500000000000007</v>
+        <v>81.25</v>
       </c>
       <c r="B197" s="4">
         <v>92.125</v>
@@ -20309,10 +20507,11 @@
       <c r="E197" s="4">
         <v>95.031000000000006</v>
       </c>
-    </row>
-    <row r="198" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F197" s="4"/>
+    </row>
+    <row r="198" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A198" s="4">
-        <v>19.600000000000009</v>
+        <v>81.666666666666671</v>
       </c>
       <c r="B198" s="4">
         <v>92.344000000000008</v>
@@ -20326,10 +20525,11 @@
       <c r="E198" s="4">
         <v>95.167999999999992</v>
       </c>
-    </row>
-    <row r="199" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F198" s="4"/>
+    </row>
+    <row r="199" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A199" s="4">
-        <v>19.70000000000001</v>
+        <v>82.083333333333329</v>
       </c>
       <c r="B199" s="4">
         <v>92.561000000000007</v>
@@ -20343,10 +20543,11 @@
       <c r="E199" s="4">
         <v>95.302999999999997</v>
       </c>
-    </row>
-    <row r="200" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F199" s="4"/>
+    </row>
+    <row r="200" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A200" s="4">
-        <v>19.800000000000011</v>
+        <v>82.5</v>
       </c>
       <c r="B200" s="4">
         <v>92.775999999999996</v>
@@ -20360,10 +20561,11 @@
       <c r="E200" s="4">
         <v>95.437000000000012</v>
       </c>
-    </row>
-    <row r="201" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F200" s="4"/>
+    </row>
+    <row r="201" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A201" s="4">
-        <v>19.900000000000013</v>
+        <v>82.916666666666657</v>
       </c>
       <c r="B201" s="4">
         <v>92.989000000000004</v>
@@ -20377,10 +20579,11 @@
       <c r="E201" s="4">
         <v>95.569000000000003</v>
       </c>
-    </row>
-    <row r="202" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F201" s="4"/>
+    </row>
+    <row r="202" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A202" s="4">
-        <v>20.000000000000014</v>
+        <v>83.333333333333343</v>
       </c>
       <c r="B202" s="4">
         <v>93.2</v>
@@ -20394,10 +20597,11 @@
       <c r="E202" s="4">
         <v>95.7</v>
       </c>
-    </row>
-    <row r="203" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F202" s="4"/>
+    </row>
+    <row r="203" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A203" s="4">
-        <v>20.100000000000016</v>
+        <v>83.75</v>
       </c>
       <c r="B203" s="4">
         <v>93.408999999999992</v>
@@ -20411,10 +20615,11 @@
       <c r="E203" s="4">
         <v>95.828999999999994</v>
       </c>
-    </row>
-    <row r="204" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F203" s="4"/>
+    </row>
+    <row r="204" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A204" s="4">
-        <v>20.200000000000017</v>
+        <v>84.166666666666671</v>
       </c>
       <c r="B204" s="4">
         <v>93.616</v>
@@ -20428,10 +20633,11 @@
       <c r="E204" s="4">
         <v>95.957999999999998</v>
       </c>
-    </row>
-    <row r="205" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F204" s="4"/>
+    </row>
+    <row r="205" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A205" s="4">
-        <v>20.300000000000018</v>
+        <v>84.583333333333329</v>
       </c>
       <c r="B205" s="4">
         <v>93.820999999999998</v>
@@ -20445,10 +20651,11 @@
       <c r="E205" s="4">
         <v>96.084999999999994</v>
       </c>
-    </row>
-    <row r="206" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F205" s="4"/>
+    </row>
+    <row r="206" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A206" s="4">
-        <v>20.40000000000002</v>
+        <v>85</v>
       </c>
       <c r="B206" s="4">
         <v>94.024000000000001</v>
@@ -20462,10 +20669,11 @@
       <c r="E206" s="4">
         <v>96.210999999999999</v>
       </c>
-    </row>
-    <row r="207" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F206" s="4"/>
+    </row>
+    <row r="207" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A207" s="4">
-        <v>20.500000000000021</v>
+        <v>85.416666666666657</v>
       </c>
       <c r="B207" s="4">
         <v>94.225000000000009</v>
@@ -20479,10 +20687,11 @@
       <c r="E207" s="4">
         <v>96.335999999999999</v>
       </c>
-    </row>
-    <row r="208" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F207" s="4"/>
+    </row>
+    <row r="208" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A208" s="4">
-        <v>20.600000000000023</v>
+        <v>85.833333333333343</v>
       </c>
       <c r="B208" s="4">
         <v>94.423999999999992</v>
@@ -20496,10 +20705,11 @@
       <c r="E208" s="4">
         <v>96.460000000000008</v>
       </c>
-    </row>
-    <row r="209" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F208" s="4"/>
+    </row>
+    <row r="209" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A209" s="4">
-        <v>20.700000000000024</v>
+        <v>86.25</v>
       </c>
       <c r="B209" s="4">
         <v>94.620999999999995</v>
@@ -20513,10 +20723,11 @@
       <c r="E209" s="4">
         <v>96.582000000000008</v>
       </c>
-    </row>
-    <row r="210" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F209" s="4"/>
+    </row>
+    <row r="210" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A210" s="4">
-        <v>20.800000000000026</v>
+        <v>86.666666666666671</v>
       </c>
       <c r="B210" s="4">
         <v>94.816000000000003</v>
@@ -20530,10 +20741,11 @@
       <c r="E210" s="4">
         <v>96.704000000000008</v>
       </c>
-    </row>
-    <row r="211" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F210" s="4"/>
+    </row>
+    <row r="211" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A211" s="4">
-        <v>20.900000000000027</v>
+        <v>87.083333333333329</v>
       </c>
       <c r="B211" s="4">
         <v>95.009</v>
@@ -20547,10 +20759,11 @@
       <c r="E211" s="4">
         <v>96.823999999999998</v>
       </c>
-    </row>
-    <row r="212" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F211" s="4"/>
+    </row>
+    <row r="212" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A212" s="4">
-        <v>21.000000000000028</v>
+        <v>87.5</v>
       </c>
       <c r="B212" s="4">
         <v>95.199999999999989</v>
@@ -20564,10 +20777,11 @@
       <c r="E212" s="4">
         <v>96.944000000000003</v>
       </c>
-    </row>
-    <row r="213" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F212" s="4"/>
+    </row>
+    <row r="213" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A213" s="4">
-        <v>21.10000000000003</v>
+        <v>87.916666666666671</v>
       </c>
       <c r="B213" s="4">
         <v>95.388999999999996</v>
@@ -20581,10 +20795,11 @@
       <c r="E213" s="4">
         <v>97.061999999999998</v>
       </c>
-    </row>
-    <row r="214" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F213" s="4"/>
+    </row>
+    <row r="214" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A214" s="4">
-        <v>21.200000000000031</v>
+        <v>88.333333333333329</v>
       </c>
       <c r="B214" s="4">
         <v>95.576000000000008</v>
@@ -20598,10 +20813,11 @@
       <c r="E214" s="4">
         <v>97.179000000000002</v>
       </c>
-    </row>
-    <row r="215" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F214" s="4"/>
+    </row>
+    <row r="215" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A215" s="4">
-        <v>21.300000000000033</v>
+        <v>88.75</v>
       </c>
       <c r="B215" s="4">
         <v>95.760999999999996</v>
@@ -20615,10 +20831,11 @@
       <c r="E215" s="4">
         <v>97.295000000000002</v>
       </c>
-    </row>
-    <row r="216" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F215" s="4"/>
+    </row>
+    <row r="216" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A216" s="4">
-        <v>21.400000000000034</v>
+        <v>89.166666666666657</v>
       </c>
       <c r="B216" s="4">
         <v>95.944000000000003</v>
@@ -20632,10 +20849,11 @@
       <c r="E216" s="4">
         <v>97.41</v>
       </c>
-    </row>
-    <row r="217" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F216" s="4"/>
+    </row>
+    <row r="217" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A217" s="4">
-        <v>21.500000000000036</v>
+        <v>89.583333333333343</v>
       </c>
       <c r="B217" s="4">
         <v>96.125</v>
@@ -20649,10 +20867,11 @@
       <c r="E217" s="4">
         <v>97.52300000000001</v>
       </c>
-    </row>
-    <row r="218" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F217" s="4"/>
+    </row>
+    <row r="218" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A218" s="4">
-        <v>21.600000000000037</v>
+        <v>90</v>
       </c>
       <c r="B218" s="4">
         <v>96.304000000000002</v>
@@ -20666,10 +20885,11 @@
       <c r="E218" s="4">
         <v>97.635999999999996</v>
       </c>
-    </row>
-    <row r="219" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F218" s="4"/>
+    </row>
+    <row r="219" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A219" s="4">
-        <v>21.700000000000038</v>
+        <v>90.416666666666671</v>
       </c>
       <c r="B219" s="4">
         <v>96.480999999999995</v>
@@ -20683,10 +20903,11 @@
       <c r="E219" s="4">
         <v>97.747</v>
       </c>
-    </row>
-    <row r="220" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F219" s="4"/>
+    </row>
+    <row r="220" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A220" s="4">
-        <v>21.80000000000004</v>
+        <v>90.833333333333329</v>
       </c>
       <c r="B220" s="4">
         <v>96.655999999999992</v>
@@ -20700,10 +20921,11 @@
       <c r="E220" s="4">
         <v>97.858000000000004</v>
       </c>
-    </row>
-    <row r="221" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F220" s="4"/>
+    </row>
+    <row r="221" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A221" s="4">
-        <v>21.900000000000041</v>
+        <v>91.25</v>
       </c>
       <c r="B221" s="4">
         <v>96.828999999999994</v>
@@ -20717,10 +20939,11 @@
       <c r="E221" s="4">
         <v>97.966999999999999</v>
       </c>
-    </row>
-    <row r="222" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F221" s="4"/>
+    </row>
+    <row r="222" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A222" s="4">
-        <v>22.000000000000043</v>
+        <v>91.666666666666657</v>
       </c>
       <c r="B222" s="4">
         <v>97</v>
@@ -20734,10 +20957,11 @@
       <c r="E222" s="4">
         <v>98.075000000000003</v>
       </c>
-    </row>
-    <row r="223" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F222" s="4"/>
+    </row>
+    <row r="223" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A223" s="4">
-        <v>22.100000000000044</v>
+        <v>92.083333333333343</v>
       </c>
       <c r="B223" s="4">
         <v>97.169000000000011</v>
@@ -20751,10 +20975,11 @@
       <c r="E223" s="4">
         <v>98.182000000000002</v>
       </c>
-    </row>
-    <row r="224" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F223" s="4"/>
+    </row>
+    <row r="224" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A224" s="4">
-        <v>22.200000000000045</v>
+        <v>92.5</v>
       </c>
       <c r="B224" s="4">
         <v>97.335999999999999</v>
@@ -20768,10 +20993,11 @@
       <c r="E224" s="4">
         <v>98.287999999999997</v>
       </c>
-    </row>
-    <row r="225" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F224" s="4"/>
+    </row>
+    <row r="225" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A225" s="4">
-        <v>22.300000000000047</v>
+        <v>92.916666666666671</v>
       </c>
       <c r="B225" s="4">
         <v>97.501000000000005</v>
@@ -20785,10 +21011,11 @@
       <c r="E225" s="4">
         <v>98.391999999999996</v>
       </c>
-    </row>
-    <row r="226" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F225" s="4"/>
+    </row>
+    <row r="226" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A226" s="4">
-        <v>22.400000000000048</v>
+        <v>93.333333333333329</v>
       </c>
       <c r="B226" s="4">
         <v>97.664000000000001</v>
@@ -20802,10 +21029,11 @@
       <c r="E226" s="4">
         <v>98.495999999999995</v>
       </c>
-    </row>
-    <row r="227" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F226" s="4"/>
+    </row>
+    <row r="227" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A227" s="4">
-        <v>22.50000000000005</v>
+        <v>93.75</v>
       </c>
       <c r="B227" s="4">
         <v>97.824999999999989</v>
@@ -20819,10 +21047,11 @@
       <c r="E227" s="4">
         <v>98.597999999999999</v>
       </c>
-    </row>
-    <row r="228" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F227" s="4"/>
+    </row>
+    <row r="228" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A228" s="4">
-        <v>22.600000000000051</v>
+        <v>94.166666666666671</v>
       </c>
       <c r="B228" s="4">
         <v>97.984000000000009</v>
@@ -20836,10 +21065,11 @@
       <c r="E228" s="4">
         <v>98.7</v>
       </c>
-    </row>
-    <row r="229" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F228" s="4"/>
+    </row>
+    <row r="229" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A229" s="4">
-        <v>22.700000000000053</v>
+        <v>94.583333333333329</v>
       </c>
       <c r="B229" s="4">
         <v>98.141000000000005</v>
@@ -20853,10 +21083,11 @@
       <c r="E229" s="4">
         <v>98.8</v>
       </c>
-    </row>
-    <row r="230" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F229" s="4"/>
+    </row>
+    <row r="230" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A230" s="4">
-        <v>22.800000000000054</v>
+        <v>95</v>
       </c>
       <c r="B230" s="4">
         <v>98.295999999999992</v>
@@ -20870,10 +21101,11 @@
       <c r="E230" s="4">
         <v>98.899000000000001</v>
       </c>
-    </row>
-    <row r="231" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F230" s="4"/>
+    </row>
+    <row r="231" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A231" s="4">
-        <v>22.900000000000055</v>
+        <v>95.416666666666657</v>
       </c>
       <c r="B231" s="4">
         <v>98.448999999999998</v>
@@ -20887,10 +21119,11 @@
       <c r="E231" s="4">
         <v>98.997</v>
       </c>
-    </row>
-    <row r="232" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F231" s="4"/>
+    </row>
+    <row r="232" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A232" s="4">
-        <v>23.000000000000057</v>
+        <v>95.833333333333343</v>
       </c>
       <c r="B232" s="4">
         <v>98.6</v>
@@ -20904,10 +21137,11 @@
       <c r="E232" s="4">
         <v>99.094000000000008</v>
       </c>
-    </row>
-    <row r="233" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F232" s="4"/>
+    </row>
+    <row r="233" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A233" s="4">
-        <v>23.100000000000058</v>
+        <v>96.25</v>
       </c>
       <c r="B233" s="4">
         <v>98.748999999999995</v>
@@ -20921,10 +21155,11 @@
       <c r="E233" s="4">
         <v>99.189000000000007</v>
       </c>
-    </row>
-    <row r="234" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F233" s="4"/>
+    </row>
+    <row r="234" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A234" s="4">
-        <v>23.20000000000006</v>
+        <v>96.666666666666671</v>
       </c>
       <c r="B234" s="4">
         <v>98.896000000000001</v>
@@ -20938,10 +21173,11 @@
       <c r="E234" s="4">
         <v>99.283999999999992</v>
       </c>
-    </row>
-    <row r="235" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F234" s="4"/>
+    </row>
+    <row r="235" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A235" s="4">
-        <v>23.300000000000061</v>
+        <v>97.083333333333329</v>
       </c>
       <c r="B235" s="4">
         <v>99.040999999999997</v>
@@ -20955,10 +21191,11 @@
       <c r="E235" s="4">
         <v>99.37700000000001</v>
       </c>
-    </row>
-    <row r="236" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F235" s="4"/>
+    </row>
+    <row r="236" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A236" s="4">
-        <v>23.400000000000063</v>
+        <v>97.5</v>
       </c>
       <c r="B236" s="4">
         <v>99.184000000000012</v>
@@ -20972,10 +21209,11 @@
       <c r="E236" s="4">
         <v>99.47</v>
       </c>
-    </row>
-    <row r="237" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F236" s="4"/>
+    </row>
+    <row r="237" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A237" s="4">
-        <v>23.500000000000064</v>
+        <v>97.916666666666657</v>
       </c>
       <c r="B237" s="4">
         <v>99.325000000000003</v>
@@ -20989,10 +21227,11 @@
       <c r="E237" s="4">
         <v>99.560999999999993</v>
       </c>
-    </row>
-    <row r="238" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F237" s="4"/>
+    </row>
+    <row r="238" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A238" s="4">
-        <v>23.600000000000065</v>
+        <v>98.333333333333343</v>
       </c>
       <c r="B238" s="4">
         <v>99.463999999999999</v>
@@ -21006,10 +21245,11 @@
       <c r="E238" s="4">
         <v>99.650999999999996</v>
       </c>
-    </row>
-    <row r="239" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F238" s="4"/>
+    </row>
+    <row r="239" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A239" s="4">
-        <v>23.700000000000067</v>
+        <v>98.75</v>
       </c>
       <c r="B239" s="4">
         <v>99.600999999999999</v>
@@ -21023,10 +21263,11 @@
       <c r="E239" s="4">
         <v>99.74</v>
       </c>
-    </row>
-    <row r="240" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F239" s="4"/>
+    </row>
+    <row r="240" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A240" s="4">
-        <v>23.800000000000068</v>
+        <v>99.166666666666671</v>
       </c>
       <c r="B240" s="4">
         <v>99.736000000000004</v>
@@ -21040,10 +21281,11 @@
       <c r="E240" s="4">
         <v>99.827999999999989</v>
       </c>
-    </row>
-    <row r="241" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F240" s="4"/>
+    </row>
+    <row r="241" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A241" s="4">
-        <v>23.90000000000007</v>
+        <v>99.583333333333329</v>
       </c>
       <c r="B241" s="4">
         <v>99.869</v>
@@ -21057,10 +21299,11 @@
       <c r="E241" s="4">
         <v>99.914000000000001</v>
       </c>
-    </row>
-    <row r="242" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F241" s="4"/>
+    </row>
+    <row r="242" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A242" s="4">
-        <v>24.000000000000071</v>
+        <v>100</v>
       </c>
       <c r="B242" s="4">
         <v>100</v>
@@ -21074,6 +21317,7 @@
       <c r="E242" s="4">
         <v>100</v>
       </c>
+      <c r="F242" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Cambio en calculo Tb y UPDATE codigo con calculo Ratios HU y lista de tiempos
</commit_message>
<xml_diff>
--- a/Inputs.xlsx
+++ b/Inputs.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Codigos\HU_SCS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72404BA4-EBF0-4ED1-9610-FA9E114747AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{20375231-82F5-4FFA-A8A3-DAA884BF7866}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Info Cuencas" sheetId="1" r:id="rId1"/>
@@ -18,6 +18,7 @@
     <sheet name="Pp Max" sheetId="3" r:id="rId3"/>
     <sheet name="CD" sheetId="4" r:id="rId4"/>
     <sheet name="DT_USCS" sheetId="5" r:id="rId5"/>
+    <sheet name="Ratios" sheetId="6" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -62,7 +63,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="34">
   <si>
     <t>Cuenca</t>
   </si>
@@ -156,6 +157,15 @@
   <si>
     <t>% Tiempo</t>
   </si>
+  <si>
+    <t>Time ratios (t/Tp)</t>
+  </si>
+  <si>
+    <t>Discharge ratios (q/qp)</t>
+  </si>
+  <si>
+    <t>Mass curve ratios (Qa/Q)</t>
+  </si>
 </sst>
 </file>
 
@@ -214,7 +224,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -249,6 +259,8 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -9194,7 +9206,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7ED18635-56AF-4151-A8F0-4CF2F4B95CB7}">
   <sheetPr codeName="Sheet2"/>
-  <dimension ref="A1:G100"/>
+  <dimension ref="A1:I100"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14.6640625" customWidth="1"/>
@@ -9203,7 +9215,7 @@
     <col min="16" max="16" width="11" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="55.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" ht="55.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="7" t="s">
         <v>0</v>
       </c>
@@ -9223,7 +9235,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A2),"",'Info Cuencas'!A2)</f>
         <v>C_01_CL</v>
@@ -9240,16 +9252,17 @@
         <v>3.4568774162111535</v>
       </c>
       <c r="E2" s="6">
-        <f>IF(A2="","",2.67*D2)</f>
-        <v>9.2298627012837802</v>
+        <f>IF(A2="","",5*D2)</f>
+        <v>17.284387081055769</v>
       </c>
       <c r="F2" s="6">
         <f>IF(A2="","",0.208*'Info Cuencas'!B2/HUS!D2)</f>
         <v>7.0561854133476336</v>
       </c>
       <c r="G2" s="6"/>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="I2" s="5"/>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A3),"",'Info Cuencas'!A3)</f>
         <v>C_02_CL</v>
@@ -9266,8 +9279,8 @@
         <v>4.9620108707170507</v>
       </c>
       <c r="E3" s="6">
-        <f t="shared" ref="E3:E11" si="0">IF(A3="","",2.67*D3)</f>
-        <v>13.248569024814525</v>
+        <f>IF(A3="","",5*D3)</f>
+        <v>24.810054353585254</v>
       </c>
       <c r="F3" s="6">
         <f>IF(A3="","",0.208*'Info Cuencas'!B3/HUS!D3)</f>
@@ -9275,7 +9288,7 @@
       </c>
       <c r="G3" s="6"/>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A4" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A4),"",'Info Cuencas'!A4)</f>
         <v/>
@@ -9290,7 +9303,7 @@
         <v/>
       </c>
       <c r="E4" s="6" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" ref="E4" si="0">IF(A4="","",5*D4)</f>
         <v/>
       </c>
       <c r="F4" s="6" t="str">
@@ -9299,7 +9312,7 @@
       </c>
       <c r="G4" s="6"/>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A5" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A5),"",'Info Cuencas'!A5)</f>
         <v/>
@@ -9314,7 +9327,7 @@
         <v/>
       </c>
       <c r="E5" s="6" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(A5="","",5*D5)</f>
         <v/>
       </c>
       <c r="F5" s="6" t="str">
@@ -9323,7 +9336,7 @@
       </c>
       <c r="G5" s="6"/>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A6" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A6),"",'Info Cuencas'!A6)</f>
         <v/>
@@ -9338,7 +9351,7 @@
         <v/>
       </c>
       <c r="E6" s="6" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" ref="E6:E11" si="1">IF(A6="","",5*D6)</f>
         <v/>
       </c>
       <c r="F6" s="6" t="str">
@@ -9347,7 +9360,7 @@
       </c>
       <c r="G6" s="6"/>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A7" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A7),"",'Info Cuencas'!A7)</f>
         <v/>
@@ -9362,7 +9375,7 @@
         <v/>
       </c>
       <c r="E7" s="6" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="F7" s="6" t="str">
@@ -9371,7 +9384,7 @@
       </c>
       <c r="G7" s="6"/>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A8" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A8),"",'Info Cuencas'!A8)</f>
         <v/>
@@ -9386,7 +9399,7 @@
         <v/>
       </c>
       <c r="E8" s="6" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(A8="","",5*D8)</f>
         <v/>
       </c>
       <c r="F8" s="6" t="str">
@@ -9395,7 +9408,7 @@
       </c>
       <c r="G8" s="6"/>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A9" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A9),"",'Info Cuencas'!A9)</f>
         <v/>
@@ -9410,7 +9423,7 @@
         <v/>
       </c>
       <c r="E9" s="6" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="F9" s="6" t="str">
@@ -9419,7 +9432,7 @@
       </c>
       <c r="G9" s="6"/>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A10" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A10),"",'Info Cuencas'!A10)</f>
         <v/>
@@ -9434,7 +9447,7 @@
         <v/>
       </c>
       <c r="E10" s="6" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="F10" s="6" t="str">
@@ -9443,7 +9456,7 @@
       </c>
       <c r="G10" s="6"/>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A11" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A11),"",'Info Cuencas'!A11)</f>
         <v/>
@@ -9458,7 +9471,7 @@
         <v/>
       </c>
       <c r="E11" s="6" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="F11" s="6" t="str">
@@ -9467,7 +9480,7 @@
       </c>
       <c r="G11" s="6"/>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A12" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A12),"",'Info Cuencas'!A12)</f>
         <v/>
@@ -9482,7 +9495,7 @@
         <v/>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A13" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A13),"",'Info Cuencas'!A13)</f>
         <v/>
@@ -9497,7 +9510,7 @@
         <v/>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A14" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A14),"",'Info Cuencas'!A14)</f>
         <v/>
@@ -9512,7 +9525,7 @@
         <v/>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A15" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A15),"",'Info Cuencas'!A15)</f>
         <v/>
@@ -9526,7 +9539,7 @@
         <v/>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A16" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A16),"",'Info Cuencas'!A16)</f>
         <v/>
@@ -10723,6 +10736,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4529BBB4-B484-4DEC-873C-57082AA401DF}">
+  <sheetPr codeName="Sheet3"/>
   <dimension ref="A1:ALL10"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
@@ -13835,6 +13849,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F0A2C426-DF10-4E3D-8B05-2AE55E972C60}">
+  <sheetPr codeName="Sheet4"/>
   <dimension ref="A1:ALL11"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
@@ -16958,6 +16973,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CC7FBFDF-ABB4-4287-9F76-768D0CF54D44}">
+  <sheetPr codeName="Sheet5"/>
   <dimension ref="A1:F242"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -21324,18 +21340,392 @@
 </worksheet>
 </file>
 
-<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="40414187-dd76-4ef8-b04f-ccddae734140" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="63768118-86e2-4829-8a12-b72c47658d02">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{999D9F95-56CA-420C-A8F3-E6555BAE56CD}">
+  <sheetPr codeName="Sheet6"/>
+  <dimension ref="A1:C34"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>31</v>
+      </c>
+      <c r="B1" t="s">
+        <v>32</v>
+      </c>
+      <c r="C1" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" s="14">
+        <v>0</v>
+      </c>
+      <c r="B2" s="15">
+        <v>0</v>
+      </c>
+      <c r="C2" s="15">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3">
+        <v>0.1</v>
+      </c>
+      <c r="B3" s="15">
+        <v>0.03</v>
+      </c>
+      <c r="C3">
+        <v>1E-3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4">
+        <v>0.2</v>
+      </c>
+      <c r="B4" s="15">
+        <v>0.1</v>
+      </c>
+      <c r="C4">
+        <v>6.0000000000000001E-3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5">
+        <v>0.3</v>
+      </c>
+      <c r="B5" s="15">
+        <v>0.19</v>
+      </c>
+      <c r="C5">
+        <v>1.7000000000000001E-2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6">
+        <v>0.4</v>
+      </c>
+      <c r="B6" s="15">
+        <v>0.31</v>
+      </c>
+      <c r="C6">
+        <v>3.5000000000000003E-2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7">
+        <v>0.5</v>
+      </c>
+      <c r="B7" s="15">
+        <v>0.47</v>
+      </c>
+      <c r="C7">
+        <v>6.5000000000000002E-2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8">
+        <v>0.6</v>
+      </c>
+      <c r="B8" s="15">
+        <v>0.66</v>
+      </c>
+      <c r="C8">
+        <v>0.107</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A9">
+        <v>0.7</v>
+      </c>
+      <c r="B9" s="15">
+        <v>0.82</v>
+      </c>
+      <c r="C9">
+        <v>0.16300000000000001</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A10">
+        <v>0.8</v>
+      </c>
+      <c r="B10" s="15">
+        <v>0.93</v>
+      </c>
+      <c r="C10" s="15">
+        <v>0.22800000000000001</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A11">
+        <v>0.9</v>
+      </c>
+      <c r="B11" s="15">
+        <v>0.99</v>
+      </c>
+      <c r="C11" s="15">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A12" s="14">
+        <v>1</v>
+      </c>
+      <c r="B12" s="15">
+        <v>1</v>
+      </c>
+      <c r="C12">
+        <v>0.375</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A13">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="B13" s="15">
+        <v>0.99</v>
+      </c>
+      <c r="C13" s="15">
+        <v>0.45</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A14">
+        <v>1.2</v>
+      </c>
+      <c r="B14" s="15">
+        <v>0.93</v>
+      </c>
+      <c r="C14">
+        <v>0.52200000000000002</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A15">
+        <v>1.3</v>
+      </c>
+      <c r="B15" s="15">
+        <v>0.86</v>
+      </c>
+      <c r="C15">
+        <v>0.58899999999999997</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A16">
+        <v>1.4</v>
+      </c>
+      <c r="B16" s="15">
+        <v>0.78</v>
+      </c>
+      <c r="C16" s="15">
+        <v>0.65</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A17">
+        <v>1.5</v>
+      </c>
+      <c r="B17" s="15">
+        <v>0.68</v>
+      </c>
+      <c r="C17">
+        <v>0.70499999999999996</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A18">
+        <v>1.6</v>
+      </c>
+      <c r="B18" s="15">
+        <v>0.56000000000000005</v>
+      </c>
+      <c r="C18">
+        <v>0.751</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A19">
+        <v>1.7</v>
+      </c>
+      <c r="B19" s="15">
+        <v>0.46</v>
+      </c>
+      <c r="C19" s="15">
+        <v>0.79</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A20">
+        <v>1.8</v>
+      </c>
+      <c r="B20" s="15">
+        <v>0.39</v>
+      </c>
+      <c r="C20">
+        <v>0.82199999999999995</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A21">
+        <v>1.9</v>
+      </c>
+      <c r="B21" s="15">
+        <v>0.33</v>
+      </c>
+      <c r="C21">
+        <v>0.84899999999999998</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A22" s="14">
+        <v>2</v>
+      </c>
+      <c r="B22" s="15">
+        <v>0.28000000000000003</v>
+      </c>
+      <c r="C22">
+        <v>0.871</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A23">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="B23" s="15">
+        <v>0.20699999999999999</v>
+      </c>
+      <c r="C23">
+        <v>0.90800000000000003</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A24">
+        <v>2.4</v>
+      </c>
+      <c r="B24" s="15">
+        <v>0.14699999999999999</v>
+      </c>
+      <c r="C24">
+        <v>0.93400000000000005</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A25">
+        <v>2.6</v>
+      </c>
+      <c r="B25" s="15">
+        <v>0.107</v>
+      </c>
+      <c r="C25">
+        <v>0.95299999999999996</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A26">
+        <v>2.8</v>
+      </c>
+      <c r="B26" s="15">
+        <v>7.6999999999999999E-2</v>
+      </c>
+      <c r="C26">
+        <v>0.96699999999999997</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A27" s="14">
+        <v>3</v>
+      </c>
+      <c r="B27" s="15">
+        <v>5.5E-2</v>
+      </c>
+      <c r="C27">
+        <v>0.97699999999999998</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A28">
+        <v>3.2</v>
+      </c>
+      <c r="B28" s="15">
+        <v>0.04</v>
+      </c>
+      <c r="C28">
+        <v>0.98399999999999999</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A29">
+        <v>3.4</v>
+      </c>
+      <c r="B29" s="15">
+        <v>2.9000000000000001E-2</v>
+      </c>
+      <c r="C29">
+        <v>0.98899999999999999</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A30">
+        <v>3.6</v>
+      </c>
+      <c r="B30" s="15">
+        <v>2.1000000000000001E-2</v>
+      </c>
+      <c r="C30">
+        <v>0.99299999999999999</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A31">
+        <v>3.8</v>
+      </c>
+      <c r="B31" s="15">
+        <v>1.4999999999999999E-2</v>
+      </c>
+      <c r="C31">
+        <v>0.995</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A32" s="14">
+        <v>4</v>
+      </c>
+      <c r="B32" s="15">
+        <v>1.0999999999999999E-2</v>
+      </c>
+      <c r="C32">
+        <v>0.997</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A33">
+        <v>4.5</v>
+      </c>
+      <c r="B33" s="15">
+        <v>5.0000000000000001E-3</v>
+      </c>
+      <c r="C33">
+        <v>0.999</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A34" s="14">
+        <v>5</v>
+      </c>
+      <c r="B34" s="15">
+        <v>0</v>
+      </c>
+      <c r="C34" s="15">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100CCB1C2B958A07241A317F5A881DFD30C" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ec29f518eb9a62149baea9c73f5411cd">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="63768118-86e2-4829-8a12-b72c47658d02" xmlns:ns3="40414187-dd76-4ef8-b04f-ccddae734140" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="29f6242226419d82ce7554acb1ee2c31" ns2:_="" ns3:_="">
     <xsd:import namespace="63768118-86e2-4829-8a12-b72c47658d02"/>
@@ -21590,7 +21980,7 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
@@ -21599,18 +21989,18 @@
 </FormTemplates>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2A4DA3E6-B8B6-48A6-81EC-CAAD4DEE707B}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="40414187-dd76-4ef8-b04f-ccddae734140"/>
-    <ds:schemaRef ds:uri="63768118-86e2-4829-8a12-b72c47658d02"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="40414187-dd76-4ef8-b04f-ccddae734140" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="63768118-86e2-4829-8a12-b72c47658d02">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{124384BF-B442-43EF-BEBD-26F0C03197F3}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -21629,10 +22019,21 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{26BC43C4-0DE4-4398-8C07-F13A3433226F}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2A4DA3E6-B8B6-48A6-81EC-CAAD4DEE707B}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="40414187-dd76-4ef8-b04f-ccddae734140"/>
+    <ds:schemaRef ds:uri="63768118-86e2-4829-8a12-b72c47658d02"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
UPDATE comentario en codigo para cuando se retome
</commit_message>
<xml_diff>
--- a/Inputs.xlsx
+++ b/Inputs.xlsx
@@ -21726,6 +21726,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="40414187-dd76-4ef8-b04f-ccddae734140" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="63768118-86e2-4829-8a12-b72c47658d02">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100CCB1C2B958A07241A317F5A881DFD30C" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ec29f518eb9a62149baea9c73f5411cd">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="63768118-86e2-4829-8a12-b72c47658d02" xmlns:ns3="40414187-dd76-4ef8-b04f-ccddae734140" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="29f6242226419d82ce7554acb1ee2c31" ns2:_="" ns3:_="">
     <xsd:import namespace="63768118-86e2-4829-8a12-b72c47658d02"/>
@@ -21980,27 +22000,26 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2A4DA3E6-B8B6-48A6-81EC-CAAD4DEE707B}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="40414187-dd76-4ef8-b04f-ccddae734140"/>
+    <ds:schemaRef ds:uri="63768118-86e2-4829-8a12-b72c47658d02"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="40414187-dd76-4ef8-b04f-ccddae734140" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="63768118-86e2-4829-8a12-b72c47658d02">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{26BC43C4-0DE4-4398-8C07-F13A3433226F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{124384BF-B442-43EF-BEBD-26F0C03197F3}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -22017,23 +22036,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{26BC43C4-0DE4-4398-8C07-F13A3433226F}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2A4DA3E6-B8B6-48A6-81EC-CAAD4DEE707B}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="40414187-dd76-4ef8-b04f-ccddae734140"/>
-    <ds:schemaRef ds:uri="63768118-86e2-4829-8a12-b72c47658d02"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
UPDATE qp y qp_
</commit_message>
<xml_diff>
--- a/Inputs.xlsx
+++ b/Inputs.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Codigos\HU_SCS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{20375231-82F5-4FFA-A8A3-DAA884BF7866}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0AB5798-EAE0-49E7-B8C5-7742832A7B26}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Info Cuencas" sheetId="1" r:id="rId1"/>
@@ -63,7 +63,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="34">
   <si>
     <t>Cuenca</t>
   </si>
@@ -9206,1526 +9206,1925 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7ED18635-56AF-4151-A8F0-4CF2F4B95CB7}">
   <sheetPr codeName="Sheet2"/>
-  <dimension ref="A1:I100"/>
+  <dimension ref="A1:J100"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14.6640625" customWidth="1"/>
-    <col min="2" max="6" width="12.6640625" customWidth="1"/>
-    <col min="13" max="13" width="10" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="11" bestFit="1" customWidth="1"/>
+    <col min="2" max="7" width="12.6640625" customWidth="1"/>
+    <col min="14" max="14" width="10" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="55.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" ht="55.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="7" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="8" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="C1" s="8" t="s">
+      <c r="D1" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="E1" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="F1" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="G1" s="2" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A2" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A2),"",'Info Cuencas'!A2)</f>
         <v>C_01_CL</v>
       </c>
-      <c r="B2" s="6">
+      <c r="B2" s="4">
+        <f>IF(A2="","",'Info Cuencas'!B2)</f>
+        <v>117.271</v>
+      </c>
+      <c r="C2" s="6">
         <f>IF(A2="","",0.133*'Info Cuencas'!R2)</f>
         <v>0.76073282726013913</v>
       </c>
-      <c r="C2" s="11">
+      <c r="D2" s="11">
         <v>0.05</v>
       </c>
-      <c r="D2" s="6">
-        <f>IF(A2="","",0.6*'Info Cuencas'!R2+HUS!C2/2)</f>
+      <c r="E2" s="6">
+        <f>IF(A2="","",0.6*'Info Cuencas'!R2+HUS!D2/2)</f>
         <v>3.4568774162111535</v>
       </c>
-      <c r="E2" s="6">
-        <f>IF(A2="","",5*D2)</f>
+      <c r="F2" s="6">
+        <f>IF(A2="","",5*E2)</f>
         <v>17.284387081055769</v>
       </c>
-      <c r="F2" s="6">
-        <f>IF(A2="","",0.208*'Info Cuencas'!B2/HUS!D2)</f>
+      <c r="G2" s="6">
+        <f>IF(A2="","",0.208*'Info Cuencas'!B2/HUS!E2)</f>
         <v>7.0561854133476336</v>
       </c>
-      <c r="G2" s="6"/>
-      <c r="I2" s="5"/>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="H2" s="6"/>
+      <c r="J2" s="5"/>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A3),"",'Info Cuencas'!A3)</f>
         <v>C_02_CL</v>
       </c>
-      <c r="B3" s="6">
+      <c r="B3" s="4">
+        <f>IF(A3="","",'Info Cuencas'!B3)</f>
+        <v>447.74</v>
+      </c>
+      <c r="C3" s="6">
         <f>IF(A3="","",0.133*'Info Cuencas'!R3)</f>
         <v>1.0943707430089464</v>
       </c>
-      <c r="C3" s="11">
+      <c r="D3" s="11">
         <v>0.05</v>
       </c>
-      <c r="D3" s="6">
-        <f>IF(A3="","",0.6*'Info Cuencas'!R3+HUS!C3/2)</f>
+      <c r="E3" s="6">
+        <f>IF(A3="","",0.6*'Info Cuencas'!R3+HUS!D3/2)</f>
         <v>4.9620108707170507</v>
       </c>
-      <c r="E3" s="6">
-        <f>IF(A3="","",5*D3)</f>
+      <c r="F3" s="6">
+        <f>IF(A3="","",5*E3)</f>
         <v>24.810054353585254</v>
       </c>
-      <c r="F3" s="6">
-        <f>IF(A3="","",0.208*'Info Cuencas'!B3/HUS!D3)</f>
+      <c r="G3" s="6">
+        <f>IF(A3="","",0.208*'Info Cuencas'!B3/HUS!E3)</f>
         <v>18.768584436120346</v>
       </c>
-      <c r="G3" s="6"/>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="H3" s="6"/>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A4" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A4),"",'Info Cuencas'!A4)</f>
         <v/>
       </c>
-      <c r="B4" s="6" t="str">
+      <c r="B4" s="4" t="str">
+        <f>IF(A4="","",'Info Cuencas'!B4)</f>
+        <v/>
+      </c>
+      <c r="C4" s="6" t="str">
         <f>IF(A4="","",0.133*'Info Cuencas'!R4)</f>
         <v/>
       </c>
-      <c r="C4" s="9"/>
-      <c r="D4" s="6" t="str">
-        <f>IF(A4="","",0.6*'Info Cuencas'!R4+HUS!C4/2)</f>
-        <v/>
-      </c>
+      <c r="D4" s="9"/>
       <c r="E4" s="6" t="str">
-        <f t="shared" ref="E4" si="0">IF(A4="","",5*D4)</f>
+        <f>IF(A4="","",0.6*'Info Cuencas'!R4+HUS!D4/2)</f>
         <v/>
       </c>
       <c r="F4" s="6" t="str">
-        <f>IF(A4="","",0.208*'Info Cuencas'!B4/HUS!D4)</f>
-        <v/>
-      </c>
-      <c r="G4" s="6"/>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
+        <f t="shared" ref="F4" si="0">IF(A4="","",5*E4)</f>
+        <v/>
+      </c>
+      <c r="G4" s="6" t="str">
+        <f>IF(A4="","",0.208*'Info Cuencas'!B4/HUS!E4)</f>
+        <v/>
+      </c>
+      <c r="H4" s="6"/>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A5" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A5),"",'Info Cuencas'!A5)</f>
         <v/>
       </c>
-      <c r="B5" s="6" t="str">
+      <c r="B5" s="4" t="str">
+        <f>IF(A5="","",'Info Cuencas'!B5)</f>
+        <v/>
+      </c>
+      <c r="C5" s="6" t="str">
         <f>IF(A5="","",0.133*'Info Cuencas'!R5)</f>
         <v/>
       </c>
-      <c r="C5" s="9"/>
-      <c r="D5" s="6" t="str">
-        <f>IF(A5="","",0.6*'Info Cuencas'!R5+HUS!C5/2)</f>
-        <v/>
-      </c>
+      <c r="D5" s="9"/>
       <c r="E5" s="6" t="str">
-        <f>IF(A5="","",5*D5)</f>
+        <f>IF(A5="","",0.6*'Info Cuencas'!R5+HUS!D5/2)</f>
         <v/>
       </c>
       <c r="F5" s="6" t="str">
-        <f>IF(A5="","",0.208*'Info Cuencas'!B5/HUS!D5)</f>
-        <v/>
-      </c>
-      <c r="G5" s="6"/>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
+        <f>IF(A5="","",5*E5)</f>
+        <v/>
+      </c>
+      <c r="G5" s="6" t="str">
+        <f>IF(A5="","",0.208*'Info Cuencas'!B5/HUS!E5)</f>
+        <v/>
+      </c>
+      <c r="H5" s="6"/>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A6" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A6),"",'Info Cuencas'!A6)</f>
         <v/>
       </c>
-      <c r="B6" s="6" t="str">
+      <c r="B6" s="4" t="str">
+        <f>IF(A6="","",'Info Cuencas'!B6)</f>
+        <v/>
+      </c>
+      <c r="C6" s="6" t="str">
         <f>IF(A6="","",0.133*'Info Cuencas'!R6)</f>
         <v/>
       </c>
-      <c r="C6" s="9"/>
-      <c r="D6" s="6" t="str">
-        <f>IF(A6="","",0.6*'Info Cuencas'!R6+HUS!C6/2)</f>
-        <v/>
-      </c>
+      <c r="D6" s="9"/>
       <c r="E6" s="6" t="str">
-        <f t="shared" ref="E6:E11" si="1">IF(A6="","",5*D6)</f>
+        <f>IF(A6="","",0.6*'Info Cuencas'!R6+HUS!D6/2)</f>
         <v/>
       </c>
       <c r="F6" s="6" t="str">
-        <f>IF(A6="","",0.208*'Info Cuencas'!B6/HUS!D6)</f>
-        <v/>
-      </c>
-      <c r="G6" s="6"/>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
+        <f t="shared" ref="F6:F11" si="1">IF(A6="","",5*E6)</f>
+        <v/>
+      </c>
+      <c r="G6" s="6" t="str">
+        <f>IF(A6="","",0.208*'Info Cuencas'!B6/HUS!E6)</f>
+        <v/>
+      </c>
+      <c r="H6" s="6"/>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A7" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A7),"",'Info Cuencas'!A7)</f>
         <v/>
       </c>
-      <c r="B7" s="6" t="str">
+      <c r="B7" s="4" t="str">
+        <f>IF(A7="","",'Info Cuencas'!B7)</f>
+        <v/>
+      </c>
+      <c r="C7" s="6" t="str">
         <f>IF(A7="","",0.133*'Info Cuencas'!R7)</f>
         <v/>
       </c>
-      <c r="C7" s="9"/>
-      <c r="D7" s="6" t="str">
-        <f>IF(A7="","",0.6*'Info Cuencas'!R7+HUS!C7/2)</f>
-        <v/>
-      </c>
+      <c r="D7" s="9"/>
       <c r="E7" s="6" t="str">
+        <f>IF(A7="","",0.6*'Info Cuencas'!R7+HUS!D7/2)</f>
+        <v/>
+      </c>
+      <c r="F7" s="6" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="F7" s="6" t="str">
-        <f>IF(A7="","",0.208*'Info Cuencas'!B7/HUS!D7)</f>
-        <v/>
-      </c>
-      <c r="G7" s="6"/>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="G7" s="6" t="str">
+        <f>IF(A7="","",0.208*'Info Cuencas'!B7/HUS!E7)</f>
+        <v/>
+      </c>
+      <c r="H7" s="6"/>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A8" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A8),"",'Info Cuencas'!A8)</f>
         <v/>
       </c>
-      <c r="B8" s="6" t="str">
+      <c r="B8" s="4" t="str">
+        <f>IF(A8="","",'Info Cuencas'!B8)</f>
+        <v/>
+      </c>
+      <c r="C8" s="6" t="str">
         <f>IF(A8="","",0.133*'Info Cuencas'!R8)</f>
         <v/>
       </c>
-      <c r="C8" s="9"/>
-      <c r="D8" s="6" t="str">
-        <f>IF(A8="","",0.6*'Info Cuencas'!R8+HUS!C8/2)</f>
-        <v/>
-      </c>
+      <c r="D8" s="9"/>
       <c r="E8" s="6" t="str">
-        <f>IF(A8="","",5*D8)</f>
+        <f>IF(A8="","",0.6*'Info Cuencas'!R8+HUS!D8/2)</f>
         <v/>
       </c>
       <c r="F8" s="6" t="str">
-        <f>IF(A8="","",0.208*'Info Cuencas'!B8/HUS!D8)</f>
-        <v/>
-      </c>
-      <c r="G8" s="6"/>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
+        <f>IF(A8="","",5*E8)</f>
+        <v/>
+      </c>
+      <c r="G8" s="6" t="str">
+        <f>IF(A8="","",0.208*'Info Cuencas'!B8/HUS!E8)</f>
+        <v/>
+      </c>
+      <c r="H8" s="6"/>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A9" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A9),"",'Info Cuencas'!A9)</f>
         <v/>
       </c>
-      <c r="B9" s="6" t="str">
+      <c r="B9" s="4" t="str">
+        <f>IF(A9="","",'Info Cuencas'!B9)</f>
+        <v/>
+      </c>
+      <c r="C9" s="6" t="str">
         <f>IF(A9="","",0.133*'Info Cuencas'!R9)</f>
         <v/>
       </c>
-      <c r="C9" s="9"/>
-      <c r="D9" s="6" t="str">
-        <f>IF(A9="","",0.6*'Info Cuencas'!R9+HUS!C9/2)</f>
-        <v/>
-      </c>
+      <c r="D9" s="9"/>
       <c r="E9" s="6" t="str">
+        <f>IF(A9="","",0.6*'Info Cuencas'!R9+HUS!D9/2)</f>
+        <v/>
+      </c>
+      <c r="F9" s="6" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="F9" s="6" t="str">
-        <f>IF(A9="","",0.208*'Info Cuencas'!B9/HUS!D9)</f>
-        <v/>
-      </c>
-      <c r="G9" s="6"/>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="G9" s="6" t="str">
+        <f>IF(A9="","",0.208*'Info Cuencas'!B9/HUS!E9)</f>
+        <v/>
+      </c>
+      <c r="H9" s="6"/>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A10" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A10),"",'Info Cuencas'!A10)</f>
         <v/>
       </c>
-      <c r="B10" s="6" t="str">
+      <c r="B10" s="4" t="str">
+        <f>IF(A10="","",'Info Cuencas'!B10)</f>
+        <v/>
+      </c>
+      <c r="C10" s="6" t="str">
         <f>IF(A10="","",0.133*'Info Cuencas'!R10)</f>
         <v/>
       </c>
-      <c r="C10" s="9"/>
-      <c r="D10" s="6" t="str">
-        <f>IF(A10="","",0.6*'Info Cuencas'!R10+HUS!C10/2)</f>
-        <v/>
-      </c>
+      <c r="D10" s="9"/>
       <c r="E10" s="6" t="str">
+        <f>IF(A10="","",0.6*'Info Cuencas'!R10+HUS!D10/2)</f>
+        <v/>
+      </c>
+      <c r="F10" s="6" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="F10" s="6" t="str">
-        <f>IF(A10="","",0.208*'Info Cuencas'!B10/HUS!D10)</f>
-        <v/>
-      </c>
-      <c r="G10" s="6"/>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="G10" s="6" t="str">
+        <f>IF(A10="","",0.208*'Info Cuencas'!B10/HUS!E10)</f>
+        <v/>
+      </c>
+      <c r="H10" s="6"/>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A11" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A11),"",'Info Cuencas'!A11)</f>
         <v/>
       </c>
-      <c r="B11" s="6" t="str">
+      <c r="B11" s="4" t="str">
+        <f>IF(A11="","",'Info Cuencas'!B11)</f>
+        <v/>
+      </c>
+      <c r="C11" s="6" t="str">
         <f>IF(A11="","",0.133*'Info Cuencas'!R11)</f>
         <v/>
       </c>
-      <c r="C11" s="9"/>
-      <c r="D11" s="6" t="str">
-        <f>IF(A11="","",0.6*'Info Cuencas'!R11+HUS!C11/2)</f>
-        <v/>
-      </c>
+      <c r="D11" s="9"/>
       <c r="E11" s="6" t="str">
+        <f>IF(A11="","",0.6*'Info Cuencas'!R11+HUS!D11/2)</f>
+        <v/>
+      </c>
+      <c r="F11" s="6" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="F11" s="6" t="str">
-        <f>IF(A11="","",0.208*'Info Cuencas'!B11/HUS!D11)</f>
-        <v/>
-      </c>
-      <c r="G11" s="6"/>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="G11" s="6" t="str">
+        <f>IF(A11="","",0.208*'Info Cuencas'!B11/HUS!E11)</f>
+        <v/>
+      </c>
+      <c r="H11" s="6"/>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A12" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A12),"",'Info Cuencas'!A12)</f>
         <v/>
       </c>
-      <c r="B12" t="str">
+      <c r="B12" s="4" t="str">
+        <f>IF(A12="","",'Info Cuencas'!B12)</f>
+        <v/>
+      </c>
+      <c r="C12" t="str">
         <f>IF(A12="","",0.133*'Info Cuencas'!R12)</f>
         <v/>
       </c>
-      <c r="C12" s="9"/>
-      <c r="D12" s="6" t="str">
-        <f>IF(A12="","",0.6*'Info Cuencas'!R12+HUS!C12/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="D12" s="9"/>
+      <c r="E12" s="6" t="str">
+        <f>IF(A12="","",0.6*'Info Cuencas'!R12+HUS!D12/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A13" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A13),"",'Info Cuencas'!A13)</f>
         <v/>
       </c>
-      <c r="B13" t="str">
+      <c r="B13" s="4" t="str">
+        <f>IF(A13="","",'Info Cuencas'!B13)</f>
+        <v/>
+      </c>
+      <c r="C13" t="str">
         <f>IF(A13="","",0.133*'Info Cuencas'!R13)</f>
         <v/>
       </c>
-      <c r="C13" s="9"/>
-      <c r="D13" s="6" t="str">
-        <f>IF(A13="","",0.6*'Info Cuencas'!R13+HUS!C13/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="D13" s="9"/>
+      <c r="E13" s="6" t="str">
+        <f>IF(A13="","",0.6*'Info Cuencas'!R13+HUS!D13/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A14" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A14),"",'Info Cuencas'!A14)</f>
         <v/>
       </c>
-      <c r="B14" t="str">
+      <c r="B14" s="4" t="str">
+        <f>IF(A14="","",'Info Cuencas'!B14)</f>
+        <v/>
+      </c>
+      <c r="C14" t="str">
         <f>IF(A14="","",0.133*'Info Cuencas'!R14)</f>
         <v/>
       </c>
-      <c r="C14" s="9"/>
-      <c r="D14" s="6" t="str">
-        <f>IF(A14="","",0.6*'Info Cuencas'!R14+HUS!C14/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="D14" s="9"/>
+      <c r="E14" s="6" t="str">
+        <f>IF(A14="","",0.6*'Info Cuencas'!R14+HUS!D14/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A15" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A15),"",'Info Cuencas'!A15)</f>
         <v/>
       </c>
-      <c r="B15" t="str">
+      <c r="B15" s="4" t="str">
+        <f>IF(A15="","",'Info Cuencas'!B15)</f>
+        <v/>
+      </c>
+      <c r="C15" t="str">
         <f>IF(A15="","",0.133*'Info Cuencas'!R15)</f>
         <v/>
       </c>
-      <c r="D15" s="6" t="str">
-        <f>IF(A15="","",0.6*'Info Cuencas'!R15+HUS!C15/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="E15" s="6" t="str">
+        <f>IF(A15="","",0.6*'Info Cuencas'!R15+HUS!D15/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A16" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A16),"",'Info Cuencas'!A16)</f>
         <v/>
       </c>
-      <c r="B16" t="str">
+      <c r="B16" s="4" t="str">
+        <f>IF(A16="","",'Info Cuencas'!B16)</f>
+        <v/>
+      </c>
+      <c r="C16" t="str">
         <f>IF(A16="","",0.133*'Info Cuencas'!R16)</f>
         <v/>
       </c>
-      <c r="D16" s="6" t="str">
-        <f>IF(A16="","",0.6*'Info Cuencas'!R16+HUS!C16/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E16" s="6" t="str">
+        <f>IF(A16="","",0.6*'Info Cuencas'!R16+HUS!D16/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A17" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A17),"",'Info Cuencas'!A17)</f>
         <v/>
       </c>
-      <c r="B17" t="str">
+      <c r="B17" s="4" t="str">
+        <f>IF(A17="","",'Info Cuencas'!B17)</f>
+        <v/>
+      </c>
+      <c r="C17" t="str">
         <f>IF(A17="","",0.133*'Info Cuencas'!R17)</f>
         <v/>
       </c>
-      <c r="D17" s="6" t="str">
-        <f>IF(A17="","",0.6*'Info Cuencas'!R17+HUS!C17/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E17" s="6" t="str">
+        <f>IF(A17="","",0.6*'Info Cuencas'!R17+HUS!D17/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A18" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A18),"",'Info Cuencas'!A18)</f>
         <v/>
       </c>
-      <c r="B18" t="str">
+      <c r="B18" s="4" t="str">
+        <f>IF(A18="","",'Info Cuencas'!B18)</f>
+        <v/>
+      </c>
+      <c r="C18" t="str">
         <f>IF(A18="","",0.133*'Info Cuencas'!R18)</f>
         <v/>
       </c>
-      <c r="D18" s="6" t="str">
-        <f>IF(A18="","",0.6*'Info Cuencas'!R18+HUS!C18/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E18" s="6" t="str">
+        <f>IF(A18="","",0.6*'Info Cuencas'!R18+HUS!D18/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A19" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A19),"",'Info Cuencas'!A19)</f>
         <v/>
       </c>
-      <c r="B19" t="str">
+      <c r="B19" s="4" t="str">
+        <f>IF(A19="","",'Info Cuencas'!B19)</f>
+        <v/>
+      </c>
+      <c r="C19" t="str">
         <f>IF(A19="","",0.133*'Info Cuencas'!R19)</f>
         <v/>
       </c>
-      <c r="D19" s="6" t="str">
-        <f>IF(A19="","",0.6*'Info Cuencas'!R19+HUS!C19/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E19" s="6" t="str">
+        <f>IF(A19="","",0.6*'Info Cuencas'!R19+HUS!D19/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A20" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A20),"",'Info Cuencas'!A20)</f>
         <v/>
       </c>
-      <c r="B20" t="str">
+      <c r="B20" s="4" t="str">
+        <f>IF(A20="","",'Info Cuencas'!B20)</f>
+        <v/>
+      </c>
+      <c r="C20" t="str">
         <f>IF(A20="","",0.133*'Info Cuencas'!R20)</f>
         <v/>
       </c>
-      <c r="D20" s="6" t="str">
-        <f>IF(A20="","",0.6*'Info Cuencas'!R20+HUS!C20/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E20" s="6" t="str">
+        <f>IF(A20="","",0.6*'Info Cuencas'!R20+HUS!D20/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A21" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A21),"",'Info Cuencas'!A21)</f>
         <v/>
       </c>
-      <c r="B21" t="str">
+      <c r="B21" s="4" t="str">
+        <f>IF(A21="","",'Info Cuencas'!B21)</f>
+        <v/>
+      </c>
+      <c r="C21" t="str">
         <f>IF(A21="","",0.133*'Info Cuencas'!R21)</f>
         <v/>
       </c>
-      <c r="D21" s="6" t="str">
-        <f>IF(A21="","",0.6*'Info Cuencas'!R21+HUS!C21/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E21" s="6" t="str">
+        <f>IF(A21="","",0.6*'Info Cuencas'!R21+HUS!D21/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A22" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A22),"",'Info Cuencas'!A22)</f>
         <v/>
       </c>
-      <c r="B22" t="str">
+      <c r="B22" s="4" t="str">
+        <f>IF(A22="","",'Info Cuencas'!B22)</f>
+        <v/>
+      </c>
+      <c r="C22" t="str">
         <f>IF(A22="","",0.133*'Info Cuencas'!R22)</f>
         <v/>
       </c>
-      <c r="D22" s="6" t="str">
-        <f>IF(A22="","",0.6*'Info Cuencas'!R22+HUS!C22/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E22" s="6" t="str">
+        <f>IF(A22="","",0.6*'Info Cuencas'!R22+HUS!D22/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A23" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A23),"",'Info Cuencas'!A23)</f>
         <v/>
       </c>
-      <c r="B23" t="str">
+      <c r="B23" s="4" t="str">
+        <f>IF(A23="","",'Info Cuencas'!B23)</f>
+        <v/>
+      </c>
+      <c r="C23" t="str">
         <f>IF(A23="","",0.133*'Info Cuencas'!R23)</f>
         <v/>
       </c>
-      <c r="D23" s="6" t="str">
-        <f>IF(A23="","",0.6*'Info Cuencas'!R23+HUS!C23/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E23" s="6" t="str">
+        <f>IF(A23="","",0.6*'Info Cuencas'!R23+HUS!D23/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A24" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A24),"",'Info Cuencas'!A24)</f>
         <v/>
       </c>
-      <c r="B24" t="str">
+      <c r="B24" s="4" t="str">
+        <f>IF(A24="","",'Info Cuencas'!B24)</f>
+        <v/>
+      </c>
+      <c r="C24" t="str">
         <f>IF(A24="","",0.133*'Info Cuencas'!R24)</f>
         <v/>
       </c>
-      <c r="D24" s="6" t="str">
-        <f>IF(A24="","",0.6*'Info Cuencas'!R24+HUS!C24/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E24" s="6" t="str">
+        <f>IF(A24="","",0.6*'Info Cuencas'!R24+HUS!D24/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A25" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A25),"",'Info Cuencas'!A25)</f>
         <v/>
       </c>
-      <c r="B25" t="str">
+      <c r="B25" s="4" t="str">
+        <f>IF(A25="","",'Info Cuencas'!B25)</f>
+        <v/>
+      </c>
+      <c r="C25" t="str">
         <f>IF(A25="","",0.133*'Info Cuencas'!R25)</f>
         <v/>
       </c>
-      <c r="D25" s="6" t="str">
-        <f>IF(A25="","",0.6*'Info Cuencas'!R25+HUS!C25/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E25" s="6" t="str">
+        <f>IF(A25="","",0.6*'Info Cuencas'!R25+HUS!D25/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A26" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A26),"",'Info Cuencas'!A26)</f>
         <v/>
       </c>
-      <c r="B26" t="str">
+      <c r="B26" s="4" t="str">
+        <f>IF(A26="","",'Info Cuencas'!B26)</f>
+        <v/>
+      </c>
+      <c r="C26" t="str">
         <f>IF(A26="","",0.133*'Info Cuencas'!R26)</f>
         <v/>
       </c>
-      <c r="D26" s="6" t="str">
-        <f>IF(A26="","",0.6*'Info Cuencas'!R26+HUS!C26/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E26" s="6" t="str">
+        <f>IF(A26="","",0.6*'Info Cuencas'!R26+HUS!D26/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A27" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A27),"",'Info Cuencas'!A27)</f>
         <v/>
       </c>
-      <c r="B27" t="str">
+      <c r="B27" s="4" t="str">
+        <f>IF(A27="","",'Info Cuencas'!B27)</f>
+        <v/>
+      </c>
+      <c r="C27" t="str">
         <f>IF(A27="","",0.133*'Info Cuencas'!R27)</f>
         <v/>
       </c>
-      <c r="D27" s="6" t="str">
-        <f>IF(A27="","",0.6*'Info Cuencas'!R27+HUS!C27/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E27" s="6" t="str">
+        <f>IF(A27="","",0.6*'Info Cuencas'!R27+HUS!D27/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A28" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A28),"",'Info Cuencas'!A28)</f>
         <v/>
       </c>
-      <c r="B28" t="str">
+      <c r="B28" s="4" t="str">
+        <f>IF(A28="","",'Info Cuencas'!B28)</f>
+        <v/>
+      </c>
+      <c r="C28" t="str">
         <f>IF(A28="","",0.133*'Info Cuencas'!R28)</f>
         <v/>
       </c>
-      <c r="D28" s="6" t="str">
-        <f>IF(A28="","",0.6*'Info Cuencas'!R28+HUS!C28/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E28" s="6" t="str">
+        <f>IF(A28="","",0.6*'Info Cuencas'!R28+HUS!D28/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A29" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A29),"",'Info Cuencas'!A29)</f>
         <v/>
       </c>
-      <c r="B29" t="str">
+      <c r="B29" s="4" t="str">
+        <f>IF(A29="","",'Info Cuencas'!B29)</f>
+        <v/>
+      </c>
+      <c r="C29" t="str">
         <f>IF(A29="","",0.133*'Info Cuencas'!R29)</f>
         <v/>
       </c>
-      <c r="D29" s="6" t="str">
-        <f>IF(A29="","",0.6*'Info Cuencas'!R29+HUS!C29/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E29" s="6" t="str">
+        <f>IF(A29="","",0.6*'Info Cuencas'!R29+HUS!D29/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A30" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A30),"",'Info Cuencas'!A30)</f>
         <v/>
       </c>
-      <c r="B30" t="str">
+      <c r="B30" s="4" t="str">
+        <f>IF(A30="","",'Info Cuencas'!B30)</f>
+        <v/>
+      </c>
+      <c r="C30" t="str">
         <f>IF(A30="","",0.133*'Info Cuencas'!R30)</f>
         <v/>
       </c>
-      <c r="D30" s="6" t="str">
-        <f>IF(A30="","",0.6*'Info Cuencas'!R30+HUS!C30/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E30" s="6" t="str">
+        <f>IF(A30="","",0.6*'Info Cuencas'!R30+HUS!D30/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A31" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A31),"",'Info Cuencas'!A31)</f>
         <v/>
       </c>
-      <c r="B31" t="str">
+      <c r="B31" s="4" t="str">
+        <f>IF(A31="","",'Info Cuencas'!B31)</f>
+        <v/>
+      </c>
+      <c r="C31" t="str">
         <f>IF(A31="","",0.133*'Info Cuencas'!R31)</f>
         <v/>
       </c>
-      <c r="D31" s="6" t="str">
-        <f>IF(A31="","",0.6*'Info Cuencas'!R31+HUS!C31/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E31" s="6" t="str">
+        <f>IF(A31="","",0.6*'Info Cuencas'!R31+HUS!D31/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A32" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A32),"",'Info Cuencas'!A32)</f>
         <v/>
       </c>
-      <c r="B32" t="str">
+      <c r="B32" s="4" t="str">
+        <f>IF(A32="","",'Info Cuencas'!B32)</f>
+        <v/>
+      </c>
+      <c r="C32" t="str">
         <f>IF(A32="","",0.133*'Info Cuencas'!R32)</f>
         <v/>
       </c>
-      <c r="D32" s="6" t="str">
-        <f>IF(A32="","",0.6*'Info Cuencas'!R32+HUS!C32/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E32" s="6" t="str">
+        <f>IF(A32="","",0.6*'Info Cuencas'!R32+HUS!D32/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A33" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A33),"",'Info Cuencas'!A33)</f>
         <v/>
       </c>
-      <c r="B33" t="str">
+      <c r="B33" s="4" t="str">
+        <f>IF(A33="","",'Info Cuencas'!B33)</f>
+        <v/>
+      </c>
+      <c r="C33" t="str">
         <f>IF(A33="","",0.133*'Info Cuencas'!R33)</f>
         <v/>
       </c>
-      <c r="D33" s="6" t="str">
-        <f>IF(A33="","",0.6*'Info Cuencas'!R33+HUS!C33/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E33" s="6" t="str">
+        <f>IF(A33="","",0.6*'Info Cuencas'!R33+HUS!D33/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A34" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A34),"",'Info Cuencas'!A34)</f>
         <v/>
       </c>
-      <c r="B34" t="str">
+      <c r="B34" s="4" t="str">
+        <f>IF(A34="","",'Info Cuencas'!B34)</f>
+        <v/>
+      </c>
+      <c r="C34" t="str">
         <f>IF(A34="","",0.133*'Info Cuencas'!R34)</f>
         <v/>
       </c>
-      <c r="D34" s="6" t="str">
-        <f>IF(A34="","",0.6*'Info Cuencas'!R34+HUS!C34/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E34" s="6" t="str">
+        <f>IF(A34="","",0.6*'Info Cuencas'!R34+HUS!D34/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A35" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A35),"",'Info Cuencas'!A35)</f>
         <v/>
       </c>
-      <c r="B35" t="str">
+      <c r="B35" s="4" t="str">
+        <f>IF(A35="","",'Info Cuencas'!B35)</f>
+        <v/>
+      </c>
+      <c r="C35" t="str">
         <f>IF(A35="","",0.133*'Info Cuencas'!R35)</f>
         <v/>
       </c>
-      <c r="D35" s="6" t="str">
-        <f>IF(A35="","",0.6*'Info Cuencas'!R35+HUS!C35/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E35" s="6" t="str">
+        <f>IF(A35="","",0.6*'Info Cuencas'!R35+HUS!D35/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A36" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A36),"",'Info Cuencas'!A36)</f>
         <v/>
       </c>
-      <c r="B36" t="str">
+      <c r="B36" s="4" t="str">
+        <f>IF(A36="","",'Info Cuencas'!B36)</f>
+        <v/>
+      </c>
+      <c r="C36" t="str">
         <f>IF(A36="","",0.133*'Info Cuencas'!R36)</f>
         <v/>
       </c>
-      <c r="D36" s="6" t="str">
-        <f>IF(A36="","",0.6*'Info Cuencas'!R36+HUS!C36/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E36" s="6" t="str">
+        <f>IF(A36="","",0.6*'Info Cuencas'!R36+HUS!D36/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A37" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A37),"",'Info Cuencas'!A37)</f>
         <v/>
       </c>
-      <c r="B37" t="str">
+      <c r="B37" s="4" t="str">
+        <f>IF(A37="","",'Info Cuencas'!B37)</f>
+        <v/>
+      </c>
+      <c r="C37" t="str">
         <f>IF(A37="","",0.133*'Info Cuencas'!R37)</f>
         <v/>
       </c>
-      <c r="D37" s="6" t="str">
-        <f>IF(A37="","",0.6*'Info Cuencas'!R37+HUS!C37/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E37" s="6" t="str">
+        <f>IF(A37="","",0.6*'Info Cuencas'!R37+HUS!D37/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A38" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A38),"",'Info Cuencas'!A38)</f>
         <v/>
       </c>
-      <c r="B38" t="str">
+      <c r="B38" s="4" t="str">
+        <f>IF(A38="","",'Info Cuencas'!B38)</f>
+        <v/>
+      </c>
+      <c r="C38" t="str">
         <f>IF(A38="","",0.133*'Info Cuencas'!R38)</f>
         <v/>
       </c>
-      <c r="D38" s="6" t="str">
-        <f>IF(A38="","",0.6*'Info Cuencas'!R38+HUS!C38/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E38" s="6" t="str">
+        <f>IF(A38="","",0.6*'Info Cuencas'!R38+HUS!D38/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A39" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A39),"",'Info Cuencas'!A39)</f>
         <v/>
       </c>
-      <c r="B39" t="str">
+      <c r="B39" s="4" t="str">
+        <f>IF(A39="","",'Info Cuencas'!B39)</f>
+        <v/>
+      </c>
+      <c r="C39" t="str">
         <f>IF(A39="","",0.133*'Info Cuencas'!R39)</f>
         <v/>
       </c>
-      <c r="D39" s="6" t="str">
-        <f>IF(A39="","",0.6*'Info Cuencas'!R39+HUS!C39/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E39" s="6" t="str">
+        <f>IF(A39="","",0.6*'Info Cuencas'!R39+HUS!D39/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A40" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A40),"",'Info Cuencas'!A40)</f>
         <v/>
       </c>
-      <c r="B40" t="str">
+      <c r="B40" s="4" t="str">
+        <f>IF(A40="","",'Info Cuencas'!B40)</f>
+        <v/>
+      </c>
+      <c r="C40" t="str">
         <f>IF(A40="","",0.133*'Info Cuencas'!R40)</f>
         <v/>
       </c>
-      <c r="D40" s="6" t="str">
-        <f>IF(A40="","",0.6*'Info Cuencas'!R40+HUS!C40/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E40" s="6" t="str">
+        <f>IF(A40="","",0.6*'Info Cuencas'!R40+HUS!D40/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A41" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A41),"",'Info Cuencas'!A41)</f>
         <v/>
       </c>
-      <c r="B41" t="str">
+      <c r="B41" s="4" t="str">
+        <f>IF(A41="","",'Info Cuencas'!B41)</f>
+        <v/>
+      </c>
+      <c r="C41" t="str">
         <f>IF(A41="","",0.133*'Info Cuencas'!R41)</f>
         <v/>
       </c>
-      <c r="D41" s="6" t="str">
-        <f>IF(A41="","",0.6*'Info Cuencas'!R41+HUS!C41/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E41" s="6" t="str">
+        <f>IF(A41="","",0.6*'Info Cuencas'!R41+HUS!D41/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A42" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A42),"",'Info Cuencas'!A42)</f>
         <v/>
       </c>
-      <c r="B42" t="str">
+      <c r="B42" s="4" t="str">
+        <f>IF(A42="","",'Info Cuencas'!B42)</f>
+        <v/>
+      </c>
+      <c r="C42" t="str">
         <f>IF(A42="","",0.133*'Info Cuencas'!R42)</f>
         <v/>
       </c>
-      <c r="D42" s="6" t="str">
-        <f>IF(A42="","",0.6*'Info Cuencas'!R42+HUS!C42/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E42" s="6" t="str">
+        <f>IF(A42="","",0.6*'Info Cuencas'!R42+HUS!D42/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A43" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A43),"",'Info Cuencas'!A43)</f>
         <v/>
       </c>
-      <c r="B43" t="str">
+      <c r="B43" s="4" t="str">
+        <f>IF(A43="","",'Info Cuencas'!B43)</f>
+        <v/>
+      </c>
+      <c r="C43" t="str">
         <f>IF(A43="","",0.133*'Info Cuencas'!R43)</f>
         <v/>
       </c>
-      <c r="D43" s="6" t="str">
-        <f>IF(A43="","",0.6*'Info Cuencas'!R43+HUS!C43/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E43" s="6" t="str">
+        <f>IF(A43="","",0.6*'Info Cuencas'!R43+HUS!D43/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A44" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A44),"",'Info Cuencas'!A44)</f>
         <v/>
       </c>
-      <c r="B44" t="str">
+      <c r="B44" s="4" t="str">
+        <f>IF(A44="","",'Info Cuencas'!B44)</f>
+        <v/>
+      </c>
+      <c r="C44" t="str">
         <f>IF(A44="","",0.133*'Info Cuencas'!R44)</f>
         <v/>
       </c>
-      <c r="D44" s="6" t="str">
-        <f>IF(A44="","",0.6*'Info Cuencas'!R44+HUS!C44/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E44" s="6" t="str">
+        <f>IF(A44="","",0.6*'Info Cuencas'!R44+HUS!D44/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="45" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A45" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A45),"",'Info Cuencas'!A45)</f>
         <v/>
       </c>
-      <c r="B45" t="str">
+      <c r="B45" s="4" t="str">
+        <f>IF(A45="","",'Info Cuencas'!B45)</f>
+        <v/>
+      </c>
+      <c r="C45" t="str">
         <f>IF(A45="","",0.133*'Info Cuencas'!R45)</f>
         <v/>
       </c>
-      <c r="D45" s="6" t="str">
-        <f>IF(A45="","",0.6*'Info Cuencas'!R45+HUS!C45/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E45" s="6" t="str">
+        <f>IF(A45="","",0.6*'Info Cuencas'!R45+HUS!D45/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A46" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A46),"",'Info Cuencas'!A46)</f>
         <v/>
       </c>
-      <c r="B46" t="str">
+      <c r="B46" s="4" t="str">
+        <f>IF(A46="","",'Info Cuencas'!B46)</f>
+        <v/>
+      </c>
+      <c r="C46" t="str">
         <f>IF(A46="","",0.133*'Info Cuencas'!R46)</f>
         <v/>
       </c>
-      <c r="D46" s="6" t="str">
-        <f>IF(A46="","",0.6*'Info Cuencas'!R46+HUS!C46/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E46" s="6" t="str">
+        <f>IF(A46="","",0.6*'Info Cuencas'!R46+HUS!D46/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A47" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A47),"",'Info Cuencas'!A47)</f>
         <v/>
       </c>
-      <c r="B47" t="str">
+      <c r="B47" s="4" t="str">
+        <f>IF(A47="","",'Info Cuencas'!B47)</f>
+        <v/>
+      </c>
+      <c r="C47" t="str">
         <f>IF(A47="","",0.133*'Info Cuencas'!R47)</f>
         <v/>
       </c>
-      <c r="D47" s="6" t="str">
-        <f>IF(A47="","",0.6*'Info Cuencas'!R47+HUS!C47/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E47" s="6" t="str">
+        <f>IF(A47="","",0.6*'Info Cuencas'!R47+HUS!D47/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="48" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A48" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A48),"",'Info Cuencas'!A48)</f>
         <v/>
       </c>
-      <c r="B48" t="str">
+      <c r="B48" s="4" t="str">
+        <f>IF(A48="","",'Info Cuencas'!B48)</f>
+        <v/>
+      </c>
+      <c r="C48" t="str">
         <f>IF(A48="","",0.133*'Info Cuencas'!R48)</f>
         <v/>
       </c>
-      <c r="D48" s="6" t="str">
-        <f>IF(A48="","",0.6*'Info Cuencas'!R48+HUS!C48/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E48" s="6" t="str">
+        <f>IF(A48="","",0.6*'Info Cuencas'!R48+HUS!D48/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="49" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A49" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A49),"",'Info Cuencas'!A49)</f>
         <v/>
       </c>
-      <c r="B49" t="str">
+      <c r="B49" s="4" t="str">
+        <f>IF(A49="","",'Info Cuencas'!B49)</f>
+        <v/>
+      </c>
+      <c r="C49" t="str">
         <f>IF(A49="","",0.133*'Info Cuencas'!R49)</f>
         <v/>
       </c>
-      <c r="D49" s="6" t="str">
-        <f>IF(A49="","",0.6*'Info Cuencas'!R49+HUS!C49/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E49" s="6" t="str">
+        <f>IF(A49="","",0.6*'Info Cuencas'!R49+HUS!D49/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A50" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A50),"",'Info Cuencas'!A50)</f>
         <v/>
       </c>
-      <c r="B50" t="str">
+      <c r="B50" s="4" t="str">
+        <f>IF(A50="","",'Info Cuencas'!B50)</f>
+        <v/>
+      </c>
+      <c r="C50" t="str">
         <f>IF(A50="","",0.133*'Info Cuencas'!R50)</f>
         <v/>
       </c>
-      <c r="D50" s="6" t="str">
-        <f>IF(A50="","",0.6*'Info Cuencas'!R50+HUS!C50/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E50" s="6" t="str">
+        <f>IF(A50="","",0.6*'Info Cuencas'!R50+HUS!D50/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="51" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A51" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A51),"",'Info Cuencas'!A51)</f>
         <v/>
       </c>
-      <c r="B51" t="str">
+      <c r="B51" s="4" t="str">
+        <f>IF(A51="","",'Info Cuencas'!B51)</f>
+        <v/>
+      </c>
+      <c r="C51" t="str">
         <f>IF(A51="","",0.133*'Info Cuencas'!R51)</f>
         <v/>
       </c>
-      <c r="D51" s="6" t="str">
-        <f>IF(A51="","",0.6*'Info Cuencas'!R51+HUS!C51/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E51" s="6" t="str">
+        <f>IF(A51="","",0.6*'Info Cuencas'!R51+HUS!D51/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="52" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A52" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A52),"",'Info Cuencas'!A52)</f>
         <v/>
       </c>
-      <c r="B52" t="str">
+      <c r="B52" s="4" t="str">
+        <f>IF(A52="","",'Info Cuencas'!B52)</f>
+        <v/>
+      </c>
+      <c r="C52" t="str">
         <f>IF(A52="","",0.133*'Info Cuencas'!R52)</f>
         <v/>
       </c>
-      <c r="D52" s="6" t="str">
-        <f>IF(A52="","",0.6*'Info Cuencas'!R52+HUS!C52/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E52" s="6" t="str">
+        <f>IF(A52="","",0.6*'Info Cuencas'!R52+HUS!D52/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="53" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A53" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A53),"",'Info Cuencas'!A53)</f>
         <v/>
       </c>
-      <c r="B53" t="str">
+      <c r="B53" s="4" t="str">
+        <f>IF(A53="","",'Info Cuencas'!B53)</f>
+        <v/>
+      </c>
+      <c r="C53" t="str">
         <f>IF(A53="","",0.133*'Info Cuencas'!R53)</f>
         <v/>
       </c>
-      <c r="D53" s="6" t="str">
-        <f>IF(A53="","",0.6*'Info Cuencas'!R53+HUS!C53/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E53" s="6" t="str">
+        <f>IF(A53="","",0.6*'Info Cuencas'!R53+HUS!D53/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="54" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A54" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A54),"",'Info Cuencas'!A54)</f>
         <v/>
       </c>
-      <c r="B54" t="str">
+      <c r="B54" s="4" t="str">
+        <f>IF(A54="","",'Info Cuencas'!B54)</f>
+        <v/>
+      </c>
+      <c r="C54" t="str">
         <f>IF(A54="","",0.133*'Info Cuencas'!R54)</f>
         <v/>
       </c>
-      <c r="D54" s="6" t="str">
-        <f>IF(A54="","",0.6*'Info Cuencas'!R54+HUS!C54/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E54" s="6" t="str">
+        <f>IF(A54="","",0.6*'Info Cuencas'!R54+HUS!D54/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="55" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A55" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A55),"",'Info Cuencas'!A55)</f>
         <v/>
       </c>
-      <c r="B55" t="str">
+      <c r="B55" s="4" t="str">
+        <f>IF(A55="","",'Info Cuencas'!B55)</f>
+        <v/>
+      </c>
+      <c r="C55" t="str">
         <f>IF(A55="","",0.133*'Info Cuencas'!R55)</f>
         <v/>
       </c>
-      <c r="D55" s="6" t="str">
-        <f>IF(A55="","",0.6*'Info Cuencas'!R55+HUS!C55/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E55" s="6" t="str">
+        <f>IF(A55="","",0.6*'Info Cuencas'!R55+HUS!D55/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="56" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A56" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A56),"",'Info Cuencas'!A56)</f>
         <v/>
       </c>
-      <c r="B56" t="str">
+      <c r="B56" s="4" t="str">
+        <f>IF(A56="","",'Info Cuencas'!B56)</f>
+        <v/>
+      </c>
+      <c r="C56" t="str">
         <f>IF(A56="","",0.133*'Info Cuencas'!R56)</f>
         <v/>
       </c>
-      <c r="D56" s="6" t="str">
-        <f>IF(A56="","",0.6*'Info Cuencas'!R56+HUS!C56/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E56" s="6" t="str">
+        <f>IF(A56="","",0.6*'Info Cuencas'!R56+HUS!D56/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="57" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A57" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A57),"",'Info Cuencas'!A57)</f>
         <v/>
       </c>
-      <c r="B57" t="str">
+      <c r="B57" s="4" t="str">
+        <f>IF(A57="","",'Info Cuencas'!B57)</f>
+        <v/>
+      </c>
+      <c r="C57" t="str">
         <f>IF(A57="","",0.133*'Info Cuencas'!R57)</f>
         <v/>
       </c>
-      <c r="D57" s="6" t="str">
-        <f>IF(A57="","",0.6*'Info Cuencas'!R57+HUS!C57/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E57" s="6" t="str">
+        <f>IF(A57="","",0.6*'Info Cuencas'!R57+HUS!D57/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="58" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A58" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A58),"",'Info Cuencas'!A58)</f>
         <v/>
       </c>
-      <c r="B58" t="str">
+      <c r="B58" s="4" t="str">
+        <f>IF(A58="","",'Info Cuencas'!B58)</f>
+        <v/>
+      </c>
+      <c r="C58" t="str">
         <f>IF(A58="","",0.133*'Info Cuencas'!R58)</f>
         <v/>
       </c>
-      <c r="D58" s="6" t="str">
-        <f>IF(A58="","",0.6*'Info Cuencas'!R58+HUS!C58/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E58" s="6" t="str">
+        <f>IF(A58="","",0.6*'Info Cuencas'!R58+HUS!D58/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="59" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A59" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A59),"",'Info Cuencas'!A59)</f>
         <v/>
       </c>
-      <c r="B59" t="str">
+      <c r="B59" s="4" t="str">
+        <f>IF(A59="","",'Info Cuencas'!B59)</f>
+        <v/>
+      </c>
+      <c r="C59" t="str">
         <f>IF(A59="","",0.133*'Info Cuencas'!R59)</f>
         <v/>
       </c>
-      <c r="D59" s="6" t="str">
-        <f>IF(A59="","",0.6*'Info Cuencas'!R59+HUS!C59/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E59" s="6" t="str">
+        <f>IF(A59="","",0.6*'Info Cuencas'!R59+HUS!D59/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="60" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A60" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A60),"",'Info Cuencas'!A60)</f>
         <v/>
       </c>
-      <c r="B60" t="str">
+      <c r="B60" s="4" t="str">
+        <f>IF(A60="","",'Info Cuencas'!B60)</f>
+        <v/>
+      </c>
+      <c r="C60" t="str">
         <f>IF(A60="","",0.133*'Info Cuencas'!R60)</f>
         <v/>
       </c>
-      <c r="D60" s="6" t="str">
-        <f>IF(A60="","",0.6*'Info Cuencas'!R60+HUS!C60/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E60" s="6" t="str">
+        <f>IF(A60="","",0.6*'Info Cuencas'!R60+HUS!D60/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="61" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A61" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A61),"",'Info Cuencas'!A61)</f>
         <v/>
       </c>
-      <c r="B61" t="str">
+      <c r="B61" s="4" t="str">
+        <f>IF(A61="","",'Info Cuencas'!B61)</f>
+        <v/>
+      </c>
+      <c r="C61" t="str">
         <f>IF(A61="","",0.133*'Info Cuencas'!R61)</f>
         <v/>
       </c>
-      <c r="D61" s="6" t="str">
-        <f>IF(A61="","",0.6*'Info Cuencas'!R61+HUS!C61/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E61" s="6" t="str">
+        <f>IF(A61="","",0.6*'Info Cuencas'!R61+HUS!D61/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="62" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A62" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A62),"",'Info Cuencas'!A62)</f>
         <v/>
       </c>
-      <c r="B62" t="str">
+      <c r="B62" s="4" t="str">
+        <f>IF(A62="","",'Info Cuencas'!B62)</f>
+        <v/>
+      </c>
+      <c r="C62" t="str">
         <f>IF(A62="","",0.133*'Info Cuencas'!R62)</f>
         <v/>
       </c>
-      <c r="D62" s="6" t="str">
-        <f>IF(A62="","",0.6*'Info Cuencas'!R62+HUS!C62/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E62" s="6" t="str">
+        <f>IF(A62="","",0.6*'Info Cuencas'!R62+HUS!D62/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="63" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A63" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A63),"",'Info Cuencas'!A63)</f>
         <v/>
       </c>
-      <c r="B63" t="str">
+      <c r="B63" s="4" t="str">
+        <f>IF(A63="","",'Info Cuencas'!B63)</f>
+        <v/>
+      </c>
+      <c r="C63" t="str">
         <f>IF(A63="","",0.133*'Info Cuencas'!R63)</f>
         <v/>
       </c>
-      <c r="D63" s="6" t="str">
-        <f>IF(A63="","",0.6*'Info Cuencas'!R63+HUS!C63/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="64" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E63" s="6" t="str">
+        <f>IF(A63="","",0.6*'Info Cuencas'!R63+HUS!D63/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="64" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A64" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A64),"",'Info Cuencas'!A64)</f>
         <v/>
       </c>
-      <c r="B64" t="str">
+      <c r="B64" s="4" t="str">
+        <f>IF(A64="","",'Info Cuencas'!B64)</f>
+        <v/>
+      </c>
+      <c r="C64" t="str">
         <f>IF(A64="","",0.133*'Info Cuencas'!R64)</f>
         <v/>
       </c>
-      <c r="D64" s="6" t="str">
-        <f>IF(A64="","",0.6*'Info Cuencas'!R64+HUS!C64/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="65" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E64" s="6" t="str">
+        <f>IF(A64="","",0.6*'Info Cuencas'!R64+HUS!D64/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="65" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A65" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A65),"",'Info Cuencas'!A65)</f>
         <v/>
       </c>
-      <c r="B65" t="str">
+      <c r="B65" s="4" t="str">
+        <f>IF(A65="","",'Info Cuencas'!B65)</f>
+        <v/>
+      </c>
+      <c r="C65" t="str">
         <f>IF(A65="","",0.133*'Info Cuencas'!R65)</f>
         <v/>
       </c>
-      <c r="D65" s="6" t="str">
-        <f>IF(A65="","",0.6*'Info Cuencas'!R65+HUS!C65/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="66" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E65" s="6" t="str">
+        <f>IF(A65="","",0.6*'Info Cuencas'!R65+HUS!D65/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="66" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A66" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A66),"",'Info Cuencas'!A66)</f>
         <v/>
       </c>
-      <c r="B66" t="str">
+      <c r="B66" s="4" t="str">
+        <f>IF(A66="","",'Info Cuencas'!B66)</f>
+        <v/>
+      </c>
+      <c r="C66" t="str">
         <f>IF(A66="","",0.133*'Info Cuencas'!R66)</f>
         <v/>
       </c>
-      <c r="D66" s="6" t="str">
-        <f>IF(A66="","",0.6*'Info Cuencas'!R66+HUS!C66/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="67" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E66" s="6" t="str">
+        <f>IF(A66="","",0.6*'Info Cuencas'!R66+HUS!D66/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="67" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A67" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A67),"",'Info Cuencas'!A67)</f>
         <v/>
       </c>
-      <c r="B67" t="str">
+      <c r="B67" s="4" t="str">
+        <f>IF(A67="","",'Info Cuencas'!B67)</f>
+        <v/>
+      </c>
+      <c r="C67" t="str">
         <f>IF(A67="","",0.133*'Info Cuencas'!R67)</f>
         <v/>
       </c>
-      <c r="D67" s="6" t="str">
-        <f>IF(A67="","",0.6*'Info Cuencas'!R67+HUS!C67/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="68" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E67" s="6" t="str">
+        <f>IF(A67="","",0.6*'Info Cuencas'!R67+HUS!D67/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="68" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A68" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A68),"",'Info Cuencas'!A68)</f>
         <v/>
       </c>
-      <c r="B68" t="str">
+      <c r="B68" s="4" t="str">
+        <f>IF(A68="","",'Info Cuencas'!B68)</f>
+        <v/>
+      </c>
+      <c r="C68" t="str">
         <f>IF(A68="","",0.133*'Info Cuencas'!R68)</f>
         <v/>
       </c>
-      <c r="D68" s="6" t="str">
-        <f>IF(A68="","",0.6*'Info Cuencas'!R68+HUS!C68/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="69" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E68" s="6" t="str">
+        <f>IF(A68="","",0.6*'Info Cuencas'!R68+HUS!D68/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="69" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A69" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A69),"",'Info Cuencas'!A69)</f>
         <v/>
       </c>
-      <c r="B69" t="str">
+      <c r="B69" s="4" t="str">
+        <f>IF(A69="","",'Info Cuencas'!B69)</f>
+        <v/>
+      </c>
+      <c r="C69" t="str">
         <f>IF(A69="","",0.133*'Info Cuencas'!R69)</f>
         <v/>
       </c>
-      <c r="D69" s="6" t="str">
-        <f>IF(A69="","",0.6*'Info Cuencas'!R69+HUS!C69/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="70" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E69" s="6" t="str">
+        <f>IF(A69="","",0.6*'Info Cuencas'!R69+HUS!D69/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="70" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A70" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A70),"",'Info Cuencas'!A70)</f>
         <v/>
       </c>
-      <c r="B70" t="str">
+      <c r="B70" s="4" t="str">
+        <f>IF(A70="","",'Info Cuencas'!B70)</f>
+        <v/>
+      </c>
+      <c r="C70" t="str">
         <f>IF(A70="","",0.133*'Info Cuencas'!R70)</f>
         <v/>
       </c>
-      <c r="D70" s="6" t="str">
-        <f>IF(A70="","",0.6*'Info Cuencas'!R70+HUS!C70/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="71" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E70" s="6" t="str">
+        <f>IF(A70="","",0.6*'Info Cuencas'!R70+HUS!D70/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="71" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A71" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A71),"",'Info Cuencas'!A71)</f>
         <v/>
       </c>
-      <c r="B71" t="str">
+      <c r="B71" s="4" t="str">
+        <f>IF(A71="","",'Info Cuencas'!B71)</f>
+        <v/>
+      </c>
+      <c r="C71" t="str">
         <f>IF(A71="","",0.133*'Info Cuencas'!R71)</f>
         <v/>
       </c>
-      <c r="D71" s="6" t="str">
-        <f>IF(A71="","",0.6*'Info Cuencas'!R71+HUS!C71/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="72" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E71" s="6" t="str">
+        <f>IF(A71="","",0.6*'Info Cuencas'!R71+HUS!D71/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="72" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A72" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A72),"",'Info Cuencas'!A72)</f>
         <v/>
       </c>
-      <c r="B72" t="str">
+      <c r="B72" s="4" t="str">
+        <f>IF(A72="","",'Info Cuencas'!B72)</f>
+        <v/>
+      </c>
+      <c r="C72" t="str">
         <f>IF(A72="","",0.133*'Info Cuencas'!R72)</f>
         <v/>
       </c>
-      <c r="D72" s="6" t="str">
-        <f>IF(A72="","",0.6*'Info Cuencas'!R72+HUS!C72/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="73" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E72" s="6" t="str">
+        <f>IF(A72="","",0.6*'Info Cuencas'!R72+HUS!D72/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="73" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A73" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A73),"",'Info Cuencas'!A73)</f>
         <v/>
       </c>
-      <c r="B73" t="str">
+      <c r="B73" s="4" t="str">
+        <f>IF(A73="","",'Info Cuencas'!B73)</f>
+        <v/>
+      </c>
+      <c r="C73" t="str">
         <f>IF(A73="","",0.133*'Info Cuencas'!R73)</f>
         <v/>
       </c>
-      <c r="D73" s="6" t="str">
-        <f>IF(A73="","",0.6*'Info Cuencas'!R73+HUS!C73/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="74" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E73" s="6" t="str">
+        <f>IF(A73="","",0.6*'Info Cuencas'!R73+HUS!D73/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="74" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A74" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A74),"",'Info Cuencas'!A74)</f>
         <v/>
       </c>
-      <c r="B74" t="str">
+      <c r="B74" s="4" t="str">
+        <f>IF(A74="","",'Info Cuencas'!B74)</f>
+        <v/>
+      </c>
+      <c r="C74" t="str">
         <f>IF(A74="","",0.133*'Info Cuencas'!R74)</f>
         <v/>
       </c>
-      <c r="D74" s="6" t="str">
-        <f>IF(A74="","",0.6*'Info Cuencas'!R74+HUS!C74/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="75" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E74" s="6" t="str">
+        <f>IF(A74="","",0.6*'Info Cuencas'!R74+HUS!D74/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="75" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A75" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A75),"",'Info Cuencas'!A75)</f>
         <v/>
       </c>
-      <c r="B75" t="str">
+      <c r="B75" s="4" t="str">
+        <f>IF(A75="","",'Info Cuencas'!B75)</f>
+        <v/>
+      </c>
+      <c r="C75" t="str">
         <f>IF(A75="","",0.133*'Info Cuencas'!R75)</f>
         <v/>
       </c>
-      <c r="D75" s="6" t="str">
-        <f>IF(A75="","",0.6*'Info Cuencas'!R75+HUS!C75/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="76" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E75" s="6" t="str">
+        <f>IF(A75="","",0.6*'Info Cuencas'!R75+HUS!D75/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="76" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A76" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A76),"",'Info Cuencas'!A76)</f>
         <v/>
       </c>
-      <c r="B76" t="str">
+      <c r="B76" s="4" t="str">
+        <f>IF(A76="","",'Info Cuencas'!B76)</f>
+        <v/>
+      </c>
+      <c r="C76" t="str">
         <f>IF(A76="","",0.133*'Info Cuencas'!R76)</f>
         <v/>
       </c>
-      <c r="D76" s="6" t="str">
-        <f>IF(A76="","",0.6*'Info Cuencas'!R76+HUS!C76/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="77" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E76" s="6" t="str">
+        <f>IF(A76="","",0.6*'Info Cuencas'!R76+HUS!D76/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="77" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A77" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A77),"",'Info Cuencas'!A77)</f>
         <v/>
       </c>
-      <c r="B77" t="str">
+      <c r="B77" s="4" t="str">
+        <f>IF(A77="","",'Info Cuencas'!B77)</f>
+        <v/>
+      </c>
+      <c r="C77" t="str">
         <f>IF(A77="","",0.133*'Info Cuencas'!R77)</f>
         <v/>
       </c>
-      <c r="D77" s="6" t="str">
-        <f>IF(A77="","",0.6*'Info Cuencas'!R77+HUS!C77/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="78" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E77" s="6" t="str">
+        <f>IF(A77="","",0.6*'Info Cuencas'!R77+HUS!D77/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="78" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A78" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A78),"",'Info Cuencas'!A78)</f>
         <v/>
       </c>
-      <c r="B78" t="str">
+      <c r="B78" s="4" t="str">
+        <f>IF(A78="","",'Info Cuencas'!B78)</f>
+        <v/>
+      </c>
+      <c r="C78" t="str">
         <f>IF(A78="","",0.133*'Info Cuencas'!R78)</f>
         <v/>
       </c>
-      <c r="D78" s="6" t="str">
-        <f>IF(A78="","",0.6*'Info Cuencas'!R78+HUS!C78/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="79" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E78" s="6" t="str">
+        <f>IF(A78="","",0.6*'Info Cuencas'!R78+HUS!D78/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="79" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A79" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A79),"",'Info Cuencas'!A79)</f>
         <v/>
       </c>
-      <c r="B79" t="str">
+      <c r="B79" s="4" t="str">
+        <f>IF(A79="","",'Info Cuencas'!B79)</f>
+        <v/>
+      </c>
+      <c r="C79" t="str">
         <f>IF(A79="","",0.133*'Info Cuencas'!R79)</f>
         <v/>
       </c>
-      <c r="D79" s="6" t="str">
-        <f>IF(A79="","",0.6*'Info Cuencas'!R79+HUS!C79/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="80" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E79" s="6" t="str">
+        <f>IF(A79="","",0.6*'Info Cuencas'!R79+HUS!D79/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="80" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A80" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A80),"",'Info Cuencas'!A80)</f>
         <v/>
       </c>
-      <c r="B80" t="str">
+      <c r="B80" s="4" t="str">
+        <f>IF(A80="","",'Info Cuencas'!B80)</f>
+        <v/>
+      </c>
+      <c r="C80" t="str">
         <f>IF(A80="","",0.133*'Info Cuencas'!R80)</f>
         <v/>
       </c>
-      <c r="D80" s="6" t="str">
-        <f>IF(A80="","",0.6*'Info Cuencas'!R80+HUS!C80/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="81" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E80" s="6" t="str">
+        <f>IF(A80="","",0.6*'Info Cuencas'!R80+HUS!D80/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="81" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A81" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A81),"",'Info Cuencas'!A81)</f>
         <v/>
       </c>
-      <c r="B81" t="str">
+      <c r="B81" s="4" t="str">
+        <f>IF(A81="","",'Info Cuencas'!B81)</f>
+        <v/>
+      </c>
+      <c r="C81" t="str">
         <f>IF(A81="","",0.133*'Info Cuencas'!R81)</f>
         <v/>
       </c>
-      <c r="D81" s="6" t="str">
-        <f>IF(A81="","",0.6*'Info Cuencas'!R81+HUS!C81/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="82" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E81" s="6" t="str">
+        <f>IF(A81="","",0.6*'Info Cuencas'!R81+HUS!D81/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="82" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A82" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A82),"",'Info Cuencas'!A82)</f>
         <v/>
       </c>
-      <c r="B82" t="str">
+      <c r="B82" s="4" t="str">
+        <f>IF(A82="","",'Info Cuencas'!B82)</f>
+        <v/>
+      </c>
+      <c r="C82" t="str">
         <f>IF(A82="","",0.133*'Info Cuencas'!R82)</f>
         <v/>
       </c>
-      <c r="D82" s="6" t="str">
-        <f>IF(A82="","",0.6*'Info Cuencas'!R82+HUS!C82/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="83" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E82" s="6" t="str">
+        <f>IF(A82="","",0.6*'Info Cuencas'!R82+HUS!D82/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="83" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A83" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A83),"",'Info Cuencas'!A83)</f>
         <v/>
       </c>
-      <c r="B83" t="str">
+      <c r="B83" s="4" t="str">
+        <f>IF(A83="","",'Info Cuencas'!B83)</f>
+        <v/>
+      </c>
+      <c r="C83" t="str">
         <f>IF(A83="","",0.133*'Info Cuencas'!R83)</f>
         <v/>
       </c>
-      <c r="D83" s="6" t="str">
-        <f>IF(A83="","",0.6*'Info Cuencas'!R83+HUS!C83/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="84" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E83" s="6" t="str">
+        <f>IF(A83="","",0.6*'Info Cuencas'!R83+HUS!D83/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="84" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A84" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A84),"",'Info Cuencas'!A84)</f>
         <v/>
       </c>
-      <c r="B84" t="str">
+      <c r="B84" s="4" t="str">
+        <f>IF(A84="","",'Info Cuencas'!B84)</f>
+        <v/>
+      </c>
+      <c r="C84" t="str">
         <f>IF(A84="","",0.133*'Info Cuencas'!R84)</f>
         <v/>
       </c>
-      <c r="D84" s="6" t="str">
-        <f>IF(A84="","",0.6*'Info Cuencas'!R84+HUS!C84/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="85" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E84" s="6" t="str">
+        <f>IF(A84="","",0.6*'Info Cuencas'!R84+HUS!D84/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="85" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A85" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A85),"",'Info Cuencas'!A85)</f>
         <v/>
       </c>
-      <c r="B85" t="str">
+      <c r="B85" s="4" t="str">
+        <f>IF(A85="","",'Info Cuencas'!B85)</f>
+        <v/>
+      </c>
+      <c r="C85" t="str">
         <f>IF(A85="","",0.133*'Info Cuencas'!R85)</f>
         <v/>
       </c>
-      <c r="D85" s="6" t="str">
-        <f>IF(A85="","",0.6*'Info Cuencas'!R85+HUS!C85/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="86" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E85" s="6" t="str">
+        <f>IF(A85="","",0.6*'Info Cuencas'!R85+HUS!D85/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="86" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A86" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A86),"",'Info Cuencas'!A86)</f>
         <v/>
       </c>
-      <c r="B86" t="str">
+      <c r="B86" s="4" t="str">
+        <f>IF(A86="","",'Info Cuencas'!B86)</f>
+        <v/>
+      </c>
+      <c r="C86" t="str">
         <f>IF(A86="","",0.133*'Info Cuencas'!R86)</f>
         <v/>
       </c>
-      <c r="D86" s="6" t="str">
-        <f>IF(A86="","",0.6*'Info Cuencas'!R86+HUS!C86/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="87" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E86" s="6" t="str">
+        <f>IF(A86="","",0.6*'Info Cuencas'!R86+HUS!D86/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="87" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A87" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A87),"",'Info Cuencas'!A87)</f>
         <v/>
       </c>
-      <c r="B87" t="str">
+      <c r="B87" s="4" t="str">
+        <f>IF(A87="","",'Info Cuencas'!B87)</f>
+        <v/>
+      </c>
+      <c r="C87" t="str">
         <f>IF(A87="","",0.133*'Info Cuencas'!R87)</f>
         <v/>
       </c>
-      <c r="D87" s="6" t="str">
-        <f>IF(A87="","",0.6*'Info Cuencas'!R87+HUS!C87/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="88" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E87" s="6" t="str">
+        <f>IF(A87="","",0.6*'Info Cuencas'!R87+HUS!D87/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="88" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A88" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A88),"",'Info Cuencas'!A88)</f>
         <v/>
       </c>
-      <c r="B88" t="str">
+      <c r="B88" s="4" t="str">
+        <f>IF(A88="","",'Info Cuencas'!B88)</f>
+        <v/>
+      </c>
+      <c r="C88" t="str">
         <f>IF(A88="","",0.133*'Info Cuencas'!R88)</f>
         <v/>
       </c>
-      <c r="D88" s="6" t="str">
-        <f>IF(A88="","",0.6*'Info Cuencas'!R88+HUS!C88/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="89" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E88" s="6" t="str">
+        <f>IF(A88="","",0.6*'Info Cuencas'!R88+HUS!D88/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="89" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A89" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A89),"",'Info Cuencas'!A89)</f>
         <v/>
       </c>
-      <c r="B89" t="str">
+      <c r="B89" s="4" t="str">
+        <f>IF(A89="","",'Info Cuencas'!B89)</f>
+        <v/>
+      </c>
+      <c r="C89" t="str">
         <f>IF(A89="","",0.133*'Info Cuencas'!R89)</f>
         <v/>
       </c>
-      <c r="D89" s="6" t="str">
-        <f>IF(A89="","",0.6*'Info Cuencas'!R89+HUS!C89/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="90" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E89" s="6" t="str">
+        <f>IF(A89="","",0.6*'Info Cuencas'!R89+HUS!D89/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="90" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A90" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A90),"",'Info Cuencas'!A90)</f>
         <v/>
       </c>
-      <c r="B90" t="str">
+      <c r="B90" s="4" t="str">
+        <f>IF(A90="","",'Info Cuencas'!B90)</f>
+        <v/>
+      </c>
+      <c r="C90" t="str">
         <f>IF(A90="","",0.133*'Info Cuencas'!R90)</f>
         <v/>
       </c>
-      <c r="D90" s="6" t="str">
-        <f>IF(A90="","",0.6*'Info Cuencas'!R90+HUS!C90/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="91" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E90" s="6" t="str">
+        <f>IF(A90="","",0.6*'Info Cuencas'!R90+HUS!D90/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="91" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A91" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A91),"",'Info Cuencas'!A91)</f>
         <v/>
       </c>
-      <c r="B91" t="str">
+      <c r="B91" s="4" t="str">
+        <f>IF(A91="","",'Info Cuencas'!B91)</f>
+        <v/>
+      </c>
+      <c r="C91" t="str">
         <f>IF(A91="","",0.133*'Info Cuencas'!R91)</f>
         <v/>
       </c>
-      <c r="D91" s="6" t="str">
-        <f>IF(A91="","",0.6*'Info Cuencas'!R91+HUS!C91/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="92" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E91" s="6" t="str">
+        <f>IF(A91="","",0.6*'Info Cuencas'!R91+HUS!D91/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="92" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A92" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A92),"",'Info Cuencas'!A92)</f>
         <v/>
       </c>
-      <c r="B92" t="str">
+      <c r="B92" s="4" t="str">
+        <f>IF(A92="","",'Info Cuencas'!B92)</f>
+        <v/>
+      </c>
+      <c r="C92" t="str">
         <f>IF(A92="","",0.133*'Info Cuencas'!R92)</f>
         <v/>
       </c>
-      <c r="D92" s="6" t="str">
-        <f>IF(A92="","",0.6*'Info Cuencas'!R92+HUS!C92/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="93" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E92" s="6" t="str">
+        <f>IF(A92="","",0.6*'Info Cuencas'!R92+HUS!D92/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="93" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A93" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A93),"",'Info Cuencas'!A93)</f>
         <v/>
       </c>
-      <c r="B93" t="str">
+      <c r="B93" s="4" t="str">
+        <f>IF(A93="","",'Info Cuencas'!B93)</f>
+        <v/>
+      </c>
+      <c r="C93" t="str">
         <f>IF(A93="","",0.133*'Info Cuencas'!R93)</f>
         <v/>
       </c>
-      <c r="D93" s="6" t="str">
-        <f>IF(A93="","",0.6*'Info Cuencas'!R93+HUS!C93/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="94" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E93" s="6" t="str">
+        <f>IF(A93="","",0.6*'Info Cuencas'!R93+HUS!D93/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="94" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A94" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A94),"",'Info Cuencas'!A94)</f>
         <v/>
       </c>
-      <c r="B94" t="str">
+      <c r="B94" s="4" t="str">
+        <f>IF(A94="","",'Info Cuencas'!B94)</f>
+        <v/>
+      </c>
+      <c r="C94" t="str">
         <f>IF(A94="","",0.133*'Info Cuencas'!R94)</f>
         <v/>
       </c>
-      <c r="D94" s="6" t="str">
-        <f>IF(A94="","",0.6*'Info Cuencas'!R94+HUS!C94/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="95" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E94" s="6" t="str">
+        <f>IF(A94="","",0.6*'Info Cuencas'!R94+HUS!D94/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="95" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A95" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A95),"",'Info Cuencas'!A95)</f>
         <v/>
       </c>
-      <c r="B95" t="str">
+      <c r="B95" s="4" t="str">
+        <f>IF(A95="","",'Info Cuencas'!B95)</f>
+        <v/>
+      </c>
+      <c r="C95" t="str">
         <f>IF(A95="","",0.133*'Info Cuencas'!R95)</f>
         <v/>
       </c>
-      <c r="D95" s="6" t="str">
-        <f>IF(A95="","",0.6*'Info Cuencas'!R95+HUS!C95/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="96" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E95" s="6" t="str">
+        <f>IF(A95="","",0.6*'Info Cuencas'!R95+HUS!D95/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="96" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A96" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A96),"",'Info Cuencas'!A96)</f>
         <v/>
       </c>
-      <c r="B96" t="str">
+      <c r="B96" s="4" t="str">
+        <f>IF(A96="","",'Info Cuencas'!B96)</f>
+        <v/>
+      </c>
+      <c r="C96" t="str">
         <f>IF(A96="","",0.133*'Info Cuencas'!R96)</f>
         <v/>
       </c>
-      <c r="D96" s="6" t="str">
-        <f>IF(A96="","",0.6*'Info Cuencas'!R96+HUS!C96/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="97" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E96" s="6" t="str">
+        <f>IF(A96="","",0.6*'Info Cuencas'!R96+HUS!D96/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="97" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A97" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A97),"",'Info Cuencas'!A97)</f>
         <v/>
       </c>
-      <c r="B97" t="str">
+      <c r="B97" s="4" t="str">
+        <f>IF(A97="","",'Info Cuencas'!B97)</f>
+        <v/>
+      </c>
+      <c r="C97" t="str">
         <f>IF(A97="","",0.133*'Info Cuencas'!R97)</f>
         <v/>
       </c>
-      <c r="D97" s="6" t="str">
-        <f>IF(A97="","",0.6*'Info Cuencas'!R97+HUS!C97/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="98" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E97" s="6" t="str">
+        <f>IF(A97="","",0.6*'Info Cuencas'!R97+HUS!D97/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="98" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A98" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A98),"",'Info Cuencas'!A98)</f>
         <v/>
       </c>
-      <c r="B98" t="str">
+      <c r="B98" s="4" t="str">
+        <f>IF(A98="","",'Info Cuencas'!B98)</f>
+        <v/>
+      </c>
+      <c r="C98" t="str">
         <f>IF(A98="","",0.133*'Info Cuencas'!R98)</f>
         <v/>
       </c>
-      <c r="D98" s="6" t="str">
-        <f>IF(A98="","",0.6*'Info Cuencas'!R98+HUS!C98/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="99" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E98" s="6" t="str">
+        <f>IF(A98="","",0.6*'Info Cuencas'!R98+HUS!D98/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="99" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A99" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A99),"",'Info Cuencas'!A99)</f>
         <v/>
       </c>
-      <c r="B99" t="str">
+      <c r="B99" s="4" t="str">
+        <f>IF(A99="","",'Info Cuencas'!B99)</f>
+        <v/>
+      </c>
+      <c r="C99" t="str">
         <f>IF(A99="","",0.133*'Info Cuencas'!R99)</f>
         <v/>
       </c>
-      <c r="D99" s="6" t="str">
-        <f>IF(A99="","",0.6*'Info Cuencas'!R99+HUS!C99/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="100" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E99" s="6" t="str">
+        <f>IF(A99="","",0.6*'Info Cuencas'!R99+HUS!D99/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="100" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A100" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A100),"",'Info Cuencas'!A100)</f>
         <v/>
       </c>
-      <c r="B100" t="str">
+      <c r="B100" s="4" t="str">
+        <f>IF(A100="","",'Info Cuencas'!B100)</f>
+        <v/>
+      </c>
+      <c r="C100" t="str">
         <f>IF(A100="","",0.133*'Info Cuencas'!R100)</f>
         <v/>
       </c>
-      <c r="D100" s="6" t="str">
-        <f>IF(A100="","",0.6*'Info Cuencas'!R100+HUS!C100/2)</f>
+      <c r="E100" s="6" t="str">
+        <f>IF(A100="","",0.6*'Info Cuencas'!R100+HUS!D100/2)</f>
         <v/>
       </c>
     </row>
@@ -21737,15 +22136,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100CCB1C2B958A07241A317F5A881DFD30C" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ec29f518eb9a62149baea9c73f5411cd">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="63768118-86e2-4829-8a12-b72c47658d02" xmlns:ns3="40414187-dd76-4ef8-b04f-ccddae734140" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="29f6242226419d82ce7554acb1ee2c31" ns2:_="" ns3:_="">
     <xsd:import namespace="63768118-86e2-4829-8a12-b72c47658d02"/>
@@ -22000,6 +22390,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2A4DA3E6-B8B6-48A6-81EC-CAAD4DEE707B}">
   <ds:schemaRefs>
@@ -22012,14 +22411,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{26BC43C4-0DE4-4398-8C07-F13A3433226F}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{124384BF-B442-43EF-BEBD-26F0C03197F3}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -22036,4 +22427,12 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{26BC43C4-0DE4-4398-8C07-F13A3433226F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
UPDATE comentarios en Inputs y se han realizado hietogramas con la discretización temporal escogida para los hidrogramas
</commit_message>
<xml_diff>
--- a/Inputs.xlsx
+++ b/Inputs.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Codigos\HU_SCS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{23BFEA37-CE9B-4DF6-BBFD-9A7A266769B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0873C22F-FC01-464E-8899-90B38A3D86B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Info Cuencas" sheetId="1" r:id="rId1"/>
@@ -449,15 +449,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>8</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:colOff>11430</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>129540</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>15</xdr:col>
-      <xdr:colOff>7620</xdr:colOff>
-      <xdr:row>4</xdr:row>
-      <xdr:rowOff>28575</xdr:rowOff>
+      <xdr:colOff>15240</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>161925</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -472,8 +472,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="6819900" y="704850"/>
-          <a:ext cx="4351020" cy="571500"/>
+          <a:off x="6831330" y="1558290"/>
+          <a:ext cx="4347210" cy="575310"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -527,6 +527,112 @@
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
             <a:t> y enviar mensaje de alerta.</a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="es-CL" sz="1100" b="1" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+          </a:br>
+          <a:endParaRPr lang="es-CL" sz="1100" b="1">
+            <a:solidFill>
+              <a:srgbClr val="FF0000"/>
+            </a:solidFill>
+            <a:latin typeface="+mn-lt"/>
+            <a:ea typeface="+mn-ea"/>
+            <a:cs typeface="+mn-cs"/>
+          </a:endParaRPr>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>9525</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>26670</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="3" name="TextBox 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4BB0B733-C4CE-472E-8143-82D4BFF38A7B}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="6819900" y="704850"/>
+          <a:ext cx="4352925" cy="569595"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+        <a:ln w="38100" cmpd="sng">
+          <a:solidFill>
+            <a:srgbClr val="FF0000"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr marL="0" indent="0"/>
+          <a:r>
+            <a:rPr lang="es-CL" sz="1100" b="1">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>En esta pestaña se debe rellenar el valor de ∆D adoptado en horas. Se recomienda que el</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="es-CL" sz="1100" b="1" baseline="0">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t> valor en minutos sea divisor de 60.</a:t>
           </a:r>
           <a:br>
             <a:rPr lang="es-CL" sz="1100" b="1" baseline="0">
@@ -736,6 +842,125 @@
     </xdr:sp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>19</xdr:col>
+      <xdr:colOff>81915</xdr:colOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>97156</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="2" name="TextBox 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9ACE1258-6722-4F98-9FA6-6BA08DCA017C}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="7315200" y="180975"/>
+          <a:ext cx="4349115" cy="1544956"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+        <a:ln w="38100" cmpd="sng">
+          <a:solidFill>
+            <a:srgbClr val="FF0000"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr marL="0" indent="0"/>
+          <a:r>
+            <a:rPr lang="es-CL" sz="1100" b="1" baseline="0">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>Nota para el codigo:</a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="es-CL" sz="1100" b="1" baseline="0">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+          </a:br>
+          <a:r>
+            <a:rPr lang="es-CL" sz="1100" b="1" baseline="0">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>Preguntar a copilot si habría problemas con que en "T" se rellenen dos períodos de retorno iguales, o si habría problemas con poner un string acá (como por ejemplo "T=2-CC")</a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="es-CL" sz="1100" b="1" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+          </a:br>
+          <a:endParaRPr lang="es-CL" sz="1100" b="1">
+            <a:solidFill>
+              <a:srgbClr val="FF0000"/>
+            </a:solidFill>
+            <a:latin typeface="+mn-lt"/>
+            <a:ea typeface="+mn-ea"/>
+            <a:cs typeface="+mn-cs"/>
+          </a:endParaRPr>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -907,6 +1132,125 @@
             </a:rPr>
             <a:t> el codigo y enviar mensaje de alerta.</a:t>
           </a:r>
+          <a:endParaRPr lang="es-CL" sz="1100" b="1">
+            <a:solidFill>
+              <a:srgbClr val="FF0000"/>
+            </a:solidFill>
+            <a:latin typeface="+mn-lt"/>
+            <a:ea typeface="+mn-ea"/>
+            <a:cs typeface="+mn-cs"/>
+          </a:endParaRPr>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>17</xdr:col>
+      <xdr:colOff>83820</xdr:colOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>93346</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="3" name="TextBox 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{3C2A0A9D-A96A-4588-9008-7CD268890179}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="6096000" y="180975"/>
+          <a:ext cx="4351020" cy="1541146"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+        <a:ln w="38100" cmpd="sng">
+          <a:solidFill>
+            <a:srgbClr val="FF0000"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr marL="0" indent="0"/>
+          <a:r>
+            <a:rPr lang="es-CL" sz="1100" b="1" baseline="0">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>Nota para el codigo:</a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="es-CL" sz="1100" b="1" baseline="0">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+          </a:br>
+          <a:r>
+            <a:rPr lang="es-CL" sz="1100" b="1" baseline="0">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>Preguntar a copilot si habría problemas con que en "Horas" se rellenen dos duraciones iguales, o si habría problemas con poner un string o un número que no sea entero (aunque esto ultimo no se si se dé en hidrología).</a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="es-CL" sz="1100" b="1" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+          </a:br>
           <a:endParaRPr lang="es-CL" sz="1100" b="1">
             <a:solidFill>
               <a:srgbClr val="FF0000"/>
@@ -22582,6 +22926,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="40414187-dd76-4ef8-b04f-ccddae734140" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="63768118-86e2-4829-8a12-b72c47658d02">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100CCB1C2B958A07241A317F5A881DFD30C" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ec29f518eb9a62149baea9c73f5411cd">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="63768118-86e2-4829-8a12-b72c47658d02" xmlns:ns3="40414187-dd76-4ef8-b04f-ccddae734140" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="29f6242226419d82ce7554acb1ee2c31" ns2:_="" ns3:_="">
     <xsd:import namespace="63768118-86e2-4829-8a12-b72c47658d02"/>
@@ -22836,27 +23200,26 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2A4DA3E6-B8B6-48A6-81EC-CAAD4DEE707B}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="40414187-dd76-4ef8-b04f-ccddae734140"/>
+    <ds:schemaRef ds:uri="63768118-86e2-4829-8a12-b72c47658d02"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="40414187-dd76-4ef8-b04f-ccddae734140" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="63768118-86e2-4829-8a12-b72c47658d02">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{26BC43C4-0DE4-4398-8C07-F13A3433226F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{124384BF-B442-43EF-BEBD-26F0C03197F3}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -22873,23 +23236,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{26BC43C4-0DE4-4398-8C07-F13A3433226F}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2A4DA3E6-B8B6-48A6-81EC-CAAD4DEE707B}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="40414187-dd76-4ef8-b04f-ccddae734140"/>
-    <ds:schemaRef ds:uri="63768118-86e2-4829-8a12-b72c47658d02"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
UPDATE planilla y codigo para leer valor de CN por cuenca
</commit_message>
<xml_diff>
--- a/Inputs.xlsx
+++ b/Inputs.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Codigos\HU_SCS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0873C22F-FC01-464E-8899-90B38A3D86B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9675E104-ED50-4A54-876F-6109ED75FCEA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Info Cuencas" sheetId="1" r:id="rId1"/>
@@ -63,7 +63,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="42">
   <si>
     <t>Cuenca</t>
   </si>
@@ -186,6 +186,9 @@
   </si>
   <si>
     <t>SCS - Tipo IA</t>
+  </si>
+  <si>
+    <t>CN</t>
   </si>
 </sst>
 </file>
@@ -448,13 +451,13 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>8</xdr:col>
+      <xdr:col>9</xdr:col>
       <xdr:colOff>11430</xdr:colOff>
       <xdr:row>5</xdr:row>
       <xdr:rowOff>129540</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>15</xdr:col>
+      <xdr:col>16</xdr:col>
       <xdr:colOff>15240</xdr:colOff>
       <xdr:row>8</xdr:row>
       <xdr:rowOff>161925</xdr:rowOff>
@@ -554,13 +557,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>8</xdr:col>
+      <xdr:col>9</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>1</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>15</xdr:col>
+      <xdr:col>16</xdr:col>
       <xdr:colOff>9525</xdr:colOff>
       <xdr:row>4</xdr:row>
       <xdr:rowOff>26670</xdr:rowOff>
@@ -10317,16 +10320,16 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7ED18635-56AF-4151-A8F0-4CF2F4B95CB7}">
   <sheetPr codeName="Sheet2"/>
-  <dimension ref="A1:J100"/>
+  <dimension ref="A1:K100"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14.6640625" customWidth="1"/>
-    <col min="2" max="7" width="12.6640625" customWidth="1"/>
-    <col min="14" max="14" width="10" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11" bestFit="1" customWidth="1"/>
+    <col min="2" max="8" width="12.6640625" customWidth="1"/>
+    <col min="15" max="15" width="10" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="11" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="55.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" ht="55.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="7" t="s">
         <v>0</v>
       </c>
@@ -10334,22 +10337,25 @@
         <v>1</v>
       </c>
       <c r="C1" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="D1" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="D1" s="8" t="s">
+      <c r="E1" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="F1" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="G1" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="H1" s="2" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A2" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A2),"",'Info Cuencas'!A2)</f>
         <v>C_01_CL</v>
@@ -10358,29 +10364,33 @@
         <f>IF(A2="","",'Info Cuencas'!B2)</f>
         <v>117.271</v>
       </c>
-      <c r="C2" s="6">
+      <c r="C2" s="4">
+        <f>IF(A2="","",'Info Cuencas'!C2)</f>
+        <v>75</v>
+      </c>
+      <c r="D2" s="6">
         <f>IF(A2="","",0.133*'Info Cuencas'!R2)</f>
         <v>0.76073282726013913</v>
       </c>
-      <c r="D2" s="11">
+      <c r="E2" s="11">
         <v>0.05</v>
       </c>
-      <c r="E2" s="6">
-        <f>IF(A2="","",0.6*'Info Cuencas'!R2+HUS!D2/2)</f>
+      <c r="F2" s="6">
+        <f>IF(A2="","",0.6*'Info Cuencas'!R2+HUS!E2/2)</f>
         <v>3.4568774162111535</v>
       </c>
-      <c r="F2" s="6">
-        <f>IF(A2="","",5*E2)</f>
+      <c r="G2" s="6">
+        <f>IF(A2="","",5*F2)</f>
         <v>17.284387081055769</v>
       </c>
-      <c r="G2" s="6">
-        <f>IF(A2="","",0.208*'Info Cuencas'!B2/HUS!E2)</f>
+      <c r="H2" s="6">
+        <f>IF(A2="","",0.208*'Info Cuencas'!B2/HUS!F2)</f>
         <v>7.0561854133476336</v>
       </c>
-      <c r="H2" s="6"/>
-      <c r="J2" s="5"/>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="I2" s="6"/>
+      <c r="K2" s="5"/>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A3" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A3),"",'Info Cuencas'!A3)</f>
         <v>C_02_CL</v>
@@ -10389,28 +10399,32 @@
         <f>IF(A3="","",'Info Cuencas'!B3)</f>
         <v>447.74</v>
       </c>
-      <c r="C3" s="6">
+      <c r="C3" s="4">
+        <f>IF(A3="","",'Info Cuencas'!C3)</f>
+        <v>75</v>
+      </c>
+      <c r="D3" s="6">
         <f>IF(A3="","",0.133*'Info Cuencas'!R3)</f>
         <v>1.0943707430089464</v>
       </c>
-      <c r="D3" s="11">
+      <c r="E3" s="11">
         <v>0.05</v>
       </c>
-      <c r="E3" s="6">
-        <f>IF(A3="","",0.6*'Info Cuencas'!R3+HUS!D3/2)</f>
+      <c r="F3" s="6">
+        <f>IF(A3="","",0.6*'Info Cuencas'!R3+HUS!E3/2)</f>
         <v>4.9620108707170507</v>
       </c>
-      <c r="F3" s="6">
-        <f>IF(A3="","",5*E3)</f>
+      <c r="G3" s="6">
+        <f>IF(A3="","",5*F3)</f>
         <v>24.810054353585254</v>
       </c>
-      <c r="G3" s="6">
-        <f>IF(A3="","",0.208*'Info Cuencas'!B3/HUS!E3)</f>
+      <c r="H3" s="6">
+        <f>IF(A3="","",0.208*'Info Cuencas'!B3/HUS!F3)</f>
         <v>18.768584436120346</v>
       </c>
-      <c r="H3" s="6"/>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="I3" s="6"/>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A4" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A4),"",'Info Cuencas'!A4)</f>
         <v/>
@@ -10419,26 +10433,30 @@
         <f>IF(A4="","",'Info Cuencas'!B4)</f>
         <v/>
       </c>
-      <c r="C4" s="6" t="str">
+      <c r="C4" s="4" t="str">
+        <f>IF(A4="","",'Info Cuencas'!C4)</f>
+        <v/>
+      </c>
+      <c r="D4" s="6" t="str">
         <f>IF(A4="","",0.133*'Info Cuencas'!R4)</f>
         <v/>
       </c>
-      <c r="D4" s="9"/>
-      <c r="E4" s="6" t="str">
-        <f>IF(A4="","",0.6*'Info Cuencas'!R4+HUS!D4/2)</f>
-        <v/>
-      </c>
+      <c r="E4" s="9"/>
       <c r="F4" s="6" t="str">
-        <f t="shared" ref="F4" si="0">IF(A4="","",5*E4)</f>
+        <f>IF(A4="","",0.6*'Info Cuencas'!R4+HUS!E4/2)</f>
         <v/>
       </c>
       <c r="G4" s="6" t="str">
-        <f>IF(A4="","",0.208*'Info Cuencas'!B4/HUS!E4)</f>
-        <v/>
-      </c>
-      <c r="H4" s="6"/>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+        <f t="shared" ref="G4" si="0">IF(A4="","",5*F4)</f>
+        <v/>
+      </c>
+      <c r="H4" s="6" t="str">
+        <f>IF(A4="","",0.208*'Info Cuencas'!B4/HUS!F4)</f>
+        <v/>
+      </c>
+      <c r="I4" s="6"/>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A5" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A5),"",'Info Cuencas'!A5)</f>
         <v/>
@@ -10447,26 +10465,30 @@
         <f>IF(A5="","",'Info Cuencas'!B5)</f>
         <v/>
       </c>
-      <c r="C5" s="6" t="str">
+      <c r="C5" s="4" t="str">
+        <f>IF(A5="","",'Info Cuencas'!C5)</f>
+        <v/>
+      </c>
+      <c r="D5" s="6" t="str">
         <f>IF(A5="","",0.133*'Info Cuencas'!R5)</f>
         <v/>
       </c>
-      <c r="D5" s="9"/>
-      <c r="E5" s="6" t="str">
-        <f>IF(A5="","",0.6*'Info Cuencas'!R5+HUS!D5/2)</f>
-        <v/>
-      </c>
+      <c r="E5" s="9"/>
       <c r="F5" s="6" t="str">
-        <f>IF(A5="","",5*E5)</f>
+        <f>IF(A5="","",0.6*'Info Cuencas'!R5+HUS!E5/2)</f>
         <v/>
       </c>
       <c r="G5" s="6" t="str">
-        <f>IF(A5="","",0.208*'Info Cuencas'!B5/HUS!E5)</f>
-        <v/>
-      </c>
-      <c r="H5" s="6"/>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+        <f>IF(A5="","",5*F5)</f>
+        <v/>
+      </c>
+      <c r="H5" s="6" t="str">
+        <f>IF(A5="","",0.208*'Info Cuencas'!B5/HUS!F5)</f>
+        <v/>
+      </c>
+      <c r="I5" s="6"/>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A6" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A6),"",'Info Cuencas'!A6)</f>
         <v/>
@@ -10475,26 +10497,30 @@
         <f>IF(A6="","",'Info Cuencas'!B6)</f>
         <v/>
       </c>
-      <c r="C6" s="6" t="str">
+      <c r="C6" s="4" t="str">
+        <f>IF(A6="","",'Info Cuencas'!C6)</f>
+        <v/>
+      </c>
+      <c r="D6" s="6" t="str">
         <f>IF(A6="","",0.133*'Info Cuencas'!R6)</f>
         <v/>
       </c>
-      <c r="D6" s="9"/>
-      <c r="E6" s="6" t="str">
-        <f>IF(A6="","",0.6*'Info Cuencas'!R6+HUS!D6/2)</f>
-        <v/>
-      </c>
+      <c r="E6" s="9"/>
       <c r="F6" s="6" t="str">
-        <f t="shared" ref="F6:F11" si="1">IF(A6="","",5*E6)</f>
+        <f>IF(A6="","",0.6*'Info Cuencas'!R6+HUS!E6/2)</f>
         <v/>
       </c>
       <c r="G6" s="6" t="str">
-        <f>IF(A6="","",0.208*'Info Cuencas'!B6/HUS!E6)</f>
-        <v/>
-      </c>
-      <c r="H6" s="6"/>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
+        <f t="shared" ref="G6:G11" si="1">IF(A6="","",5*F6)</f>
+        <v/>
+      </c>
+      <c r="H6" s="6" t="str">
+        <f>IF(A6="","",0.208*'Info Cuencas'!B6/HUS!F6)</f>
+        <v/>
+      </c>
+      <c r="I6" s="6"/>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A7" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A7),"",'Info Cuencas'!A7)</f>
         <v/>
@@ -10503,26 +10529,30 @@
         <f>IF(A7="","",'Info Cuencas'!B7)</f>
         <v/>
       </c>
-      <c r="C7" s="6" t="str">
+      <c r="C7" s="4" t="str">
+        <f>IF(A7="","",'Info Cuencas'!C7)</f>
+        <v/>
+      </c>
+      <c r="D7" s="6" t="str">
         <f>IF(A7="","",0.133*'Info Cuencas'!R7)</f>
         <v/>
       </c>
-      <c r="D7" s="9"/>
-      <c r="E7" s="6" t="str">
-        <f>IF(A7="","",0.6*'Info Cuencas'!R7+HUS!D7/2)</f>
-        <v/>
-      </c>
+      <c r="E7" s="9"/>
       <c r="F7" s="6" t="str">
+        <f>IF(A7="","",0.6*'Info Cuencas'!R7+HUS!E7/2)</f>
+        <v/>
+      </c>
+      <c r="G7" s="6" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="G7" s="6" t="str">
-        <f>IF(A7="","",0.208*'Info Cuencas'!B7/HUS!E7)</f>
-        <v/>
-      </c>
-      <c r="H7" s="6"/>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="H7" s="6" t="str">
+        <f>IF(A7="","",0.208*'Info Cuencas'!B7/HUS!F7)</f>
+        <v/>
+      </c>
+      <c r="I7" s="6"/>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A8" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A8),"",'Info Cuencas'!A8)</f>
         <v/>
@@ -10531,26 +10561,30 @@
         <f>IF(A8="","",'Info Cuencas'!B8)</f>
         <v/>
       </c>
-      <c r="C8" s="6" t="str">
+      <c r="C8" s="4" t="str">
+        <f>IF(A8="","",'Info Cuencas'!C8)</f>
+        <v/>
+      </c>
+      <c r="D8" s="6" t="str">
         <f>IF(A8="","",0.133*'Info Cuencas'!R8)</f>
         <v/>
       </c>
-      <c r="D8" s="9"/>
-      <c r="E8" s="6" t="str">
-        <f>IF(A8="","",0.6*'Info Cuencas'!R8+HUS!D8/2)</f>
-        <v/>
-      </c>
+      <c r="E8" s="9"/>
       <c r="F8" s="6" t="str">
-        <f>IF(A8="","",5*E8)</f>
+        <f>IF(A8="","",0.6*'Info Cuencas'!R8+HUS!E8/2)</f>
         <v/>
       </c>
       <c r="G8" s="6" t="str">
-        <f>IF(A8="","",0.208*'Info Cuencas'!B8/HUS!E8)</f>
-        <v/>
-      </c>
-      <c r="H8" s="6"/>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
+        <f>IF(A8="","",5*F8)</f>
+        <v/>
+      </c>
+      <c r="H8" s="6" t="str">
+        <f>IF(A8="","",0.208*'Info Cuencas'!B8/HUS!F8)</f>
+        <v/>
+      </c>
+      <c r="I8" s="6"/>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A9" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A9),"",'Info Cuencas'!A9)</f>
         <v/>
@@ -10559,26 +10593,30 @@
         <f>IF(A9="","",'Info Cuencas'!B9)</f>
         <v/>
       </c>
-      <c r="C9" s="6" t="str">
+      <c r="C9" s="4" t="str">
+        <f>IF(A9="","",'Info Cuencas'!C9)</f>
+        <v/>
+      </c>
+      <c r="D9" s="6" t="str">
         <f>IF(A9="","",0.133*'Info Cuencas'!R9)</f>
         <v/>
       </c>
-      <c r="D9" s="9"/>
-      <c r="E9" s="6" t="str">
-        <f>IF(A9="","",0.6*'Info Cuencas'!R9+HUS!D9/2)</f>
-        <v/>
-      </c>
+      <c r="E9" s="9"/>
       <c r="F9" s="6" t="str">
+        <f>IF(A9="","",0.6*'Info Cuencas'!R9+HUS!E9/2)</f>
+        <v/>
+      </c>
+      <c r="G9" s="6" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="G9" s="6" t="str">
-        <f>IF(A9="","",0.208*'Info Cuencas'!B9/HUS!E9)</f>
-        <v/>
-      </c>
-      <c r="H9" s="6"/>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="H9" s="6" t="str">
+        <f>IF(A9="","",0.208*'Info Cuencas'!B9/HUS!F9)</f>
+        <v/>
+      </c>
+      <c r="I9" s="6"/>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A10" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A10),"",'Info Cuencas'!A10)</f>
         <v/>
@@ -10587,26 +10625,30 @@
         <f>IF(A10="","",'Info Cuencas'!B10)</f>
         <v/>
       </c>
-      <c r="C10" s="6" t="str">
+      <c r="C10" s="4" t="str">
+        <f>IF(A10="","",'Info Cuencas'!C10)</f>
+        <v/>
+      </c>
+      <c r="D10" s="6" t="str">
         <f>IF(A10="","",0.133*'Info Cuencas'!R10)</f>
         <v/>
       </c>
-      <c r="D10" s="9"/>
-      <c r="E10" s="6" t="str">
-        <f>IF(A10="","",0.6*'Info Cuencas'!R10+HUS!D10/2)</f>
-        <v/>
-      </c>
+      <c r="E10" s="9"/>
       <c r="F10" s="6" t="str">
+        <f>IF(A10="","",0.6*'Info Cuencas'!R10+HUS!E10/2)</f>
+        <v/>
+      </c>
+      <c r="G10" s="6" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="G10" s="6" t="str">
-        <f>IF(A10="","",0.208*'Info Cuencas'!B10/HUS!E10)</f>
-        <v/>
-      </c>
-      <c r="H10" s="6"/>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="H10" s="6" t="str">
+        <f>IF(A10="","",0.208*'Info Cuencas'!B10/HUS!F10)</f>
+        <v/>
+      </c>
+      <c r="I10" s="6"/>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A11" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A11),"",'Info Cuencas'!A11)</f>
         <v/>
@@ -10615,26 +10657,30 @@
         <f>IF(A11="","",'Info Cuencas'!B11)</f>
         <v/>
       </c>
-      <c r="C11" s="6" t="str">
+      <c r="C11" s="4" t="str">
+        <f>IF(A11="","",'Info Cuencas'!C11)</f>
+        <v/>
+      </c>
+      <c r="D11" s="6" t="str">
         <f>IF(A11="","",0.133*'Info Cuencas'!R11)</f>
         <v/>
       </c>
-      <c r="D11" s="9"/>
-      <c r="E11" s="6" t="str">
-        <f>IF(A11="","",0.6*'Info Cuencas'!R11+HUS!D11/2)</f>
-        <v/>
-      </c>
+      <c r="E11" s="9"/>
       <c r="F11" s="6" t="str">
+        <f>IF(A11="","",0.6*'Info Cuencas'!R11+HUS!E11/2)</f>
+        <v/>
+      </c>
+      <c r="G11" s="6" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="G11" s="6" t="str">
-        <f>IF(A11="","",0.208*'Info Cuencas'!B11/HUS!E11)</f>
-        <v/>
-      </c>
-      <c r="H11" s="6"/>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="H11" s="6" t="str">
+        <f>IF(A11="","",0.208*'Info Cuencas'!B11/HUS!F11)</f>
+        <v/>
+      </c>
+      <c r="I11" s="6"/>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A12" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A12),"",'Info Cuencas'!A12)</f>
         <v/>
@@ -10643,17 +10689,21 @@
         <f>IF(A12="","",'Info Cuencas'!B12)</f>
         <v/>
       </c>
-      <c r="C12" t="str">
+      <c r="C12" s="4" t="str">
+        <f>IF(A12="","",'Info Cuencas'!C12)</f>
+        <v/>
+      </c>
+      <c r="D12" t="str">
         <f>IF(A12="","",0.133*'Info Cuencas'!R12)</f>
         <v/>
       </c>
-      <c r="D12" s="9"/>
-      <c r="E12" s="6" t="str">
-        <f>IF(A12="","",0.6*'Info Cuencas'!R12+HUS!D12/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="E12" s="9"/>
+      <c r="F12" s="6" t="str">
+        <f>IF(A12="","",0.6*'Info Cuencas'!R12+HUS!E12/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A13" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A13),"",'Info Cuencas'!A13)</f>
         <v/>
@@ -10662,17 +10712,21 @@
         <f>IF(A13="","",'Info Cuencas'!B13)</f>
         <v/>
       </c>
-      <c r="C13" t="str">
+      <c r="C13" s="4" t="str">
+        <f>IF(A13="","",'Info Cuencas'!C13)</f>
+        <v/>
+      </c>
+      <c r="D13" t="str">
         <f>IF(A13="","",0.133*'Info Cuencas'!R13)</f>
         <v/>
       </c>
-      <c r="D13" s="9"/>
-      <c r="E13" s="6" t="str">
-        <f>IF(A13="","",0.6*'Info Cuencas'!R13+HUS!D13/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="E13" s="9"/>
+      <c r="F13" s="6" t="str">
+        <f>IF(A13="","",0.6*'Info Cuencas'!R13+HUS!E13/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A14" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A14),"",'Info Cuencas'!A14)</f>
         <v/>
@@ -10681,17 +10735,21 @@
         <f>IF(A14="","",'Info Cuencas'!B14)</f>
         <v/>
       </c>
-      <c r="C14" t="str">
+      <c r="C14" s="4" t="str">
+        <f>IF(A14="","",'Info Cuencas'!C14)</f>
+        <v/>
+      </c>
+      <c r="D14" t="str">
         <f>IF(A14="","",0.133*'Info Cuencas'!R14)</f>
         <v/>
       </c>
-      <c r="D14" s="9"/>
-      <c r="E14" s="6" t="str">
-        <f>IF(A14="","",0.6*'Info Cuencas'!R14+HUS!D14/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="E14" s="9"/>
+      <c r="F14" s="6" t="str">
+        <f>IF(A14="","",0.6*'Info Cuencas'!R14+HUS!E14/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A15" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A15),"",'Info Cuencas'!A15)</f>
         <v/>
@@ -10700,16 +10758,20 @@
         <f>IF(A15="","",'Info Cuencas'!B15)</f>
         <v/>
       </c>
-      <c r="C15" t="str">
+      <c r="C15" s="4" t="str">
+        <f>IF(A15="","",'Info Cuencas'!C15)</f>
+        <v/>
+      </c>
+      <c r="D15" t="str">
         <f>IF(A15="","",0.133*'Info Cuencas'!R15)</f>
         <v/>
       </c>
-      <c r="E15" s="6" t="str">
-        <f>IF(A15="","",0.6*'Info Cuencas'!R15+HUS!D15/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="F15" s="6" t="str">
+        <f>IF(A15="","",0.6*'Info Cuencas'!R15+HUS!E15/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A16" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A16),"",'Info Cuencas'!A16)</f>
         <v/>
@@ -10718,16 +10780,20 @@
         <f>IF(A16="","",'Info Cuencas'!B16)</f>
         <v/>
       </c>
-      <c r="C16" t="str">
+      <c r="C16" s="4" t="str">
+        <f>IF(A16="","",'Info Cuencas'!C16)</f>
+        <v/>
+      </c>
+      <c r="D16" t="str">
         <f>IF(A16="","",0.133*'Info Cuencas'!R16)</f>
         <v/>
       </c>
-      <c r="E16" s="6" t="str">
-        <f>IF(A16="","",0.6*'Info Cuencas'!R16+HUS!D16/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F16" s="6" t="str">
+        <f>IF(A16="","",0.6*'Info Cuencas'!R16+HUS!E16/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A17" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A17),"",'Info Cuencas'!A17)</f>
         <v/>
@@ -10736,16 +10802,20 @@
         <f>IF(A17="","",'Info Cuencas'!B17)</f>
         <v/>
       </c>
-      <c r="C17" t="str">
+      <c r="C17" s="4" t="str">
+        <f>IF(A17="","",'Info Cuencas'!C17)</f>
+        <v/>
+      </c>
+      <c r="D17" t="str">
         <f>IF(A17="","",0.133*'Info Cuencas'!R17)</f>
         <v/>
       </c>
-      <c r="E17" s="6" t="str">
-        <f>IF(A17="","",0.6*'Info Cuencas'!R17+HUS!D17/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F17" s="6" t="str">
+        <f>IF(A17="","",0.6*'Info Cuencas'!R17+HUS!E17/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A18" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A18),"",'Info Cuencas'!A18)</f>
         <v/>
@@ -10754,16 +10824,20 @@
         <f>IF(A18="","",'Info Cuencas'!B18)</f>
         <v/>
       </c>
-      <c r="C18" t="str">
+      <c r="C18" s="4" t="str">
+        <f>IF(A18="","",'Info Cuencas'!C18)</f>
+        <v/>
+      </c>
+      <c r="D18" t="str">
         <f>IF(A18="","",0.133*'Info Cuencas'!R18)</f>
         <v/>
       </c>
-      <c r="E18" s="6" t="str">
-        <f>IF(A18="","",0.6*'Info Cuencas'!R18+HUS!D18/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F18" s="6" t="str">
+        <f>IF(A18="","",0.6*'Info Cuencas'!R18+HUS!E18/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A19" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A19),"",'Info Cuencas'!A19)</f>
         <v/>
@@ -10772,16 +10846,20 @@
         <f>IF(A19="","",'Info Cuencas'!B19)</f>
         <v/>
       </c>
-      <c r="C19" t="str">
+      <c r="C19" s="4" t="str">
+        <f>IF(A19="","",'Info Cuencas'!C19)</f>
+        <v/>
+      </c>
+      <c r="D19" t="str">
         <f>IF(A19="","",0.133*'Info Cuencas'!R19)</f>
         <v/>
       </c>
-      <c r="E19" s="6" t="str">
-        <f>IF(A19="","",0.6*'Info Cuencas'!R19+HUS!D19/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F19" s="6" t="str">
+        <f>IF(A19="","",0.6*'Info Cuencas'!R19+HUS!E19/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A20" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A20),"",'Info Cuencas'!A20)</f>
         <v/>
@@ -10790,16 +10868,20 @@
         <f>IF(A20="","",'Info Cuencas'!B20)</f>
         <v/>
       </c>
-      <c r="C20" t="str">
+      <c r="C20" s="4" t="str">
+        <f>IF(A20="","",'Info Cuencas'!C20)</f>
+        <v/>
+      </c>
+      <c r="D20" t="str">
         <f>IF(A20="","",0.133*'Info Cuencas'!R20)</f>
         <v/>
       </c>
-      <c r="E20" s="6" t="str">
-        <f>IF(A20="","",0.6*'Info Cuencas'!R20+HUS!D20/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F20" s="6" t="str">
+        <f>IF(A20="","",0.6*'Info Cuencas'!R20+HUS!E20/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A21" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A21),"",'Info Cuencas'!A21)</f>
         <v/>
@@ -10808,16 +10890,20 @@
         <f>IF(A21="","",'Info Cuencas'!B21)</f>
         <v/>
       </c>
-      <c r="C21" t="str">
+      <c r="C21" s="4" t="str">
+        <f>IF(A21="","",'Info Cuencas'!C21)</f>
+        <v/>
+      </c>
+      <c r="D21" t="str">
         <f>IF(A21="","",0.133*'Info Cuencas'!R21)</f>
         <v/>
       </c>
-      <c r="E21" s="6" t="str">
-        <f>IF(A21="","",0.6*'Info Cuencas'!R21+HUS!D21/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F21" s="6" t="str">
+        <f>IF(A21="","",0.6*'Info Cuencas'!R21+HUS!E21/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A22" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A22),"",'Info Cuencas'!A22)</f>
         <v/>
@@ -10826,16 +10912,20 @@
         <f>IF(A22="","",'Info Cuencas'!B22)</f>
         <v/>
       </c>
-      <c r="C22" t="str">
+      <c r="C22" s="4" t="str">
+        <f>IF(A22="","",'Info Cuencas'!C22)</f>
+        <v/>
+      </c>
+      <c r="D22" t="str">
         <f>IF(A22="","",0.133*'Info Cuencas'!R22)</f>
         <v/>
       </c>
-      <c r="E22" s="6" t="str">
-        <f>IF(A22="","",0.6*'Info Cuencas'!R22+HUS!D22/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F22" s="6" t="str">
+        <f>IF(A22="","",0.6*'Info Cuencas'!R22+HUS!E22/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A23" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A23),"",'Info Cuencas'!A23)</f>
         <v/>
@@ -10844,16 +10934,20 @@
         <f>IF(A23="","",'Info Cuencas'!B23)</f>
         <v/>
       </c>
-      <c r="C23" t="str">
+      <c r="C23" s="4" t="str">
+        <f>IF(A23="","",'Info Cuencas'!C23)</f>
+        <v/>
+      </c>
+      <c r="D23" t="str">
         <f>IF(A23="","",0.133*'Info Cuencas'!R23)</f>
         <v/>
       </c>
-      <c r="E23" s="6" t="str">
-        <f>IF(A23="","",0.6*'Info Cuencas'!R23+HUS!D23/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F23" s="6" t="str">
+        <f>IF(A23="","",0.6*'Info Cuencas'!R23+HUS!E23/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A24" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A24),"",'Info Cuencas'!A24)</f>
         <v/>
@@ -10862,16 +10956,20 @@
         <f>IF(A24="","",'Info Cuencas'!B24)</f>
         <v/>
       </c>
-      <c r="C24" t="str">
+      <c r="C24" s="4" t="str">
+        <f>IF(A24="","",'Info Cuencas'!C24)</f>
+        <v/>
+      </c>
+      <c r="D24" t="str">
         <f>IF(A24="","",0.133*'Info Cuencas'!R24)</f>
         <v/>
       </c>
-      <c r="E24" s="6" t="str">
-        <f>IF(A24="","",0.6*'Info Cuencas'!R24+HUS!D24/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F24" s="6" t="str">
+        <f>IF(A24="","",0.6*'Info Cuencas'!R24+HUS!E24/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A25" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A25),"",'Info Cuencas'!A25)</f>
         <v/>
@@ -10880,16 +10978,20 @@
         <f>IF(A25="","",'Info Cuencas'!B25)</f>
         <v/>
       </c>
-      <c r="C25" t="str">
+      <c r="C25" s="4" t="str">
+        <f>IF(A25="","",'Info Cuencas'!C25)</f>
+        <v/>
+      </c>
+      <c r="D25" t="str">
         <f>IF(A25="","",0.133*'Info Cuencas'!R25)</f>
         <v/>
       </c>
-      <c r="E25" s="6" t="str">
-        <f>IF(A25="","",0.6*'Info Cuencas'!R25+HUS!D25/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F25" s="6" t="str">
+        <f>IF(A25="","",0.6*'Info Cuencas'!R25+HUS!E25/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A26" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A26),"",'Info Cuencas'!A26)</f>
         <v/>
@@ -10898,16 +11000,20 @@
         <f>IF(A26="","",'Info Cuencas'!B26)</f>
         <v/>
       </c>
-      <c r="C26" t="str">
+      <c r="C26" s="4" t="str">
+        <f>IF(A26="","",'Info Cuencas'!C26)</f>
+        <v/>
+      </c>
+      <c r="D26" t="str">
         <f>IF(A26="","",0.133*'Info Cuencas'!R26)</f>
         <v/>
       </c>
-      <c r="E26" s="6" t="str">
-        <f>IF(A26="","",0.6*'Info Cuencas'!R26+HUS!D26/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F26" s="6" t="str">
+        <f>IF(A26="","",0.6*'Info Cuencas'!R26+HUS!E26/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A27" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A27),"",'Info Cuencas'!A27)</f>
         <v/>
@@ -10916,16 +11022,20 @@
         <f>IF(A27="","",'Info Cuencas'!B27)</f>
         <v/>
       </c>
-      <c r="C27" t="str">
+      <c r="C27" s="4" t="str">
+        <f>IF(A27="","",'Info Cuencas'!C27)</f>
+        <v/>
+      </c>
+      <c r="D27" t="str">
         <f>IF(A27="","",0.133*'Info Cuencas'!R27)</f>
         <v/>
       </c>
-      <c r="E27" s="6" t="str">
-        <f>IF(A27="","",0.6*'Info Cuencas'!R27+HUS!D27/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F27" s="6" t="str">
+        <f>IF(A27="","",0.6*'Info Cuencas'!R27+HUS!E27/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A28" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A28),"",'Info Cuencas'!A28)</f>
         <v/>
@@ -10934,16 +11044,20 @@
         <f>IF(A28="","",'Info Cuencas'!B28)</f>
         <v/>
       </c>
-      <c r="C28" t="str">
+      <c r="C28" s="4" t="str">
+        <f>IF(A28="","",'Info Cuencas'!C28)</f>
+        <v/>
+      </c>
+      <c r="D28" t="str">
         <f>IF(A28="","",0.133*'Info Cuencas'!R28)</f>
         <v/>
       </c>
-      <c r="E28" s="6" t="str">
-        <f>IF(A28="","",0.6*'Info Cuencas'!R28+HUS!D28/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F28" s="6" t="str">
+        <f>IF(A28="","",0.6*'Info Cuencas'!R28+HUS!E28/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A29" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A29),"",'Info Cuencas'!A29)</f>
         <v/>
@@ -10952,16 +11066,20 @@
         <f>IF(A29="","",'Info Cuencas'!B29)</f>
         <v/>
       </c>
-      <c r="C29" t="str">
+      <c r="C29" s="4" t="str">
+        <f>IF(A29="","",'Info Cuencas'!C29)</f>
+        <v/>
+      </c>
+      <c r="D29" t="str">
         <f>IF(A29="","",0.133*'Info Cuencas'!R29)</f>
         <v/>
       </c>
-      <c r="E29" s="6" t="str">
-        <f>IF(A29="","",0.6*'Info Cuencas'!R29+HUS!D29/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F29" s="6" t="str">
+        <f>IF(A29="","",0.6*'Info Cuencas'!R29+HUS!E29/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A30" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A30),"",'Info Cuencas'!A30)</f>
         <v/>
@@ -10970,16 +11088,20 @@
         <f>IF(A30="","",'Info Cuencas'!B30)</f>
         <v/>
       </c>
-      <c r="C30" t="str">
+      <c r="C30" s="4" t="str">
+        <f>IF(A30="","",'Info Cuencas'!C30)</f>
+        <v/>
+      </c>
+      <c r="D30" t="str">
         <f>IF(A30="","",0.133*'Info Cuencas'!R30)</f>
         <v/>
       </c>
-      <c r="E30" s="6" t="str">
-        <f>IF(A30="","",0.6*'Info Cuencas'!R30+HUS!D30/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F30" s="6" t="str">
+        <f>IF(A30="","",0.6*'Info Cuencas'!R30+HUS!E30/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A31" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A31),"",'Info Cuencas'!A31)</f>
         <v/>
@@ -10988,16 +11110,20 @@
         <f>IF(A31="","",'Info Cuencas'!B31)</f>
         <v/>
       </c>
-      <c r="C31" t="str">
+      <c r="C31" s="4" t="str">
+        <f>IF(A31="","",'Info Cuencas'!C31)</f>
+        <v/>
+      </c>
+      <c r="D31" t="str">
         <f>IF(A31="","",0.133*'Info Cuencas'!R31)</f>
         <v/>
       </c>
-      <c r="E31" s="6" t="str">
-        <f>IF(A31="","",0.6*'Info Cuencas'!R31+HUS!D31/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F31" s="6" t="str">
+        <f>IF(A31="","",0.6*'Info Cuencas'!R31+HUS!E31/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A32" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A32),"",'Info Cuencas'!A32)</f>
         <v/>
@@ -11006,16 +11132,20 @@
         <f>IF(A32="","",'Info Cuencas'!B32)</f>
         <v/>
       </c>
-      <c r="C32" t="str">
+      <c r="C32" s="4" t="str">
+        <f>IF(A32="","",'Info Cuencas'!C32)</f>
+        <v/>
+      </c>
+      <c r="D32" t="str">
         <f>IF(A32="","",0.133*'Info Cuencas'!R32)</f>
         <v/>
       </c>
-      <c r="E32" s="6" t="str">
-        <f>IF(A32="","",0.6*'Info Cuencas'!R32+HUS!D32/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F32" s="6" t="str">
+        <f>IF(A32="","",0.6*'Info Cuencas'!R32+HUS!E32/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A33" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A33),"",'Info Cuencas'!A33)</f>
         <v/>
@@ -11024,16 +11154,20 @@
         <f>IF(A33="","",'Info Cuencas'!B33)</f>
         <v/>
       </c>
-      <c r="C33" t="str">
+      <c r="C33" s="4" t="str">
+        <f>IF(A33="","",'Info Cuencas'!C33)</f>
+        <v/>
+      </c>
+      <c r="D33" t="str">
         <f>IF(A33="","",0.133*'Info Cuencas'!R33)</f>
         <v/>
       </c>
-      <c r="E33" s="6" t="str">
-        <f>IF(A33="","",0.6*'Info Cuencas'!R33+HUS!D33/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F33" s="6" t="str">
+        <f>IF(A33="","",0.6*'Info Cuencas'!R33+HUS!E33/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A34" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A34),"",'Info Cuencas'!A34)</f>
         <v/>
@@ -11042,16 +11176,20 @@
         <f>IF(A34="","",'Info Cuencas'!B34)</f>
         <v/>
       </c>
-      <c r="C34" t="str">
+      <c r="C34" s="4" t="str">
+        <f>IF(A34="","",'Info Cuencas'!C34)</f>
+        <v/>
+      </c>
+      <c r="D34" t="str">
         <f>IF(A34="","",0.133*'Info Cuencas'!R34)</f>
         <v/>
       </c>
-      <c r="E34" s="6" t="str">
-        <f>IF(A34="","",0.6*'Info Cuencas'!R34+HUS!D34/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F34" s="6" t="str">
+        <f>IF(A34="","",0.6*'Info Cuencas'!R34+HUS!E34/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A35" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A35),"",'Info Cuencas'!A35)</f>
         <v/>
@@ -11060,16 +11198,20 @@
         <f>IF(A35="","",'Info Cuencas'!B35)</f>
         <v/>
       </c>
-      <c r="C35" t="str">
+      <c r="C35" s="4" t="str">
+        <f>IF(A35="","",'Info Cuencas'!C35)</f>
+        <v/>
+      </c>
+      <c r="D35" t="str">
         <f>IF(A35="","",0.133*'Info Cuencas'!R35)</f>
         <v/>
       </c>
-      <c r="E35" s="6" t="str">
-        <f>IF(A35="","",0.6*'Info Cuencas'!R35+HUS!D35/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F35" s="6" t="str">
+        <f>IF(A35="","",0.6*'Info Cuencas'!R35+HUS!E35/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A36" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A36),"",'Info Cuencas'!A36)</f>
         <v/>
@@ -11078,16 +11220,20 @@
         <f>IF(A36="","",'Info Cuencas'!B36)</f>
         <v/>
       </c>
-      <c r="C36" t="str">
+      <c r="C36" s="4" t="str">
+        <f>IF(A36="","",'Info Cuencas'!C36)</f>
+        <v/>
+      </c>
+      <c r="D36" t="str">
         <f>IF(A36="","",0.133*'Info Cuencas'!R36)</f>
         <v/>
       </c>
-      <c r="E36" s="6" t="str">
-        <f>IF(A36="","",0.6*'Info Cuencas'!R36+HUS!D36/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F36" s="6" t="str">
+        <f>IF(A36="","",0.6*'Info Cuencas'!R36+HUS!E36/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A37" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A37),"",'Info Cuencas'!A37)</f>
         <v/>
@@ -11096,16 +11242,20 @@
         <f>IF(A37="","",'Info Cuencas'!B37)</f>
         <v/>
       </c>
-      <c r="C37" t="str">
+      <c r="C37" s="4" t="str">
+        <f>IF(A37="","",'Info Cuencas'!C37)</f>
+        <v/>
+      </c>
+      <c r="D37" t="str">
         <f>IF(A37="","",0.133*'Info Cuencas'!R37)</f>
         <v/>
       </c>
-      <c r="E37" s="6" t="str">
-        <f>IF(A37="","",0.6*'Info Cuencas'!R37+HUS!D37/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F37" s="6" t="str">
+        <f>IF(A37="","",0.6*'Info Cuencas'!R37+HUS!E37/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A38" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A38),"",'Info Cuencas'!A38)</f>
         <v/>
@@ -11114,16 +11264,20 @@
         <f>IF(A38="","",'Info Cuencas'!B38)</f>
         <v/>
       </c>
-      <c r="C38" t="str">
+      <c r="C38" s="4" t="str">
+        <f>IF(A38="","",'Info Cuencas'!C38)</f>
+        <v/>
+      </c>
+      <c r="D38" t="str">
         <f>IF(A38="","",0.133*'Info Cuencas'!R38)</f>
         <v/>
       </c>
-      <c r="E38" s="6" t="str">
-        <f>IF(A38="","",0.6*'Info Cuencas'!R38+HUS!D38/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F38" s="6" t="str">
+        <f>IF(A38="","",0.6*'Info Cuencas'!R38+HUS!E38/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A39" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A39),"",'Info Cuencas'!A39)</f>
         <v/>
@@ -11132,16 +11286,20 @@
         <f>IF(A39="","",'Info Cuencas'!B39)</f>
         <v/>
       </c>
-      <c r="C39" t="str">
+      <c r="C39" s="4" t="str">
+        <f>IF(A39="","",'Info Cuencas'!C39)</f>
+        <v/>
+      </c>
+      <c r="D39" t="str">
         <f>IF(A39="","",0.133*'Info Cuencas'!R39)</f>
         <v/>
       </c>
-      <c r="E39" s="6" t="str">
-        <f>IF(A39="","",0.6*'Info Cuencas'!R39+HUS!D39/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F39" s="6" t="str">
+        <f>IF(A39="","",0.6*'Info Cuencas'!R39+HUS!E39/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A40" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A40),"",'Info Cuencas'!A40)</f>
         <v/>
@@ -11150,16 +11308,20 @@
         <f>IF(A40="","",'Info Cuencas'!B40)</f>
         <v/>
       </c>
-      <c r="C40" t="str">
+      <c r="C40" s="4" t="str">
+        <f>IF(A40="","",'Info Cuencas'!C40)</f>
+        <v/>
+      </c>
+      <c r="D40" t="str">
         <f>IF(A40="","",0.133*'Info Cuencas'!R40)</f>
         <v/>
       </c>
-      <c r="E40" s="6" t="str">
-        <f>IF(A40="","",0.6*'Info Cuencas'!R40+HUS!D40/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F40" s="6" t="str">
+        <f>IF(A40="","",0.6*'Info Cuencas'!R40+HUS!E40/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A41" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A41),"",'Info Cuencas'!A41)</f>
         <v/>
@@ -11168,16 +11330,20 @@
         <f>IF(A41="","",'Info Cuencas'!B41)</f>
         <v/>
       </c>
-      <c r="C41" t="str">
+      <c r="C41" s="4" t="str">
+        <f>IF(A41="","",'Info Cuencas'!C41)</f>
+        <v/>
+      </c>
+      <c r="D41" t="str">
         <f>IF(A41="","",0.133*'Info Cuencas'!R41)</f>
         <v/>
       </c>
-      <c r="E41" s="6" t="str">
-        <f>IF(A41="","",0.6*'Info Cuencas'!R41+HUS!D41/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F41" s="6" t="str">
+        <f>IF(A41="","",0.6*'Info Cuencas'!R41+HUS!E41/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A42" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A42),"",'Info Cuencas'!A42)</f>
         <v/>
@@ -11186,16 +11352,20 @@
         <f>IF(A42="","",'Info Cuencas'!B42)</f>
         <v/>
       </c>
-      <c r="C42" t="str">
+      <c r="C42" s="4" t="str">
+        <f>IF(A42="","",'Info Cuencas'!C42)</f>
+        <v/>
+      </c>
+      <c r="D42" t="str">
         <f>IF(A42="","",0.133*'Info Cuencas'!R42)</f>
         <v/>
       </c>
-      <c r="E42" s="6" t="str">
-        <f>IF(A42="","",0.6*'Info Cuencas'!R42+HUS!D42/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F42" s="6" t="str">
+        <f>IF(A42="","",0.6*'Info Cuencas'!R42+HUS!E42/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A43" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A43),"",'Info Cuencas'!A43)</f>
         <v/>
@@ -11204,16 +11374,20 @@
         <f>IF(A43="","",'Info Cuencas'!B43)</f>
         <v/>
       </c>
-      <c r="C43" t="str">
+      <c r="C43" s="4" t="str">
+        <f>IF(A43="","",'Info Cuencas'!C43)</f>
+        <v/>
+      </c>
+      <c r="D43" t="str">
         <f>IF(A43="","",0.133*'Info Cuencas'!R43)</f>
         <v/>
       </c>
-      <c r="E43" s="6" t="str">
-        <f>IF(A43="","",0.6*'Info Cuencas'!R43+HUS!D43/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F43" s="6" t="str">
+        <f>IF(A43="","",0.6*'Info Cuencas'!R43+HUS!E43/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A44" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A44),"",'Info Cuencas'!A44)</f>
         <v/>
@@ -11222,16 +11396,20 @@
         <f>IF(A44="","",'Info Cuencas'!B44)</f>
         <v/>
       </c>
-      <c r="C44" t="str">
+      <c r="C44" s="4" t="str">
+        <f>IF(A44="","",'Info Cuencas'!C44)</f>
+        <v/>
+      </c>
+      <c r="D44" t="str">
         <f>IF(A44="","",0.133*'Info Cuencas'!R44)</f>
         <v/>
       </c>
-      <c r="E44" s="6" t="str">
-        <f>IF(A44="","",0.6*'Info Cuencas'!R44+HUS!D44/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F44" s="6" t="str">
+        <f>IF(A44="","",0.6*'Info Cuencas'!R44+HUS!E44/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A45" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A45),"",'Info Cuencas'!A45)</f>
         <v/>
@@ -11240,16 +11418,20 @@
         <f>IF(A45="","",'Info Cuencas'!B45)</f>
         <v/>
       </c>
-      <c r="C45" t="str">
+      <c r="C45" s="4" t="str">
+        <f>IF(A45="","",'Info Cuencas'!C45)</f>
+        <v/>
+      </c>
+      <c r="D45" t="str">
         <f>IF(A45="","",0.133*'Info Cuencas'!R45)</f>
         <v/>
       </c>
-      <c r="E45" s="6" t="str">
-        <f>IF(A45="","",0.6*'Info Cuencas'!R45+HUS!D45/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F45" s="6" t="str">
+        <f>IF(A45="","",0.6*'Info Cuencas'!R45+HUS!E45/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A46" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A46),"",'Info Cuencas'!A46)</f>
         <v/>
@@ -11258,16 +11440,20 @@
         <f>IF(A46="","",'Info Cuencas'!B46)</f>
         <v/>
       </c>
-      <c r="C46" t="str">
+      <c r="C46" s="4" t="str">
+        <f>IF(A46="","",'Info Cuencas'!C46)</f>
+        <v/>
+      </c>
+      <c r="D46" t="str">
         <f>IF(A46="","",0.133*'Info Cuencas'!R46)</f>
         <v/>
       </c>
-      <c r="E46" s="6" t="str">
-        <f>IF(A46="","",0.6*'Info Cuencas'!R46+HUS!D46/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F46" s="6" t="str">
+        <f>IF(A46="","",0.6*'Info Cuencas'!R46+HUS!E46/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A47" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A47),"",'Info Cuencas'!A47)</f>
         <v/>
@@ -11276,16 +11462,20 @@
         <f>IF(A47="","",'Info Cuencas'!B47)</f>
         <v/>
       </c>
-      <c r="C47" t="str">
+      <c r="C47" s="4" t="str">
+        <f>IF(A47="","",'Info Cuencas'!C47)</f>
+        <v/>
+      </c>
+      <c r="D47" t="str">
         <f>IF(A47="","",0.133*'Info Cuencas'!R47)</f>
         <v/>
       </c>
-      <c r="E47" s="6" t="str">
-        <f>IF(A47="","",0.6*'Info Cuencas'!R47+HUS!D47/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F47" s="6" t="str">
+        <f>IF(A47="","",0.6*'Info Cuencas'!R47+HUS!E47/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A48" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A48),"",'Info Cuencas'!A48)</f>
         <v/>
@@ -11294,16 +11484,20 @@
         <f>IF(A48="","",'Info Cuencas'!B48)</f>
         <v/>
       </c>
-      <c r="C48" t="str">
+      <c r="C48" s="4" t="str">
+        <f>IF(A48="","",'Info Cuencas'!C48)</f>
+        <v/>
+      </c>
+      <c r="D48" t="str">
         <f>IF(A48="","",0.133*'Info Cuencas'!R48)</f>
         <v/>
       </c>
-      <c r="E48" s="6" t="str">
-        <f>IF(A48="","",0.6*'Info Cuencas'!R48+HUS!D48/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F48" s="6" t="str">
+        <f>IF(A48="","",0.6*'Info Cuencas'!R48+HUS!E48/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A49" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A49),"",'Info Cuencas'!A49)</f>
         <v/>
@@ -11312,16 +11506,20 @@
         <f>IF(A49="","",'Info Cuencas'!B49)</f>
         <v/>
       </c>
-      <c r="C49" t="str">
+      <c r="C49" s="4" t="str">
+        <f>IF(A49="","",'Info Cuencas'!C49)</f>
+        <v/>
+      </c>
+      <c r="D49" t="str">
         <f>IF(A49="","",0.133*'Info Cuencas'!R49)</f>
         <v/>
       </c>
-      <c r="E49" s="6" t="str">
-        <f>IF(A49="","",0.6*'Info Cuencas'!R49+HUS!D49/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F49" s="6" t="str">
+        <f>IF(A49="","",0.6*'Info Cuencas'!R49+HUS!E49/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A50" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A50),"",'Info Cuencas'!A50)</f>
         <v/>
@@ -11330,16 +11528,20 @@
         <f>IF(A50="","",'Info Cuencas'!B50)</f>
         <v/>
       </c>
-      <c r="C50" t="str">
+      <c r="C50" s="4" t="str">
+        <f>IF(A50="","",'Info Cuencas'!C50)</f>
+        <v/>
+      </c>
+      <c r="D50" t="str">
         <f>IF(A50="","",0.133*'Info Cuencas'!R50)</f>
         <v/>
       </c>
-      <c r="E50" s="6" t="str">
-        <f>IF(A50="","",0.6*'Info Cuencas'!R50+HUS!D50/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F50" s="6" t="str">
+        <f>IF(A50="","",0.6*'Info Cuencas'!R50+HUS!E50/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A51" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A51),"",'Info Cuencas'!A51)</f>
         <v/>
@@ -11348,16 +11550,20 @@
         <f>IF(A51="","",'Info Cuencas'!B51)</f>
         <v/>
       </c>
-      <c r="C51" t="str">
+      <c r="C51" s="4" t="str">
+        <f>IF(A51="","",'Info Cuencas'!C51)</f>
+        <v/>
+      </c>
+      <c r="D51" t="str">
         <f>IF(A51="","",0.133*'Info Cuencas'!R51)</f>
         <v/>
       </c>
-      <c r="E51" s="6" t="str">
-        <f>IF(A51="","",0.6*'Info Cuencas'!R51+HUS!D51/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F51" s="6" t="str">
+        <f>IF(A51="","",0.6*'Info Cuencas'!R51+HUS!E51/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A52" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A52),"",'Info Cuencas'!A52)</f>
         <v/>
@@ -11366,16 +11572,20 @@
         <f>IF(A52="","",'Info Cuencas'!B52)</f>
         <v/>
       </c>
-      <c r="C52" t="str">
+      <c r="C52" s="4" t="str">
+        <f>IF(A52="","",'Info Cuencas'!C52)</f>
+        <v/>
+      </c>
+      <c r="D52" t="str">
         <f>IF(A52="","",0.133*'Info Cuencas'!R52)</f>
         <v/>
       </c>
-      <c r="E52" s="6" t="str">
-        <f>IF(A52="","",0.6*'Info Cuencas'!R52+HUS!D52/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F52" s="6" t="str">
+        <f>IF(A52="","",0.6*'Info Cuencas'!R52+HUS!E52/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A53" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A53),"",'Info Cuencas'!A53)</f>
         <v/>
@@ -11384,16 +11594,20 @@
         <f>IF(A53="","",'Info Cuencas'!B53)</f>
         <v/>
       </c>
-      <c r="C53" t="str">
+      <c r="C53" s="4" t="str">
+        <f>IF(A53="","",'Info Cuencas'!C53)</f>
+        <v/>
+      </c>
+      <c r="D53" t="str">
         <f>IF(A53="","",0.133*'Info Cuencas'!R53)</f>
         <v/>
       </c>
-      <c r="E53" s="6" t="str">
-        <f>IF(A53="","",0.6*'Info Cuencas'!R53+HUS!D53/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F53" s="6" t="str">
+        <f>IF(A53="","",0.6*'Info Cuencas'!R53+HUS!E53/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A54" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A54),"",'Info Cuencas'!A54)</f>
         <v/>
@@ -11402,16 +11616,20 @@
         <f>IF(A54="","",'Info Cuencas'!B54)</f>
         <v/>
       </c>
-      <c r="C54" t="str">
+      <c r="C54" s="4" t="str">
+        <f>IF(A54="","",'Info Cuencas'!C54)</f>
+        <v/>
+      </c>
+      <c r="D54" t="str">
         <f>IF(A54="","",0.133*'Info Cuencas'!R54)</f>
         <v/>
       </c>
-      <c r="E54" s="6" t="str">
-        <f>IF(A54="","",0.6*'Info Cuencas'!R54+HUS!D54/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F54" s="6" t="str">
+        <f>IF(A54="","",0.6*'Info Cuencas'!R54+HUS!E54/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A55" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A55),"",'Info Cuencas'!A55)</f>
         <v/>
@@ -11420,16 +11638,20 @@
         <f>IF(A55="","",'Info Cuencas'!B55)</f>
         <v/>
       </c>
-      <c r="C55" t="str">
+      <c r="C55" s="4" t="str">
+        <f>IF(A55="","",'Info Cuencas'!C55)</f>
+        <v/>
+      </c>
+      <c r="D55" t="str">
         <f>IF(A55="","",0.133*'Info Cuencas'!R55)</f>
         <v/>
       </c>
-      <c r="E55" s="6" t="str">
-        <f>IF(A55="","",0.6*'Info Cuencas'!R55+HUS!D55/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F55" s="6" t="str">
+        <f>IF(A55="","",0.6*'Info Cuencas'!R55+HUS!E55/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A56" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A56),"",'Info Cuencas'!A56)</f>
         <v/>
@@ -11438,16 +11660,20 @@
         <f>IF(A56="","",'Info Cuencas'!B56)</f>
         <v/>
       </c>
-      <c r="C56" t="str">
+      <c r="C56" s="4" t="str">
+        <f>IF(A56="","",'Info Cuencas'!C56)</f>
+        <v/>
+      </c>
+      <c r="D56" t="str">
         <f>IF(A56="","",0.133*'Info Cuencas'!R56)</f>
         <v/>
       </c>
-      <c r="E56" s="6" t="str">
-        <f>IF(A56="","",0.6*'Info Cuencas'!R56+HUS!D56/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F56" s="6" t="str">
+        <f>IF(A56="","",0.6*'Info Cuencas'!R56+HUS!E56/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A57" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A57),"",'Info Cuencas'!A57)</f>
         <v/>
@@ -11456,16 +11682,20 @@
         <f>IF(A57="","",'Info Cuencas'!B57)</f>
         <v/>
       </c>
-      <c r="C57" t="str">
+      <c r="C57" s="4" t="str">
+        <f>IF(A57="","",'Info Cuencas'!C57)</f>
+        <v/>
+      </c>
+      <c r="D57" t="str">
         <f>IF(A57="","",0.133*'Info Cuencas'!R57)</f>
         <v/>
       </c>
-      <c r="E57" s="6" t="str">
-        <f>IF(A57="","",0.6*'Info Cuencas'!R57+HUS!D57/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F57" s="6" t="str">
+        <f>IF(A57="","",0.6*'Info Cuencas'!R57+HUS!E57/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="58" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A58" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A58),"",'Info Cuencas'!A58)</f>
         <v/>
@@ -11474,16 +11704,20 @@
         <f>IF(A58="","",'Info Cuencas'!B58)</f>
         <v/>
       </c>
-      <c r="C58" t="str">
+      <c r="C58" s="4" t="str">
+        <f>IF(A58="","",'Info Cuencas'!C58)</f>
+        <v/>
+      </c>
+      <c r="D58" t="str">
         <f>IF(A58="","",0.133*'Info Cuencas'!R58)</f>
         <v/>
       </c>
-      <c r="E58" s="6" t="str">
-        <f>IF(A58="","",0.6*'Info Cuencas'!R58+HUS!D58/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F58" s="6" t="str">
+        <f>IF(A58="","",0.6*'Info Cuencas'!R58+HUS!E58/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="59" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A59" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A59),"",'Info Cuencas'!A59)</f>
         <v/>
@@ -11492,16 +11726,20 @@
         <f>IF(A59="","",'Info Cuencas'!B59)</f>
         <v/>
       </c>
-      <c r="C59" t="str">
+      <c r="C59" s="4" t="str">
+        <f>IF(A59="","",'Info Cuencas'!C59)</f>
+        <v/>
+      </c>
+      <c r="D59" t="str">
         <f>IF(A59="","",0.133*'Info Cuencas'!R59)</f>
         <v/>
       </c>
-      <c r="E59" s="6" t="str">
-        <f>IF(A59="","",0.6*'Info Cuencas'!R59+HUS!D59/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F59" s="6" t="str">
+        <f>IF(A59="","",0.6*'Info Cuencas'!R59+HUS!E59/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="60" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A60" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A60),"",'Info Cuencas'!A60)</f>
         <v/>
@@ -11510,16 +11748,20 @@
         <f>IF(A60="","",'Info Cuencas'!B60)</f>
         <v/>
       </c>
-      <c r="C60" t="str">
+      <c r="C60" s="4" t="str">
+        <f>IF(A60="","",'Info Cuencas'!C60)</f>
+        <v/>
+      </c>
+      <c r="D60" t="str">
         <f>IF(A60="","",0.133*'Info Cuencas'!R60)</f>
         <v/>
       </c>
-      <c r="E60" s="6" t="str">
-        <f>IF(A60="","",0.6*'Info Cuencas'!R60+HUS!D60/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F60" s="6" t="str">
+        <f>IF(A60="","",0.6*'Info Cuencas'!R60+HUS!E60/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="61" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A61" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A61),"",'Info Cuencas'!A61)</f>
         <v/>
@@ -11528,16 +11770,20 @@
         <f>IF(A61="","",'Info Cuencas'!B61)</f>
         <v/>
       </c>
-      <c r="C61" t="str">
+      <c r="C61" s="4" t="str">
+        <f>IF(A61="","",'Info Cuencas'!C61)</f>
+        <v/>
+      </c>
+      <c r="D61" t="str">
         <f>IF(A61="","",0.133*'Info Cuencas'!R61)</f>
         <v/>
       </c>
-      <c r="E61" s="6" t="str">
-        <f>IF(A61="","",0.6*'Info Cuencas'!R61+HUS!D61/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F61" s="6" t="str">
+        <f>IF(A61="","",0.6*'Info Cuencas'!R61+HUS!E61/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="62" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A62" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A62),"",'Info Cuencas'!A62)</f>
         <v/>
@@ -11546,16 +11792,20 @@
         <f>IF(A62="","",'Info Cuencas'!B62)</f>
         <v/>
       </c>
-      <c r="C62" t="str">
+      <c r="C62" s="4" t="str">
+        <f>IF(A62="","",'Info Cuencas'!C62)</f>
+        <v/>
+      </c>
+      <c r="D62" t="str">
         <f>IF(A62="","",0.133*'Info Cuencas'!R62)</f>
         <v/>
       </c>
-      <c r="E62" s="6" t="str">
-        <f>IF(A62="","",0.6*'Info Cuencas'!R62+HUS!D62/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F62" s="6" t="str">
+        <f>IF(A62="","",0.6*'Info Cuencas'!R62+HUS!E62/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="63" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A63" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A63),"",'Info Cuencas'!A63)</f>
         <v/>
@@ -11564,16 +11814,20 @@
         <f>IF(A63="","",'Info Cuencas'!B63)</f>
         <v/>
       </c>
-      <c r="C63" t="str">
+      <c r="C63" s="4" t="str">
+        <f>IF(A63="","",'Info Cuencas'!C63)</f>
+        <v/>
+      </c>
+      <c r="D63" t="str">
         <f>IF(A63="","",0.133*'Info Cuencas'!R63)</f>
         <v/>
       </c>
-      <c r="E63" s="6" t="str">
-        <f>IF(A63="","",0.6*'Info Cuencas'!R63+HUS!D63/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F63" s="6" t="str">
+        <f>IF(A63="","",0.6*'Info Cuencas'!R63+HUS!E63/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="64" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A64" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A64),"",'Info Cuencas'!A64)</f>
         <v/>
@@ -11582,16 +11836,20 @@
         <f>IF(A64="","",'Info Cuencas'!B64)</f>
         <v/>
       </c>
-      <c r="C64" t="str">
+      <c r="C64" s="4" t="str">
+        <f>IF(A64="","",'Info Cuencas'!C64)</f>
+        <v/>
+      </c>
+      <c r="D64" t="str">
         <f>IF(A64="","",0.133*'Info Cuencas'!R64)</f>
         <v/>
       </c>
-      <c r="E64" s="6" t="str">
-        <f>IF(A64="","",0.6*'Info Cuencas'!R64+HUS!D64/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F64" s="6" t="str">
+        <f>IF(A64="","",0.6*'Info Cuencas'!R64+HUS!E64/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="65" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A65" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A65),"",'Info Cuencas'!A65)</f>
         <v/>
@@ -11600,16 +11858,20 @@
         <f>IF(A65="","",'Info Cuencas'!B65)</f>
         <v/>
       </c>
-      <c r="C65" t="str">
+      <c r="C65" s="4" t="str">
+        <f>IF(A65="","",'Info Cuencas'!C65)</f>
+        <v/>
+      </c>
+      <c r="D65" t="str">
         <f>IF(A65="","",0.133*'Info Cuencas'!R65)</f>
         <v/>
       </c>
-      <c r="E65" s="6" t="str">
-        <f>IF(A65="","",0.6*'Info Cuencas'!R65+HUS!D65/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F65" s="6" t="str">
+        <f>IF(A65="","",0.6*'Info Cuencas'!R65+HUS!E65/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="66" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A66" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A66),"",'Info Cuencas'!A66)</f>
         <v/>
@@ -11618,16 +11880,20 @@
         <f>IF(A66="","",'Info Cuencas'!B66)</f>
         <v/>
       </c>
-      <c r="C66" t="str">
+      <c r="C66" s="4" t="str">
+        <f>IF(A66="","",'Info Cuencas'!C66)</f>
+        <v/>
+      </c>
+      <c r="D66" t="str">
         <f>IF(A66="","",0.133*'Info Cuencas'!R66)</f>
         <v/>
       </c>
-      <c r="E66" s="6" t="str">
-        <f>IF(A66="","",0.6*'Info Cuencas'!R66+HUS!D66/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F66" s="6" t="str">
+        <f>IF(A66="","",0.6*'Info Cuencas'!R66+HUS!E66/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A67" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A67),"",'Info Cuencas'!A67)</f>
         <v/>
@@ -11636,16 +11902,20 @@
         <f>IF(A67="","",'Info Cuencas'!B67)</f>
         <v/>
       </c>
-      <c r="C67" t="str">
+      <c r="C67" s="4" t="str">
+        <f>IF(A67="","",'Info Cuencas'!C67)</f>
+        <v/>
+      </c>
+      <c r="D67" t="str">
         <f>IF(A67="","",0.133*'Info Cuencas'!R67)</f>
         <v/>
       </c>
-      <c r="E67" s="6" t="str">
-        <f>IF(A67="","",0.6*'Info Cuencas'!R67+HUS!D67/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F67" s="6" t="str">
+        <f>IF(A67="","",0.6*'Info Cuencas'!R67+HUS!E67/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="68" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A68" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A68),"",'Info Cuencas'!A68)</f>
         <v/>
@@ -11654,16 +11924,20 @@
         <f>IF(A68="","",'Info Cuencas'!B68)</f>
         <v/>
       </c>
-      <c r="C68" t="str">
+      <c r="C68" s="4" t="str">
+        <f>IF(A68="","",'Info Cuencas'!C68)</f>
+        <v/>
+      </c>
+      <c r="D68" t="str">
         <f>IF(A68="","",0.133*'Info Cuencas'!R68)</f>
         <v/>
       </c>
-      <c r="E68" s="6" t="str">
-        <f>IF(A68="","",0.6*'Info Cuencas'!R68+HUS!D68/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F68" s="6" t="str">
+        <f>IF(A68="","",0.6*'Info Cuencas'!R68+HUS!E68/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="69" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A69" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A69),"",'Info Cuencas'!A69)</f>
         <v/>
@@ -11672,16 +11946,20 @@
         <f>IF(A69="","",'Info Cuencas'!B69)</f>
         <v/>
       </c>
-      <c r="C69" t="str">
+      <c r="C69" s="4" t="str">
+        <f>IF(A69="","",'Info Cuencas'!C69)</f>
+        <v/>
+      </c>
+      <c r="D69" t="str">
         <f>IF(A69="","",0.133*'Info Cuencas'!R69)</f>
         <v/>
       </c>
-      <c r="E69" s="6" t="str">
-        <f>IF(A69="","",0.6*'Info Cuencas'!R69+HUS!D69/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F69" s="6" t="str">
+        <f>IF(A69="","",0.6*'Info Cuencas'!R69+HUS!E69/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="70" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A70" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A70),"",'Info Cuencas'!A70)</f>
         <v/>
@@ -11690,16 +11968,20 @@
         <f>IF(A70="","",'Info Cuencas'!B70)</f>
         <v/>
       </c>
-      <c r="C70" t="str">
+      <c r="C70" s="4" t="str">
+        <f>IF(A70="","",'Info Cuencas'!C70)</f>
+        <v/>
+      </c>
+      <c r="D70" t="str">
         <f>IF(A70="","",0.133*'Info Cuencas'!R70)</f>
         <v/>
       </c>
-      <c r="E70" s="6" t="str">
-        <f>IF(A70="","",0.6*'Info Cuencas'!R70+HUS!D70/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="71" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F70" s="6" t="str">
+        <f>IF(A70="","",0.6*'Info Cuencas'!R70+HUS!E70/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="71" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A71" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A71),"",'Info Cuencas'!A71)</f>
         <v/>
@@ -11708,16 +11990,20 @@
         <f>IF(A71="","",'Info Cuencas'!B71)</f>
         <v/>
       </c>
-      <c r="C71" t="str">
+      <c r="C71" s="4" t="str">
+        <f>IF(A71="","",'Info Cuencas'!C71)</f>
+        <v/>
+      </c>
+      <c r="D71" t="str">
         <f>IF(A71="","",0.133*'Info Cuencas'!R71)</f>
         <v/>
       </c>
-      <c r="E71" s="6" t="str">
-        <f>IF(A71="","",0.6*'Info Cuencas'!R71+HUS!D71/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F71" s="6" t="str">
+        <f>IF(A71="","",0.6*'Info Cuencas'!R71+HUS!E71/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="72" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A72" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A72),"",'Info Cuencas'!A72)</f>
         <v/>
@@ -11726,16 +12012,20 @@
         <f>IF(A72="","",'Info Cuencas'!B72)</f>
         <v/>
       </c>
-      <c r="C72" t="str">
+      <c r="C72" s="4" t="str">
+        <f>IF(A72="","",'Info Cuencas'!C72)</f>
+        <v/>
+      </c>
+      <c r="D72" t="str">
         <f>IF(A72="","",0.133*'Info Cuencas'!R72)</f>
         <v/>
       </c>
-      <c r="E72" s="6" t="str">
-        <f>IF(A72="","",0.6*'Info Cuencas'!R72+HUS!D72/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F72" s="6" t="str">
+        <f>IF(A72="","",0.6*'Info Cuencas'!R72+HUS!E72/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="73" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A73" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A73),"",'Info Cuencas'!A73)</f>
         <v/>
@@ -11744,16 +12034,20 @@
         <f>IF(A73="","",'Info Cuencas'!B73)</f>
         <v/>
       </c>
-      <c r="C73" t="str">
+      <c r="C73" s="4" t="str">
+        <f>IF(A73="","",'Info Cuencas'!C73)</f>
+        <v/>
+      </c>
+      <c r="D73" t="str">
         <f>IF(A73="","",0.133*'Info Cuencas'!R73)</f>
         <v/>
       </c>
-      <c r="E73" s="6" t="str">
-        <f>IF(A73="","",0.6*'Info Cuencas'!R73+HUS!D73/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F73" s="6" t="str">
+        <f>IF(A73="","",0.6*'Info Cuencas'!R73+HUS!E73/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="74" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A74" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A74),"",'Info Cuencas'!A74)</f>
         <v/>
@@ -11762,16 +12056,20 @@
         <f>IF(A74="","",'Info Cuencas'!B74)</f>
         <v/>
       </c>
-      <c r="C74" t="str">
+      <c r="C74" s="4" t="str">
+        <f>IF(A74="","",'Info Cuencas'!C74)</f>
+        <v/>
+      </c>
+      <c r="D74" t="str">
         <f>IF(A74="","",0.133*'Info Cuencas'!R74)</f>
         <v/>
       </c>
-      <c r="E74" s="6" t="str">
-        <f>IF(A74="","",0.6*'Info Cuencas'!R74+HUS!D74/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F74" s="6" t="str">
+        <f>IF(A74="","",0.6*'Info Cuencas'!R74+HUS!E74/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="75" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A75" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A75),"",'Info Cuencas'!A75)</f>
         <v/>
@@ -11780,16 +12078,20 @@
         <f>IF(A75="","",'Info Cuencas'!B75)</f>
         <v/>
       </c>
-      <c r="C75" t="str">
+      <c r="C75" s="4" t="str">
+        <f>IF(A75="","",'Info Cuencas'!C75)</f>
+        <v/>
+      </c>
+      <c r="D75" t="str">
         <f>IF(A75="","",0.133*'Info Cuencas'!R75)</f>
         <v/>
       </c>
-      <c r="E75" s="6" t="str">
-        <f>IF(A75="","",0.6*'Info Cuencas'!R75+HUS!D75/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F75" s="6" t="str">
+        <f>IF(A75="","",0.6*'Info Cuencas'!R75+HUS!E75/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="76" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A76" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A76),"",'Info Cuencas'!A76)</f>
         <v/>
@@ -11798,16 +12100,20 @@
         <f>IF(A76="","",'Info Cuencas'!B76)</f>
         <v/>
       </c>
-      <c r="C76" t="str">
+      <c r="C76" s="4" t="str">
+        <f>IF(A76="","",'Info Cuencas'!C76)</f>
+        <v/>
+      </c>
+      <c r="D76" t="str">
         <f>IF(A76="","",0.133*'Info Cuencas'!R76)</f>
         <v/>
       </c>
-      <c r="E76" s="6" t="str">
-        <f>IF(A76="","",0.6*'Info Cuencas'!R76+HUS!D76/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="77" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F76" s="6" t="str">
+        <f>IF(A76="","",0.6*'Info Cuencas'!R76+HUS!E76/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="77" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A77" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A77),"",'Info Cuencas'!A77)</f>
         <v/>
@@ -11816,16 +12122,20 @@
         <f>IF(A77="","",'Info Cuencas'!B77)</f>
         <v/>
       </c>
-      <c r="C77" t="str">
+      <c r="C77" s="4" t="str">
+        <f>IF(A77="","",'Info Cuencas'!C77)</f>
+        <v/>
+      </c>
+      <c r="D77" t="str">
         <f>IF(A77="","",0.133*'Info Cuencas'!R77)</f>
         <v/>
       </c>
-      <c r="E77" s="6" t="str">
-        <f>IF(A77="","",0.6*'Info Cuencas'!R77+HUS!D77/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="78" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F77" s="6" t="str">
+        <f>IF(A77="","",0.6*'Info Cuencas'!R77+HUS!E77/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="78" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A78" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A78),"",'Info Cuencas'!A78)</f>
         <v/>
@@ -11834,16 +12144,20 @@
         <f>IF(A78="","",'Info Cuencas'!B78)</f>
         <v/>
       </c>
-      <c r="C78" t="str">
+      <c r="C78" s="4" t="str">
+        <f>IF(A78="","",'Info Cuencas'!C78)</f>
+        <v/>
+      </c>
+      <c r="D78" t="str">
         <f>IF(A78="","",0.133*'Info Cuencas'!R78)</f>
         <v/>
       </c>
-      <c r="E78" s="6" t="str">
-        <f>IF(A78="","",0.6*'Info Cuencas'!R78+HUS!D78/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="79" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F78" s="6" t="str">
+        <f>IF(A78="","",0.6*'Info Cuencas'!R78+HUS!E78/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="79" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A79" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A79),"",'Info Cuencas'!A79)</f>
         <v/>
@@ -11852,16 +12166,20 @@
         <f>IF(A79="","",'Info Cuencas'!B79)</f>
         <v/>
       </c>
-      <c r="C79" t="str">
+      <c r="C79" s="4" t="str">
+        <f>IF(A79="","",'Info Cuencas'!C79)</f>
+        <v/>
+      </c>
+      <c r="D79" t="str">
         <f>IF(A79="","",0.133*'Info Cuencas'!R79)</f>
         <v/>
       </c>
-      <c r="E79" s="6" t="str">
-        <f>IF(A79="","",0.6*'Info Cuencas'!R79+HUS!D79/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="80" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F79" s="6" t="str">
+        <f>IF(A79="","",0.6*'Info Cuencas'!R79+HUS!E79/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="80" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A80" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A80),"",'Info Cuencas'!A80)</f>
         <v/>
@@ -11870,16 +12188,20 @@
         <f>IF(A80="","",'Info Cuencas'!B80)</f>
         <v/>
       </c>
-      <c r="C80" t="str">
+      <c r="C80" s="4" t="str">
+        <f>IF(A80="","",'Info Cuencas'!C80)</f>
+        <v/>
+      </c>
+      <c r="D80" t="str">
         <f>IF(A80="","",0.133*'Info Cuencas'!R80)</f>
         <v/>
       </c>
-      <c r="E80" s="6" t="str">
-        <f>IF(A80="","",0.6*'Info Cuencas'!R80+HUS!D80/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="81" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F80" s="6" t="str">
+        <f>IF(A80="","",0.6*'Info Cuencas'!R80+HUS!E80/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="81" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A81" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A81),"",'Info Cuencas'!A81)</f>
         <v/>
@@ -11888,16 +12210,20 @@
         <f>IF(A81="","",'Info Cuencas'!B81)</f>
         <v/>
       </c>
-      <c r="C81" t="str">
+      <c r="C81" s="4" t="str">
+        <f>IF(A81="","",'Info Cuencas'!C81)</f>
+        <v/>
+      </c>
+      <c r="D81" t="str">
         <f>IF(A81="","",0.133*'Info Cuencas'!R81)</f>
         <v/>
       </c>
-      <c r="E81" s="6" t="str">
-        <f>IF(A81="","",0.6*'Info Cuencas'!R81+HUS!D81/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="82" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F81" s="6" t="str">
+        <f>IF(A81="","",0.6*'Info Cuencas'!R81+HUS!E81/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="82" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A82" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A82),"",'Info Cuencas'!A82)</f>
         <v/>
@@ -11906,16 +12232,20 @@
         <f>IF(A82="","",'Info Cuencas'!B82)</f>
         <v/>
       </c>
-      <c r="C82" t="str">
+      <c r="C82" s="4" t="str">
+        <f>IF(A82="","",'Info Cuencas'!C82)</f>
+        <v/>
+      </c>
+      <c r="D82" t="str">
         <f>IF(A82="","",0.133*'Info Cuencas'!R82)</f>
         <v/>
       </c>
-      <c r="E82" s="6" t="str">
-        <f>IF(A82="","",0.6*'Info Cuencas'!R82+HUS!D82/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="83" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F82" s="6" t="str">
+        <f>IF(A82="","",0.6*'Info Cuencas'!R82+HUS!E82/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="83" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A83" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A83),"",'Info Cuencas'!A83)</f>
         <v/>
@@ -11924,16 +12254,20 @@
         <f>IF(A83="","",'Info Cuencas'!B83)</f>
         <v/>
       </c>
-      <c r="C83" t="str">
+      <c r="C83" s="4" t="str">
+        <f>IF(A83="","",'Info Cuencas'!C83)</f>
+        <v/>
+      </c>
+      <c r="D83" t="str">
         <f>IF(A83="","",0.133*'Info Cuencas'!R83)</f>
         <v/>
       </c>
-      <c r="E83" s="6" t="str">
-        <f>IF(A83="","",0.6*'Info Cuencas'!R83+HUS!D83/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="84" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F83" s="6" t="str">
+        <f>IF(A83="","",0.6*'Info Cuencas'!R83+HUS!E83/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="84" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A84" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A84),"",'Info Cuencas'!A84)</f>
         <v/>
@@ -11942,16 +12276,20 @@
         <f>IF(A84="","",'Info Cuencas'!B84)</f>
         <v/>
       </c>
-      <c r="C84" t="str">
+      <c r="C84" s="4" t="str">
+        <f>IF(A84="","",'Info Cuencas'!C84)</f>
+        <v/>
+      </c>
+      <c r="D84" t="str">
         <f>IF(A84="","",0.133*'Info Cuencas'!R84)</f>
         <v/>
       </c>
-      <c r="E84" s="6" t="str">
-        <f>IF(A84="","",0.6*'Info Cuencas'!R84+HUS!D84/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="85" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F84" s="6" t="str">
+        <f>IF(A84="","",0.6*'Info Cuencas'!R84+HUS!E84/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="85" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A85" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A85),"",'Info Cuencas'!A85)</f>
         <v/>
@@ -11960,16 +12298,20 @@
         <f>IF(A85="","",'Info Cuencas'!B85)</f>
         <v/>
       </c>
-      <c r="C85" t="str">
+      <c r="C85" s="4" t="str">
+        <f>IF(A85="","",'Info Cuencas'!C85)</f>
+        <v/>
+      </c>
+      <c r="D85" t="str">
         <f>IF(A85="","",0.133*'Info Cuencas'!R85)</f>
         <v/>
       </c>
-      <c r="E85" s="6" t="str">
-        <f>IF(A85="","",0.6*'Info Cuencas'!R85+HUS!D85/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="86" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F85" s="6" t="str">
+        <f>IF(A85="","",0.6*'Info Cuencas'!R85+HUS!E85/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="86" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A86" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A86),"",'Info Cuencas'!A86)</f>
         <v/>
@@ -11978,16 +12320,20 @@
         <f>IF(A86="","",'Info Cuencas'!B86)</f>
         <v/>
       </c>
-      <c r="C86" t="str">
+      <c r="C86" s="4" t="str">
+        <f>IF(A86="","",'Info Cuencas'!C86)</f>
+        <v/>
+      </c>
+      <c r="D86" t="str">
         <f>IF(A86="","",0.133*'Info Cuencas'!R86)</f>
         <v/>
       </c>
-      <c r="E86" s="6" t="str">
-        <f>IF(A86="","",0.6*'Info Cuencas'!R86+HUS!D86/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="87" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F86" s="6" t="str">
+        <f>IF(A86="","",0.6*'Info Cuencas'!R86+HUS!E86/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="87" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A87" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A87),"",'Info Cuencas'!A87)</f>
         <v/>
@@ -11996,16 +12342,20 @@
         <f>IF(A87="","",'Info Cuencas'!B87)</f>
         <v/>
       </c>
-      <c r="C87" t="str">
+      <c r="C87" s="4" t="str">
+        <f>IF(A87="","",'Info Cuencas'!C87)</f>
+        <v/>
+      </c>
+      <c r="D87" t="str">
         <f>IF(A87="","",0.133*'Info Cuencas'!R87)</f>
         <v/>
       </c>
-      <c r="E87" s="6" t="str">
-        <f>IF(A87="","",0.6*'Info Cuencas'!R87+HUS!D87/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="88" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F87" s="6" t="str">
+        <f>IF(A87="","",0.6*'Info Cuencas'!R87+HUS!E87/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="88" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A88" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A88),"",'Info Cuencas'!A88)</f>
         <v/>
@@ -12014,16 +12364,20 @@
         <f>IF(A88="","",'Info Cuencas'!B88)</f>
         <v/>
       </c>
-      <c r="C88" t="str">
+      <c r="C88" s="4" t="str">
+        <f>IF(A88="","",'Info Cuencas'!C88)</f>
+        <v/>
+      </c>
+      <c r="D88" t="str">
         <f>IF(A88="","",0.133*'Info Cuencas'!R88)</f>
         <v/>
       </c>
-      <c r="E88" s="6" t="str">
-        <f>IF(A88="","",0.6*'Info Cuencas'!R88+HUS!D88/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="89" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F88" s="6" t="str">
+        <f>IF(A88="","",0.6*'Info Cuencas'!R88+HUS!E88/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="89" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A89" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A89),"",'Info Cuencas'!A89)</f>
         <v/>
@@ -12032,16 +12386,20 @@
         <f>IF(A89="","",'Info Cuencas'!B89)</f>
         <v/>
       </c>
-      <c r="C89" t="str">
+      <c r="C89" s="4" t="str">
+        <f>IF(A89="","",'Info Cuencas'!C89)</f>
+        <v/>
+      </c>
+      <c r="D89" t="str">
         <f>IF(A89="","",0.133*'Info Cuencas'!R89)</f>
         <v/>
       </c>
-      <c r="E89" s="6" t="str">
-        <f>IF(A89="","",0.6*'Info Cuencas'!R89+HUS!D89/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="90" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F89" s="6" t="str">
+        <f>IF(A89="","",0.6*'Info Cuencas'!R89+HUS!E89/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="90" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A90" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A90),"",'Info Cuencas'!A90)</f>
         <v/>
@@ -12050,16 +12408,20 @@
         <f>IF(A90="","",'Info Cuencas'!B90)</f>
         <v/>
       </c>
-      <c r="C90" t="str">
+      <c r="C90" s="4" t="str">
+        <f>IF(A90="","",'Info Cuencas'!C90)</f>
+        <v/>
+      </c>
+      <c r="D90" t="str">
         <f>IF(A90="","",0.133*'Info Cuencas'!R90)</f>
         <v/>
       </c>
-      <c r="E90" s="6" t="str">
-        <f>IF(A90="","",0.6*'Info Cuencas'!R90+HUS!D90/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="91" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F90" s="6" t="str">
+        <f>IF(A90="","",0.6*'Info Cuencas'!R90+HUS!E90/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="91" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A91" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A91),"",'Info Cuencas'!A91)</f>
         <v/>
@@ -12068,16 +12430,20 @@
         <f>IF(A91="","",'Info Cuencas'!B91)</f>
         <v/>
       </c>
-      <c r="C91" t="str">
+      <c r="C91" s="4" t="str">
+        <f>IF(A91="","",'Info Cuencas'!C91)</f>
+        <v/>
+      </c>
+      <c r="D91" t="str">
         <f>IF(A91="","",0.133*'Info Cuencas'!R91)</f>
         <v/>
       </c>
-      <c r="E91" s="6" t="str">
-        <f>IF(A91="","",0.6*'Info Cuencas'!R91+HUS!D91/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="92" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F91" s="6" t="str">
+        <f>IF(A91="","",0.6*'Info Cuencas'!R91+HUS!E91/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="92" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A92" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A92),"",'Info Cuencas'!A92)</f>
         <v/>
@@ -12086,16 +12452,20 @@
         <f>IF(A92="","",'Info Cuencas'!B92)</f>
         <v/>
       </c>
-      <c r="C92" t="str">
+      <c r="C92" s="4" t="str">
+        <f>IF(A92="","",'Info Cuencas'!C92)</f>
+        <v/>
+      </c>
+      <c r="D92" t="str">
         <f>IF(A92="","",0.133*'Info Cuencas'!R92)</f>
         <v/>
       </c>
-      <c r="E92" s="6" t="str">
-        <f>IF(A92="","",0.6*'Info Cuencas'!R92+HUS!D92/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="93" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F92" s="6" t="str">
+        <f>IF(A92="","",0.6*'Info Cuencas'!R92+HUS!E92/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="93" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A93" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A93),"",'Info Cuencas'!A93)</f>
         <v/>
@@ -12104,16 +12474,20 @@
         <f>IF(A93="","",'Info Cuencas'!B93)</f>
         <v/>
       </c>
-      <c r="C93" t="str">
+      <c r="C93" s="4" t="str">
+        <f>IF(A93="","",'Info Cuencas'!C93)</f>
+        <v/>
+      </c>
+      <c r="D93" t="str">
         <f>IF(A93="","",0.133*'Info Cuencas'!R93)</f>
         <v/>
       </c>
-      <c r="E93" s="6" t="str">
-        <f>IF(A93="","",0.6*'Info Cuencas'!R93+HUS!D93/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="94" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F93" s="6" t="str">
+        <f>IF(A93="","",0.6*'Info Cuencas'!R93+HUS!E93/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="94" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A94" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A94),"",'Info Cuencas'!A94)</f>
         <v/>
@@ -12122,16 +12496,20 @@
         <f>IF(A94="","",'Info Cuencas'!B94)</f>
         <v/>
       </c>
-      <c r="C94" t="str">
+      <c r="C94" s="4" t="str">
+        <f>IF(A94="","",'Info Cuencas'!C94)</f>
+        <v/>
+      </c>
+      <c r="D94" t="str">
         <f>IF(A94="","",0.133*'Info Cuencas'!R94)</f>
         <v/>
       </c>
-      <c r="E94" s="6" t="str">
-        <f>IF(A94="","",0.6*'Info Cuencas'!R94+HUS!D94/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="95" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F94" s="6" t="str">
+        <f>IF(A94="","",0.6*'Info Cuencas'!R94+HUS!E94/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="95" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A95" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A95),"",'Info Cuencas'!A95)</f>
         <v/>
@@ -12140,16 +12518,20 @@
         <f>IF(A95="","",'Info Cuencas'!B95)</f>
         <v/>
       </c>
-      <c r="C95" t="str">
+      <c r="C95" s="4" t="str">
+        <f>IF(A95="","",'Info Cuencas'!C95)</f>
+        <v/>
+      </c>
+      <c r="D95" t="str">
         <f>IF(A95="","",0.133*'Info Cuencas'!R95)</f>
         <v/>
       </c>
-      <c r="E95" s="6" t="str">
-        <f>IF(A95="","",0.6*'Info Cuencas'!R95+HUS!D95/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="96" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F95" s="6" t="str">
+        <f>IF(A95="","",0.6*'Info Cuencas'!R95+HUS!E95/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="96" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A96" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A96),"",'Info Cuencas'!A96)</f>
         <v/>
@@ -12158,16 +12540,20 @@
         <f>IF(A96="","",'Info Cuencas'!B96)</f>
         <v/>
       </c>
-      <c r="C96" t="str">
+      <c r="C96" s="4" t="str">
+        <f>IF(A96="","",'Info Cuencas'!C96)</f>
+        <v/>
+      </c>
+      <c r="D96" t="str">
         <f>IF(A96="","",0.133*'Info Cuencas'!R96)</f>
         <v/>
       </c>
-      <c r="E96" s="6" t="str">
-        <f>IF(A96="","",0.6*'Info Cuencas'!R96+HUS!D96/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="97" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F96" s="6" t="str">
+        <f>IF(A96="","",0.6*'Info Cuencas'!R96+HUS!E96/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="97" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A97" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A97),"",'Info Cuencas'!A97)</f>
         <v/>
@@ -12176,16 +12562,20 @@
         <f>IF(A97="","",'Info Cuencas'!B97)</f>
         <v/>
       </c>
-      <c r="C97" t="str">
+      <c r="C97" s="4" t="str">
+        <f>IF(A97="","",'Info Cuencas'!C97)</f>
+        <v/>
+      </c>
+      <c r="D97" t="str">
         <f>IF(A97="","",0.133*'Info Cuencas'!R97)</f>
         <v/>
       </c>
-      <c r="E97" s="6" t="str">
-        <f>IF(A97="","",0.6*'Info Cuencas'!R97+HUS!D97/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="98" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F97" s="6" t="str">
+        <f>IF(A97="","",0.6*'Info Cuencas'!R97+HUS!E97/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="98" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A98" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A98),"",'Info Cuencas'!A98)</f>
         <v/>
@@ -12194,16 +12584,20 @@
         <f>IF(A98="","",'Info Cuencas'!B98)</f>
         <v/>
       </c>
-      <c r="C98" t="str">
+      <c r="C98" s="4" t="str">
+        <f>IF(A98="","",'Info Cuencas'!C98)</f>
+        <v/>
+      </c>
+      <c r="D98" t="str">
         <f>IF(A98="","",0.133*'Info Cuencas'!R98)</f>
         <v/>
       </c>
-      <c r="E98" s="6" t="str">
-        <f>IF(A98="","",0.6*'Info Cuencas'!R98+HUS!D98/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="99" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F98" s="6" t="str">
+        <f>IF(A98="","",0.6*'Info Cuencas'!R98+HUS!E98/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="99" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A99" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A99),"",'Info Cuencas'!A99)</f>
         <v/>
@@ -12212,16 +12606,20 @@
         <f>IF(A99="","",'Info Cuencas'!B99)</f>
         <v/>
       </c>
-      <c r="C99" t="str">
+      <c r="C99" s="4" t="str">
+        <f>IF(A99="","",'Info Cuencas'!C99)</f>
+        <v/>
+      </c>
+      <c r="D99" t="str">
         <f>IF(A99="","",0.133*'Info Cuencas'!R99)</f>
         <v/>
       </c>
-      <c r="E99" s="6" t="str">
-        <f>IF(A99="","",0.6*'Info Cuencas'!R99+HUS!D99/2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="100" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F99" s="6" t="str">
+        <f>IF(A99="","",0.6*'Info Cuencas'!R99+HUS!E99/2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="100" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A100" t="str">
         <f>IF(ISBLANK('Info Cuencas'!A100),"",'Info Cuencas'!A100)</f>
         <v/>
@@ -12230,12 +12628,16 @@
         <f>IF(A100="","",'Info Cuencas'!B100)</f>
         <v/>
       </c>
-      <c r="C100" t="str">
+      <c r="C100" s="4" t="str">
+        <f>IF(A100="","",'Info Cuencas'!C100)</f>
+        <v/>
+      </c>
+      <c r="D100" t="str">
         <f>IF(A100="","",0.133*'Info Cuencas'!R100)</f>
         <v/>
       </c>
-      <c r="E100" s="6" t="str">
-        <f>IF(A100="","",0.6*'Info Cuencas'!R100+HUS!D100/2)</f>
+      <c r="F100" s="6" t="str">
+        <f>IF(A100="","",0.6*'Info Cuencas'!R100+HUS!E100/2)</f>
         <v/>
       </c>
     </row>
@@ -22926,26 +23328,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="40414187-dd76-4ef8-b04f-ccddae734140" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="63768118-86e2-4829-8a12-b72c47658d02">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100CCB1C2B958A07241A317F5A881DFD30C" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ec29f518eb9a62149baea9c73f5411cd">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="63768118-86e2-4829-8a12-b72c47658d02" xmlns:ns3="40414187-dd76-4ef8-b04f-ccddae734140" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="29f6242226419d82ce7554acb1ee2c31" ns2:_="" ns3:_="">
     <xsd:import namespace="63768118-86e2-4829-8a12-b72c47658d02"/>
@@ -23200,26 +23582,27 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2A4DA3E6-B8B6-48A6-81EC-CAAD4DEE707B}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="40414187-dd76-4ef8-b04f-ccddae734140"/>
-    <ds:schemaRef ds:uri="63768118-86e2-4829-8a12-b72c47658d02"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{26BC43C4-0DE4-4398-8C07-F13A3433226F}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="40414187-dd76-4ef8-b04f-ccddae734140" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="63768118-86e2-4829-8a12-b72c47658d02">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{124384BF-B442-43EF-BEBD-26F0C03197F3}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -23236,4 +23619,23 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{26BC43C4-0DE4-4398-8C07-F13A3433226F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2A4DA3E6-B8B6-48A6-81EC-CAAD4DEE707B}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="40414187-dd76-4ef8-b04f-ccddae734140"/>
+    <ds:schemaRef ds:uri="63768118-86e2-4829-8a12-b72c47658d02"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
UPDATE codigo calcula HED mediante convolucion
</commit_message>
<xml_diff>
--- a/Inputs.xlsx
+++ b/Inputs.xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9675E104-ED50-4A54-876F-6109ED75FCEA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="588" yWindow="1704" windowWidth="21600" windowHeight="11232" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Info Cuencas" sheetId="1" r:id="rId1"/>
@@ -23328,6 +23328,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="40414187-dd76-4ef8-b04f-ccddae734140" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="63768118-86e2-4829-8a12-b72c47658d02">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100CCB1C2B958A07241A317F5A881DFD30C" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ec29f518eb9a62149baea9c73f5411cd">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="63768118-86e2-4829-8a12-b72c47658d02" xmlns:ns3="40414187-dd76-4ef8-b04f-ccddae734140" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="29f6242226419d82ce7554acb1ee2c31" ns2:_="" ns3:_="">
     <xsd:import namespace="63768118-86e2-4829-8a12-b72c47658d02"/>
@@ -23582,27 +23602,26 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2A4DA3E6-B8B6-48A6-81EC-CAAD4DEE707B}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="40414187-dd76-4ef8-b04f-ccddae734140"/>
+    <ds:schemaRef ds:uri="63768118-86e2-4829-8a12-b72c47658d02"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="40414187-dd76-4ef8-b04f-ccddae734140" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="63768118-86e2-4829-8a12-b72c47658d02">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{26BC43C4-0DE4-4398-8C07-F13A3433226F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{124384BF-B442-43EF-BEBD-26F0C03197F3}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -23619,23 +23638,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{26BC43C4-0DE4-4398-8C07-F13A3433226F}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2A4DA3E6-B8B6-48A6-81EC-CAAD4DEE707B}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="40414187-dd76-4ef8-b04f-ccddae734140"/>
-    <ds:schemaRef ds:uri="63768118-86e2-4829-8a12-b72c47658d02"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Codigo funciona, comprobado con HECHMS
</commit_message>
<xml_diff>
--- a/Inputs.xlsx
+++ b/Inputs.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Codigos\HU_SCS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9675E104-ED50-4A54-876F-6109ED75FCEA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9989D8CD-1FC5-41ED-ABB9-5A6E1611DB9B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="588" yWindow="1704" windowWidth="21600" windowHeight="11232" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Info Cuencas" sheetId="1" r:id="rId1"/>
@@ -63,7 +63,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="44">
   <si>
     <t>Cuenca</t>
   </si>
@@ -190,14 +190,21 @@
   <si>
     <t>CN</t>
   </si>
+  <si>
+    <t>Tormenta N°6</t>
+  </si>
+  <si>
+    <t>HU-Varas II</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="0.0"/>
     <numFmt numFmtId="165" formatCode="0.000"/>
+    <numFmt numFmtId="166" formatCode="0.0%"/>
   </numFmts>
   <fonts count="4" x14ac:knownFonts="1">
     <font>
@@ -256,7 +263,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -296,6 +303,7 @@
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1274,16 +1282,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>16</xdr:col>
-      <xdr:colOff>220980</xdr:colOff>
+      <xdr:col>20</xdr:col>
+      <xdr:colOff>601980</xdr:colOff>
       <xdr:row>1</xdr:row>
-      <xdr:rowOff>22860</xdr:rowOff>
+      <xdr:rowOff>53340</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>21</xdr:col>
-      <xdr:colOff>581025</xdr:colOff>
+      <xdr:col>26</xdr:col>
+      <xdr:colOff>352425</xdr:colOff>
       <xdr:row>23</xdr:row>
-      <xdr:rowOff>120016</xdr:rowOff>
+      <xdr:rowOff>150496</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -1298,7 +1306,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="13936980" y="205740"/>
+          <a:off x="16756380" y="236220"/>
           <a:ext cx="3408045" cy="4120516"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -18889,7 +18897,7 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CC7FBFDF-ABB4-4287-9F76-768D0CF54D44}">
   <sheetPr codeName="Sheet5"/>
-  <dimension ref="A1:N242"/>
+  <dimension ref="A1:R243"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12.88671875" bestFit="1" customWidth="1"/>
@@ -18905,9 +18913,11 @@
     <col min="12" max="12" width="8.88671875" customWidth="1"/>
     <col min="13" max="13" width="12.88671875" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="11.5546875" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="12.44140625" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A1" s="9" t="s">
         <v>29</v>
       </c>
@@ -18942,8 +18952,14 @@
       <c r="N1" s="9" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="P1" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="Q1" s="9" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="2" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
         <v>30</v>
       </c>
@@ -18978,8 +18994,14 @@
       <c r="N2" s="4" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="P2" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="Q2" s="4" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="3" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A3" s="16">
         <v>0</v>
       </c>
@@ -19014,8 +19036,15 @@
       <c r="N3" s="16">
         <v>0</v>
       </c>
-    </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="P3" s="17">
+        <v>0</v>
+      </c>
+      <c r="Q3" s="17">
+        <v>0</v>
+      </c>
+      <c r="R3" s="17"/>
+    </row>
+    <row r="4" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A4" s="16">
         <v>0.1</v>
       </c>
@@ -19050,8 +19079,15 @@
       <c r="N4" s="16">
         <v>0.02</v>
       </c>
-    </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="P4" s="17">
+        <v>4.1666666666666666E-3</v>
+      </c>
+      <c r="Q4" s="17">
+        <v>5.8333333333333336E-3</v>
+      </c>
+      <c r="R4" s="17"/>
+    </row>
+    <row r="5" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A5" s="16">
         <v>0.2</v>
       </c>
@@ -19086,8 +19122,15 @@
       <c r="N5" s="16">
         <v>0.05</v>
       </c>
-    </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="P5" s="17">
+        <v>8.3333333333333332E-3</v>
+      </c>
+      <c r="Q5" s="17">
+        <v>1.1666666666666667E-2</v>
+      </c>
+      <c r="R5" s="17"/>
+    </row>
+    <row r="6" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A6" s="16">
         <v>0.3</v>
       </c>
@@ -19122,8 +19165,15 @@
       <c r="N6" s="16">
         <v>8.2000000000000003E-2</v>
       </c>
-    </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="P6" s="17">
+        <v>1.2500000000000002E-2</v>
+      </c>
+      <c r="Q6" s="17">
+        <v>1.7500000000000002E-2</v>
+      </c>
+      <c r="R6" s="17"/>
+    </row>
+    <row r="7" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A7" s="16">
         <v>0.4</v>
       </c>
@@ -19158,8 +19208,15 @@
       <c r="N7" s="16">
         <v>0.11600000000000001</v>
       </c>
-    </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="P7" s="17">
+        <v>1.6666666666666666E-2</v>
+      </c>
+      <c r="Q7" s="17">
+        <v>2.3333333333333334E-2</v>
+      </c>
+      <c r="R7" s="17"/>
+    </row>
+    <row r="8" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A8" s="16">
         <v>0.5</v>
       </c>
@@ -19194,8 +19251,15 @@
       <c r="N8" s="16">
         <v>0.156</v>
       </c>
-    </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="P8" s="17">
+        <v>2.0833333333333329E-2</v>
+      </c>
+      <c r="Q8" s="17">
+        <v>2.916666666666666E-2</v>
+      </c>
+      <c r="R8" s="17"/>
+    </row>
+    <row r="9" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A9" s="16">
         <v>0.6</v>
       </c>
@@ -19230,8 +19294,15 @@
       <c r="N9" s="16">
         <v>0.20599999999999999</v>
       </c>
-    </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="P9" s="17">
+        <v>2.5000000000000001E-2</v>
+      </c>
+      <c r="Q9" s="17">
+        <v>3.5000000000000003E-2</v>
+      </c>
+      <c r="R9" s="17"/>
+    </row>
+    <row r="10" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A10" s="16">
         <v>0.7</v>
       </c>
@@ -19266,8 +19337,15 @@
       <c r="N10" s="16">
         <v>0.26800000000000002</v>
       </c>
-    </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="P10" s="17">
+        <v>2.9166666666666664E-2</v>
+      </c>
+      <c r="Q10" s="17">
+        <v>4.0833333333333333E-2</v>
+      </c>
+      <c r="R10" s="17"/>
+    </row>
+    <row r="11" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A11" s="16">
         <v>0.8</v>
       </c>
@@ -19302,8 +19380,15 @@
       <c r="N11" s="16">
         <v>0.42499999999999999</v>
       </c>
-    </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="P11" s="17">
+        <v>3.3333333333333333E-2</v>
+      </c>
+      <c r="Q11" s="17">
+        <v>4.6666666666666669E-2</v>
+      </c>
+      <c r="R11" s="17"/>
+    </row>
+    <row r="12" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A12" s="16">
         <v>0.9</v>
       </c>
@@ -19338,8 +19423,15 @@
       <c r="N12" s="16">
         <v>0.52</v>
       </c>
-    </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="P12" s="17">
+        <v>3.7499999999999999E-2</v>
+      </c>
+      <c r="Q12" s="17">
+        <v>5.2499999999999998E-2</v>
+      </c>
+      <c r="R12" s="17"/>
+    </row>
+    <row r="13" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A13" s="16">
         <v>1</v>
       </c>
@@ -19374,8 +19466,15 @@
       <c r="N13" s="16">
         <v>0.57699999999999996</v>
       </c>
-    </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="P13" s="17">
+        <v>4.1666666666666657E-2</v>
+      </c>
+      <c r="Q13" s="17">
+        <v>5.833333333333332E-2</v>
+      </c>
+      <c r="R13" s="17"/>
+    </row>
+    <row r="14" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A14" s="4"/>
       <c r="B14" s="4"/>
       <c r="C14" s="4"/>
@@ -19398,8 +19497,15 @@
       <c r="N14" s="16">
         <v>0.624</v>
       </c>
-    </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="P14" s="17">
+        <v>4.583333333333333E-2</v>
+      </c>
+      <c r="Q14" s="17">
+        <v>6.4166666666666664E-2</v>
+      </c>
+      <c r="R14" s="17"/>
+    </row>
+    <row r="15" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A15" s="4"/>
       <c r="B15" s="4"/>
       <c r="C15" s="4"/>
@@ -19422,8 +19528,15 @@
       <c r="N15" s="16">
         <v>0.66400000000000003</v>
       </c>
-    </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="P15" s="17">
+        <v>0.05</v>
+      </c>
+      <c r="Q15" s="17">
+        <v>7.0000000000000007E-2</v>
+      </c>
+      <c r="R15" s="17"/>
+    </row>
+    <row r="16" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A16" s="4"/>
       <c r="B16" s="4"/>
       <c r="C16" s="4"/>
@@ -19446,8 +19559,15 @@
       <c r="N16" s="16">
         <v>0.70099999999999996</v>
       </c>
-    </row>
-    <row r="17" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="P16" s="17">
+        <v>5.4166666666666669E-2</v>
+      </c>
+      <c r="Q16" s="17">
+        <v>7.5833333333333336E-2</v>
+      </c>
+      <c r="R16" s="17"/>
+    </row>
+    <row r="17" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A17" s="4"/>
       <c r="B17" s="4"/>
       <c r="C17" s="4"/>
@@ -19470,8 +19590,15 @@
       <c r="N17" s="16">
         <v>0.73599999999999999</v>
       </c>
-    </row>
-    <row r="18" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="P17" s="17">
+        <v>5.8333333333333341E-2</v>
+      </c>
+      <c r="Q17" s="17">
+        <v>8.1666666666666679E-2</v>
+      </c>
+      <c r="R17" s="17"/>
+    </row>
+    <row r="18" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A18" s="4"/>
       <c r="B18" s="4"/>
       <c r="C18" s="4"/>
@@ -19494,8 +19621,15 @@
       <c r="N18" s="16">
         <v>0.76900000000000002</v>
       </c>
-    </row>
-    <row r="19" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="P18" s="17">
+        <v>6.2500000000000014E-2</v>
+      </c>
+      <c r="Q18" s="17">
+        <v>8.7500000000000022E-2</v>
+      </c>
+      <c r="R18" s="17"/>
+    </row>
+    <row r="19" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A19" s="4"/>
       <c r="B19" s="4"/>
       <c r="C19" s="4"/>
@@ -19518,8 +19652,15 @@
       <c r="N19" s="16">
         <v>0.8</v>
       </c>
-    </row>
-    <row r="20" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="P19" s="17">
+        <v>6.666666666666668E-2</v>
+      </c>
+      <c r="Q19" s="17">
+        <v>9.3333333333333351E-2</v>
+      </c>
+      <c r="R19" s="17"/>
+    </row>
+    <row r="20" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A20" s="4"/>
       <c r="B20" s="4"/>
       <c r="C20" s="4"/>
@@ -19542,8 +19683,15 @@
       <c r="N20" s="16">
         <v>0.83</v>
       </c>
-    </row>
-    <row r="21" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="P20" s="17">
+        <v>7.0833333333333345E-2</v>
+      </c>
+      <c r="Q20" s="17">
+        <v>9.9166666666666681E-2</v>
+      </c>
+      <c r="R20" s="17"/>
+    </row>
+    <row r="21" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A21" s="4"/>
       <c r="B21" s="4"/>
       <c r="C21" s="4"/>
@@ -19566,8 +19714,15 @@
       <c r="N21" s="16">
         <v>0.85799999999999998</v>
       </c>
-    </row>
-    <row r="22" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="P21" s="17">
+        <v>7.5000000000000025E-2</v>
+      </c>
+      <c r="Q21" s="17">
+        <v>0.10500000000000004</v>
+      </c>
+      <c r="R21" s="17"/>
+    </row>
+    <row r="22" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A22" s="4"/>
       <c r="B22" s="4"/>
       <c r="C22" s="4"/>
@@ -19590,8 +19745,15 @@
       <c r="N22" s="16">
         <v>0.88400000000000001</v>
       </c>
-    </row>
-    <row r="23" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="P22" s="17">
+        <v>7.9166666666666691E-2</v>
+      </c>
+      <c r="Q22" s="17">
+        <v>0.11083333333333335</v>
+      </c>
+      <c r="R22" s="17"/>
+    </row>
+    <row r="23" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A23" s="4"/>
       <c r="B23" s="4"/>
       <c r="C23" s="4"/>
@@ -19614,8 +19776,15 @@
       <c r="N23" s="16">
         <v>0.90800000000000003</v>
       </c>
-    </row>
-    <row r="24" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="P23" s="17">
+        <v>8.3333333333333356E-2</v>
+      </c>
+      <c r="Q23" s="17">
+        <v>0.1166666666666667</v>
+      </c>
+      <c r="R23" s="17"/>
+    </row>
+    <row r="24" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A24" s="4"/>
       <c r="B24" s="4"/>
       <c r="C24" s="4"/>
@@ -19638,8 +19807,15 @@
       <c r="N24" s="16">
         <v>0.93200000000000005</v>
       </c>
-    </row>
-    <row r="25" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="P24" s="17">
+        <v>8.7500000000000022E-2</v>
+      </c>
+      <c r="Q24" s="17">
+        <v>0.12250000000000001</v>
+      </c>
+      <c r="R24" s="17"/>
+    </row>
+    <row r="25" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A25" s="4"/>
       <c r="B25" s="4"/>
       <c r="C25" s="4"/>
@@ -19662,8 +19838,15 @@
       <c r="N25" s="16">
         <v>0.95599999999999996</v>
       </c>
-    </row>
-    <row r="26" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="P25" s="17">
+        <v>9.1666666666666702E-2</v>
+      </c>
+      <c r="Q25" s="17">
+        <v>0.12833333333333338</v>
+      </c>
+      <c r="R25" s="17"/>
+    </row>
+    <row r="26" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A26" s="4"/>
       <c r="B26" s="4"/>
       <c r="C26" s="4"/>
@@ -19686,8 +19869,15 @@
       <c r="N26" s="16">
         <v>0.97799999999999998</v>
       </c>
-    </row>
-    <row r="27" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="P26" s="17">
+        <v>9.5833333333333381E-2</v>
+      </c>
+      <c r="Q26" s="17">
+        <v>0.13416666666666674</v>
+      </c>
+      <c r="R26" s="17"/>
+    </row>
+    <row r="27" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A27" s="4"/>
       <c r="B27" s="4"/>
       <c r="C27" s="4"/>
@@ -19710,8 +19900,15 @@
       <c r="N27" s="16">
         <v>1</v>
       </c>
-    </row>
-    <row r="28" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="P27" s="17">
+        <v>0.10000000000000003</v>
+      </c>
+      <c r="Q27" s="17">
+        <v>0.14000000000000004</v>
+      </c>
+      <c r="R27" s="17"/>
+    </row>
+    <row r="28" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A28" s="4"/>
       <c r="B28" s="4"/>
       <c r="C28" s="4"/>
@@ -19725,8 +19922,15 @@
       <c r="K28" s="4"/>
       <c r="L28" s="4"/>
       <c r="M28" s="4"/>
-    </row>
-    <row r="29" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="P28" s="17">
+        <v>0.1041666666666667</v>
+      </c>
+      <c r="Q28" s="17">
+        <v>0.14583333333333337</v>
+      </c>
+      <c r="R28" s="17"/>
+    </row>
+    <row r="29" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A29" s="4"/>
       <c r="B29" s="4"/>
       <c r="C29" s="4"/>
@@ -19740,8 +19944,15 @@
       <c r="K29" s="4"/>
       <c r="L29" s="4"/>
       <c r="M29" s="4"/>
-    </row>
-    <row r="30" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="P29" s="17">
+        <v>0.10833333333333338</v>
+      </c>
+      <c r="Q29" s="17">
+        <v>0.15166666666666673</v>
+      </c>
+      <c r="R29" s="17"/>
+    </row>
+    <row r="30" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A30" s="4"/>
       <c r="B30" s="4"/>
       <c r="C30" s="4"/>
@@ -19755,8 +19966,15 @@
       <c r="K30" s="4"/>
       <c r="L30" s="4"/>
       <c r="M30" s="4"/>
-    </row>
-    <row r="31" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="P30" s="17">
+        <v>0.11250000000000003</v>
+      </c>
+      <c r="Q30" s="17">
+        <v>0.15750000000000006</v>
+      </c>
+      <c r="R30" s="17"/>
+    </row>
+    <row r="31" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A31" s="4"/>
       <c r="B31" s="4"/>
       <c r="C31" s="4"/>
@@ -19770,8 +19988,15 @@
       <c r="K31" s="4"/>
       <c r="L31" s="4"/>
       <c r="M31" s="4"/>
-    </row>
-    <row r="32" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="P31" s="17">
+        <v>0.11666666666666671</v>
+      </c>
+      <c r="Q31" s="17">
+        <v>0.16333333333333339</v>
+      </c>
+      <c r="R31" s="17"/>
+    </row>
+    <row r="32" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A32" s="4"/>
       <c r="B32" s="4"/>
       <c r="C32" s="4"/>
@@ -19785,8 +20010,15 @@
       <c r="K32" s="4"/>
       <c r="L32" s="4"/>
       <c r="M32" s="4"/>
-    </row>
-    <row r="33" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P32" s="17">
+        <v>0.12083333333333339</v>
+      </c>
+      <c r="Q32" s="17">
+        <v>0.16916666666666674</v>
+      </c>
+      <c r="R32" s="17"/>
+    </row>
+    <row r="33" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A33" s="4"/>
       <c r="B33" s="4"/>
       <c r="C33" s="4"/>
@@ -19800,8 +20032,15 @@
       <c r="K33" s="4"/>
       <c r="L33" s="4"/>
       <c r="M33" s="4"/>
-    </row>
-    <row r="34" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P33" s="17">
+        <v>0.12500000000000006</v>
+      </c>
+      <c r="Q33" s="17">
+        <v>0.17500000000000007</v>
+      </c>
+      <c r="R33" s="17"/>
+    </row>
+    <row r="34" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A34" s="4"/>
       <c r="B34" s="4"/>
       <c r="C34" s="4"/>
@@ -19815,8 +20054,15 @@
       <c r="K34" s="4"/>
       <c r="L34" s="4"/>
       <c r="M34" s="4"/>
-    </row>
-    <row r="35" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P34" s="17">
+        <v>0.12916666666666674</v>
+      </c>
+      <c r="Q34" s="17">
+        <v>0.18083333333333343</v>
+      </c>
+      <c r="R34" s="17"/>
+    </row>
+    <row r="35" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A35" s="4"/>
       <c r="B35" s="4"/>
       <c r="C35" s="4"/>
@@ -19830,8 +20076,15 @@
       <c r="K35" s="4"/>
       <c r="L35" s="4"/>
       <c r="M35" s="4"/>
-    </row>
-    <row r="36" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P35" s="17">
+        <v>0.13333333333333339</v>
+      </c>
+      <c r="Q35" s="17">
+        <v>0.18666666666666676</v>
+      </c>
+      <c r="R35" s="17"/>
+    </row>
+    <row r="36" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A36" s="4"/>
       <c r="B36" s="4"/>
       <c r="C36" s="4"/>
@@ -19845,8 +20098,15 @@
       <c r="K36" s="4"/>
       <c r="L36" s="4"/>
       <c r="M36" s="4"/>
-    </row>
-    <row r="37" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P36" s="17">
+        <v>0.13750000000000007</v>
+      </c>
+      <c r="Q36" s="17">
+        <v>0.19250000000000012</v>
+      </c>
+      <c r="R36" s="17"/>
+    </row>
+    <row r="37" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A37" s="4"/>
       <c r="B37" s="4"/>
       <c r="C37" s="4"/>
@@ -19860,8 +20120,15 @@
       <c r="K37" s="4"/>
       <c r="L37" s="4"/>
       <c r="M37" s="4"/>
-    </row>
-    <row r="38" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P37" s="17">
+        <v>0.14166666666666675</v>
+      </c>
+      <c r="Q37" s="17">
+        <v>0.19833333333333347</v>
+      </c>
+      <c r="R37" s="17"/>
+    </row>
+    <row r="38" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A38" s="4"/>
       <c r="B38" s="4"/>
       <c r="C38" s="4"/>
@@ -19875,8 +20142,15 @@
       <c r="K38" s="4"/>
       <c r="L38" s="4"/>
       <c r="M38" s="4"/>
-    </row>
-    <row r="39" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P38" s="17">
+        <v>0.1458333333333334</v>
+      </c>
+      <c r="Q38" s="17">
+        <v>0.20416666666666675</v>
+      </c>
+      <c r="R38" s="17"/>
+    </row>
+    <row r="39" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A39" s="4"/>
       <c r="B39" s="4"/>
       <c r="C39" s="4"/>
@@ -19890,8 +20164,15 @@
       <c r="K39" s="4"/>
       <c r="L39" s="4"/>
       <c r="M39" s="4"/>
-    </row>
-    <row r="40" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P39" s="17">
+        <v>0.15000000000000008</v>
+      </c>
+      <c r="Q39" s="17">
+        <v>0.2100000000000001</v>
+      </c>
+      <c r="R39" s="17"/>
+    </row>
+    <row r="40" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A40" s="4"/>
       <c r="B40" s="4"/>
       <c r="C40" s="4"/>
@@ -19905,8 +20186,15 @@
       <c r="K40" s="4"/>
       <c r="L40" s="4"/>
       <c r="M40" s="4"/>
-    </row>
-    <row r="41" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P40" s="17">
+        <v>0.15416666666666676</v>
+      </c>
+      <c r="Q40" s="17">
+        <v>0.21583333333333346</v>
+      </c>
+      <c r="R40" s="17"/>
+    </row>
+    <row r="41" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A41" s="4"/>
       <c r="B41" s="4"/>
       <c r="C41" s="4"/>
@@ -19920,8 +20208,15 @@
       <c r="K41" s="4"/>
       <c r="L41" s="4"/>
       <c r="M41" s="4"/>
-    </row>
-    <row r="42" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P41" s="17">
+        <v>0.15833333333333341</v>
+      </c>
+      <c r="Q41" s="17">
+        <v>0.22166666666666679</v>
+      </c>
+      <c r="R41" s="17"/>
+    </row>
+    <row r="42" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A42" s="4"/>
       <c r="B42" s="4"/>
       <c r="C42" s="4"/>
@@ -19935,8 +20230,15 @@
       <c r="K42" s="4"/>
       <c r="L42" s="4"/>
       <c r="M42" s="4"/>
-    </row>
-    <row r="43" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P42" s="17">
+        <v>0.16250000000000006</v>
+      </c>
+      <c r="Q42" s="17">
+        <v>0.22750000000000012</v>
+      </c>
+      <c r="R42" s="17"/>
+    </row>
+    <row r="43" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A43" s="4"/>
       <c r="B43" s="4"/>
       <c r="C43" s="4"/>
@@ -19950,8 +20252,15 @@
       <c r="K43" s="4"/>
       <c r="L43" s="4"/>
       <c r="M43" s="4"/>
-    </row>
-    <row r="44" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P43" s="17">
+        <v>0.16666666666666674</v>
+      </c>
+      <c r="Q43" s="17">
+        <v>0.23333333333333348</v>
+      </c>
+      <c r="R43" s="17"/>
+    </row>
+    <row r="44" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A44" s="4"/>
       <c r="B44" s="4"/>
       <c r="C44" s="4"/>
@@ -19965,8 +20274,15 @@
       <c r="K44" s="4"/>
       <c r="L44" s="4"/>
       <c r="M44" s="4"/>
-    </row>
-    <row r="45" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P44" s="17">
+        <v>0.17083333333333339</v>
+      </c>
+      <c r="Q44" s="17">
+        <v>0.23916666666666675</v>
+      </c>
+      <c r="R44" s="17"/>
+    </row>
+    <row r="45" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A45" s="4"/>
       <c r="B45" s="4"/>
       <c r="C45" s="4"/>
@@ -19980,8 +20296,15 @@
       <c r="K45" s="4"/>
       <c r="L45" s="4"/>
       <c r="M45" s="4"/>
-    </row>
-    <row r="46" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P45" s="17">
+        <v>0.17500000000000004</v>
+      </c>
+      <c r="Q45" s="17">
+        <v>0.24500000000000002</v>
+      </c>
+      <c r="R45" s="17"/>
+    </row>
+    <row r="46" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A46" s="4"/>
       <c r="B46" s="4"/>
       <c r="C46" s="4"/>
@@ -19995,8 +20318,15 @@
       <c r="K46" s="4"/>
       <c r="L46" s="4"/>
       <c r="M46" s="4"/>
-    </row>
-    <row r="47" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P46" s="17">
+        <v>0.17916666666666672</v>
+      </c>
+      <c r="Q46" s="17">
+        <v>0.25083333333333341</v>
+      </c>
+      <c r="R46" s="17"/>
+    </row>
+    <row r="47" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A47" s="4"/>
       <c r="B47" s="4"/>
       <c r="C47" s="4"/>
@@ -20010,8 +20340,15 @@
       <c r="K47" s="4"/>
       <c r="L47" s="4"/>
       <c r="M47" s="4"/>
-    </row>
-    <row r="48" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P47" s="17">
+        <v>0.18333333333333335</v>
+      </c>
+      <c r="Q47" s="17">
+        <v>0.25666666666666671</v>
+      </c>
+      <c r="R47" s="17"/>
+    </row>
+    <row r="48" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A48" s="4"/>
       <c r="B48" s="4"/>
       <c r="C48" s="4"/>
@@ -20025,8 +20362,15 @@
       <c r="K48" s="4"/>
       <c r="L48" s="4"/>
       <c r="M48" s="4"/>
-    </row>
-    <row r="49" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P48" s="17">
+        <v>0.1875</v>
+      </c>
+      <c r="Q48" s="17">
+        <v>0.26250000000000001</v>
+      </c>
+      <c r="R48" s="17"/>
+    </row>
+    <row r="49" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A49" s="4"/>
       <c r="B49" s="4"/>
       <c r="C49" s="4"/>
@@ -20040,8 +20384,15 @@
       <c r="K49" s="4"/>
       <c r="L49" s="4"/>
       <c r="M49" s="4"/>
-    </row>
-    <row r="50" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P49" s="17">
+        <v>0.19166666666666665</v>
+      </c>
+      <c r="Q49" s="17">
+        <v>0.26833333333333331</v>
+      </c>
+      <c r="R49" s="17"/>
+    </row>
+    <row r="50" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A50" s="4"/>
       <c r="B50" s="4"/>
       <c r="C50" s="4"/>
@@ -20055,8 +20406,15 @@
       <c r="K50" s="4"/>
       <c r="L50" s="4"/>
       <c r="M50" s="4"/>
-    </row>
-    <row r="51" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P50" s="17">
+        <v>0.19583333333333328</v>
+      </c>
+      <c r="Q50" s="17">
+        <v>0.27416666666666661</v>
+      </c>
+      <c r="R50" s="17"/>
+    </row>
+    <row r="51" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A51" s="4"/>
       <c r="B51" s="4"/>
       <c r="C51" s="4"/>
@@ -20070,8 +20428,15 @@
       <c r="K51" s="4"/>
       <c r="L51" s="4"/>
       <c r="M51" s="4"/>
-    </row>
-    <row r="52" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P51" s="17">
+        <v>0.19999999999999996</v>
+      </c>
+      <c r="Q51" s="17">
+        <v>0.27999999999999997</v>
+      </c>
+      <c r="R51" s="17"/>
+    </row>
+    <row r="52" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A52" s="4"/>
       <c r="B52" s="4"/>
       <c r="C52" s="4"/>
@@ -20085,8 +20450,15 @@
       <c r="K52" s="4"/>
       <c r="L52" s="4"/>
       <c r="M52" s="4"/>
-    </row>
-    <row r="53" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P52" s="17">
+        <v>0.20416666666666661</v>
+      </c>
+      <c r="Q52" s="17">
+        <v>0.28583333333333327</v>
+      </c>
+      <c r="R52" s="17"/>
+    </row>
+    <row r="53" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A53" s="4"/>
       <c r="B53" s="4"/>
       <c r="C53" s="4"/>
@@ -20100,8 +20472,15 @@
       <c r="K53" s="4"/>
       <c r="L53" s="4"/>
       <c r="M53" s="4"/>
-    </row>
-    <row r="54" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P53" s="17">
+        <v>0.20833333333333326</v>
+      </c>
+      <c r="Q53" s="17">
+        <v>0.29166666666666652</v>
+      </c>
+      <c r="R53" s="17"/>
+    </row>
+    <row r="54" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A54" s="4"/>
       <c r="B54" s="4"/>
       <c r="C54" s="4"/>
@@ -20115,8 +20494,15 @@
       <c r="K54" s="4"/>
       <c r="L54" s="4"/>
       <c r="M54" s="4"/>
-    </row>
-    <row r="55" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P54" s="17">
+        <v>0.21249999999999994</v>
+      </c>
+      <c r="Q54" s="17">
+        <v>0.29749999999999988</v>
+      </c>
+      <c r="R54" s="17"/>
+    </row>
+    <row r="55" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A55" s="4"/>
       <c r="B55" s="4"/>
       <c r="C55" s="4"/>
@@ -20130,8 +20516,15 @@
       <c r="K55" s="4"/>
       <c r="L55" s="4"/>
       <c r="M55" s="4"/>
-    </row>
-    <row r="56" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P55" s="17">
+        <v>0.21666666666666656</v>
+      </c>
+      <c r="Q55" s="17">
+        <v>0.30333333333333323</v>
+      </c>
+      <c r="R55" s="17"/>
+    </row>
+    <row r="56" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A56" s="4"/>
       <c r="B56" s="4"/>
       <c r="C56" s="4"/>
@@ -20145,8 +20538,15 @@
       <c r="K56" s="4"/>
       <c r="L56" s="4"/>
       <c r="M56" s="4"/>
-    </row>
-    <row r="57" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P56" s="17">
+        <v>0.22083333333333321</v>
+      </c>
+      <c r="Q56" s="17">
+        <v>0.30916666666666648</v>
+      </c>
+      <c r="R56" s="17"/>
+    </row>
+    <row r="57" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A57" s="4"/>
       <c r="B57" s="4"/>
       <c r="C57" s="4"/>
@@ -20160,8 +20560,15 @@
       <c r="K57" s="4"/>
       <c r="L57" s="4"/>
       <c r="M57" s="4"/>
-    </row>
-    <row r="58" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P57" s="17">
+        <v>0.22499999999999987</v>
+      </c>
+      <c r="Q57" s="17">
+        <v>0.31499999999999978</v>
+      </c>
+      <c r="R57" s="17"/>
+    </row>
+    <row r="58" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A58" s="4"/>
       <c r="B58" s="4"/>
       <c r="C58" s="4"/>
@@ -20175,8 +20582,15 @@
       <c r="K58" s="4"/>
       <c r="L58" s="4"/>
       <c r="M58" s="4"/>
-    </row>
-    <row r="59" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P58" s="17">
+        <v>0.22916666666666649</v>
+      </c>
+      <c r="Q58" s="17">
+        <v>0.32083333333333308</v>
+      </c>
+      <c r="R58" s="17"/>
+    </row>
+    <row r="59" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A59" s="4"/>
       <c r="B59" s="4"/>
       <c r="C59" s="4"/>
@@ -20190,8 +20604,15 @@
       <c r="K59" s="4"/>
       <c r="L59" s="4"/>
       <c r="M59" s="4"/>
-    </row>
-    <row r="60" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P59" s="17">
+        <v>0.23333333333333317</v>
+      </c>
+      <c r="Q59" s="17">
+        <v>0.32666666666666644</v>
+      </c>
+      <c r="R59" s="17"/>
+    </row>
+    <row r="60" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A60" s="4"/>
       <c r="B60" s="4"/>
       <c r="C60" s="4"/>
@@ -20205,8 +20626,15 @@
       <c r="K60" s="4"/>
       <c r="L60" s="4"/>
       <c r="M60" s="4"/>
-    </row>
-    <row r="61" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P60" s="17">
+        <v>0.23749999999999982</v>
+      </c>
+      <c r="Q60" s="17">
+        <v>0.33249999999999974</v>
+      </c>
+      <c r="R60" s="17"/>
+    </row>
+    <row r="61" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A61" s="4"/>
       <c r="B61" s="4"/>
       <c r="C61" s="4"/>
@@ -20220,8 +20648,15 @@
       <c r="K61" s="4"/>
       <c r="L61" s="4"/>
       <c r="M61" s="4"/>
-    </row>
-    <row r="62" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P61" s="17">
+        <v>0.24166666666666647</v>
+      </c>
+      <c r="Q61" s="17">
+        <v>0.3383333333333331</v>
+      </c>
+      <c r="R61" s="17"/>
+    </row>
+    <row r="62" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A62" s="4"/>
       <c r="B62" s="4"/>
       <c r="C62" s="4"/>
@@ -20235,8 +20670,15 @@
       <c r="K62" s="4"/>
       <c r="L62" s="4"/>
       <c r="M62" s="4"/>
-    </row>
-    <row r="63" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P62" s="17">
+        <v>0.24583333333333315</v>
+      </c>
+      <c r="Q62" s="17">
+        <v>0.34416666666666645</v>
+      </c>
+      <c r="R62" s="17"/>
+    </row>
+    <row r="63" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A63" s="4"/>
       <c r="B63" s="4"/>
       <c r="C63" s="4"/>
@@ -20250,8 +20692,15 @@
       <c r="K63" s="4"/>
       <c r="L63" s="4"/>
       <c r="M63" s="4"/>
-    </row>
-    <row r="64" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P63" s="17">
+        <v>0.24999999999999978</v>
+      </c>
+      <c r="Q63" s="17">
+        <v>0.3499999999999997</v>
+      </c>
+      <c r="R63" s="17"/>
+    </row>
+    <row r="64" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A64" s="4"/>
       <c r="B64" s="4"/>
       <c r="C64" s="4"/>
@@ -20265,8 +20714,15 @@
       <c r="K64" s="4"/>
       <c r="L64" s="4"/>
       <c r="M64" s="4"/>
-    </row>
-    <row r="65" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P64" s="17">
+        <v>0.25416666666666643</v>
+      </c>
+      <c r="Q64" s="17">
+        <v>0.355833333333333</v>
+      </c>
+      <c r="R64" s="17"/>
+    </row>
+    <row r="65" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A65" s="4"/>
       <c r="B65" s="4"/>
       <c r="C65" s="4"/>
@@ -20280,8 +20736,15 @@
       <c r="K65" s="4"/>
       <c r="L65" s="4"/>
       <c r="M65" s="4"/>
-    </row>
-    <row r="66" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P65" s="17">
+        <v>0.25833333333333308</v>
+      </c>
+      <c r="Q65" s="17">
+        <v>0.3616666666666663</v>
+      </c>
+      <c r="R65" s="17"/>
+    </row>
+    <row r="66" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A66" s="4"/>
       <c r="B66" s="4"/>
       <c r="C66" s="4"/>
@@ -20295,8 +20758,15 @@
       <c r="K66" s="4"/>
       <c r="L66" s="4"/>
       <c r="M66" s="4"/>
-    </row>
-    <row r="67" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P66" s="17">
+        <v>0.26249999999999973</v>
+      </c>
+      <c r="Q66" s="17">
+        <v>0.36749999999999955</v>
+      </c>
+      <c r="R66" s="17"/>
+    </row>
+    <row r="67" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A67" s="4"/>
       <c r="B67" s="4"/>
       <c r="C67" s="4"/>
@@ -20310,8 +20780,15 @@
       <c r="K67" s="4"/>
       <c r="L67" s="4"/>
       <c r="M67" s="4"/>
-    </row>
-    <row r="68" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P67" s="17">
+        <v>0.26666666666666639</v>
+      </c>
+      <c r="Q67" s="17">
+        <v>0.37333333333333291</v>
+      </c>
+      <c r="R67" s="17"/>
+    </row>
+    <row r="68" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A68" s="4"/>
       <c r="B68" s="4"/>
       <c r="C68" s="4"/>
@@ -20325,8 +20802,15 @@
       <c r="K68" s="4"/>
       <c r="L68" s="4"/>
       <c r="M68" s="4"/>
-    </row>
-    <row r="69" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P68" s="17">
+        <v>0.27083333333333304</v>
+      </c>
+      <c r="Q68" s="17">
+        <v>0.37916666666666626</v>
+      </c>
+      <c r="R68" s="17"/>
+    </row>
+    <row r="69" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A69" s="4"/>
       <c r="B69" s="4"/>
       <c r="C69" s="4"/>
@@ -20340,8 +20824,15 @@
       <c r="K69" s="4"/>
       <c r="L69" s="4"/>
       <c r="M69" s="4"/>
-    </row>
-    <row r="70" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P69" s="17">
+        <v>0.27499999999999969</v>
+      </c>
+      <c r="Q69" s="17">
+        <v>0.38499999999999956</v>
+      </c>
+      <c r="R69" s="17"/>
+    </row>
+    <row r="70" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A70" s="4"/>
       <c r="B70" s="4"/>
       <c r="C70" s="4"/>
@@ -20355,8 +20846,15 @@
       <c r="K70" s="4"/>
       <c r="L70" s="4"/>
       <c r="M70" s="4"/>
-    </row>
-    <row r="71" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P70" s="17">
+        <v>0.27916666666666634</v>
+      </c>
+      <c r="Q70" s="17">
+        <v>0.39083333333333292</v>
+      </c>
+      <c r="R70" s="17"/>
+    </row>
+    <row r="71" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A71" s="4"/>
       <c r="B71" s="4"/>
       <c r="C71" s="4"/>
@@ -20370,8 +20868,15 @@
       <c r="K71" s="4"/>
       <c r="L71" s="4"/>
       <c r="M71" s="4"/>
-    </row>
-    <row r="72" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P71" s="17">
+        <v>0.28333333333333299</v>
+      </c>
+      <c r="Q71" s="17">
+        <v>0.39666666666666622</v>
+      </c>
+      <c r="R71" s="17"/>
+    </row>
+    <row r="72" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A72" s="4"/>
       <c r="B72" s="4"/>
       <c r="C72" s="4"/>
@@ -20385,8 +20890,15 @@
       <c r="K72" s="4"/>
       <c r="L72" s="4"/>
       <c r="M72" s="4"/>
-    </row>
-    <row r="73" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P72" s="17">
+        <v>0.28749999999999964</v>
+      </c>
+      <c r="Q72" s="17">
+        <v>0.40249999999999952</v>
+      </c>
+      <c r="R72" s="17"/>
+    </row>
+    <row r="73" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A73" s="4"/>
       <c r="B73" s="4"/>
       <c r="C73" s="4"/>
@@ -20400,8 +20912,15 @@
       <c r="K73" s="4"/>
       <c r="L73" s="4"/>
       <c r="M73" s="4"/>
-    </row>
-    <row r="74" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P73" s="17">
+        <v>0.2916666666666663</v>
+      </c>
+      <c r="Q73" s="17">
+        <v>0.40833333333333277</v>
+      </c>
+      <c r="R73" s="17"/>
+    </row>
+    <row r="74" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A74" s="4"/>
       <c r="B74" s="4"/>
       <c r="C74" s="4"/>
@@ -20415,8 +20934,15 @@
       <c r="K74" s="4"/>
       <c r="L74" s="4"/>
       <c r="M74" s="4"/>
-    </row>
-    <row r="75" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P74" s="17">
+        <v>0.29583333333333295</v>
+      </c>
+      <c r="Q74" s="17">
+        <v>0.41416666666666607</v>
+      </c>
+      <c r="R74" s="17"/>
+    </row>
+    <row r="75" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A75" s="4"/>
       <c r="B75" s="4"/>
       <c r="C75" s="4"/>
@@ -20430,8 +20956,15 @@
       <c r="K75" s="4"/>
       <c r="L75" s="4"/>
       <c r="M75" s="4"/>
-    </row>
-    <row r="76" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P75" s="17">
+        <v>0.2999999999999996</v>
+      </c>
+      <c r="Q75" s="17">
+        <v>0.41999999999999943</v>
+      </c>
+      <c r="R75" s="17"/>
+    </row>
+    <row r="76" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A76" s="4"/>
       <c r="B76" s="4"/>
       <c r="C76" s="4"/>
@@ -20445,8 +20978,15 @@
       <c r="K76" s="4"/>
       <c r="L76" s="4"/>
       <c r="M76" s="4"/>
-    </row>
-    <row r="77" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P76" s="17">
+        <v>0.30416666666666625</v>
+      </c>
+      <c r="Q76" s="17">
+        <v>0.42583333333333273</v>
+      </c>
+      <c r="R76" s="17"/>
+    </row>
+    <row r="77" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A77" s="4"/>
       <c r="B77" s="4"/>
       <c r="C77" s="4"/>
@@ -20460,8 +21000,15 @@
       <c r="K77" s="4"/>
       <c r="L77" s="4"/>
       <c r="M77" s="4"/>
-    </row>
-    <row r="78" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P77" s="17">
+        <v>0.3083333333333329</v>
+      </c>
+      <c r="Q77" s="17">
+        <v>0.43166666666666609</v>
+      </c>
+      <c r="R77" s="17"/>
+    </row>
+    <row r="78" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A78" s="4"/>
       <c r="B78" s="4"/>
       <c r="C78" s="4"/>
@@ -20475,8 +21022,15 @@
       <c r="K78" s="4"/>
       <c r="L78" s="4"/>
       <c r="M78" s="4"/>
-    </row>
-    <row r="79" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P78" s="17">
+        <v>0.31249999999999956</v>
+      </c>
+      <c r="Q78" s="17">
+        <v>0.43749999999999944</v>
+      </c>
+      <c r="R78" s="17"/>
+    </row>
+    <row r="79" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A79" s="4"/>
       <c r="B79" s="4"/>
       <c r="C79" s="4"/>
@@ -20490,8 +21044,15 @@
       <c r="K79" s="4"/>
       <c r="L79" s="4"/>
       <c r="M79" s="4"/>
-    </row>
-    <row r="80" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P79" s="17">
+        <v>0.31666666666666621</v>
+      </c>
+      <c r="Q79" s="17">
+        <v>0.44333333333333269</v>
+      </c>
+      <c r="R79" s="17"/>
+    </row>
+    <row r="80" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A80" s="4"/>
       <c r="B80" s="4"/>
       <c r="C80" s="4"/>
@@ -20505,8 +21066,15 @@
       <c r="K80" s="4"/>
       <c r="L80" s="4"/>
       <c r="M80" s="4"/>
-    </row>
-    <row r="81" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P80" s="17">
+        <v>0.32083333333333286</v>
+      </c>
+      <c r="Q80" s="17">
+        <v>0.44916666666666599</v>
+      </c>
+      <c r="R80" s="17"/>
+    </row>
+    <row r="81" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A81" s="4"/>
       <c r="B81" s="4"/>
       <c r="C81" s="4"/>
@@ -20520,8 +21088,15 @@
       <c r="K81" s="4"/>
       <c r="L81" s="4"/>
       <c r="M81" s="4"/>
-    </row>
-    <row r="82" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P81" s="17">
+        <v>0.32499999999999951</v>
+      </c>
+      <c r="Q81" s="17">
+        <v>0.45499999999999929</v>
+      </c>
+      <c r="R81" s="17"/>
+    </row>
+    <row r="82" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A82" s="4"/>
       <c r="B82" s="4"/>
       <c r="C82" s="4"/>
@@ -20535,8 +21110,15 @@
       <c r="K82" s="4"/>
       <c r="L82" s="4"/>
       <c r="M82" s="4"/>
-    </row>
-    <row r="83" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P82" s="17">
+        <v>0.32916666666666616</v>
+      </c>
+      <c r="Q82" s="17">
+        <v>0.4608333333333326</v>
+      </c>
+      <c r="R82" s="17"/>
+    </row>
+    <row r="83" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A83" s="4"/>
       <c r="B83" s="4"/>
       <c r="C83" s="4"/>
@@ -20550,8 +21132,15 @@
       <c r="K83" s="4"/>
       <c r="L83" s="4"/>
       <c r="M83" s="4"/>
-    </row>
-    <row r="84" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P83" s="17">
+        <v>0.33333333333333282</v>
+      </c>
+      <c r="Q83" s="17">
+        <v>0.46666666666666595</v>
+      </c>
+      <c r="R83" s="17"/>
+    </row>
+    <row r="84" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A84" s="4"/>
       <c r="B84" s="4"/>
       <c r="C84" s="4"/>
@@ -20565,8 +21154,15 @@
       <c r="K84" s="4"/>
       <c r="L84" s="4"/>
       <c r="M84" s="4"/>
-    </row>
-    <row r="85" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P84" s="17">
+        <v>0.33749999999999941</v>
+      </c>
+      <c r="Q84" s="17">
+        <v>0.4724999999999992</v>
+      </c>
+      <c r="R84" s="17"/>
+    </row>
+    <row r="85" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A85" s="4"/>
       <c r="B85" s="4"/>
       <c r="C85" s="4"/>
@@ -20580,8 +21176,15 @@
       <c r="K85" s="4"/>
       <c r="L85" s="4"/>
       <c r="M85" s="4"/>
-    </row>
-    <row r="86" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P85" s="17">
+        <v>0.34166666666666612</v>
+      </c>
+      <c r="Q85" s="17">
+        <v>0.47833333333333256</v>
+      </c>
+      <c r="R85" s="17"/>
+    </row>
+    <row r="86" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A86" s="4"/>
       <c r="B86" s="4"/>
       <c r="C86" s="4"/>
@@ -20595,8 +21198,15 @@
       <c r="K86" s="4"/>
       <c r="L86" s="4"/>
       <c r="M86" s="4"/>
-    </row>
-    <row r="87" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P86" s="17">
+        <v>0.34583333333333277</v>
+      </c>
+      <c r="Q86" s="17">
+        <v>0.48416666666666591</v>
+      </c>
+      <c r="R86" s="17"/>
+    </row>
+    <row r="87" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A87" s="4"/>
       <c r="B87" s="4"/>
       <c r="C87" s="4"/>
@@ -20610,8 +21220,15 @@
       <c r="K87" s="4"/>
       <c r="L87" s="4"/>
       <c r="M87" s="4"/>
-    </row>
-    <row r="88" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P87" s="17">
+        <v>0.34999999999999942</v>
+      </c>
+      <c r="Q87" s="17">
+        <v>0.48999999999999921</v>
+      </c>
+      <c r="R87" s="17"/>
+    </row>
+    <row r="88" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A88" s="4"/>
       <c r="B88" s="4"/>
       <c r="C88" s="4"/>
@@ -20625,8 +21242,15 @@
       <c r="K88" s="4"/>
       <c r="L88" s="4"/>
       <c r="M88" s="4"/>
-    </row>
-    <row r="89" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P88" s="17">
+        <v>0.35416666666666607</v>
+      </c>
+      <c r="Q88" s="17">
+        <v>0.49583333333333252</v>
+      </c>
+      <c r="R88" s="17"/>
+    </row>
+    <row r="89" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A89" s="4"/>
       <c r="B89" s="4"/>
       <c r="C89" s="4"/>
@@ -20640,8 +21264,15 @@
       <c r="K89" s="4"/>
       <c r="L89" s="4"/>
       <c r="M89" s="4"/>
-    </row>
-    <row r="90" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P89" s="17">
+        <v>0.35833333333333273</v>
+      </c>
+      <c r="Q89" s="17">
+        <v>0.50166666666666582</v>
+      </c>
+      <c r="R89" s="17"/>
+    </row>
+    <row r="90" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A90" s="4"/>
       <c r="B90" s="4"/>
       <c r="C90" s="4"/>
@@ -20655,8 +21286,15 @@
       <c r="K90" s="4"/>
       <c r="L90" s="4"/>
       <c r="M90" s="4"/>
-    </row>
-    <row r="91" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P90" s="17">
+        <v>0.36249999999999938</v>
+      </c>
+      <c r="Q90" s="17">
+        <v>0.50749999999999906</v>
+      </c>
+      <c r="R90" s="17"/>
+    </row>
+    <row r="91" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A91" s="4"/>
       <c r="B91" s="4"/>
       <c r="C91" s="4"/>
@@ -20670,8 +21308,15 @@
       <c r="K91" s="4"/>
       <c r="L91" s="4"/>
       <c r="M91" s="4"/>
-    </row>
-    <row r="92" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P91" s="17">
+        <v>0.36666666666666603</v>
+      </c>
+      <c r="Q91" s="17">
+        <v>0.51333333333333242</v>
+      </c>
+      <c r="R91" s="17"/>
+    </row>
+    <row r="92" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A92" s="4"/>
       <c r="B92" s="4"/>
       <c r="C92" s="4"/>
@@ -20685,8 +21330,15 @@
       <c r="K92" s="4"/>
       <c r="L92" s="4"/>
       <c r="M92" s="4"/>
-    </row>
-    <row r="93" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P92" s="17">
+        <v>0.37083333333333274</v>
+      </c>
+      <c r="Q92" s="17">
+        <v>0.51916666666666578</v>
+      </c>
+      <c r="R92" s="17"/>
+    </row>
+    <row r="93" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A93" s="4"/>
       <c r="B93" s="4"/>
       <c r="C93" s="4"/>
@@ -20700,8 +21352,15 @@
       <c r="K93" s="4"/>
       <c r="L93" s="4"/>
       <c r="M93" s="4"/>
-    </row>
-    <row r="94" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P93" s="17">
+        <v>0.37499999999999933</v>
+      </c>
+      <c r="Q93" s="17">
+        <v>0.52499999999999902</v>
+      </c>
+      <c r="R93" s="17"/>
+    </row>
+    <row r="94" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A94" s="4"/>
       <c r="B94" s="4"/>
       <c r="C94" s="4"/>
@@ -20715,8 +21374,15 @@
       <c r="K94" s="4"/>
       <c r="L94" s="4"/>
       <c r="M94" s="4"/>
-    </row>
-    <row r="95" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P94" s="17">
+        <v>0.37916666666666599</v>
+      </c>
+      <c r="Q94" s="17">
+        <v>0.53083333333333238</v>
+      </c>
+      <c r="R94" s="17"/>
+    </row>
+    <row r="95" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A95" s="4"/>
       <c r="B95" s="4"/>
       <c r="C95" s="4"/>
@@ -20730,8 +21396,15 @@
       <c r="K95" s="4"/>
       <c r="L95" s="4"/>
       <c r="M95" s="4"/>
-    </row>
-    <row r="96" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P95" s="17">
+        <v>0.38333333333333264</v>
+      </c>
+      <c r="Q95" s="17">
+        <v>0.53666666666666574</v>
+      </c>
+      <c r="R95" s="17"/>
+    </row>
+    <row r="96" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A96" s="4"/>
       <c r="B96" s="4"/>
       <c r="C96" s="4"/>
@@ -20745,8 +21418,15 @@
       <c r="K96" s="4"/>
       <c r="L96" s="4"/>
       <c r="M96" s="4"/>
-    </row>
-    <row r="97" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P96" s="17">
+        <v>0.38749999999999929</v>
+      </c>
+      <c r="Q96" s="17">
+        <v>0.54249999999999898</v>
+      </c>
+      <c r="R96" s="17"/>
+    </row>
+    <row r="97" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A97" s="4"/>
       <c r="B97" s="4"/>
       <c r="C97" s="4"/>
@@ -20760,8 +21440,15 @@
       <c r="K97" s="4"/>
       <c r="L97" s="4"/>
       <c r="M97" s="4"/>
-    </row>
-    <row r="98" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P97" s="17">
+        <v>0.39166666666666594</v>
+      </c>
+      <c r="Q97" s="17">
+        <v>0.54833333333333234</v>
+      </c>
+      <c r="R97" s="17"/>
+    </row>
+    <row r="98" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A98" s="4"/>
       <c r="B98" s="4"/>
       <c r="C98" s="4"/>
@@ -20775,8 +21462,15 @@
       <c r="K98" s="4"/>
       <c r="L98" s="4"/>
       <c r="M98" s="4"/>
-    </row>
-    <row r="99" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P98" s="17">
+        <v>0.39583333333333259</v>
+      </c>
+      <c r="Q98" s="17">
+        <v>0.55416666666666559</v>
+      </c>
+      <c r="R98" s="17"/>
+    </row>
+    <row r="99" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A99" s="4"/>
       <c r="B99" s="4"/>
       <c r="C99" s="4"/>
@@ -20790,8 +21484,15 @@
       <c r="K99" s="4"/>
       <c r="L99" s="4"/>
       <c r="M99" s="4"/>
-    </row>
-    <row r="100" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P99" s="17">
+        <v>0.39999999999999925</v>
+      </c>
+      <c r="Q99" s="17">
+        <v>0.55999999999999894</v>
+      </c>
+      <c r="R99" s="17"/>
+    </row>
+    <row r="100" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A100" s="4"/>
       <c r="B100" s="4"/>
       <c r="C100" s="4"/>
@@ -20805,8 +21506,15 @@
       <c r="K100" s="4"/>
       <c r="L100" s="4"/>
       <c r="M100" s="4"/>
-    </row>
-    <row r="101" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P100" s="17">
+        <v>0.40416666666666584</v>
+      </c>
+      <c r="Q100" s="17">
+        <v>0.56666666666666532</v>
+      </c>
+      <c r="R100" s="17"/>
+    </row>
+    <row r="101" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A101" s="4"/>
       <c r="B101" s="4"/>
       <c r="C101" s="4"/>
@@ -20820,8 +21528,15 @@
       <c r="K101" s="4"/>
       <c r="L101" s="4"/>
       <c r="M101" s="4"/>
-    </row>
-    <row r="102" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P101" s="17">
+        <v>0.40833333333333255</v>
+      </c>
+      <c r="Q101" s="17">
+        <v>0.57333333333333214</v>
+      </c>
+      <c r="R101" s="17"/>
+    </row>
+    <row r="102" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A102" s="4"/>
       <c r="B102" s="4"/>
       <c r="C102" s="4"/>
@@ -20835,8 +21550,15 @@
       <c r="K102" s="4"/>
       <c r="L102" s="4"/>
       <c r="M102" s="4"/>
-    </row>
-    <row r="103" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P102" s="17">
+        <v>0.4124999999999992</v>
+      </c>
+      <c r="Q102" s="17">
+        <v>0.57999999999999874</v>
+      </c>
+      <c r="R102" s="17"/>
+    </row>
+    <row r="103" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A103" s="4"/>
       <c r="B103" s="4"/>
       <c r="C103" s="4"/>
@@ -20850,8 +21572,15 @@
       <c r="K103" s="4"/>
       <c r="L103" s="4"/>
       <c r="M103" s="4"/>
-    </row>
-    <row r="104" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P103" s="17">
+        <v>0.41666666666666585</v>
+      </c>
+      <c r="Q103" s="17">
+        <v>0.58666666666666534</v>
+      </c>
+      <c r="R103" s="17"/>
+    </row>
+    <row r="104" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A104" s="4"/>
       <c r="B104" s="4"/>
       <c r="C104" s="4"/>
@@ -20865,8 +21594,15 @@
       <c r="K104" s="4"/>
       <c r="L104" s="4"/>
       <c r="M104" s="4"/>
-    </row>
-    <row r="105" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P104" s="17">
+        <v>0.4208333333333325</v>
+      </c>
+      <c r="Q104" s="17">
+        <v>0.59333333333333205</v>
+      </c>
+      <c r="R104" s="17"/>
+    </row>
+    <row r="105" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A105" s="4"/>
       <c r="B105" s="4"/>
       <c r="C105" s="4"/>
@@ -20880,8 +21616,15 @@
       <c r="K105" s="4"/>
       <c r="L105" s="4"/>
       <c r="M105" s="4"/>
-    </row>
-    <row r="106" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P105" s="17">
+        <v>0.42499999999999916</v>
+      </c>
+      <c r="Q105" s="17">
+        <v>0.59999999999999865</v>
+      </c>
+      <c r="R105" s="17"/>
+    </row>
+    <row r="106" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A106" s="4"/>
       <c r="B106" s="4"/>
       <c r="C106" s="4"/>
@@ -20895,8 +21638,15 @@
       <c r="K106" s="4"/>
       <c r="L106" s="4"/>
       <c r="M106" s="4"/>
-    </row>
-    <row r="107" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P106" s="17">
+        <v>0.42916666666666581</v>
+      </c>
+      <c r="Q106" s="17">
+        <v>0.60666666666666524</v>
+      </c>
+      <c r="R106" s="17"/>
+    </row>
+    <row r="107" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A107" s="4"/>
       <c r="B107" s="4"/>
       <c r="C107" s="4"/>
@@ -20910,8 +21660,15 @@
       <c r="K107" s="4"/>
       <c r="L107" s="4"/>
       <c r="M107" s="4"/>
-    </row>
-    <row r="108" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P107" s="17">
+        <v>0.43333333333333246</v>
+      </c>
+      <c r="Q107" s="17">
+        <v>0.61333333333333184</v>
+      </c>
+      <c r="R107" s="17"/>
+    </row>
+    <row r="108" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A108" s="4"/>
       <c r="B108" s="4"/>
       <c r="C108" s="4"/>
@@ -20925,8 +21682,15 @@
       <c r="K108" s="4"/>
       <c r="L108" s="4"/>
       <c r="M108" s="4"/>
-    </row>
-    <row r="109" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P108" s="17">
+        <v>0.43749999999999917</v>
+      </c>
+      <c r="Q108" s="17">
+        <v>0.61999999999999866</v>
+      </c>
+      <c r="R108" s="17"/>
+    </row>
+    <row r="109" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A109" s="4"/>
       <c r="B109" s="4"/>
       <c r="C109" s="4"/>
@@ -20940,8 +21704,15 @@
       <c r="K109" s="4"/>
       <c r="L109" s="4"/>
       <c r="M109" s="4"/>
-    </row>
-    <row r="110" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P109" s="17">
+        <v>0.44166666666666576</v>
+      </c>
+      <c r="Q109" s="17">
+        <v>0.62666666666666526</v>
+      </c>
+      <c r="R109" s="17"/>
+    </row>
+    <row r="110" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A110" s="4"/>
       <c r="B110" s="4"/>
       <c r="C110" s="4"/>
@@ -20955,8 +21726,15 @@
       <c r="K110" s="4"/>
       <c r="L110" s="4"/>
       <c r="M110" s="4"/>
-    </row>
-    <row r="111" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P110" s="17">
+        <v>0.44583333333333242</v>
+      </c>
+      <c r="Q110" s="17">
+        <v>0.63333333333333186</v>
+      </c>
+      <c r="R110" s="17"/>
+    </row>
+    <row r="111" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A111" s="4"/>
       <c r="B111" s="4"/>
       <c r="C111" s="4"/>
@@ -20970,8 +21748,15 @@
       <c r="K111" s="4"/>
       <c r="L111" s="4"/>
       <c r="M111" s="4"/>
-    </row>
-    <row r="112" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P111" s="17">
+        <v>0.44999999999999907</v>
+      </c>
+      <c r="Q111" s="17">
+        <v>0.63999999999999846</v>
+      </c>
+      <c r="R111" s="17"/>
+    </row>
+    <row r="112" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A112" s="4"/>
       <c r="B112" s="4"/>
       <c r="C112" s="4"/>
@@ -20985,8 +21770,15 @@
       <c r="K112" s="4"/>
       <c r="L112" s="4"/>
       <c r="M112" s="4"/>
-    </row>
-    <row r="113" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P112" s="17">
+        <v>0.45416666666666572</v>
+      </c>
+      <c r="Q112" s="17">
+        <v>0.64666666666666517</v>
+      </c>
+      <c r="R112" s="17"/>
+    </row>
+    <row r="113" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A113" s="4"/>
       <c r="B113" s="4"/>
       <c r="C113" s="4"/>
@@ -21000,8 +21792,15 @@
       <c r="K113" s="4"/>
       <c r="L113" s="4"/>
       <c r="M113" s="4"/>
-    </row>
-    <row r="114" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P113" s="17">
+        <v>0.45833333333333237</v>
+      </c>
+      <c r="Q113" s="17">
+        <v>0.65333333333333177</v>
+      </c>
+      <c r="R113" s="17"/>
+    </row>
+    <row r="114" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A114" s="4"/>
       <c r="B114" s="4"/>
       <c r="C114" s="4"/>
@@ -21015,8 +21814,15 @@
       <c r="K114" s="4"/>
       <c r="L114" s="4"/>
       <c r="M114" s="4"/>
-    </row>
-    <row r="115" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P114" s="17">
+        <v>0.46249999999999902</v>
+      </c>
+      <c r="Q114" s="17">
+        <v>0.65999999999999848</v>
+      </c>
+      <c r="R114" s="17"/>
+    </row>
+    <row r="115" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A115" s="4"/>
       <c r="B115" s="4"/>
       <c r="C115" s="4"/>
@@ -21030,8 +21836,15 @@
       <c r="K115" s="4"/>
       <c r="L115" s="4"/>
       <c r="M115" s="4"/>
-    </row>
-    <row r="116" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P115" s="17">
+        <v>0.46666666666666567</v>
+      </c>
+      <c r="Q115" s="17">
+        <v>0.66666666666666496</v>
+      </c>
+      <c r="R115" s="17"/>
+    </row>
+    <row r="116" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A116" s="4"/>
       <c r="B116" s="4"/>
       <c r="C116" s="4"/>
@@ -21045,8 +21858,15 @@
       <c r="K116" s="4"/>
       <c r="L116" s="4"/>
       <c r="M116" s="4"/>
-    </row>
-    <row r="117" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P116" s="17">
+        <v>0.47083333333333227</v>
+      </c>
+      <c r="Q116" s="17">
+        <v>0.67333333333333167</v>
+      </c>
+      <c r="R116" s="17"/>
+    </row>
+    <row r="117" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A117" s="4"/>
       <c r="B117" s="4"/>
       <c r="C117" s="4"/>
@@ -21060,8 +21880,15 @@
       <c r="K117" s="4"/>
       <c r="L117" s="4"/>
       <c r="M117" s="4"/>
-    </row>
-    <row r="118" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P117" s="17">
+        <v>0.47499999999999898</v>
+      </c>
+      <c r="Q117" s="17">
+        <v>0.67999999999999838</v>
+      </c>
+      <c r="R117" s="17"/>
+    </row>
+    <row r="118" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A118" s="4"/>
       <c r="B118" s="4"/>
       <c r="C118" s="4"/>
@@ -21075,8 +21902,15 @@
       <c r="K118" s="4"/>
       <c r="L118" s="4"/>
       <c r="M118" s="4"/>
-    </row>
-    <row r="119" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P118" s="17">
+        <v>0.47916666666666563</v>
+      </c>
+      <c r="Q118" s="17">
+        <v>0.68666666666666498</v>
+      </c>
+      <c r="R118" s="17"/>
+    </row>
+    <row r="119" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A119" s="4"/>
       <c r="B119" s="4"/>
       <c r="C119" s="4"/>
@@ -21090,8 +21924,15 @@
       <c r="K119" s="4"/>
       <c r="L119" s="4"/>
       <c r="M119" s="4"/>
-    </row>
-    <row r="120" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P119" s="17">
+        <v>0.48333333333333228</v>
+      </c>
+      <c r="Q119" s="17">
+        <v>0.69333333333333169</v>
+      </c>
+      <c r="R119" s="17"/>
+    </row>
+    <row r="120" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A120" s="4"/>
       <c r="B120" s="4"/>
       <c r="C120" s="4"/>
@@ -21105,8 +21946,15 @@
       <c r="K120" s="4"/>
       <c r="L120" s="4"/>
       <c r="M120" s="4"/>
-    </row>
-    <row r="121" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P120" s="17">
+        <v>0.48749999999999893</v>
+      </c>
+      <c r="Q120" s="17">
+        <v>0.69999999999999829</v>
+      </c>
+      <c r="R120" s="17"/>
+    </row>
+    <row r="121" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A121" s="4"/>
       <c r="B121" s="4"/>
       <c r="C121" s="4"/>
@@ -21120,8 +21968,15 @@
       <c r="K121" s="4"/>
       <c r="L121" s="4"/>
       <c r="M121" s="4"/>
-    </row>
-    <row r="122" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P121" s="17">
+        <v>0.49166666666666559</v>
+      </c>
+      <c r="Q121" s="17">
+        <v>0.70666666666666489</v>
+      </c>
+      <c r="R121" s="17"/>
+    </row>
+    <row r="122" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A122" s="4"/>
       <c r="B122" s="4"/>
       <c r="C122" s="4"/>
@@ -21135,8 +21990,15 @@
       <c r="K122" s="4"/>
       <c r="L122" s="4"/>
       <c r="M122" s="4"/>
-    </row>
-    <row r="123" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P122" s="17">
+        <v>0.49583333333333224</v>
+      </c>
+      <c r="Q122" s="17">
+        <v>0.7133333333333316</v>
+      </c>
+      <c r="R122" s="17"/>
+    </row>
+    <row r="123" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A123" s="4"/>
       <c r="B123" s="4"/>
       <c r="C123" s="4"/>
@@ -21150,8 +22012,15 @@
       <c r="K123" s="4"/>
       <c r="L123" s="4"/>
       <c r="M123" s="4"/>
-    </row>
-    <row r="124" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P123" s="17">
+        <v>0.49999999999999889</v>
+      </c>
+      <c r="Q123" s="17">
+        <v>0.7199999999999982</v>
+      </c>
+      <c r="R123" s="17"/>
+    </row>
+    <row r="124" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A124" s="4"/>
       <c r="B124" s="4"/>
       <c r="C124" s="4"/>
@@ -21165,8 +22034,15 @@
       <c r="K124" s="4"/>
       <c r="L124" s="4"/>
       <c r="M124" s="4"/>
-    </row>
-    <row r="125" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P124" s="17">
+        <v>0.50416666666666554</v>
+      </c>
+      <c r="Q124" s="17">
+        <v>0.72374999999999901</v>
+      </c>
+      <c r="R124" s="17"/>
+    </row>
+    <row r="125" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A125" s="4"/>
       <c r="B125" s="4"/>
       <c r="C125" s="4"/>
@@ -21180,8 +22056,15 @@
       <c r="K125" s="4"/>
       <c r="L125" s="4"/>
       <c r="M125" s="4"/>
-    </row>
-    <row r="126" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P125" s="17">
+        <v>0.50833333333333219</v>
+      </c>
+      <c r="Q125" s="17">
+        <v>0.72749999999999904</v>
+      </c>
+      <c r="R125" s="17"/>
+    </row>
+    <row r="126" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A126" s="4"/>
       <c r="B126" s="4"/>
       <c r="C126" s="4"/>
@@ -21195,8 +22078,15 @@
       <c r="K126" s="4"/>
       <c r="L126" s="4"/>
       <c r="M126" s="4"/>
-    </row>
-    <row r="127" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P126" s="17">
+        <v>0.51249999999999885</v>
+      </c>
+      <c r="Q126" s="17">
+        <v>0.73124999999999896</v>
+      </c>
+      <c r="R126" s="17"/>
+    </row>
+    <row r="127" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A127" s="4"/>
       <c r="B127" s="4"/>
       <c r="C127" s="4"/>
@@ -21210,8 +22100,15 @@
       <c r="K127" s="4"/>
       <c r="L127" s="4"/>
       <c r="M127" s="4"/>
-    </row>
-    <row r="128" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P127" s="17">
+        <v>0.5166666666666655</v>
+      </c>
+      <c r="Q127" s="17">
+        <v>0.73499999999999899</v>
+      </c>
+      <c r="R127" s="17"/>
+    </row>
+    <row r="128" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A128" s="4"/>
       <c r="B128" s="4"/>
       <c r="C128" s="4"/>
@@ -21225,8 +22122,15 @@
       <c r="K128" s="4"/>
       <c r="L128" s="4"/>
       <c r="M128" s="4"/>
-    </row>
-    <row r="129" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P128" s="17">
+        <v>0.52083333333333215</v>
+      </c>
+      <c r="Q128" s="17">
+        <v>0.73874999999999891</v>
+      </c>
+      <c r="R128" s="17"/>
+    </row>
+    <row r="129" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A129" s="4"/>
       <c r="B129" s="4"/>
       <c r="C129" s="4"/>
@@ -21240,8 +22144,15 @@
       <c r="K129" s="4"/>
       <c r="L129" s="4"/>
       <c r="M129" s="4"/>
-    </row>
-    <row r="130" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P129" s="17">
+        <v>0.5249999999999988</v>
+      </c>
+      <c r="Q129" s="17">
+        <v>0.74249999999999883</v>
+      </c>
+      <c r="R129" s="17"/>
+    </row>
+    <row r="130" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A130" s="4"/>
       <c r="B130" s="4"/>
       <c r="C130" s="4"/>
@@ -21255,8 +22166,15 @@
       <c r="K130" s="4"/>
       <c r="L130" s="4"/>
       <c r="M130" s="4"/>
-    </row>
-    <row r="131" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P130" s="17">
+        <v>0.52916666666666545</v>
+      </c>
+      <c r="Q130" s="17">
+        <v>0.74624999999999886</v>
+      </c>
+      <c r="R130" s="17"/>
+    </row>
+    <row r="131" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A131" s="4"/>
       <c r="B131" s="4"/>
       <c r="C131" s="4"/>
@@ -21270,8 +22188,15 @@
       <c r="K131" s="4"/>
       <c r="L131" s="4"/>
       <c r="M131" s="4"/>
-    </row>
-    <row r="132" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P131" s="17">
+        <v>0.5333333333333321</v>
+      </c>
+      <c r="Q131" s="17">
+        <v>0.74999999999999889</v>
+      </c>
+      <c r="R131" s="17"/>
+    </row>
+    <row r="132" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A132" s="4"/>
       <c r="B132" s="4"/>
       <c r="C132" s="4"/>
@@ -21285,8 +22210,15 @@
       <c r="K132" s="4"/>
       <c r="L132" s="4"/>
       <c r="M132" s="4"/>
-    </row>
-    <row r="133" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P132" s="17">
+        <v>0.53749999999999876</v>
+      </c>
+      <c r="Q132" s="17">
+        <v>0.75374999999999881</v>
+      </c>
+      <c r="R132" s="17"/>
+    </row>
+    <row r="133" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A133" s="4"/>
       <c r="B133" s="4"/>
       <c r="C133" s="4"/>
@@ -21300,8 +22232,15 @@
       <c r="K133" s="4"/>
       <c r="L133" s="4"/>
       <c r="M133" s="4"/>
-    </row>
-    <row r="134" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P133" s="17">
+        <v>0.54166666666666541</v>
+      </c>
+      <c r="Q133" s="17">
+        <v>0.75749999999999884</v>
+      </c>
+      <c r="R133" s="17"/>
+    </row>
+    <row r="134" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A134" s="4"/>
       <c r="B134" s="4"/>
       <c r="C134" s="4"/>
@@ -21315,8 +22254,15 @@
       <c r="K134" s="4"/>
       <c r="L134" s="4"/>
       <c r="M134" s="4"/>
-    </row>
-    <row r="135" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P134" s="17">
+        <v>0.54583333333333206</v>
+      </c>
+      <c r="Q134" s="17">
+        <v>0.76124999999999887</v>
+      </c>
+      <c r="R134" s="17"/>
+    </row>
+    <row r="135" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A135" s="4"/>
       <c r="B135" s="4"/>
       <c r="C135" s="4"/>
@@ -21330,8 +22276,15 @@
       <c r="K135" s="4"/>
       <c r="L135" s="4"/>
       <c r="M135" s="4"/>
-    </row>
-    <row r="136" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P135" s="17">
+        <v>0.54999999999999871</v>
+      </c>
+      <c r="Q135" s="17">
+        <v>0.7649999999999989</v>
+      </c>
+      <c r="R135" s="17"/>
+    </row>
+    <row r="136" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A136" s="4"/>
       <c r="B136" s="4"/>
       <c r="C136" s="4"/>
@@ -21345,8 +22298,15 @@
       <c r="K136" s="4"/>
       <c r="L136" s="4"/>
       <c r="M136" s="4"/>
-    </row>
-    <row r="137" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P136" s="17">
+        <v>0.55416666666666536</v>
+      </c>
+      <c r="Q136" s="17">
+        <v>0.76874999999999882</v>
+      </c>
+      <c r="R136" s="17"/>
+    </row>
+    <row r="137" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A137" s="4"/>
       <c r="B137" s="4"/>
       <c r="C137" s="4"/>
@@ -21360,8 +22320,15 @@
       <c r="K137" s="4"/>
       <c r="L137" s="4"/>
       <c r="M137" s="4"/>
-    </row>
-    <row r="138" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P137" s="17">
+        <v>0.55833333333333202</v>
+      </c>
+      <c r="Q137" s="17">
+        <v>0.77249999999999885</v>
+      </c>
+      <c r="R137" s="17"/>
+    </row>
+    <row r="138" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A138" s="4"/>
       <c r="B138" s="4"/>
       <c r="C138" s="4"/>
@@ -21375,8 +22342,15 @@
       <c r="K138" s="4"/>
       <c r="L138" s="4"/>
       <c r="M138" s="4"/>
-    </row>
-    <row r="139" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P138" s="17">
+        <v>0.56249999999999867</v>
+      </c>
+      <c r="Q138" s="17">
+        <v>0.77624999999999877</v>
+      </c>
+      <c r="R138" s="17"/>
+    </row>
+    <row r="139" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A139" s="4"/>
       <c r="B139" s="4"/>
       <c r="C139" s="4"/>
@@ -21390,8 +22364,15 @@
       <c r="K139" s="4"/>
       <c r="L139" s="4"/>
       <c r="M139" s="4"/>
-    </row>
-    <row r="140" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P139" s="17">
+        <v>0.56666666666666532</v>
+      </c>
+      <c r="Q139" s="17">
+        <v>0.77999999999999869</v>
+      </c>
+      <c r="R139" s="17"/>
+    </row>
+    <row r="140" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A140" s="4"/>
       <c r="B140" s="4"/>
       <c r="C140" s="4"/>
@@ -21405,8 +22386,15 @@
       <c r="K140" s="4"/>
       <c r="L140" s="4"/>
       <c r="M140" s="4"/>
-    </row>
-    <row r="141" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P140" s="17">
+        <v>0.57083333333333197</v>
+      </c>
+      <c r="Q140" s="17">
+        <v>0.78374999999999884</v>
+      </c>
+      <c r="R140" s="17"/>
+    </row>
+    <row r="141" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A141" s="4"/>
       <c r="B141" s="4"/>
       <c r="C141" s="4"/>
@@ -21420,8 +22408,15 @@
       <c r="K141" s="4"/>
       <c r="L141" s="4"/>
       <c r="M141" s="4"/>
-    </row>
-    <row r="142" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P141" s="17">
+        <v>0.57499999999999862</v>
+      </c>
+      <c r="Q141" s="17">
+        <v>0.78749999999999876</v>
+      </c>
+      <c r="R141" s="17"/>
+    </row>
+    <row r="142" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A142" s="4"/>
       <c r="B142" s="4"/>
       <c r="C142" s="4"/>
@@ -21435,8 +22430,15 @@
       <c r="K142" s="4"/>
       <c r="L142" s="4"/>
       <c r="M142" s="4"/>
-    </row>
-    <row r="143" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P142" s="17">
+        <v>0.57916666666666528</v>
+      </c>
+      <c r="Q142" s="17">
+        <v>0.79124999999999868</v>
+      </c>
+      <c r="R142" s="17"/>
+    </row>
+    <row r="143" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A143" s="4"/>
       <c r="B143" s="4"/>
       <c r="C143" s="4"/>
@@ -21450,8 +22452,15 @@
       <c r="K143" s="4"/>
       <c r="L143" s="4"/>
       <c r="M143" s="4"/>
-    </row>
-    <row r="144" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P143" s="17">
+        <v>0.58333333333333193</v>
+      </c>
+      <c r="Q143" s="17">
+        <v>0.79499999999999871</v>
+      </c>
+      <c r="R143" s="17"/>
+    </row>
+    <row r="144" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A144" s="4"/>
       <c r="B144" s="4"/>
       <c r="C144" s="4"/>
@@ -21465,8 +22474,15 @@
       <c r="K144" s="4"/>
       <c r="L144" s="4"/>
       <c r="M144" s="4"/>
-    </row>
-    <row r="145" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P144" s="17">
+        <v>0.58749999999999858</v>
+      </c>
+      <c r="Q144" s="17">
+        <v>0.79874999999999874</v>
+      </c>
+      <c r="R144" s="17"/>
+    </row>
+    <row r="145" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A145" s="4"/>
       <c r="B145" s="4"/>
       <c r="C145" s="4"/>
@@ -21480,8 +22496,15 @@
       <c r="K145" s="4"/>
       <c r="L145" s="4"/>
       <c r="M145" s="4"/>
-    </row>
-    <row r="146" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P145" s="17">
+        <v>0.59166666666666523</v>
+      </c>
+      <c r="Q145" s="17">
+        <v>0.80249999999999877</v>
+      </c>
+      <c r="R145" s="17"/>
+    </row>
+    <row r="146" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A146" s="4"/>
       <c r="B146" s="4"/>
       <c r="C146" s="4"/>
@@ -21495,8 +22518,15 @@
       <c r="K146" s="4"/>
       <c r="L146" s="4"/>
       <c r="M146" s="4"/>
-    </row>
-    <row r="147" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P146" s="17">
+        <v>0.59583333333333188</v>
+      </c>
+      <c r="Q146" s="17">
+        <v>0.80624999999999869</v>
+      </c>
+      <c r="R146" s="17"/>
+    </row>
+    <row r="147" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A147" s="4"/>
       <c r="B147" s="4"/>
       <c r="C147" s="4"/>
@@ -21510,8 +22540,15 @@
       <c r="K147" s="4"/>
       <c r="L147" s="4"/>
       <c r="M147" s="4"/>
-    </row>
-    <row r="148" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P147" s="17">
+        <v>0.59999999999999853</v>
+      </c>
+      <c r="Q147" s="17">
+        <v>0.80999999999999872</v>
+      </c>
+      <c r="R147" s="17"/>
+    </row>
+    <row r="148" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A148" s="4"/>
       <c r="B148" s="4"/>
       <c r="C148" s="4"/>
@@ -21525,8 +22562,15 @@
       <c r="K148" s="4"/>
       <c r="L148" s="4"/>
       <c r="M148" s="4"/>
-    </row>
-    <row r="149" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P148" s="17">
+        <v>0.60416666666666519</v>
+      </c>
+      <c r="Q148" s="17">
+        <v>0.81291666666666562</v>
+      </c>
+      <c r="R148" s="17"/>
+    </row>
+    <row r="149" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A149" s="4"/>
       <c r="B149" s="4"/>
       <c r="C149" s="4"/>
@@ -21540,8 +22584,15 @@
       <c r="K149" s="4"/>
       <c r="L149" s="4"/>
       <c r="M149" s="4"/>
-    </row>
-    <row r="150" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P149" s="17">
+        <v>0.60833333333333184</v>
+      </c>
+      <c r="Q149" s="17">
+        <v>0.8158333333333323</v>
+      </c>
+      <c r="R149" s="17"/>
+    </row>
+    <row r="150" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A150" s="4"/>
       <c r="B150" s="4"/>
       <c r="C150" s="4"/>
@@ -21555,8 +22606,15 @@
       <c r="K150" s="4"/>
       <c r="L150" s="4"/>
       <c r="M150" s="4"/>
-    </row>
-    <row r="151" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P150" s="17">
+        <v>0.61249999999999849</v>
+      </c>
+      <c r="Q150" s="17">
+        <v>0.81874999999999898</v>
+      </c>
+      <c r="R150" s="17"/>
+    </row>
+    <row r="151" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A151" s="4"/>
       <c r="B151" s="4"/>
       <c r="C151" s="4"/>
@@ -21570,8 +22628,15 @@
       <c r="K151" s="4"/>
       <c r="L151" s="4"/>
       <c r="M151" s="4"/>
-    </row>
-    <row r="152" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P151" s="17">
+        <v>0.61666666666666514</v>
+      </c>
+      <c r="Q151" s="17">
+        <v>0.82166666666666555</v>
+      </c>
+      <c r="R151" s="17"/>
+    </row>
+    <row r="152" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A152" s="4"/>
       <c r="B152" s="4"/>
       <c r="C152" s="4"/>
@@ -21585,8 +22650,15 @@
       <c r="K152" s="4"/>
       <c r="L152" s="4"/>
       <c r="M152" s="4"/>
-    </row>
-    <row r="153" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P152" s="17">
+        <v>0.62083333333333179</v>
+      </c>
+      <c r="Q152" s="17">
+        <v>0.82458333333333234</v>
+      </c>
+      <c r="R152" s="17"/>
+    </row>
+    <row r="153" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A153" s="4"/>
       <c r="B153" s="4"/>
       <c r="C153" s="4"/>
@@ -21600,8 +22672,15 @@
       <c r="K153" s="4"/>
       <c r="L153" s="4"/>
       <c r="M153" s="4"/>
-    </row>
-    <row r="154" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P153" s="17">
+        <v>0.62499999999999845</v>
+      </c>
+      <c r="Q153" s="17">
+        <v>0.8274999999999989</v>
+      </c>
+      <c r="R153" s="17"/>
+    </row>
+    <row r="154" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A154" s="4"/>
       <c r="B154" s="4"/>
       <c r="C154" s="4"/>
@@ -21615,8 +22694,15 @@
       <c r="K154" s="4"/>
       <c r="L154" s="4"/>
       <c r="M154" s="4"/>
-    </row>
-    <row r="155" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P154" s="17">
+        <v>0.6291666666666651</v>
+      </c>
+      <c r="Q154" s="17">
+        <v>0.83041666666666558</v>
+      </c>
+      <c r="R154" s="17"/>
+    </row>
+    <row r="155" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A155" s="4"/>
       <c r="B155" s="4"/>
       <c r="C155" s="4"/>
@@ -21630,8 +22716,15 @@
       <c r="K155" s="4"/>
       <c r="L155" s="4"/>
       <c r="M155" s="4"/>
-    </row>
-    <row r="156" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P155" s="17">
+        <v>0.63333333333333175</v>
+      </c>
+      <c r="Q155" s="17">
+        <v>0.83333333333333215</v>
+      </c>
+      <c r="R155" s="17"/>
+    </row>
+    <row r="156" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A156" s="4"/>
       <c r="B156" s="4"/>
       <c r="C156" s="4"/>
@@ -21645,8 +22738,15 @@
       <c r="K156" s="4"/>
       <c r="L156" s="4"/>
       <c r="M156" s="4"/>
-    </row>
-    <row r="157" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P156" s="17">
+        <v>0.6374999999999984</v>
+      </c>
+      <c r="Q156" s="17">
+        <v>0.83624999999999883</v>
+      </c>
+      <c r="R156" s="17"/>
+    </row>
+    <row r="157" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A157" s="4"/>
       <c r="B157" s="4"/>
       <c r="C157" s="4"/>
@@ -21660,8 +22760,15 @@
       <c r="K157" s="4"/>
       <c r="L157" s="4"/>
       <c r="M157" s="4"/>
-    </row>
-    <row r="158" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P157" s="17">
+        <v>0.64166666666666505</v>
+      </c>
+      <c r="Q157" s="17">
+        <v>0.8391666666666654</v>
+      </c>
+      <c r="R157" s="17"/>
+    </row>
+    <row r="158" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A158" s="4"/>
       <c r="B158" s="4"/>
       <c r="C158" s="4"/>
@@ -21675,8 +22782,15 @@
       <c r="K158" s="4"/>
       <c r="L158" s="4"/>
       <c r="M158" s="4"/>
-    </row>
-    <row r="159" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P158" s="17">
+        <v>0.64583333333333171</v>
+      </c>
+      <c r="Q158" s="17">
+        <v>0.84208333333333218</v>
+      </c>
+      <c r="R158" s="17"/>
+    </row>
+    <row r="159" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A159" s="4"/>
       <c r="B159" s="4"/>
       <c r="C159" s="4"/>
@@ -21690,8 +22804,15 @@
       <c r="K159" s="4"/>
       <c r="L159" s="4"/>
       <c r="M159" s="4"/>
-    </row>
-    <row r="160" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P159" s="17">
+        <v>0.64999999999999825</v>
+      </c>
+      <c r="Q159" s="17">
+        <v>0.84499999999999886</v>
+      </c>
+      <c r="R159" s="17"/>
+    </row>
+    <row r="160" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A160" s="4"/>
       <c r="B160" s="4"/>
       <c r="C160" s="4"/>
@@ -21705,8 +22826,15 @@
       <c r="K160" s="4"/>
       <c r="L160" s="4"/>
       <c r="M160" s="4"/>
-    </row>
-    <row r="161" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P160" s="17">
+        <v>0.65416666666666501</v>
+      </c>
+      <c r="Q160" s="17">
+        <v>0.84791666666666543</v>
+      </c>
+      <c r="R160" s="17"/>
+    </row>
+    <row r="161" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A161" s="4"/>
       <c r="B161" s="4"/>
       <c r="C161" s="4"/>
@@ -21720,8 +22848,15 @@
       <c r="K161" s="4"/>
       <c r="L161" s="4"/>
       <c r="M161" s="4"/>
-    </row>
-    <row r="162" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P161" s="17">
+        <v>0.65833333333333177</v>
+      </c>
+      <c r="Q161" s="17">
+        <v>0.85083333333333211</v>
+      </c>
+      <c r="R161" s="17"/>
+    </row>
+    <row r="162" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A162" s="4"/>
       <c r="B162" s="4"/>
       <c r="C162" s="4"/>
@@ -21735,8 +22870,15 @@
       <c r="K162" s="4"/>
       <c r="L162" s="4"/>
       <c r="M162" s="4"/>
-    </row>
-    <row r="163" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P162" s="17">
+        <v>0.66249999999999831</v>
+      </c>
+      <c r="Q162" s="17">
+        <v>0.8537499999999989</v>
+      </c>
+      <c r="R162" s="17"/>
+    </row>
+    <row r="163" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A163" s="4"/>
       <c r="B163" s="4"/>
       <c r="C163" s="4"/>
@@ -21750,8 +22892,15 @@
       <c r="K163" s="4"/>
       <c r="L163" s="4"/>
       <c r="M163" s="4"/>
-    </row>
-    <row r="164" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P163" s="17">
+        <v>0.66666666666666496</v>
+      </c>
+      <c r="Q163" s="17">
+        <v>0.85666666666666547</v>
+      </c>
+      <c r="R163" s="17"/>
+    </row>
+    <row r="164" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A164" s="4"/>
       <c r="B164" s="4"/>
       <c r="C164" s="4"/>
@@ -21765,8 +22914,15 @@
       <c r="K164" s="4"/>
       <c r="L164" s="4"/>
       <c r="M164" s="4"/>
-    </row>
-    <row r="165" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P164" s="17">
+        <v>0.67083333333333162</v>
+      </c>
+      <c r="Q164" s="17">
+        <v>0.85958333333333214</v>
+      </c>
+      <c r="R164" s="17"/>
+    </row>
+    <row r="165" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A165" s="4"/>
       <c r="B165" s="4"/>
       <c r="C165" s="4"/>
@@ -21780,8 +22936,15 @@
       <c r="K165" s="4"/>
       <c r="L165" s="4"/>
       <c r="M165" s="4"/>
-    </row>
-    <row r="166" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P165" s="17">
+        <v>0.67499999999999849</v>
+      </c>
+      <c r="Q165" s="17">
+        <v>0.86249999999999882</v>
+      </c>
+      <c r="R165" s="17"/>
+    </row>
+    <row r="166" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A166" s="4"/>
       <c r="B166" s="4"/>
       <c r="C166" s="4"/>
@@ -21795,8 +22958,15 @@
       <c r="K166" s="4"/>
       <c r="L166" s="4"/>
       <c r="M166" s="4"/>
-    </row>
-    <row r="167" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P166" s="17">
+        <v>0.67916666666666503</v>
+      </c>
+      <c r="Q166" s="17">
+        <v>0.86541666666666539</v>
+      </c>
+      <c r="R166" s="17"/>
+    </row>
+    <row r="167" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A167" s="4"/>
       <c r="B167" s="4"/>
       <c r="C167" s="4"/>
@@ -21810,8 +22980,15 @@
       <c r="K167" s="4"/>
       <c r="L167" s="4"/>
       <c r="M167" s="4"/>
-    </row>
-    <row r="168" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P167" s="17">
+        <v>0.68333333333333168</v>
+      </c>
+      <c r="Q167" s="17">
+        <v>0.86833333333333218</v>
+      </c>
+      <c r="R167" s="17"/>
+    </row>
+    <row r="168" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A168" s="4"/>
       <c r="B168" s="4"/>
       <c r="C168" s="4"/>
@@ -21825,8 +23002,15 @@
       <c r="K168" s="4"/>
       <c r="L168" s="4"/>
       <c r="M168" s="4"/>
-    </row>
-    <row r="169" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P168" s="17">
+        <v>0.68749999999999856</v>
+      </c>
+      <c r="Q168" s="17">
+        <v>0.87124999999999897</v>
+      </c>
+      <c r="R168" s="17"/>
+    </row>
+    <row r="169" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A169" s="4"/>
       <c r="B169" s="4"/>
       <c r="C169" s="4"/>
@@ -21840,8 +23024,15 @@
       <c r="K169" s="4"/>
       <c r="L169" s="4"/>
       <c r="M169" s="4"/>
-    </row>
-    <row r="170" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P169" s="17">
+        <v>0.6916666666666651</v>
+      </c>
+      <c r="Q169" s="17">
+        <v>0.87416666666666554</v>
+      </c>
+      <c r="R169" s="17"/>
+    </row>
+    <row r="170" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A170" s="4"/>
       <c r="B170" s="4"/>
       <c r="C170" s="4"/>
@@ -21855,8 +23046,15 @@
       <c r="K170" s="4"/>
       <c r="L170" s="4"/>
       <c r="M170" s="4"/>
-    </row>
-    <row r="171" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P170" s="17">
+        <v>0.69583333333333197</v>
+      </c>
+      <c r="Q170" s="17">
+        <v>0.87708333333333244</v>
+      </c>
+      <c r="R170" s="17"/>
+    </row>
+    <row r="171" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A171" s="4"/>
       <c r="B171" s="4"/>
       <c r="C171" s="4"/>
@@ -21870,8 +23068,15 @@
       <c r="K171" s="4"/>
       <c r="L171" s="4"/>
       <c r="M171" s="4"/>
-    </row>
-    <row r="172" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P171" s="17">
+        <v>0.69999999999999873</v>
+      </c>
+      <c r="Q171" s="17">
+        <v>0.87999999999999912</v>
+      </c>
+      <c r="R171" s="17"/>
+    </row>
+    <row r="172" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A172" s="4"/>
       <c r="B172" s="4"/>
       <c r="C172" s="4"/>
@@ -21885,8 +23090,15 @@
       <c r="K172" s="4"/>
       <c r="L172" s="4"/>
       <c r="M172" s="4"/>
-    </row>
-    <row r="173" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P172" s="17">
+        <v>0.70416666666666539</v>
+      </c>
+      <c r="Q172" s="17">
+        <v>0.88249999999999929</v>
+      </c>
+      <c r="R172" s="17"/>
+    </row>
+    <row r="173" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A173" s="4"/>
       <c r="B173" s="4"/>
       <c r="C173" s="4"/>
@@ -21900,8 +23112,15 @@
       <c r="K173" s="4"/>
       <c r="L173" s="4"/>
       <c r="M173" s="4"/>
-    </row>
-    <row r="174" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P173" s="17">
+        <v>0.70833333333333215</v>
+      </c>
+      <c r="Q173" s="17">
+        <v>0.88499999999999934</v>
+      </c>
+      <c r="R173" s="17"/>
+    </row>
+    <row r="174" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A174" s="4"/>
       <c r="B174" s="4"/>
       <c r="C174" s="4"/>
@@ -21915,8 +23134,15 @@
       <c r="K174" s="4"/>
       <c r="L174" s="4"/>
       <c r="M174" s="4"/>
-    </row>
-    <row r="175" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P174" s="17">
+        <v>0.71249999999999891</v>
+      </c>
+      <c r="Q174" s="17">
+        <v>0.88749999999999929</v>
+      </c>
+      <c r="R174" s="17"/>
+    </row>
+    <row r="175" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A175" s="4"/>
       <c r="B175" s="4"/>
       <c r="C175" s="4"/>
@@ -21930,8 +23156,15 @@
       <c r="K175" s="4"/>
       <c r="L175" s="4"/>
       <c r="M175" s="4"/>
-    </row>
-    <row r="176" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P175" s="17">
+        <v>0.71666666666666556</v>
+      </c>
+      <c r="Q175" s="17">
+        <v>0.88999999999999924</v>
+      </c>
+      <c r="R175" s="17"/>
+    </row>
+    <row r="176" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A176" s="4"/>
       <c r="B176" s="4"/>
       <c r="C176" s="4"/>
@@ -21945,8 +23178,15 @@
       <c r="K176" s="4"/>
       <c r="L176" s="4"/>
       <c r="M176" s="4"/>
-    </row>
-    <row r="177" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P176" s="17">
+        <v>0.72083333333333233</v>
+      </c>
+      <c r="Q176" s="17">
+        <v>0.8924999999999994</v>
+      </c>
+      <c r="R176" s="17"/>
+    </row>
+    <row r="177" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A177" s="4"/>
       <c r="B177" s="4"/>
       <c r="C177" s="4"/>
@@ -21960,8 +23200,15 @@
       <c r="K177" s="4"/>
       <c r="L177" s="4"/>
       <c r="M177" s="4"/>
-    </row>
-    <row r="178" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P177" s="17">
+        <v>0.7249999999999992</v>
+      </c>
+      <c r="Q177" s="17">
+        <v>0.89499999999999946</v>
+      </c>
+      <c r="R177" s="17"/>
+    </row>
+    <row r="178" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A178" s="4"/>
       <c r="B178" s="4"/>
       <c r="C178" s="4"/>
@@ -21975,8 +23222,15 @@
       <c r="K178" s="4"/>
       <c r="L178" s="4"/>
       <c r="M178" s="4"/>
-    </row>
-    <row r="179" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P178" s="17">
+        <v>0.72916666666666574</v>
+      </c>
+      <c r="Q178" s="17">
+        <v>0.89749999999999941</v>
+      </c>
+      <c r="R178" s="17"/>
+    </row>
+    <row r="179" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A179" s="4"/>
       <c r="B179" s="4"/>
       <c r="C179" s="4"/>
@@ -21990,8 +23244,15 @@
       <c r="K179" s="4"/>
       <c r="L179" s="4"/>
       <c r="M179" s="4"/>
-    </row>
-    <row r="180" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P179" s="17">
+        <v>0.73333333333333262</v>
+      </c>
+      <c r="Q179" s="17">
+        <v>0.89999999999999958</v>
+      </c>
+      <c r="R179" s="17"/>
+    </row>
+    <row r="180" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A180" s="4"/>
       <c r="B180" s="4"/>
       <c r="C180" s="4"/>
@@ -22005,8 +23266,15 @@
       <c r="K180" s="4"/>
       <c r="L180" s="4"/>
       <c r="M180" s="4"/>
-    </row>
-    <row r="181" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P180" s="17">
+        <v>0.73749999999999927</v>
+      </c>
+      <c r="Q180" s="17">
+        <v>0.90249999999999952</v>
+      </c>
+      <c r="R180" s="17"/>
+    </row>
+    <row r="181" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A181" s="4"/>
       <c r="B181" s="4"/>
       <c r="C181" s="4"/>
@@ -22020,8 +23288,15 @@
       <c r="K181" s="4"/>
       <c r="L181" s="4"/>
       <c r="M181" s="4"/>
-    </row>
-    <row r="182" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P181" s="17">
+        <v>0.74166666666666581</v>
+      </c>
+      <c r="Q181" s="17">
+        <v>0.90499999999999958</v>
+      </c>
+      <c r="R181" s="17"/>
+    </row>
+    <row r="182" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A182" s="4"/>
       <c r="B182" s="4"/>
       <c r="C182" s="4"/>
@@ -22035,8 +23310,15 @@
       <c r="K182" s="4"/>
       <c r="L182" s="4"/>
       <c r="M182" s="4"/>
-    </row>
-    <row r="183" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P182" s="17">
+        <v>0.74583333333333268</v>
+      </c>
+      <c r="Q182" s="17">
+        <v>0.90749999999999953</v>
+      </c>
+      <c r="R182" s="17"/>
+    </row>
+    <row r="183" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A183" s="4"/>
       <c r="B183" s="4"/>
       <c r="C183" s="4"/>
@@ -22050,8 +23332,15 @@
       <c r="K183" s="4"/>
       <c r="L183" s="4"/>
       <c r="M183" s="4"/>
-    </row>
-    <row r="184" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P183" s="17">
+        <v>0.74999999999999944</v>
+      </c>
+      <c r="Q183" s="17">
+        <v>0.9099999999999997</v>
+      </c>
+      <c r="R183" s="17"/>
+    </row>
+    <row r="184" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A184" s="4"/>
       <c r="B184" s="4"/>
       <c r="C184" s="4"/>
@@ -22065,8 +23354,15 @@
       <c r="K184" s="4"/>
       <c r="L184" s="4"/>
       <c r="M184" s="4"/>
-    </row>
-    <row r="185" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P184" s="17">
+        <v>0.7541666666666661</v>
+      </c>
+      <c r="Q184" s="17">
+        <v>0.91249999999999976</v>
+      </c>
+      <c r="R184" s="17"/>
+    </row>
+    <row r="185" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A185" s="4"/>
       <c r="B185" s="4"/>
       <c r="C185" s="4"/>
@@ -22080,8 +23376,15 @@
       <c r="K185" s="4"/>
       <c r="L185" s="4"/>
       <c r="M185" s="4"/>
-    </row>
-    <row r="186" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P185" s="17">
+        <v>0.75833333333333286</v>
+      </c>
+      <c r="Q185" s="17">
+        <v>0.9149999999999997</v>
+      </c>
+      <c r="R185" s="17"/>
+    </row>
+    <row r="186" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A186" s="4"/>
       <c r="B186" s="4"/>
       <c r="C186" s="4"/>
@@ -22095,8 +23398,15 @@
       <c r="K186" s="4"/>
       <c r="L186" s="4"/>
       <c r="M186" s="4"/>
-    </row>
-    <row r="187" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P186" s="17">
+        <v>0.76249999999999962</v>
+      </c>
+      <c r="Q186" s="17">
+        <v>0.91749999999999976</v>
+      </c>
+      <c r="R186" s="17"/>
+    </row>
+    <row r="187" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A187" s="4"/>
       <c r="B187" s="4"/>
       <c r="C187" s="4"/>
@@ -22110,8 +23420,15 @@
       <c r="K187" s="4"/>
       <c r="L187" s="4"/>
       <c r="M187" s="4"/>
-    </row>
-    <row r="188" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P187" s="17">
+        <v>0.76666666666666627</v>
+      </c>
+      <c r="Q187" s="17">
+        <v>0.91999999999999971</v>
+      </c>
+      <c r="R187" s="17"/>
+    </row>
+    <row r="188" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A188" s="4"/>
       <c r="B188" s="4"/>
       <c r="C188" s="4"/>
@@ -22125,8 +23442,15 @@
       <c r="K188" s="4"/>
       <c r="L188" s="4"/>
       <c r="M188" s="4"/>
-    </row>
-    <row r="189" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P188" s="17">
+        <v>0.77083333333333304</v>
+      </c>
+      <c r="Q188" s="17">
+        <v>0.92249999999999988</v>
+      </c>
+      <c r="R188" s="17"/>
+    </row>
+    <row r="189" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A189" s="4"/>
       <c r="B189" s="4"/>
       <c r="C189" s="4"/>
@@ -22140,8 +23464,15 @@
       <c r="K189" s="4"/>
       <c r="L189" s="4"/>
       <c r="M189" s="4"/>
-    </row>
-    <row r="190" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P189" s="17">
+        <v>0.77499999999999991</v>
+      </c>
+      <c r="Q189" s="17">
+        <v>0.92499999999999982</v>
+      </c>
+      <c r="R189" s="17"/>
+    </row>
+    <row r="190" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A190" s="4"/>
       <c r="B190" s="4"/>
       <c r="C190" s="4"/>
@@ -22155,8 +23486,15 @@
       <c r="K190" s="4"/>
       <c r="L190" s="4"/>
       <c r="M190" s="4"/>
-    </row>
-    <row r="191" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P190" s="17">
+        <v>0.77916666666666645</v>
+      </c>
+      <c r="Q190" s="17">
+        <v>0.92749999999999988</v>
+      </c>
+      <c r="R190" s="17"/>
+    </row>
+    <row r="191" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A191" s="4"/>
       <c r="B191" s="4"/>
       <c r="C191" s="4"/>
@@ -22170,8 +23508,15 @@
       <c r="K191" s="4"/>
       <c r="L191" s="4"/>
       <c r="M191" s="4"/>
-    </row>
-    <row r="192" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P191" s="17">
+        <v>0.7833333333333331</v>
+      </c>
+      <c r="Q191" s="17">
+        <v>0.92999999999999983</v>
+      </c>
+      <c r="R191" s="17"/>
+    </row>
+    <row r="192" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A192" s="4"/>
       <c r="B192" s="4"/>
       <c r="C192" s="4"/>
@@ -22185,8 +23530,15 @@
       <c r="K192" s="4"/>
       <c r="L192" s="4"/>
       <c r="M192" s="4"/>
-    </row>
-    <row r="193" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P192" s="17">
+        <v>0.78749999999999998</v>
+      </c>
+      <c r="Q192" s="17">
+        <v>0.9325</v>
+      </c>
+      <c r="R192" s="17"/>
+    </row>
+    <row r="193" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A193" s="4"/>
       <c r="B193" s="4"/>
       <c r="C193" s="4"/>
@@ -22200,8 +23552,15 @@
       <c r="K193" s="4"/>
       <c r="L193" s="4"/>
       <c r="M193" s="4"/>
-    </row>
-    <row r="194" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P193" s="17">
+        <v>0.79166666666666652</v>
+      </c>
+      <c r="Q193" s="17">
+        <v>0.93500000000000005</v>
+      </c>
+      <c r="R193" s="17"/>
+    </row>
+    <row r="194" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A194" s="4"/>
       <c r="B194" s="4"/>
       <c r="C194" s="4"/>
@@ -22215,8 +23574,15 @@
       <c r="K194" s="4"/>
       <c r="L194" s="4"/>
       <c r="M194" s="4"/>
-    </row>
-    <row r="195" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P194" s="17">
+        <v>0.79583333333333339</v>
+      </c>
+      <c r="Q194" s="17">
+        <v>0.9375</v>
+      </c>
+      <c r="R194" s="17"/>
+    </row>
+    <row r="195" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A195" s="4"/>
       <c r="B195" s="4"/>
       <c r="C195" s="4"/>
@@ -22230,8 +23596,15 @@
       <c r="K195" s="4"/>
       <c r="L195" s="4"/>
       <c r="M195" s="4"/>
-    </row>
-    <row r="196" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P195" s="17">
+        <v>0.80000000000000016</v>
+      </c>
+      <c r="Q195" s="17">
+        <v>0.94</v>
+      </c>
+      <c r="R195" s="17"/>
+    </row>
+    <row r="196" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A196" s="4"/>
       <c r="B196" s="4"/>
       <c r="C196" s="4"/>
@@ -22245,8 +23618,15 @@
       <c r="K196" s="4"/>
       <c r="L196" s="4"/>
       <c r="M196" s="4"/>
-    </row>
-    <row r="197" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P196" s="17">
+        <v>0.80416666666666681</v>
+      </c>
+      <c r="Q196" s="17">
+        <v>0.94125000000000003</v>
+      </c>
+      <c r="R196" s="17"/>
+    </row>
+    <row r="197" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A197" s="4"/>
       <c r="B197" s="4"/>
       <c r="C197" s="4"/>
@@ -22260,8 +23640,15 @@
       <c r="K197" s="4"/>
       <c r="L197" s="4"/>
       <c r="M197" s="4"/>
-    </row>
-    <row r="198" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P197" s="17">
+        <v>0.80833333333333357</v>
+      </c>
+      <c r="Q197" s="17">
+        <v>0.9425</v>
+      </c>
+      <c r="R197" s="17"/>
+    </row>
+    <row r="198" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A198" s="4"/>
       <c r="B198" s="4"/>
       <c r="C198" s="4"/>
@@ -22275,8 +23662,15 @@
       <c r="K198" s="4"/>
       <c r="L198" s="4"/>
       <c r="M198" s="4"/>
-    </row>
-    <row r="199" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P198" s="17">
+        <v>0.81250000000000033</v>
+      </c>
+      <c r="Q198" s="17">
+        <v>0.94375000000000009</v>
+      </c>
+      <c r="R198" s="17"/>
+    </row>
+    <row r="199" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A199" s="4"/>
       <c r="B199" s="4"/>
       <c r="C199" s="4"/>
@@ -22290,8 +23684,15 @@
       <c r="K199" s="4"/>
       <c r="L199" s="4"/>
       <c r="M199" s="4"/>
-    </row>
-    <row r="200" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P199" s="17">
+        <v>0.81666666666666698</v>
+      </c>
+      <c r="Q199" s="17">
+        <v>0.94500000000000017</v>
+      </c>
+      <c r="R199" s="17"/>
+    </row>
+    <row r="200" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A200" s="4"/>
       <c r="B200" s="4"/>
       <c r="C200" s="4"/>
@@ -22305,8 +23706,15 @@
       <c r="K200" s="4"/>
       <c r="L200" s="4"/>
       <c r="M200" s="4"/>
-    </row>
-    <row r="201" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P200" s="17">
+        <v>0.82083333333333375</v>
+      </c>
+      <c r="Q200" s="17">
+        <v>0.94625000000000015</v>
+      </c>
+      <c r="R200" s="17"/>
+    </row>
+    <row r="201" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A201" s="4"/>
       <c r="B201" s="4"/>
       <c r="C201" s="4"/>
@@ -22320,8 +23728,15 @@
       <c r="K201" s="4"/>
       <c r="L201" s="4"/>
       <c r="M201" s="4"/>
-    </row>
-    <row r="202" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P201" s="17">
+        <v>0.82500000000000062</v>
+      </c>
+      <c r="Q201" s="17">
+        <v>0.94750000000000012</v>
+      </c>
+      <c r="R201" s="17"/>
+    </row>
+    <row r="202" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A202" s="4"/>
       <c r="B202" s="4"/>
       <c r="C202" s="4"/>
@@ -22335,8 +23750,15 @@
       <c r="K202" s="4"/>
       <c r="L202" s="4"/>
       <c r="M202" s="4"/>
-    </row>
-    <row r="203" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P202" s="17">
+        <v>0.82916666666666716</v>
+      </c>
+      <c r="Q202" s="17">
+        <v>0.94875000000000009</v>
+      </c>
+      <c r="R202" s="17"/>
+    </row>
+    <row r="203" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A203" s="4"/>
       <c r="B203" s="4"/>
       <c r="C203" s="4"/>
@@ -22350,8 +23772,15 @@
       <c r="K203" s="4"/>
       <c r="L203" s="4"/>
       <c r="M203" s="4"/>
-    </row>
-    <row r="204" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P203" s="17">
+        <v>0.83333333333333404</v>
+      </c>
+      <c r="Q203" s="17">
+        <v>0.95000000000000018</v>
+      </c>
+      <c r="R203" s="17"/>
+    </row>
+    <row r="204" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A204" s="4"/>
       <c r="B204" s="4"/>
       <c r="C204" s="4"/>
@@ -22365,8 +23794,15 @@
       <c r="K204" s="4"/>
       <c r="L204" s="4"/>
       <c r="M204" s="4"/>
-    </row>
-    <row r="205" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P204" s="17">
+        <v>0.83750000000000069</v>
+      </c>
+      <c r="Q204" s="17">
+        <v>0.95125000000000026</v>
+      </c>
+      <c r="R204" s="17"/>
+    </row>
+    <row r="205" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A205" s="4"/>
       <c r="B205" s="4"/>
       <c r="C205" s="4"/>
@@ -22380,8 +23816,15 @@
       <c r="K205" s="4"/>
       <c r="L205" s="4"/>
       <c r="M205" s="4"/>
-    </row>
-    <row r="206" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P205" s="17">
+        <v>0.84166666666666723</v>
+      </c>
+      <c r="Q205" s="17">
+        <v>0.95250000000000012</v>
+      </c>
+      <c r="R205" s="17"/>
+    </row>
+    <row r="206" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A206" s="4"/>
       <c r="B206" s="4"/>
       <c r="C206" s="4"/>
@@ -22395,8 +23838,15 @@
       <c r="K206" s="4"/>
       <c r="L206" s="4"/>
       <c r="M206" s="4"/>
-    </row>
-    <row r="207" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P206" s="17">
+        <v>0.8458333333333341</v>
+      </c>
+      <c r="Q206" s="17">
+        <v>0.95375000000000032</v>
+      </c>
+      <c r="R206" s="17"/>
+    </row>
+    <row r="207" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A207" s="4"/>
       <c r="B207" s="4"/>
       <c r="C207" s="4"/>
@@ -22410,8 +23860,15 @@
       <c r="K207" s="4"/>
       <c r="L207" s="4"/>
       <c r="M207" s="4"/>
-    </row>
-    <row r="208" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P207" s="17">
+        <v>0.85000000000000087</v>
+      </c>
+      <c r="Q207" s="17">
+        <v>0.95500000000000029</v>
+      </c>
+      <c r="R207" s="17"/>
+    </row>
+    <row r="208" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A208" s="4"/>
       <c r="B208" s="4"/>
       <c r="C208" s="4"/>
@@ -22425,8 +23882,15 @@
       <c r="K208" s="4"/>
       <c r="L208" s="4"/>
       <c r="M208" s="4"/>
-    </row>
-    <row r="209" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P208" s="17">
+        <v>0.85416666666666752</v>
+      </c>
+      <c r="Q208" s="17">
+        <v>0.95625000000000027</v>
+      </c>
+      <c r="R208" s="17"/>
+    </row>
+    <row r="209" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A209" s="4"/>
       <c r="B209" s="4"/>
       <c r="C209" s="4"/>
@@ -22440,8 +23904,15 @@
       <c r="K209" s="4"/>
       <c r="L209" s="4"/>
       <c r="M209" s="4"/>
-    </row>
-    <row r="210" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P209" s="17">
+        <v>0.85833333333333428</v>
+      </c>
+      <c r="Q209" s="17">
+        <v>0.95750000000000024</v>
+      </c>
+      <c r="R209" s="17"/>
+    </row>
+    <row r="210" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A210" s="4"/>
       <c r="B210" s="4"/>
       <c r="C210" s="4"/>
@@ -22455,8 +23926,15 @@
       <c r="K210" s="4"/>
       <c r="L210" s="4"/>
       <c r="M210" s="4"/>
-    </row>
-    <row r="211" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P210" s="17">
+        <v>0.86250000000000104</v>
+      </c>
+      <c r="Q210" s="17">
+        <v>0.95875000000000032</v>
+      </c>
+      <c r="R210" s="17"/>
+    </row>
+    <row r="211" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A211" s="4"/>
       <c r="B211" s="4"/>
       <c r="C211" s="4"/>
@@ -22470,8 +23948,15 @@
       <c r="K211" s="4"/>
       <c r="L211" s="4"/>
       <c r="M211" s="4"/>
-    </row>
-    <row r="212" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P211" s="17">
+        <v>0.8666666666666677</v>
+      </c>
+      <c r="Q211" s="17">
+        <v>0.9600000000000003</v>
+      </c>
+      <c r="R211" s="17"/>
+    </row>
+    <row r="212" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A212" s="4"/>
       <c r="B212" s="4"/>
       <c r="C212" s="4"/>
@@ -22485,8 +23970,15 @@
       <c r="K212" s="4"/>
       <c r="L212" s="4"/>
       <c r="M212" s="4"/>
-    </row>
-    <row r="213" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P212" s="17">
+        <v>0.87083333333333446</v>
+      </c>
+      <c r="Q212" s="17">
+        <v>0.96125000000000027</v>
+      </c>
+      <c r="R212" s="17"/>
+    </row>
+    <row r="213" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A213" s="4"/>
       <c r="B213" s="4"/>
       <c r="C213" s="4"/>
@@ -22500,8 +23992,15 @@
       <c r="K213" s="4"/>
       <c r="L213" s="4"/>
       <c r="M213" s="4"/>
-    </row>
-    <row r="214" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P213" s="17">
+        <v>0.87500000000000133</v>
+      </c>
+      <c r="Q213" s="17">
+        <v>0.96250000000000047</v>
+      </c>
+      <c r="R213" s="17"/>
+    </row>
+    <row r="214" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A214" s="4"/>
       <c r="B214" s="4"/>
       <c r="C214" s="4"/>
@@ -22515,8 +24014,15 @@
       <c r="K214" s="4"/>
       <c r="L214" s="4"/>
       <c r="M214" s="4"/>
-    </row>
-    <row r="215" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P214" s="17">
+        <v>0.87916666666666787</v>
+      </c>
+      <c r="Q214" s="17">
+        <v>0.96375000000000033</v>
+      </c>
+      <c r="R214" s="17"/>
+    </row>
+    <row r="215" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A215" s="4"/>
       <c r="B215" s="4"/>
       <c r="C215" s="4"/>
@@ -22530,8 +24036,15 @@
       <c r="K215" s="4"/>
       <c r="L215" s="4"/>
       <c r="M215" s="4"/>
-    </row>
-    <row r="216" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P215" s="17">
+        <v>0.88333333333333452</v>
+      </c>
+      <c r="Q215" s="17">
+        <v>0.96500000000000041</v>
+      </c>
+      <c r="R215" s="17"/>
+    </row>
+    <row r="216" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A216" s="4"/>
       <c r="B216" s="4"/>
       <c r="C216" s="4"/>
@@ -22545,8 +24058,15 @@
       <c r="K216" s="4"/>
       <c r="L216" s="4"/>
       <c r="M216" s="4"/>
-    </row>
-    <row r="217" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P216" s="17">
+        <v>0.8875000000000014</v>
+      </c>
+      <c r="Q216" s="17">
+        <v>0.96625000000000039</v>
+      </c>
+      <c r="R216" s="17"/>
+    </row>
+    <row r="217" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A217" s="4"/>
       <c r="B217" s="4"/>
       <c r="C217" s="4"/>
@@ -22560,8 +24080,15 @@
       <c r="K217" s="4"/>
       <c r="L217" s="4"/>
       <c r="M217" s="4"/>
-    </row>
-    <row r="218" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P217" s="17">
+        <v>0.89166666666666794</v>
+      </c>
+      <c r="Q217" s="17">
+        <v>0.96750000000000047</v>
+      </c>
+      <c r="R217" s="17"/>
+    </row>
+    <row r="218" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A218" s="4"/>
       <c r="B218" s="4"/>
       <c r="C218" s="4"/>
@@ -22575,8 +24102,15 @@
       <c r="K218" s="4"/>
       <c r="L218" s="4"/>
       <c r="M218" s="4"/>
-    </row>
-    <row r="219" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P218" s="17">
+        <v>0.89583333333333481</v>
+      </c>
+      <c r="Q218" s="17">
+        <v>0.96875000000000044</v>
+      </c>
+      <c r="R218" s="17"/>
+    </row>
+    <row r="219" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A219" s="4"/>
       <c r="B219" s="4"/>
       <c r="C219" s="4"/>
@@ -22590,8 +24124,15 @@
       <c r="K219" s="4"/>
       <c r="L219" s="4"/>
       <c r="M219" s="4"/>
-    </row>
-    <row r="220" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P219" s="17">
+        <v>0.90000000000000158</v>
+      </c>
+      <c r="Q219" s="17">
+        <v>0.97000000000000042</v>
+      </c>
+      <c r="R219" s="17"/>
+    </row>
+    <row r="220" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A220" s="4"/>
       <c r="B220" s="4"/>
       <c r="C220" s="4"/>
@@ -22605,8 +24146,15 @@
       <c r="K220" s="4"/>
       <c r="L220" s="4"/>
       <c r="M220" s="4"/>
-    </row>
-    <row r="221" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P220" s="17">
+        <v>0.90416666666666823</v>
+      </c>
+      <c r="Q220" s="17">
+        <v>0.97125000000000039</v>
+      </c>
+      <c r="R220" s="17"/>
+    </row>
+    <row r="221" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A221" s="4"/>
       <c r="B221" s="4"/>
       <c r="C221" s="4"/>
@@ -22620,8 +24168,15 @@
       <c r="K221" s="4"/>
       <c r="L221" s="4"/>
       <c r="M221" s="4"/>
-    </row>
-    <row r="222" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P221" s="17">
+        <v>0.90833333333333499</v>
+      </c>
+      <c r="Q221" s="17">
+        <v>0.97250000000000059</v>
+      </c>
+      <c r="R221" s="17"/>
+    </row>
+    <row r="222" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A222" s="4"/>
       <c r="B222" s="4"/>
       <c r="C222" s="4"/>
@@ -22635,8 +24190,15 @@
       <c r="K222" s="4"/>
       <c r="L222" s="4"/>
       <c r="M222" s="4"/>
-    </row>
-    <row r="223" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P222" s="17">
+        <v>0.91250000000000175</v>
+      </c>
+      <c r="Q222" s="17">
+        <v>0.97375000000000056</v>
+      </c>
+      <c r="R222" s="17"/>
+    </row>
+    <row r="223" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A223" s="4"/>
       <c r="B223" s="4"/>
       <c r="C223" s="4"/>
@@ -22650,8 +24212,15 @@
       <c r="K223" s="4"/>
       <c r="L223" s="4"/>
       <c r="M223" s="4"/>
-    </row>
-    <row r="224" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P223" s="17">
+        <v>0.91666666666666841</v>
+      </c>
+      <c r="Q223" s="17">
+        <v>0.97500000000000053</v>
+      </c>
+      <c r="R223" s="17"/>
+    </row>
+    <row r="224" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A224" s="4"/>
       <c r="B224" s="4"/>
       <c r="C224" s="4"/>
@@ -22665,8 +24234,15 @@
       <c r="K224" s="4"/>
       <c r="L224" s="4"/>
       <c r="M224" s="4"/>
-    </row>
-    <row r="225" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P224" s="17">
+        <v>0.92083333333333517</v>
+      </c>
+      <c r="Q224" s="17">
+        <v>0.97625000000000062</v>
+      </c>
+      <c r="R224" s="17"/>
+    </row>
+    <row r="225" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A225" s="4"/>
       <c r="B225" s="4"/>
       <c r="C225" s="4"/>
@@ -22680,8 +24256,15 @@
       <c r="K225" s="4"/>
       <c r="L225" s="4"/>
       <c r="M225" s="4"/>
-    </row>
-    <row r="226" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P225" s="17">
+        <v>0.92500000000000204</v>
+      </c>
+      <c r="Q225" s="17">
+        <v>0.97750000000000059</v>
+      </c>
+      <c r="R225" s="17"/>
+    </row>
+    <row r="226" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A226" s="4"/>
       <c r="B226" s="4"/>
       <c r="C226" s="4"/>
@@ -22695,8 +24278,15 @@
       <c r="K226" s="4"/>
       <c r="L226" s="4"/>
       <c r="M226" s="4"/>
-    </row>
-    <row r="227" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P226" s="17">
+        <v>0.92916666666666858</v>
+      </c>
+      <c r="Q226" s="17">
+        <v>0.97875000000000056</v>
+      </c>
+      <c r="R226" s="17"/>
+    </row>
+    <row r="227" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A227" s="4"/>
       <c r="B227" s="4"/>
       <c r="C227" s="4"/>
@@ -22710,8 +24300,15 @@
       <c r="K227" s="4"/>
       <c r="L227" s="4"/>
       <c r="M227" s="4"/>
-    </row>
-    <row r="228" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P227" s="17">
+        <v>0.93333333333333546</v>
+      </c>
+      <c r="Q227" s="17">
+        <v>0.98000000000000054</v>
+      </c>
+      <c r="R227" s="17"/>
+    </row>
+    <row r="228" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A228" s="4"/>
       <c r="B228" s="4"/>
       <c r="C228" s="4"/>
@@ -22725,8 +24322,15 @@
       <c r="K228" s="4"/>
       <c r="L228" s="4"/>
       <c r="M228" s="4"/>
-    </row>
-    <row r="229" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P228" s="17">
+        <v>0.93750000000000211</v>
+      </c>
+      <c r="Q228" s="17">
+        <v>0.98125000000000062</v>
+      </c>
+      <c r="R228" s="17"/>
+    </row>
+    <row r="229" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A229" s="4"/>
       <c r="B229" s="4"/>
       <c r="C229" s="4"/>
@@ -22740,8 +24344,15 @@
       <c r="K229" s="4"/>
       <c r="L229" s="4"/>
       <c r="M229" s="4"/>
-    </row>
-    <row r="230" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P229" s="17">
+        <v>0.94166666666666865</v>
+      </c>
+      <c r="Q229" s="17">
+        <v>0.9825000000000006</v>
+      </c>
+      <c r="R229" s="17"/>
+    </row>
+    <row r="230" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A230" s="4"/>
       <c r="B230" s="4"/>
       <c r="C230" s="4"/>
@@ -22755,8 +24366,15 @@
       <c r="K230" s="4"/>
       <c r="L230" s="4"/>
       <c r="M230" s="4"/>
-    </row>
-    <row r="231" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P230" s="17">
+        <v>0.94583333333333552</v>
+      </c>
+      <c r="Q230" s="17">
+        <v>0.98375000000000068</v>
+      </c>
+      <c r="R230" s="17"/>
+    </row>
+    <row r="231" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A231" s="4"/>
       <c r="B231" s="4"/>
       <c r="C231" s="4"/>
@@ -22770,8 +24388,15 @@
       <c r="K231" s="4"/>
       <c r="L231" s="4"/>
       <c r="M231" s="4"/>
-    </row>
-    <row r="232" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P231" s="17">
+        <v>0.95000000000000229</v>
+      </c>
+      <c r="Q231" s="17">
+        <v>0.98500000000000076</v>
+      </c>
+      <c r="R231" s="17"/>
+    </row>
+    <row r="232" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A232" s="4"/>
       <c r="B232" s="4"/>
       <c r="C232" s="4"/>
@@ -22785,8 +24410,15 @@
       <c r="K232" s="4"/>
       <c r="L232" s="4"/>
       <c r="M232" s="4"/>
-    </row>
-    <row r="233" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P232" s="17">
+        <v>0.95416666666666894</v>
+      </c>
+      <c r="Q232" s="17">
+        <v>0.98625000000000074</v>
+      </c>
+      <c r="R232" s="17"/>
+    </row>
+    <row r="233" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A233" s="4"/>
       <c r="B233" s="4"/>
       <c r="C233" s="4"/>
@@ -22800,8 +24432,15 @@
       <c r="K233" s="4"/>
       <c r="L233" s="4"/>
       <c r="M233" s="4"/>
-    </row>
-    <row r="234" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P233" s="17">
+        <v>0.9583333333333357</v>
+      </c>
+      <c r="Q233" s="17">
+        <v>0.98750000000000071</v>
+      </c>
+      <c r="R233" s="17"/>
+    </row>
+    <row r="234" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A234" s="4"/>
       <c r="B234" s="4"/>
       <c r="C234" s="4"/>
@@ -22815,8 +24454,15 @@
       <c r="K234" s="4"/>
       <c r="L234" s="4"/>
       <c r="M234" s="4"/>
-    </row>
-    <row r="235" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P234" s="17">
+        <v>0.96250000000000246</v>
+      </c>
+      <c r="Q234" s="17">
+        <v>0.98875000000000068</v>
+      </c>
+      <c r="R234" s="17"/>
+    </row>
+    <row r="235" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A235" s="4"/>
       <c r="B235" s="4"/>
       <c r="C235" s="4"/>
@@ -22830,8 +24476,15 @@
       <c r="K235" s="4"/>
       <c r="L235" s="4"/>
       <c r="M235" s="4"/>
-    </row>
-    <row r="236" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P235" s="17">
+        <v>0.96666666666666912</v>
+      </c>
+      <c r="Q235" s="17">
+        <v>0.99000000000000066</v>
+      </c>
+      <c r="R235" s="17"/>
+    </row>
+    <row r="236" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A236" s="4"/>
       <c r="B236" s="4"/>
       <c r="C236" s="4"/>
@@ -22845,8 +24498,15 @@
       <c r="K236" s="4"/>
       <c r="L236" s="4"/>
       <c r="M236" s="4"/>
-    </row>
-    <row r="237" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P236" s="17">
+        <v>0.97083333333333588</v>
+      </c>
+      <c r="Q236" s="17">
+        <v>0.99125000000000074</v>
+      </c>
+      <c r="R236" s="17"/>
+    </row>
+    <row r="237" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A237" s="4"/>
       <c r="B237" s="4"/>
       <c r="C237" s="4"/>
@@ -22860,8 +24520,15 @@
       <c r="K237" s="4"/>
       <c r="L237" s="4"/>
       <c r="M237" s="4"/>
-    </row>
-    <row r="238" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P237" s="17">
+        <v>0.97500000000000275</v>
+      </c>
+      <c r="Q237" s="17">
+        <v>0.99250000000000083</v>
+      </c>
+      <c r="R237" s="17"/>
+    </row>
+    <row r="238" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A238" s="4"/>
       <c r="B238" s="4"/>
       <c r="C238" s="4"/>
@@ -22875,8 +24542,15 @@
       <c r="K238" s="4"/>
       <c r="L238" s="4"/>
       <c r="M238" s="4"/>
-    </row>
-    <row r="239" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P238" s="17">
+        <v>0.97916666666666929</v>
+      </c>
+      <c r="Q238" s="17">
+        <v>0.9937500000000008</v>
+      </c>
+      <c r="R238" s="17"/>
+    </row>
+    <row r="239" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A239" s="4"/>
       <c r="B239" s="4"/>
       <c r="C239" s="4"/>
@@ -22890,8 +24564,15 @@
       <c r="K239" s="4"/>
       <c r="L239" s="4"/>
       <c r="M239" s="4"/>
-    </row>
-    <row r="240" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P239" s="17">
+        <v>0.98333333333333595</v>
+      </c>
+      <c r="Q239" s="17">
+        <v>0.99500000000000088</v>
+      </c>
+      <c r="R239" s="17"/>
+    </row>
+    <row r="240" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A240" s="4"/>
       <c r="B240" s="4"/>
       <c r="C240" s="4"/>
@@ -22905,8 +24586,15 @@
       <c r="K240" s="4"/>
       <c r="L240" s="4"/>
       <c r="M240" s="4"/>
-    </row>
-    <row r="241" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P240" s="17">
+        <v>0.98750000000000282</v>
+      </c>
+      <c r="Q240" s="17">
+        <v>0.99625000000000086</v>
+      </c>
+      <c r="R240" s="17"/>
+    </row>
+    <row r="241" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A241" s="4"/>
       <c r="B241" s="4"/>
       <c r="C241" s="4"/>
@@ -22920,8 +24608,15 @@
       <c r="K241" s="4"/>
       <c r="L241" s="4"/>
       <c r="M241" s="4"/>
-    </row>
-    <row r="242" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="P241" s="17">
+        <v>0.99166666666666936</v>
+      </c>
+      <c r="Q241" s="17">
+        <v>0.99750000000000083</v>
+      </c>
+      <c r="R241" s="17"/>
+    </row>
+    <row r="242" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A242" s="4"/>
       <c r="B242" s="4"/>
       <c r="C242" s="4"/>
@@ -22935,6 +24630,22 @@
       <c r="K242" s="4"/>
       <c r="L242" s="4"/>
       <c r="M242" s="4"/>
+      <c r="P242" s="17">
+        <v>0.99583333333333623</v>
+      </c>
+      <c r="Q242" s="17">
+        <v>0.9987500000000008</v>
+      </c>
+      <c r="R242" s="17"/>
+    </row>
+    <row r="243" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="P243" s="17">
+        <v>1.0000000000000029</v>
+      </c>
+      <c r="Q243" s="17">
+        <v>1.0000000000000009</v>
+      </c>
+      <c r="R243" s="17"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -23328,26 +25039,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="40414187-dd76-4ef8-b04f-ccddae734140" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="63768118-86e2-4829-8a12-b72c47658d02">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100CCB1C2B958A07241A317F5A881DFD30C" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ec29f518eb9a62149baea9c73f5411cd">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="63768118-86e2-4829-8a12-b72c47658d02" xmlns:ns3="40414187-dd76-4ef8-b04f-ccddae734140" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="29f6242226419d82ce7554acb1ee2c31" ns2:_="" ns3:_="">
     <xsd:import namespace="63768118-86e2-4829-8a12-b72c47658d02"/>
@@ -23602,26 +25293,27 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2A4DA3E6-B8B6-48A6-81EC-CAAD4DEE707B}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="40414187-dd76-4ef8-b04f-ccddae734140"/>
-    <ds:schemaRef ds:uri="63768118-86e2-4829-8a12-b72c47658d02"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{26BC43C4-0DE4-4398-8C07-F13A3433226F}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="40414187-dd76-4ef8-b04f-ccddae734140" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="63768118-86e2-4829-8a12-b72c47658d02">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{124384BF-B442-43EF-BEBD-26F0C03197F3}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -23638,4 +25330,23 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{26BC43C4-0DE4-4398-8C07-F13A3433226F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2A4DA3E6-B8B6-48A6-81EC-CAAD4DEE707B}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="40414187-dd76-4ef8-b04f-ccddae734140"/>
+    <ds:schemaRef ds:uri="63768118-86e2-4829-8a12-b72c47658d02"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>